<commit_message>
Add per-complex Presnensky data and declared lot counts
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Bv8NELxW2W7udnb3XUFGS2
</commit_message>
<xml_diff>
--- a/docs/premium-cao/premium-zhk-cao.xlsx
+++ b/docs/premium-cao/premium-zhk-cao.xlsx
@@ -7141,13 +7141,13 @@
         </is>
       </c>
       <c r="J10" s="3" t="n">
-        <v>5980861</v>
+        <v>4318135</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>5980861</v>
+        <v>6843436</v>
       </c>
       <c r="L10" s="3" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
@@ -8158,7 +8158,7 @@
         <v>2800000</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>5500000</v>
+        <v>4189200</v>
       </c>
       <c r="L25" s="3" t="n">
         <v>16</v>
@@ -8168,10 +8168,14 @@
           <t>бетон</t>
         </is>
       </c>
-      <c r="N25" s="2" t="inlineStr"/>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cian.ru/sale/flat/332401547/</t>
+        </is>
+      </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>таблица заказчика</t>
+          <t>таблица заказчика + Циан 2026-09-07</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
@@ -8451,36 +8455,40 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Клубные резиденции Лёвшинский, 19</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr"/>
+          <t>ЖК «Фрунзенская набережная»</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Sminex</t>
+        </is>
+      </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>2028</t>
+          <t>3 кв. 2027</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Москва, Большой Левшинский, 19</t>
+          <t>Москва, Фрунзенская набережная, 30</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
+          <t>Фрунзенская</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
           <t>Хамовники</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>Хамовники</t>
-        </is>
-      </c>
       <c r="G30" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10-13</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
@@ -8489,23 +8497,27 @@
         </is>
       </c>
       <c r="J30" s="3" t="n">
-        <v>2844930</v>
+        <v>2180740</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>2844930</v>
+        <v>6898288</v>
       </c>
       <c r="L30" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="M30" s="2" t="inlineStr"/>
+        <v>97</v>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>бетон</t>
+        </is>
+      </c>
       <c r="N30" s="2" t="inlineStr">
         <is>
-          <t>https://www.cian.ru/sale/flat/328904518/</t>
+          <t>https://www.cian.ru/sale/flat/333537451/</t>
         </is>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>Циан 2026-09-07</t>
+          <t>таблица заказчика + Циан 2026-09-07</t>
         </is>
       </c>
       <c r="P30" s="2" t="inlineStr"/>
@@ -8513,27 +8525,27 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>ЖК «Фрунзенская набережная»</t>
+          <t>ЖК «Коллекция Лужники»</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Sminex</t>
+          <t>Absolute Premium</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>3 кв. 2027</t>
+          <t>4 кв. 2027</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Москва, Фрунзенская набережная, 30</t>
+          <t>Москва, Лужнецкая набережная</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Фрунзенская</t>
+          <t>Воробьёвы горы</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -8542,11 +8554,11 @@
         </is>
       </c>
       <c r="G31" s="3" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>10-13</t>
+          <t>12-18</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
@@ -8555,13 +8567,13 @@
         </is>
       </c>
       <c r="J31" s="3" t="n">
-        <v>2180740</v>
+        <v>1218182</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>6898288</v>
+        <v>4200000</v>
       </c>
       <c r="L31" s="3" t="n">
-        <v>97</v>
+        <v>59</v>
       </c>
       <c r="M31" s="2" t="inlineStr">
         <is>
@@ -8570,7 +8582,7 @@
       </c>
       <c r="N31" s="2" t="inlineStr">
         <is>
-          <t>https://www.cian.ru/sale/flat/333537451/</t>
+          <t>https://www.cian.ru/sale/flat/333460103/</t>
         </is>
       </c>
       <c r="O31" s="2" t="inlineStr">
@@ -8578,32 +8590,36 @@
           <t>таблица заказчика + Циан 2026-09-07</t>
         </is>
       </c>
-      <c r="P31" s="2" t="inlineStr"/>
+      <c r="P31" s="2" t="inlineStr">
+        <is>
+          <t>пометка «Изучить»</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>ЖК «Коллекция Лужники»</t>
+          <t>ЖК «Узоры»</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Absolute Premium</t>
+          <t>Capital Group</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>4 кв. 2027</t>
+          <t>4 кв. 2028</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Москва, Лужнецкая набережная</t>
+          <t>Москва, 2-й Вражский переулок, 8с2</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Воробьёвы горы</t>
+          <t>Киевская</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -8612,11 +8628,11 @@
         </is>
       </c>
       <c r="G32" s="3" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>12-18</t>
+          <t>9-10</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
@@ -8625,13 +8641,13 @@
         </is>
       </c>
       <c r="J32" s="3" t="n">
-        <v>1218182</v>
+        <v>3177900</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>4200000</v>
+        <v>4559310</v>
       </c>
       <c r="L32" s="3" t="n">
-        <v>59</v>
+        <v>4</v>
       </c>
       <c r="M32" s="2" t="inlineStr">
         <is>
@@ -8640,7 +8656,7 @@
       </c>
       <c r="N32" s="2" t="inlineStr">
         <is>
-          <t>https://www.cian.ru/sale/flat/333460103/</t>
+          <t>https://www.cian.ru/sale/flat/333082541/</t>
         </is>
       </c>
       <c r="O32" s="2" t="inlineStr">
@@ -8650,19 +8666,19 @@
       </c>
       <c r="P32" s="2" t="inlineStr">
         <is>
-          <t>пометка «Изучить»</t>
+          <t>пометка «Изучить! +»; по РБК Компании: старт продаж 2026, стройка начата (котлован)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>ЖК «Узоры»</t>
+          <t>ЖК «Погодинская»</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Capital Group</t>
+          <t>Веспер</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -8672,12 +8688,12 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Москва, 2-й Вражский переулок, 8с2</t>
+          <t>Москва, Погодинская улица</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Киевская</t>
+          <t>Спортивная</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -8690,7 +8706,7 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>9-10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
@@ -8699,13 +8715,13 @@
         </is>
       </c>
       <c r="J33" s="3" t="n">
-        <v>3177900</v>
+        <v>3003600</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>4559310</v>
+        <v>4855100</v>
       </c>
       <c r="L33" s="3" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="M33" s="2" t="inlineStr">
         <is>
@@ -8714,7 +8730,7 @@
       </c>
       <c r="N33" s="2" t="inlineStr">
         <is>
-          <t>https://www.cian.ru/sale/flat/333082541/</t>
+          <t>https://www.cian.ru/sale/flat/332519714/</t>
         </is>
       </c>
       <c r="O33" s="2" t="inlineStr">
@@ -8724,39 +8740,39 @@
       </c>
       <c r="P33" s="2" t="inlineStr">
         <is>
-          <t>пометка «Изучить! +»; по РБК Компании: старт продаж 2026, стройка начата (котлован)</t>
+          <t>РНС получено в ноябре 2025, закрытый старт продаж апрель–май 2026</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>ЖК «Погодинская»</t>
+          <t>ЖК «Дом Дау»</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Веспер</t>
+          <t>1-й Красногвардейский</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>4 кв. 2028</t>
+          <t>2 кв. 2027</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Москва, Погодинская улица</t>
+          <t>Москва, Краснопресненская набережная</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Спортивная</t>
+          <t>Москва-Сити</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Хамовники</t>
+          <t>Сити</t>
         </is>
       </c>
       <c r="G34" s="3" t="n">
@@ -8764,7 +8780,7 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>87</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
@@ -8773,13 +8789,13 @@
         </is>
       </c>
       <c r="J34" s="3" t="n">
-        <v>3003600</v>
+        <v>807900</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>4855100</v>
+        <v>1995800</v>
       </c>
       <c r="L34" s="3" t="n">
-        <v>13</v>
+        <v>295</v>
       </c>
       <c r="M34" s="2" t="inlineStr">
         <is>
@@ -8788,7 +8804,7 @@
       </c>
       <c r="N34" s="2" t="inlineStr">
         <is>
-          <t>https://www.cian.ru/sale/flat/332519714/</t>
+          <t>https://www.cian.ru/sale/flat/331233664/</t>
         </is>
       </c>
       <c r="O34" s="2" t="inlineStr">
@@ -8796,49 +8812,41 @@
           <t>таблица заказчика + Циан 2026-09-07</t>
         </is>
       </c>
-      <c r="P34" s="2" t="inlineStr">
-        <is>
-          <t>РНС получено в ноябре 2025, закрытый старт продаж апрель–май 2026</t>
-        </is>
-      </c>
+      <c r="P34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>ЖК «Дом Дау»</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>1-й КРАСНОГВАРДЕЙСКИЙ</t>
-        </is>
-      </c>
+          <t>Дом 56</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr"/>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>2 кв. 2027</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Москва, Краснопресненская набережная</t>
+          <t>Москва, Фридриха Энгельса, 56</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Москва-Сити</t>
+          <t>Басманный</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Сити</t>
+          <t>Басманный (вне Садового)</t>
         </is>
       </c>
       <c r="G35" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>20-27</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
@@ -8847,23 +8855,23 @@
         </is>
       </c>
       <c r="J35" s="3" t="n">
-        <v>855000</v>
+        <v>609244</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>1184000</v>
+        <v>1043429</v>
       </c>
       <c r="L35" s="3" t="n">
-        <v>232</v>
-      </c>
-      <c r="M35" s="2" t="inlineStr">
-        <is>
-          <t>бетон</t>
-        </is>
-      </c>
-      <c r="N35" s="2" t="inlineStr"/>
+        <v>61</v>
+      </c>
+      <c r="M35" s="2" t="inlineStr"/>
+      <c r="N35" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cian.ru/sale/flat/333461162/</t>
+        </is>
+      </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>таблица заказчика</t>
+          <t>Циан 2026-09-07</t>
         </is>
       </c>
       <c r="P35" s="2" t="inlineStr"/>
@@ -8871,23 +8879,27 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Дом 56</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr"/>
+          <t>ЖК «Новая, 11»</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2029</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Москва, Фридриха Энгельса, 56</t>
+          <t>Москва, улица Новая Дорога, 11Бс1</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Басманный</t>
+          <t>Электрозаводская</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -8896,11 +8908,11 @@
         </is>
       </c>
       <c r="G36" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>20-27</t>
+          <t>9-15</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
@@ -8909,23 +8921,27 @@
         </is>
       </c>
       <c r="J36" s="3" t="n">
-        <v>609244</v>
+        <v>664831</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>1043429</v>
+        <v>1500000</v>
       </c>
       <c r="L36" s="3" t="n">
-        <v>61</v>
-      </c>
-      <c r="M36" s="2" t="inlineStr"/>
+        <v>40</v>
+      </c>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>бетон</t>
+        </is>
+      </c>
       <c r="N36" s="2" t="inlineStr">
         <is>
-          <t>https://www.cian.ru/sale/flat/333461162/</t>
+          <t>https://www.cian.ru/sale/flat/333531308/</t>
         </is>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>Циан 2026-09-07</t>
+          <t>таблица заказчика + Циан 2026-09-07</t>
         </is>
       </c>
       <c r="P36" s="2" t="inlineStr"/>
@@ -8933,32 +8949,28 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>ЖК «Новая, 11»</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>Element</t>
-        </is>
-      </c>
+          <t>Vernissage (Апартаменты премиум-класса) (Вернисаж)</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr"/>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>2029</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Москва, улица Новая Дорога, 11Бс1</t>
+          <t>Москва, Щипок, 26С2</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Электрозаводская</t>
+          <t>Замоскворечье</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Басманный (вне Садового)</t>
+          <t>Замоскворечье (вне Садового)</t>
         </is>
       </c>
       <c r="G37" s="3" t="n">
@@ -8966,36 +8978,32 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>9-15</t>
+          <t>5-8</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>квартиры</t>
+          <t>апартаменты</t>
         </is>
       </c>
       <c r="J37" s="3" t="n">
-        <v>664831</v>
+        <v>696124</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>1500000</v>
+        <v>962085</v>
       </c>
       <c r="L37" s="3" t="n">
-        <v>40</v>
-      </c>
-      <c r="M37" s="2" t="inlineStr">
-        <is>
-          <t>бетон</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="M37" s="2" t="inlineStr"/>
       <c r="N37" s="2" t="inlineStr">
         <is>
-          <t>https://www.cian.ru/sale/flat/333531308/</t>
+          <t>https://www.cian.ru/sale/flat/326325222/</t>
         </is>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>таблица заказчика + Циан 2026-09-07</t>
+          <t>Циан 2026-09-07</t>
         </is>
       </c>
       <c r="P37" s="2" t="inlineStr"/>
@@ -9003,69 +9011,81 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Vernissage (Апартаменты премиум-класса) (Вернисаж)</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr"/>
+          <t>ЖК «Квартал Life Time»</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Sminex</t>
+        </is>
+      </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2 кв. 2026</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Москва, Щипок, 26С2</t>
+          <t>Москва, улица Сергея Макеева</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Замоскворечье</t>
+          <t>1905 года</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Замоскворечье (вне Садового)</t>
+          <t>Пресненский (вне Садового)</t>
         </is>
       </c>
       <c r="G38" s="3" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>5-8</t>
+          <t>9-23</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>апартаменты</t>
+          <t>квартиры</t>
         </is>
       </c>
       <c r="J38" s="3" t="n">
-        <v>696124</v>
+        <v>1019417</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>962085</v>
+        <v>2290000</v>
       </c>
       <c r="L38" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="M38" s="2" t="inlineStr"/>
+        <v>232</v>
+      </c>
+      <c r="M38" s="2" t="inlineStr">
+        <is>
+          <t>бетон</t>
+        </is>
+      </c>
       <c r="N38" s="2" t="inlineStr">
         <is>
-          <t>https://www.cian.ru/sale/flat/326325222/</t>
+          <t>https://www.cian.ru/sale/flat/333570956/</t>
         </is>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>Циан 2026-09-07</t>
-        </is>
-      </c>
-      <c r="P38" s="2" t="inlineStr"/>
+          <t>таблица заказчика + Циан 2026-09-07</t>
+        </is>
+      </c>
+      <c r="P38" s="2" t="inlineStr">
+        <is>
+          <t>по Циан дом сдан</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>ЖК «Квартал Life Time»</t>
+          <t>ЖК «Элитный квартал Тишинский бульвар»</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -9075,17 +9095,17 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>2 кв. 2026</t>
+          <t>2027–2028</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Москва, улица Сергея Макеева</t>
+          <t>Москва, Электрический переулок</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>1905 года</t>
+          <t>Белорусская</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -9094,11 +9114,11 @@
         </is>
       </c>
       <c r="G39" s="3" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>9-23</t>
+          <t>3-14</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
@@ -9107,13 +9127,13 @@
         </is>
       </c>
       <c r="J39" s="3" t="n">
-        <v>1025225</v>
+        <v>1239934</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>1539792</v>
+        <v>3044646</v>
       </c>
       <c r="L39" s="3" t="n">
-        <v>3</v>
+        <v>229</v>
       </c>
       <c r="M39" s="2" t="inlineStr">
         <is>
@@ -9122,7 +9142,7 @@
       </c>
       <c r="N39" s="2" t="inlineStr">
         <is>
-          <t>https://www.cian.ru/sale/flat/333570956/</t>
+          <t>https://www.cian.ru/sale/flat/333476988/</t>
         </is>
       </c>
       <c r="O39" s="2" t="inlineStr">
@@ -9130,36 +9150,32 @@
           <t>таблица заказчика + Циан 2026-09-07</t>
         </is>
       </c>
-      <c r="P39" s="2" t="inlineStr">
-        <is>
-          <t>по Циан дом сдан</t>
-        </is>
-      </c>
+      <c r="P39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>ЖК «Элитный квартал Тишинский бульвар»</t>
+          <t>ЖК «Начало»</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Sminex</t>
+          <t>ДОНСТРОЙ</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>2027–2028</t>
+          <t>2029</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Москва, Электрический переулок</t>
+          <t>Москва, улица Сергея Макеева, 7</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Белорусская</t>
+          <t>Ул. 1905 года</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -9168,11 +9184,11 @@
         </is>
       </c>
       <c r="G40" s="3" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>3-14</t>
+          <t>11-48</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
@@ -9181,36 +9197,44 @@
         </is>
       </c>
       <c r="J40" s="3" t="n">
-        <v>1341000</v>
+        <v>925200</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>3900000</v>
+        <v>1352000</v>
       </c>
       <c r="L40" s="3" t="n">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="M40" s="2" t="inlineStr">
         <is>
           <t>бетон</t>
         </is>
       </c>
-      <c r="N40" s="2" t="inlineStr"/>
+      <c r="N40" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cian.ru/sale/flat/332534047/</t>
+        </is>
+      </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>таблица заказчика</t>
-        </is>
-      </c>
-      <c r="P40" s="2" t="inlineStr"/>
+          <t>таблица заказчика + Циан 2026-09-07</t>
+        </is>
+      </c>
+      <c r="P40" s="2" t="inlineStr">
+        <is>
+          <t>знак вопроса</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>ЖК «Начало»</t>
+          <t>Дом Спорта</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>ДОНСТРОЙ</t>
+          <t>Capital Group</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -9220,12 +9244,12 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Москва, улица Сергея Макеева, 7</t>
+          <t>Москва, Дружинниковская, 18</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Ул. 1905 года</t>
+          <t>Пресненский</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -9234,11 +9258,11 @@
         </is>
       </c>
       <c r="G41" s="3" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>11-48</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
@@ -9247,28 +9271,28 @@
         </is>
       </c>
       <c r="J41" s="3" t="n">
-        <v>975000</v>
+        <v>2281650</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>1900000</v>
+        <v>3174937</v>
       </c>
       <c r="L41" s="3" t="n">
-        <v>204</v>
-      </c>
-      <c r="M41" s="2" t="inlineStr">
-        <is>
-          <t>бетон</t>
-        </is>
-      </c>
-      <c r="N41" s="2" t="inlineStr"/>
+        <v>13</v>
+      </c>
+      <c r="M41" s="2" t="inlineStr"/>
+      <c r="N41" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cian.ru/sale/flat/333577651/</t>
+        </is>
+      </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
-          <t>таблица заказчика</t>
+          <t>Циан 2026-09-07</t>
         </is>
       </c>
       <c r="P41" s="2" t="inlineStr">
         <is>
-          <t>знак вопроса</t>
+          <t>старт продаж 2026, стройка начата (Ведомости)</t>
         </is>
       </c>
     </row>
@@ -9317,23 +9341,27 @@
         </is>
       </c>
       <c r="J42" s="3" t="n">
-        <v>1800000</v>
+        <v>1581360</v>
       </c>
       <c r="K42" s="3" t="n">
         <v>2550000</v>
       </c>
       <c r="L42" s="3" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M42" s="2" t="inlineStr">
         <is>
           <t>бетон</t>
         </is>
       </c>
-      <c r="N42" s="2" t="inlineStr"/>
+      <c r="N42" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cian.ru/sale/flat/331232083/</t>
+        </is>
+      </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
-          <t>таблица заказчика</t>
+          <t>таблица заказчика + Циан 2026-09-07</t>
         </is>
       </c>
       <c r="P42" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Extend planning sheet with developer follow-up research
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Bv8NELxW2W7udnb3XUFGS2
</commit_message>
<xml_diff>
--- a/docs/premium-cao/premium-zhk-cao.xlsx
+++ b/docs/premium-cao/premium-zhk-cao.xlsx
@@ -18,9 +18,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2. Строится'!$A$3:$P$51</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'2. Строится'!$3:$3</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'2. Строится'!$A$1:$P$53</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'3. Проектирование'!$A$3:$Q$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'3. Проектирование'!$A$3:$Q$39</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'3. Проектирование'!$3:$3</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'3. Проектирование'!$A$1:$Q$36</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'3. Проектирование'!$A$1:$Q$41</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -11252,7 +11252,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q36"/>
+  <dimension ref="A1:Q41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -11455,17 +11455,17 @@
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Берниковская набережная, 12</t>
+          <t>Большая Ордынка, 25</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Берниковская наб., 12</t>
+          <t>ул. Большая Ордынка, 25, стр. 1</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Таганский</t>
+          <t>Замоскворечье</t>
         </is>
       </c>
       <c r="D5" s="28" t="inlineStr">
@@ -11473,33 +11473,35 @@
           <t>Садовое кольцо</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>не раскрыт</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>проектирование</t>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Aurix Development (Группа «Эталон»)</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>концепция одобрена ГЗК, подготовка к строительству, старт продаж 2026</t>
         </is>
       </c>
       <c r="G5" s="7" t="n">
-        <v>23000</v>
+        <v>17000</v>
       </c>
       <c r="H5" s="5" t="n"/>
       <c r="I5" s="7" t="n">
-        <v>13</v>
-      </c>
-      <c r="J5" s="7" t="n">
-        <v>166</v>
-      </c>
-      <c r="K5" s="5" t="n"/>
+        <v>8</v>
+      </c>
+      <c r="J5" s="5" t="n"/>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
       <c r="L5" s="5" t="n"/>
       <c r="M5" s="5" t="n"/>
       <c r="N5" s="5" t="n"/>
       <c r="O5" s="4" t="inlineStr">
         <is>
-          <t>kvartiravmoskve.ru (также mskdeluxe.ru/start)</t>
+          <t>официальный сайт проекта (также whitewill.ru)</t>
         </is>
       </c>
       <c r="P5" s="8" t="inlineStr">
@@ -11509,24 +11511,24 @@
       </c>
       <c r="Q5" s="4" t="inlineStr">
         <is>
-          <t>Участок 0,6 га на первой линии Яузы, два корпуса 9–13 этажей, ~23 тыс. м², 166 квартир, «органический неоклассицизм». Делюкс. Застройщик не назван.</t>
+          <t>7 этажей + мансардный уровень, &gt;17 тыс. м², на месте конструктивистской АТС 1927 г. Де-люкс. Одобрение ГЗК упоминает whitewill.ru.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Большая Ордынка, 25</t>
+          <t>Большой Козихинский, 22</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>ул. Большая Ордынка, 25, стр. 1</t>
+          <t>Большой Козихинский пер., 22</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Замоскворечье</t>
+          <t>Пресненский</t>
         </is>
       </c>
       <c r="D6" s="28" t="inlineStr">
@@ -11534,24 +11536,26 @@
           <t>Садовое кольцо</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>Aurix Development (Группа «Эталон»)</t>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>КОЛДИ / Доминанта</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>концепция одобрена ГЗК, подготовка к строительству, старт продаж 2026</t>
+          <t>проект, продажи не начаты</t>
         </is>
       </c>
       <c r="G6" s="7" t="n">
-        <v>17000</v>
+        <v>9377</v>
       </c>
       <c r="H6" s="5" t="n"/>
       <c r="I6" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="J6" s="5" t="n"/>
+        <v>9</v>
+      </c>
+      <c r="J6" s="7" t="n">
+        <v>98</v>
+      </c>
       <c r="K6" s="5" t="inlineStr">
         <is>
           <t>2026</t>
@@ -11560,9 +11564,9 @@
       <c r="L6" s="5" t="n"/>
       <c r="M6" s="5" t="n"/>
       <c r="N6" s="5" t="n"/>
-      <c r="O6" s="4" t="inlineStr">
-        <is>
-          <t>официальный сайт проекта (также whitewill.ru)</t>
+      <c r="O6" s="5" t="inlineStr">
+        <is>
+          <t>novostroev.ru</t>
         </is>
       </c>
       <c r="P6" s="8" t="inlineStr">
@@ -11572,24 +11576,24 @@
       </c>
       <c r="Q6" s="4" t="inlineStr">
         <is>
-          <t>7 этажей + мансардный уровень, &gt;17 тыс. м², на месте конструктивистской АТС 1927 г. Де-люкс. Одобрение ГЗК упоминает whitewill.ru.</t>
+          <t>Патриаршие пруды. Статус «Проект / продажи не начаты» подтверждён novostroev.ru на 01.09.2026; включён в список перспективных стартов делюкс-класса 2026 (novostroev.ru). Официальный сайт kozihinsky22.ru недоступен (403).</t>
         </is>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Большой Козихинский, 22</t>
+          <t>Воздвиженка 7/6</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Большой Козихинский пер., 22</t>
+          <t>ул. Воздвиженка, 7/6</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Пресненский</t>
+          <t>Арбат</t>
         </is>
       </c>
       <c r="D7" s="28" t="inlineStr">
@@ -11597,29 +11601,23 @@
           <t>Садовое кольцо</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>КОЛДИ / Доминанта</t>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>АПРИ (по данным vozdvizhenka7.ru)</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>проект, продажи не начаты</t>
-        </is>
-      </c>
-      <c r="G7" s="7" t="n">
-        <v>9377</v>
-      </c>
+          <t>анонсирован, старт продаж ожидается</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="n"/>
       <c r="H7" s="5" t="n"/>
-      <c r="I7" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="J7" s="7" t="n">
-        <v>98</v>
-      </c>
+      <c r="I7" s="5" t="n"/>
+      <c r="J7" s="5" t="n"/>
       <c r="K7" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2026–2027</t>
         </is>
       </c>
       <c r="L7" s="5" t="n"/>
@@ -11627,7 +11625,7 @@
       <c r="N7" s="5" t="n"/>
       <c r="O7" s="5" t="inlineStr">
         <is>
-          <t>novostroev.ru</t>
+          <t>mskdeluxe.ru</t>
         </is>
       </c>
       <c r="P7" s="8" t="inlineStr">
@@ -11637,24 +11635,24 @@
       </c>
       <c r="Q7" s="4" t="inlineStr">
         <is>
-          <t>Патриаршие пруды. Статус «Проект / продажи не начаты» подтверждён novostroev.ru на 01.09.2026; включён в список перспективных стартов делюкс-класса 2026 (novostroev.ru). Официальный сайт kozihinsky22.ru недоступен (403).</t>
+          <t>Указан в базе делюкс-стартов 2026–2027 mskdeluxe.ru. Агрегаторы описывают как бутик-дом на 10–15 квартир; ранее указывалась сдача 1 кв. 2025 — данные противоречивы, официальный сайт vozdvizhenka7.ru недоступен (503). Требует верификации.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Воздвиженка 7/6</t>
+          <t>Клубные дома на Берниковской набережной, 12 (Sminex)</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>ул. Воздвиженка, 7/6</t>
+          <t>Берниковская набережная, 12, стр. 1 (здание бывшей школы №1685, 1936 г., арх. А. Машинский)</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Арбат</t>
+          <t>Таганский</t>
         </is>
       </c>
       <c r="D8" s="28" t="inlineStr">
@@ -11662,31 +11660,41 @@
           <t>Садовое кольцо</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>АПРИ (по данным vozdvizhenka7.ru)</t>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Sminex</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>анонсирован, старт продаж ожидается</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="n"/>
-      <c r="H8" s="5" t="n"/>
-      <c r="I8" s="5" t="n"/>
-      <c r="J8" s="5" t="n"/>
-      <c r="K8" s="5" t="inlineStr">
-        <is>
-          <t>2026–2027</t>
-        </is>
-      </c>
+          <t>проектирование; предварительная архитектурная концепция (бюро 80/88) опубликована в марте 2026</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="n">
+        <v>23336</v>
+      </c>
+      <c r="H8" s="7" t="n">
+        <v>13000</v>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>9–13 (два корпуса; 9-этажный многосекционный вдоль набережной, 13-этажный в глубине со стороны Берникова переулка)</t>
+        </is>
+      </c>
+      <c r="J8" s="7" t="n">
+        <v>166</v>
+      </c>
+      <c r="K8" s="5" t="n"/>
       <c r="L8" s="5" t="n"/>
       <c r="M8" s="5" t="n"/>
-      <c r="N8" s="5" t="n"/>
-      <c r="O8" s="5" t="inlineStr">
-        <is>
-          <t>mskdeluxe.ru</t>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>2025-03-18</t>
+        </is>
+      </c>
+      <c r="O8" s="4" t="inlineStr">
+        <is>
+          <t>Novostroy-M.ru (пресс-релиз Sminex, 18.03.2025); Москвич Mag (17.03.2026)</t>
         </is>
       </c>
       <c r="P8" s="8" t="inlineStr">
@@ -11696,24 +11704,24 @@
       </c>
       <c r="Q8" s="4" t="inlineStr">
         <is>
-          <t>Указан в базе делюкс-стартов 2026–2027 mskdeluxe.ru. Агрегаторы описывают как бутик-дом на 10–15 квартир; ранее указывалась сдача 1 кв. 2025 — данные противоречивы, официальный сайт vozdvizhenka7.ru недоступен (503). Требует верификации.</t>
+          <t>Участок 0,6 га на первой линии Яузы, два корпуса 9–13 этажей, ~23 тыс. м², 166 квартир, «органический неоклассицизм». Делюкс. Застройщик не назван.; Sminex приобрел площадку в конце 2024 г.; по пресс-релизу — два элитных клубных дома 7–13 этажей, общая площадь 21,4 тыс. м², из них ~13 тыс. м² жилья. По концепции 80/88 (Москвич Mag, https://moskvichmag.ru/gorod/poyavilsya-proekt-mnogosektsionnogo-zhk-na-bernikovskoj-naberezhnoj-na-meste-zakrytoj-shkoly) — 23 336 м², 166 квартир; участок 0,6 га; отмечается, что окончательная реализация именно этого проекта не гарантирована. Агрегатор kvartiravmoskve.ru: стадия «проектирование», монолит-кирпич, подземный паркинг.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Малая Дмитровка, 5/9</t>
+          <t>Клубный дом Duo (Софийская набережная, усадьба Кокорева)</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>ул. Малая Дмитровка, 5/9</t>
+          <t>Софийская набережная (бывшая усадьба Кокорева), напротив Кремля</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Тверской</t>
+          <t>Якиманка</t>
         </is>
       </c>
       <c r="D9" s="28" t="inlineStr">
@@ -11721,35 +11729,37 @@
           <t>Садовое кольцо</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>Группа «Эталон»</t>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>V2 Group (владелец площадки; fee-девелопер Hutton вышел из проекта в июне 2026)</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>анонсирован, старт продаж ожидается в 2026 г.</t>
+          <t>строительство завершается; сдача II кв. 2026, выдача ключей до конца декабря 2026; продано ~27%; ищется новый партнер</t>
         </is>
       </c>
       <c r="G9" s="7" t="n">
-        <v>12000</v>
+        <v>18700</v>
       </c>
       <c r="H9" s="5" t="n"/>
-      <c r="I9" s="7" t="n">
-        <v>9</v>
-      </c>
+      <c r="I9" s="5" t="n"/>
       <c r="J9" s="5" t="n"/>
-      <c r="K9" s="5" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="L9" s="5" t="n"/>
+      <c r="K9" s="5" t="n"/>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t>2026 Q2 (ключи — декабрь 2026)</t>
+        </is>
+      </c>
       <c r="M9" s="5" t="n"/>
-      <c r="N9" s="5" t="n"/>
+      <c r="N9" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
       <c r="O9" s="4" t="inlineStr">
         <is>
-          <t>sosedi.life (также mskdeluxe.ru/start, anwin.ru)</t>
+          <t>Коммерсантъ (17.06.2026)</t>
         </is>
       </c>
       <c r="P9" s="8" t="inlineStr">
@@ -11759,19 +11769,19 @@
       </c>
       <c r="Q9" s="4" t="inlineStr">
         <is>
-          <t>Участок ~0,4 га у сада «Эрмитаж», 2 корпуса 7–9 этажей, волнообразные фасады, делюкс-класс.</t>
+          <t>Не новая очередь Golden Island, а смена управляющего девелопера на Софийской набережной: Hutton (И. Давыдик, А. Антонов) вышел из проекта; собственник V2 Group (В. Фоминых, В. Грознов) купил площадку у MR Group в 2023 за ~4,5–5 млрд руб. Новых очередей «Золотого острова» (Capital Group, ЖК «Золотой») в 2025–2026 не анонсировано.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Малая Никитская, 27</t>
+          <t>Клубный дом «Большая Никитская, 16» (R4S)</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Малая Никитская ул., 27</t>
+          <t>Большая Никитская улица, 16 (реконструкция доходного дома, объект культурного наследия)</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -11784,33 +11794,43 @@
           <t>Садовое кольцо</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>не раскрыт</t>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>R4S Group (генподрядчик — Спецжилремонт)</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>проект на согласовании, старт продаж ожидается</t>
+          <t>реконструкция; старт продаж I кв. 2026; ввод III кв. 2026</t>
         </is>
       </c>
       <c r="G10" s="5" t="n"/>
       <c r="H10" s="5" t="n"/>
-      <c r="I10" s="5" t="n"/>
-      <c r="J10" s="5" t="n"/>
-      <c r="K10" s="5" t="n"/>
-      <c r="L10" s="5" t="n"/>
-      <c r="M10" s="7" t="n">
-        <v>3000000</v>
-      </c>
+      <c r="I10" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="J10" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="K10" s="4" t="inlineStr">
+        <is>
+          <t>2026 Q1 (старт продаж)</t>
+        </is>
+      </c>
+      <c r="L10" s="5" t="inlineStr">
+        <is>
+          <t>2026 Q3</t>
+        </is>
+      </c>
+      <c r="M10" s="5" t="n"/>
       <c r="N10" s="5" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="O10" s="4" t="inlineStr">
         <is>
-          <t>sosedi.life (также moskvichmag.ru, 31.03.2024)</t>
+          <t>Novostroev.ru (19.01.2026); sosedi.life</t>
         </is>
       </c>
       <c r="P10" s="8" t="inlineStr">
@@ -11820,24 +11840,24 @@
       </c>
       <c r="Q10" s="4" t="inlineStr">
         <is>
-          <t>Клубный дом высотой 33 м по проекту бюро WALL на месте двух двухэтажных особняков (бывший отель Club 27). Ориентировочная цена «от ~3 млн руб./м²» — оценка источника, не подтверждена застройщиком. В базе mskdeluxe.ru фигурирует как «Малая Никитская, 29-31».</t>
+          <t>Единственная публичная новинка на Большой Никитской в 2025–2026: 4 квартиры 139,4 / 141,4 / 151 / 234 м². Другие участки на Большой Никитской в открытых анонсах не найдены.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Малая Ордынка, 14/1</t>
+          <t>Клубный дом «Малая Никитская, 27»</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>ул. Малая Ордынка, 14/1</t>
+          <t>Малая Никитская улица, 27 (два двухэтажных особняка 1861 г., бывший «Клуб 27»)</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Замоскворечье</t>
+          <t>Пресненский</t>
         </is>
       </c>
       <c r="D11" s="28" t="inlineStr">
@@ -11845,41 +11865,33 @@
           <t>Садовое кольцо</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>Гута-Девелопмент</t>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>не раскрыт (по данным форума pronovostroy.ru — Mono/ПИК; официально не подтверждено)</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>старт продаж 06.04.2026</t>
-        </is>
-      </c>
-      <c r="G11" s="7" t="n">
-        <v>3000</v>
-      </c>
+          <t>проект на согласовании (высотность 33 м); продажи не открыты</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="n"/>
       <c r="H11" s="5" t="n"/>
-      <c r="I11" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="J11" s="7" t="n">
-        <v>11</v>
-      </c>
-      <c r="K11" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-06</t>
-        </is>
-      </c>
+      <c r="I11" s="5" t="n"/>
+      <c r="J11" s="5" t="n"/>
+      <c r="K11" s="5" t="n"/>
       <c r="L11" s="5" t="n"/>
-      <c r="M11" s="5" t="n"/>
+      <c r="M11" s="7" t="n">
+        <v>3000000</v>
+      </c>
       <c r="N11" s="5" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2024-03-31</t>
         </is>
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
-          <t>sosedi.life (также novostroev.ru обзор делюкс-стартов 2026)</t>
+          <t>Москвич Mag (31.03.2024); sosedi.life (07.04.2026); pronovostroy.ru</t>
         </is>
       </c>
       <c r="P11" s="8" t="inlineStr">
@@ -11889,19 +11901,19 @@
       </c>
       <c r="Q11" s="4" t="inlineStr">
         <is>
-          <t>Участок 0,1 га, 11 квартир, 14 подземных м/м, архитектура A2M. Делюкс.</t>
+          <t>Клубный дом высотой 33 м по проекту бюро WALL на месте двух двухэтажных особняков (бывший отель Club 27). Ориентировочная цена «от ~3 млн руб./м²» — оценка источника, не подтверждена застройщиком. В базе mskdeluxe.ru фигурирует как «Малая Никитская, 29-31».; Архитектура — бюро WALL (ярусные объемы, черно-белые фасады). Существующие здания ~4 000 м² сносятся. Цена ~3 млн руб./м² — предварительное рыночное ожидание (sosedi.life, https://sosedi.life/news/zhk-malaya-nikitskaya-27/), не оферта. Restate.ru (2025–2026) отмечал неопределенность со стартом: возможна продажа площадки вместо запуска.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="24" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Палашёвский 11 (Большой Палашёвский, 11–13/15)</t>
+          <t>Малая Дмитровка, 5/9</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Большой Палашёвский пер., 11–13</t>
+          <t>ул. Малая Дмитровка, 5/9</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -11914,47 +11926,35 @@
           <t>Садовое кольцо</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>Sminex (СЗ «Смайнэкс Палашёвский 11»)</t>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Группа «Эталон»</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>старт продаж без стройки (закрытый старт 22.04.2026)</t>
+          <t>анонсирован, старт продаж ожидается в 2026 г.</t>
         </is>
       </c>
       <c r="G12" s="7" t="n">
-        <v>15600</v>
+        <v>12000</v>
       </c>
       <c r="H12" s="5" t="n"/>
       <c r="I12" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="J12" s="7" t="n">
-        <v>43</v>
-      </c>
+      <c r="J12" s="5" t="n"/>
       <c r="K12" s="5" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
-        </is>
-      </c>
-      <c r="L12" s="5" t="inlineStr">
-        <is>
-          <t>1 кв. 2030</t>
-        </is>
-      </c>
-      <c r="M12" s="7" t="n">
-        <v>3500000</v>
-      </c>
-      <c r="N12" s="5" t="inlineStr">
-        <is>
-          <t>2026-04</t>
-        </is>
-      </c>
-      <c r="O12" s="5" t="inlineStr">
-        <is>
-          <t>novostroev.ru</t>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L12" s="5" t="n"/>
+      <c r="M12" s="5" t="n"/>
+      <c r="N12" s="5" t="n"/>
+      <c r="O12" s="4" t="inlineStr">
+        <is>
+          <t>sosedi.life (также mskdeluxe.ru/start, anwin.ru)</t>
         </is>
       </c>
       <c r="P12" s="8" t="inlineStr">
@@ -11964,24 +11964,24 @@
       </c>
       <c r="Q12" s="4" t="inlineStr">
         <is>
-          <t>Три корпуса 8–9 этажей с контрастными фасадами у Патриарших. Старт продаж 22.04.2026, лоты от 222,4 млн руб. (nngm.ru), от ~3,5 млн руб./м². Сдача 1 кв. 2030 (novostroev.ru, обзор делюкс-стартов 2026).</t>
+          <t>Участок ~0,4 га у сада «Эрмитаж», 2 корпуса 7–9 этажей, волнообразные фасады, делюкс-класс.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="24" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Полянка-3</t>
+          <t>Малая Дмитровка, 5/9 (ожидаемый делюкс-старт)</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>ул. Малая Полянка, 3</t>
+          <t>Малая Дмитровка, 5/9</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Якиманка</t>
+          <t>Тверской</t>
         </is>
       </c>
       <c r="D13" s="28" t="inlineStr">
@@ -11989,35 +11989,27 @@
           <t>Садовое кольцо</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>Aurix Development (Группа «Эталон»)</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>старт продаж 2026</t>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>не раскрыт</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>в списке ожидаемых стартов делюкс-класса 2026 (агрегатор); подробностей нет</t>
         </is>
       </c>
       <c r="G13" s="5" t="n"/>
       <c r="H13" s="5" t="n"/>
-      <c r="I13" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="J13" s="7" t="n">
-        <v>34</v>
-      </c>
-      <c r="K13" s="5" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
+      <c r="I13" s="5" t="n"/>
+      <c r="J13" s="5" t="n"/>
+      <c r="K13" s="5" t="n"/>
       <c r="L13" s="5" t="n"/>
       <c r="M13" s="5" t="n"/>
       <c r="N13" s="5" t="n"/>
       <c r="O13" s="4" t="inlineStr">
         <is>
-          <t>официальный сайт проекта (также mskdeluxe.ru/start)</t>
+          <t>mskdeluxe.ru (список стартов делюкс 2026)</t>
         </is>
       </c>
       <c r="P13" s="8" t="inlineStr">
@@ -12027,24 +12019,24 @@
       </c>
       <c r="Q13" s="4" t="inlineStr">
         <is>
-          <t>9 этажей, 34 квартиры, паркинг на 36 м/м, проект Etalon Project. Продажи открыты в 2026 г.; стадия строительства в открытых источниках не уточнена.</t>
+          <t>Единственное упоминание новой площадки в зоне Петровка/Дмитровка; по Петровке и Большой Дмитровке в 2025–2026 новых анонсов не найдено (только реализуемые «Советник» (Insigma) и Petrovsky).</t>
         </is>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Роден (ранее анонсировался как Veil)</t>
+          <t>Малая Никитская, 29–31 (ожидаемый делюкс-старт)</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Большой Харитоньевский пер., 13А</t>
+          <t>Малая Никитская улица, 29–31</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Басманный</t>
+          <t>Пресненский</t>
         </is>
       </c>
       <c r="D14" s="28" t="inlineStr">
@@ -12054,35 +12046,25 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>MR Group</t>
+          <t>не раскрыт</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>старт продаж июль–август 2026</t>
+          <t>в списке ожидаемых стартов делюкс-класса 2026 (агрегатор); подробностей нет</t>
         </is>
       </c>
       <c r="G14" s="5" t="n"/>
       <c r="H14" s="5" t="n"/>
-      <c r="I14" s="7" t="n">
-        <v>7</v>
-      </c>
+      <c r="I14" s="5" t="n"/>
       <c r="J14" s="5" t="n"/>
-      <c r="K14" s="5" t="inlineStr">
-        <is>
-          <t>2026-07</t>
-        </is>
-      </c>
+      <c r="K14" s="5" t="n"/>
       <c r="L14" s="5" t="n"/>
       <c r="M14" s="5" t="n"/>
-      <c r="N14" s="5" t="inlineStr">
-        <is>
-          <t>2026-07</t>
-        </is>
-      </c>
+      <c r="N14" s="5" t="n"/>
       <c r="O14" s="4" t="inlineStr">
         <is>
-          <t>novostroev.ru (также roden.moscow)</t>
+          <t>mskdeluxe.ru (список стартов делюкс 2026)</t>
         </is>
       </c>
       <c r="P14" s="8" t="inlineStr">
@@ -12092,24 +12074,24 @@
       </c>
       <c r="Q14" s="4" t="inlineStr">
         <is>
-          <t>Клубный дом делюкс-класса у Чистых прудов, 1 монолитный корпус 7 этажей, архитектура WALL. В обзоре делюкс-стартов 2026 novostroev.ru фигурировал как Veil, 9 этажей.</t>
+          <t>В том же списке mskdeluxe.ru: М. Дмитровка 5/9, Льва Толстого 14, Хилков 3, Б. Пироговская 51, Б. Харитоньевский 13, Олсуфьевский 10, Большая Ордынка 25, Воздвиженка 7/6, Малая Полянка 3 — без параметров и девелоперов.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="24" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Рождественка 8</t>
+          <t>Малая Ордынка, 14/1</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>ул. Рождественка / Кузнецкий Мост / Варсонофьевский пер.</t>
+          <t>ул. Малая Ордынка, 14/1</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Мещанский</t>
+          <t>Замоскворечье</t>
         </is>
       </c>
       <c r="D15" s="28" t="inlineStr">
@@ -12117,39 +12099,41 @@
           <t>Садовое кольцо</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>Sminex (проект выкуплен у «Галс-Девелопмент»)</t>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Гута-Девелопмент</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>проект приобретён, старт продаж ожидается</t>
+          <t>старт продаж 06.04.2026</t>
         </is>
       </c>
       <c r="G15" s="7" t="n">
-        <v>36400</v>
-      </c>
-      <c r="H15" s="7" t="n">
-        <v>18000</v>
-      </c>
+        <v>3000</v>
+      </c>
+      <c r="H15" s="5" t="n"/>
       <c r="I15" s="7" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>115</v>
-      </c>
-      <c r="K15" s="5" t="n"/>
+        <v>11</v>
+      </c>
+      <c r="K15" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
       <c r="L15" s="5" t="n"/>
       <c r="M15" s="5" t="n"/>
       <c r="N15" s="5" t="inlineStr">
         <is>
-          <t>2025-12-12</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="O15" s="4" t="inlineStr">
         <is>
-          <t>РИА Недвижимость (также kommersant.ru/doc/8291907, cre.ru)</t>
+          <t>sosedi.life (также novostroev.ru обзор делюкс-стартов 2026)</t>
         </is>
       </c>
       <c r="P15" s="8" t="inlineStr">
@@ -12159,320 +12143,348 @@
       </c>
       <c r="Q15" s="4" t="inlineStr">
         <is>
-          <t>Семь корпусов 2–10 этажей, 115 квартир 61–426 м², таунхаусы и пентхаусы, двор-парк Scape, реставрация особняка конца XIX в. Сделка 12.12.2025.</t>
+          <t>Участок 0,1 га, 11 квартир, 14 подземных м/м, архитектура A2M. Делюкс.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
+          <t>Палашёвский 11 (Большой Палашёвский, 11–13/15)</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Большой Палашёвский пер., 11–13</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Тверской</t>
+        </is>
+      </c>
+      <c r="D16" s="28" t="inlineStr">
+        <is>
+          <t>Садовое кольцо</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Sminex (СЗ «Смайнэкс Палашёвский 11»)</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>старт продаж без стройки (закрытый старт 22.04.2026)</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="n">
+        <v>15600</v>
+      </c>
+      <c r="H16" s="5" t="n"/>
+      <c r="I16" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="J16" s="7" t="n">
+        <v>43</v>
+      </c>
+      <c r="K16" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="L16" s="5" t="inlineStr">
+        <is>
+          <t>1 кв. 2030</t>
+        </is>
+      </c>
+      <c r="M16" s="7" t="n">
+        <v>3500000</v>
+      </c>
+      <c r="N16" s="5" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="O16" s="5" t="inlineStr">
+        <is>
+          <t>novostroev.ru</t>
+        </is>
+      </c>
+      <c r="P16" s="8" t="inlineStr">
+        <is>
+          <t>ссылка</t>
+        </is>
+      </c>
+      <c r="Q16" s="4" t="inlineStr">
+        <is>
+          <t>Три корпуса 8–9 этажей с контрастными фасадами у Патриарших. Старт продаж 22.04.2026, лоты от 222,4 млн руб. (nngm.ru), от ~3,5 млн руб./м². Сдача 1 кв. 2030 (novostroev.ru, обзор делюкс-стартов 2026).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Полянка-3</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>ул. Малая Полянка, 3</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Якиманка</t>
+        </is>
+      </c>
+      <c r="D17" s="28" t="inlineStr">
+        <is>
+          <t>Садовое кольцо</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Aurix Development (Группа «Эталон»)</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>старт продаж 2026</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="n"/>
+      <c r="H17" s="5" t="n"/>
+      <c r="I17" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="J17" s="7" t="n">
+        <v>34</v>
+      </c>
+      <c r="K17" s="5" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L17" s="5" t="n"/>
+      <c r="M17" s="5" t="n"/>
+      <c r="N17" s="5" t="n"/>
+      <c r="O17" s="4" t="inlineStr">
+        <is>
+          <t>официальный сайт проекта (также mskdeluxe.ru/start)</t>
+        </is>
+      </c>
+      <c r="P17" s="8" t="inlineStr">
+        <is>
+          <t>ссылка</t>
+        </is>
+      </c>
+      <c r="Q17" s="4" t="inlineStr">
+        <is>
+          <t>9 этажей, 34 квартиры, паркинг на 36 м/м, проект Etalon Project. Продажи открыты в 2026 г.; стадия строительства в открытых источниках не уточнена.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Роден (ранее анонсировался как Veil)</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Большой Харитоньевский пер., 13А</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Басманный</t>
+        </is>
+      </c>
+      <c r="D18" s="28" t="inlineStr">
+        <is>
+          <t>Садовое кольцо</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>MR Group</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>старт продаж июль–август 2026</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="n"/>
+      <c r="H18" s="5" t="n"/>
+      <c r="I18" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="J18" s="5" t="n"/>
+      <c r="K18" s="5" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="L18" s="5" t="n"/>
+      <c r="M18" s="5" t="n"/>
+      <c r="N18" s="5" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="O18" s="4" t="inlineStr">
+        <is>
+          <t>novostroev.ru (также roden.moscow)</t>
+        </is>
+      </c>
+      <c r="P18" s="8" t="inlineStr">
+        <is>
+          <t>ссылка</t>
+        </is>
+      </c>
+      <c r="Q18" s="4" t="inlineStr">
+        <is>
+          <t>Клубный дом делюкс-класса у Чистых прудов, 1 монолитный корпус 7 этажей, архитектура WALL. В обзоре делюкс-стартов 2026 novostroev.ru фигурировал как Veil, 9 этажей.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Рождественка 8</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>ул. Рождественка / Кузнецкий Мост / Варсонофьевский пер.</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Мещанский</t>
+        </is>
+      </c>
+      <c r="D19" s="28" t="inlineStr">
+        <is>
+          <t>Садовое кольцо</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Sminex (проект выкуплен у «Галс-Девелопмент»)</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>проект приобретён, старт продаж ожидается</t>
+        </is>
+      </c>
+      <c r="G19" s="7" t="n">
+        <v>36400</v>
+      </c>
+      <c r="H19" s="7" t="n">
+        <v>18000</v>
+      </c>
+      <c r="I19" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="J19" s="7" t="n">
+        <v>115</v>
+      </c>
+      <c r="K19" s="5" t="n"/>
+      <c r="L19" s="5" t="n"/>
+      <c r="M19" s="5" t="n"/>
+      <c r="N19" s="5" t="inlineStr">
+        <is>
+          <t>2025-12-12</t>
+        </is>
+      </c>
+      <c r="O19" s="4" t="inlineStr">
+        <is>
+          <t>РИА Недвижимость (также kommersant.ru/doc/8291907, cre.ru)</t>
+        </is>
+      </c>
+      <c r="P19" s="8" t="inlineStr">
+        <is>
+          <t>ссылка</t>
+        </is>
+      </c>
+      <c r="Q19" s="4" t="inlineStr">
+        <is>
+          <t>Семь корпусов 2–10 этажей, 115 квартир 61–426 м², таунхаусы и пентхаусы, двор-парк Scape, реставрация особняка конца XIX в. Сделка 12.12.2025.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="24" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
           <t>Типография Сытина (Пятницкая, 71/5)</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>ул. Пятницкая, 71/5 (2-й Монетчиковский пер., 5)</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C20" s="5" t="inlineStr">
         <is>
           <t>Замоскворечье</t>
         </is>
       </c>
-      <c r="D16" s="28" t="inlineStr">
+      <c r="D20" s="28" t="inlineStr">
         <is>
           <t>Садовое кольцо</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr">
+      <c r="E20" s="5" t="inlineStr">
         <is>
           <t>Sminex</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr">
+      <c r="F20" s="4" t="inlineStr">
         <is>
           <t>участок приобретён (март 2026), проектирование</t>
         </is>
       </c>
-      <c r="G16" s="5" t="n"/>
-      <c r="H16" s="5" t="n"/>
-      <c r="I16" s="5" t="n"/>
-      <c r="J16" s="5" t="n"/>
-      <c r="K16" s="5" t="n"/>
-      <c r="L16" s="5" t="n"/>
-      <c r="M16" s="5" t="n"/>
-      <c r="N16" s="5" t="inlineStr">
+      <c r="G20" s="5" t="n"/>
+      <c r="H20" s="5" t="n"/>
+      <c r="I20" s="5" t="n"/>
+      <c r="J20" s="5" t="n"/>
+      <c r="K20" s="5" t="n"/>
+      <c r="L20" s="5" t="n"/>
+      <c r="M20" s="5" t="n"/>
+      <c r="N20" s="5" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
       </c>
-      <c r="O16" s="4" t="inlineStr">
+      <c r="O20" s="4" t="inlineStr">
         <is>
           <t>РИА Недвижимость (также sminex.com, mperspektiva.ru)</t>
         </is>
       </c>
-      <c r="P16" s="8" t="inlineStr">
-        <is>
-          <t>ссылка</t>
-        </is>
-      </c>
-      <c r="Q16" s="4" t="inlineStr">
+      <c r="P20" s="8" t="inlineStr">
+        <is>
+          <t>ссылка</t>
+        </is>
+      </c>
+      <c r="Q20" s="4" t="inlineStr">
         <is>
           <t>Участок 1,8 га, 8 зданий 38,5 тыс. м², в т.ч. 3 корпуса типографии Сытина (ОКН, арх. Эрихсон/Шухов). Продавец — В. Погребенко, оценка сделки 12–14 млрд руб., инвестиции 25–30 млрд руб. План: реставрация + новые элитные клубные дома. Участок у Садового кольца (Валовая ул.).</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="24" customHeight="1">
-      <c r="A17" s="9" t="inlineStr">
-        <is>
-          <t>Большая Пироговская, 51 (общежития Института красной профессуры)</t>
-        </is>
-      </c>
-      <c r="B17" s="9" t="inlineStr">
-        <is>
-          <t>ул. Большая Пироговская, 51</t>
-        </is>
-      </c>
-      <c r="C17" s="10" t="inlineStr">
-        <is>
-          <t>Хамовники</t>
-        </is>
-      </c>
-      <c r="D17" s="29" t="inlineStr">
-        <is>
-          <t>Хамовники</t>
-        </is>
-      </c>
-      <c r="E17" s="9" t="inlineStr">
-        <is>
-          <t>Vesper (fee-девелопер) / собственник Capital Group</t>
-        </is>
-      </c>
-      <c r="F17" s="9" t="inlineStr">
-        <is>
-          <t>анонсирован (fee-development), концепция</t>
-        </is>
-      </c>
-      <c r="G17" s="12" t="n">
-        <v>46700</v>
-      </c>
-      <c r="H17" s="10" t="n"/>
-      <c r="I17" s="10" t="n"/>
-      <c r="J17" s="10" t="n"/>
-      <c r="K17" s="10" t="n"/>
-      <c r="L17" s="10" t="n"/>
-      <c r="M17" s="10" t="n"/>
-      <c r="N17" s="10" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-      <c r="O17" s="9" t="inlineStr">
-        <is>
-          <t>РИА Недвижимость (также vedomosti.ru 18.06.2026)</t>
-        </is>
-      </c>
-      <c r="P17" s="13" t="inlineStr">
-        <is>
-          <t>ссылка</t>
-        </is>
-      </c>
-      <c r="Q17" s="9" t="inlineStr">
-        <is>
-          <t>Участок 1,5 га, ансамбль восьми 6-этажных корпусов 1929–32 гг. (арх. Осипов, Рухлядев; статус памятника утрачен в 2000-х). Планируемая площадь выросла с 39 до 46,7 тыс. м². Vesper — концепция, продукт и управление реализацией. В базе mskdeluxe.ru — «Б.Пироговская, 51».</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="24" customHeight="1">
-      <c r="A18" s="9" t="inlineStr">
-        <is>
-          <t>Земледельческий, 15</t>
-        </is>
-      </c>
-      <c r="B18" s="9" t="inlineStr">
-        <is>
-          <t>Земледельческий пер., 15</t>
-        </is>
-      </c>
-      <c r="C18" s="10" t="inlineStr">
-        <is>
-          <t>Хамовники</t>
-        </is>
-      </c>
-      <c r="D18" s="29" t="inlineStr">
-        <is>
-          <t>Хамовники</t>
-        </is>
-      </c>
-      <c r="E18" s="10" t="inlineStr">
-        <is>
-          <t>не раскрыт</t>
-        </is>
-      </c>
-      <c r="F18" s="10" t="inlineStr">
-        <is>
-          <t>проектирование</t>
-        </is>
-      </c>
-      <c r="G18" s="12" t="n">
-        <v>8000</v>
-      </c>
-      <c r="H18" s="10" t="n"/>
-      <c r="I18" s="10" t="n"/>
-      <c r="J18" s="12" t="n">
-        <v>77</v>
-      </c>
-      <c r="K18" s="10" t="inlineStr">
-        <is>
-          <t>2026–2027</t>
-        </is>
-      </c>
-      <c r="L18" s="10" t="n"/>
-      <c r="M18" s="10" t="n"/>
-      <c r="N18" s="10" t="n"/>
-      <c r="O18" s="9" t="inlineStr">
-        <is>
-          <t>kvartiravmoskve.ru (также mskdeluxe.ru/start)</t>
-        </is>
-      </c>
-      <c r="P18" s="13" t="inlineStr">
-        <is>
-          <t>ссылка</t>
-        </is>
-      </c>
-      <c r="Q18" s="9" t="inlineStr">
-        <is>
-          <t>Участок 0,3 га (сейчас административное здание 1975 г., 5 эт., 5,7 тыс. м²), клубный дом ~8 тыс. м², 77 квартир, коммерция, подземный паркинг. Делюкс.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="24" customHeight="1">
-      <c r="A19" s="9" t="inlineStr">
-        <is>
-          <t>Квартал на Савинской набережной («Московский шёлк»)</t>
-        </is>
-      </c>
-      <c r="B19" s="9" t="inlineStr">
-        <is>
-          <t>Савинская наб. (территория БЦ «Московский шёлк»)</t>
-        </is>
-      </c>
-      <c r="C19" s="10" t="inlineStr">
-        <is>
-          <t>Хамовники</t>
-        </is>
-      </c>
-      <c r="D19" s="29" t="inlineStr">
-        <is>
-          <t>Хамовники</t>
-        </is>
-      </c>
-      <c r="E19" s="10" t="inlineStr">
-        <is>
-          <t>Sminex</t>
-        </is>
-      </c>
-      <c r="F19" s="10" t="inlineStr">
-        <is>
-          <t>проектирование</t>
-        </is>
-      </c>
-      <c r="G19" s="12" t="n">
-        <v>125000</v>
-      </c>
-      <c r="H19" s="10" t="n"/>
-      <c r="I19" s="10" t="n"/>
-      <c r="J19" s="10" t="n"/>
-      <c r="K19" s="10" t="n"/>
-      <c r="L19" s="10" t="n"/>
-      <c r="M19" s="10" t="n"/>
-      <c r="N19" s="10" t="inlineStr">
-        <is>
-          <t>2024-03-12</t>
-        </is>
-      </c>
-      <c r="O19" s="9" t="inlineStr">
-        <is>
-          <t>РИА Недвижимость (стадия подтверждена mperspektiva.ru 18.12.2025)</t>
-        </is>
-      </c>
-      <c r="P19" s="13" t="inlineStr">
-        <is>
-          <t>ссылка</t>
-        </is>
-      </c>
-      <c r="Q19" s="9" t="inlineStr">
-        <is>
-          <t>ЖК ~125 тыс. м² на территории делового квартала «Московский шёлк». По данным Sminex на декабрь 2025 г. находится в стадии проектирования (вместе с Лужнецкой).</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="24" customHeight="1">
-      <c r="A20" s="9" t="inlineStr">
-        <is>
-          <t>Курсовой, 15</t>
-        </is>
-      </c>
-      <c r="B20" s="9" t="inlineStr">
-        <is>
-          <t>Курсовой пер., 15 (Остоженка)</t>
-        </is>
-      </c>
-      <c r="C20" s="10" t="inlineStr">
-        <is>
-          <t>Хамовники</t>
-        </is>
-      </c>
-      <c r="D20" s="29" t="inlineStr">
-        <is>
-          <t>Хамовники</t>
-        </is>
-      </c>
-      <c r="E20" s="9" t="inlineStr">
-        <is>
-          <t>не раскрыт (проект бюро Дмитрия Великовского)</t>
-        </is>
-      </c>
-      <c r="F20" s="9" t="inlineStr">
-        <is>
-          <t>анонсирован, старт продаж ожидается</t>
-        </is>
-      </c>
-      <c r="G20" s="10" t="n"/>
-      <c r="H20" s="10" t="n"/>
-      <c r="I20" s="12" t="n">
-        <v>6</v>
-      </c>
-      <c r="J20" s="10" t="n"/>
-      <c r="K20" s="10" t="n"/>
-      <c r="L20" s="10" t="n"/>
-      <c r="M20" s="10" t="n"/>
-      <c r="N20" s="10" t="n"/>
-      <c r="O20" s="10" t="inlineStr">
-        <is>
-          <t>anwin.ru</t>
-        </is>
-      </c>
-      <c r="P20" s="13" t="inlineStr">
-        <is>
-          <t>ссылка</t>
-        </is>
-      </c>
-      <c r="Q20" s="9" t="inlineStr">
-        <is>
-          <t>«Золотая миля», 6 этажей, камерный клубный дом. Подробные параметры и застройщик в открытых источниках не раскрыты.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="24" customHeight="1">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>Льва Толстого, 14–16 (три клубных дома Sminex)</t>
+          <t>Большая Пироговская, 51 (общежития Института красной профессуры)</t>
         </is>
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>ул. Льва Толстого, 14</t>
+          <t>ул. Большая Пироговская, 51</t>
         </is>
       </c>
       <c r="C21" s="10" t="inlineStr">
@@ -12485,22 +12497,20 @@
           <t>Хамовники</t>
         </is>
       </c>
-      <c r="E21" s="10" t="inlineStr">
-        <is>
-          <t>Sminex</t>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>Vesper (fee-девелопер) / собственник Capital Group</t>
         </is>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
-          <t>участок приобретён (декабрь 2025), концепция в финальной стадии, старт продаж не объявлен</t>
+          <t>анонсирован (fee-development), концепция</t>
         </is>
       </c>
       <c r="G21" s="12" t="n">
-        <v>20300</v>
-      </c>
-      <c r="H21" s="12" t="n">
-        <v>12400</v>
-      </c>
+        <v>46700</v>
+      </c>
+      <c r="H21" s="10" t="n"/>
       <c r="I21" s="10" t="n"/>
       <c r="J21" s="10" t="n"/>
       <c r="K21" s="10" t="n"/>
@@ -12508,12 +12518,12 @@
       <c r="M21" s="10" t="n"/>
       <c r="N21" s="10" t="inlineStr">
         <is>
-          <t>2025-12-18</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="O21" s="9" t="inlineStr">
         <is>
-          <t>Московская перспектива (также rbc.ru 18.12.2025, sosedi.life 07.04.2026)</t>
+          <t>РИА Недвижимость (также vedomosti.ru 18.06.2026)</t>
         </is>
       </c>
       <c r="P21" s="13" t="inlineStr">
@@ -12523,19 +12533,19 @@
       </c>
       <c r="Q21" s="9" t="inlineStr">
         <is>
-          <t>Участок ~0,6 га у делового квартала «Красная Роза», куплен у структур А. Клячина. Три камерных клубных дома, надземная площадь 20,3 тыс. м², квартиры 12,4 тыс. м². Сохраняется фасад бывшего доходного дома Трындина-Жиро.</t>
+          <t>Участок 1,5 га, ансамбль восьми 6-этажных корпусов 1929–32 гг. (арх. Осипов, Рухлядев; статус памятника утрачен в 2000-х). Планируемая площадь выросла с 39 до 46,7 тыс. м². Vesper — концепция, продукт и управление реализацией. В базе mskdeluxe.ru — «Б.Пироговская, 51».</t>
         </is>
       </c>
     </row>
     <row r="22" ht="24" customHeight="1">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>Лёвшинский, 19</t>
+          <t>Квартал на Савинской набережной («Московский шёлк»)</t>
         </is>
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>Большой Лёвшинский пер., 19</t>
+          <t>Савинская наб. (территория БЦ «Московский шёлк»)</t>
         </is>
       </c>
       <c r="C22" s="10" t="inlineStr">
@@ -12548,39 +12558,33 @@
           <t>Хамовники</t>
         </is>
       </c>
-      <c r="E22" s="9" t="inlineStr">
-        <is>
-          <t>ТСИ Девелопмент (ГК «Трансстройинвест»)</t>
-        </is>
-      </c>
-      <c r="F22" s="9" t="inlineStr">
-        <is>
-          <t>старт бронирования, старт продаж</t>
-        </is>
-      </c>
-      <c r="G22" s="10" t="n"/>
+      <c r="E22" s="10" t="inlineStr">
+        <is>
+          <t>Sminex</t>
+        </is>
+      </c>
+      <c r="F22" s="10" t="inlineStr">
+        <is>
+          <t>проектирование</t>
+        </is>
+      </c>
+      <c r="G22" s="12" t="n">
+        <v>125000</v>
+      </c>
       <c r="H22" s="10" t="n"/>
-      <c r="I22" s="12" t="n">
-        <v>8</v>
-      </c>
-      <c r="J22" s="12" t="n">
-        <v>16</v>
-      </c>
-      <c r="K22" s="10" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="L22" s="10" t="inlineStr">
-        <is>
-          <t>2 кв. 2028</t>
-        </is>
-      </c>
+      <c r="I22" s="10" t="n"/>
+      <c r="J22" s="10" t="n"/>
+      <c r="K22" s="10" t="n"/>
+      <c r="L22" s="10" t="n"/>
       <c r="M22" s="10" t="n"/>
-      <c r="N22" s="10" t="n"/>
+      <c r="N22" s="10" t="inlineStr">
+        <is>
+          <t>2024-03-12</t>
+        </is>
+      </c>
       <c r="O22" s="9" t="inlineStr">
         <is>
-          <t>whitewill.ru (также tehne.com, levshinsky-19.ru)</t>
+          <t>РИА Недвижимость (стадия подтверждена mperspektiva.ru 18.12.2025)</t>
         </is>
       </c>
       <c r="P22" s="13" t="inlineStr">
@@ -12590,19 +12594,19 @@
       </c>
       <c r="Q22" s="9" t="inlineStr">
         <is>
-          <t>Воссоздание фасада доходного дома Духовских (1904, арх. Мейснер), проект HADAA Architects. 16 резиденций 70–239 м², паркинг 18 м/м. Цена от 197,12 млн руб. за лот. Стадия стройки в источниках не подтверждена.</t>
+          <t>ЖК ~125 тыс. м² на территории делового квартала «Московский шёлк». По данным Sminex на декабрь 2025 г. находится в стадии проектирования (вместе с Лужнецкой).</t>
         </is>
       </c>
     </row>
     <row r="23" ht="24" customHeight="1">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>Олсуфьевский 10</t>
+          <t>Клубный дом «Земледельческий, 15»</t>
         </is>
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>Олсуфьевский пер., 10</t>
+          <t>Земледельческий переулок, 15 (на месте административного здания 1975 г., 5 этажей, 5 744 м²)</t>
         </is>
       </c>
       <c r="C23" s="10" t="inlineStr">
@@ -12617,20 +12621,22 @@
       </c>
       <c r="E23" s="10" t="inlineStr">
         <is>
-          <t>Грандор (Grandor)</t>
+          <t>не раскрыт</t>
         </is>
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
-          <t>ГПЗУ получен (апрель 2021), старт продаж ожидается</t>
-        </is>
-      </c>
-      <c r="G23" s="10" t="n"/>
+          <t>проектирование (агрегаторы; в списке ожидаемых стартов делюкс-класса 2026 на mskdeluxe.ru)</t>
+        </is>
+      </c>
+      <c r="G23" s="12" t="n">
+        <v>8000</v>
+      </c>
       <c r="H23" s="10" t="n"/>
-      <c r="I23" s="12" t="n">
-        <v>8</v>
-      </c>
-      <c r="J23" s="10" t="n"/>
+      <c r="I23" s="10" t="n"/>
+      <c r="J23" s="12" t="n">
+        <v>77</v>
+      </c>
       <c r="K23" s="10" t="inlineStr">
         <is>
           <t>2026–2027</t>
@@ -12638,10 +12644,14 @@
       </c>
       <c r="L23" s="10" t="n"/>
       <c r="M23" s="10" t="n"/>
-      <c r="N23" s="10" t="n"/>
+      <c r="N23" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
       <c r="O23" s="9" t="inlineStr">
         <is>
-          <t>официальный сайт проекта (также novostroy.ru, mskdeluxe.ru/start)</t>
+          <t>kvartiravmoskve.ru (обновлено 21.06.2026); mskdeluxe.ru/start</t>
         </is>
       </c>
       <c r="P23" s="13" t="inlineStr">
@@ -12651,60 +12661,54 @@
       </c>
       <c r="Q23" s="9" t="inlineStr">
         <is>
-          <t>Участок 0,4 га, семь корпусов 5–8 этажей в индивидуальной архитектуре. В базе делюкс-стартов 2026–2027 mskdeluxe.ru.</t>
+          <t>Участок 0,3 га (сейчас административное здание 1975 г., 5 эт., 5,7 тыс. м²), клубный дом ~8 тыс. м², 77 квартир, коммерция, подземный паркинг. Делюкс.; Участок 0,3 га; делюкс; 77 квартир + коммерческая часть; подземный паркинг; монолит-кирпич; 1 км до м. Смоленская. Сделок по продаже БЦ и решений Москомархитектуры в открытых источниках не найдено.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="24" customHeight="1">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>Премиальный квартал на Лужнецкой набережной, 10А</t>
+          <t>Клубный дом на Курсовом переулке, 15 (проект бюро Дмитрия Великовского)</t>
         </is>
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>Лужнецкая наб., вл. 10А</t>
-        </is>
-      </c>
-      <c r="C24" s="10" t="inlineStr">
+          <t>Курсовой переулок, 15</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>Хамовники (Остоженка)</t>
+        </is>
+      </c>
+      <c r="D24" s="29" t="inlineStr">
         <is>
           <t>Хамовники</t>
         </is>
       </c>
-      <c r="D24" s="29" t="inlineStr">
-        <is>
-          <t>Хамовники</t>
-        </is>
-      </c>
-      <c r="E24" s="10" t="inlineStr">
-        <is>
-          <t>Sminex</t>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
+          <t>не раскрыт (проект бюро Дмитрия Великовского)</t>
         </is>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
-          <t>проект утверждён (АГР, май 2026), начало строительства 2027</t>
+          <t>проект / предстарт; в открытых источниках только страница агрегатора</t>
         </is>
       </c>
       <c r="G24" s="10" t="n"/>
       <c r="H24" s="10" t="n"/>
-      <c r="I24" s="10" t="n"/>
+      <c r="I24" s="12" t="n">
+        <v>6</v>
+      </c>
       <c r="J24" s="10" t="n"/>
-      <c r="K24" s="10" t="inlineStr">
-        <is>
-          <t>2027 (стройка)</t>
-        </is>
-      </c>
+      <c r="K24" s="10" t="n"/>
       <c r="L24" s="10" t="n"/>
       <c r="M24" s="10" t="n"/>
-      <c r="N24" s="10" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
+      <c r="N24" s="10" t="n"/>
       <c r="O24" s="9" t="inlineStr">
         <is>
-          <t>РИА Недвижимость (также anwin.ru)</t>
+          <t>Anwin (агрегатор элитной недвижимости)</t>
         </is>
       </c>
       <c r="P24" s="13" t="inlineStr">
@@ -12714,19 +12718,19 @@
       </c>
       <c r="Q24" s="9" t="inlineStr">
         <is>
-          <t>Два жилых корпуса переменной этажности в неоклассике + эллиптический БЦ 26 тыс. м² («яйцо Фаберже»). Концепция согласована Департаментом градостроительной политики (В. Овчинский). Параметры жилой части не раскрыты.</t>
+          <t>«Золотая миля», 6 этажей, камерный клубный дом. Подробные параметры и застройщик в открытых источниках не раскрыты.; По описанию агрегатора: 6-этажный дом по проекту бюро Дмитрия Великовского, панорамное остекление, локация «Золотой мили» рядом с Зачатьевским монастырем. Сейчас по адресу — детский клуб-студия «Пречистенские ворота». Пресса (Коммерсант, РБК, Ведомости, Москвич Mag) и Москомархитектура публикаций по площадке не имеют; девелопер и параметры не подтверждены.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="24" customHeight="1">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t>Тимура Фрунзе, 11 (клубный дом Sminex)</t>
+          <t>Льва Толстого, 14–16 (три клубных дома Sminex)</t>
         </is>
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>ул. Тимура Фрунзе, 11, стр. 7, 19, 33, 50</t>
+          <t>ул. Льва Толстого, 14</t>
         </is>
       </c>
       <c r="C25" s="10" t="inlineStr">
@@ -12746,14 +12750,14 @@
       </c>
       <c r="F25" s="9" t="inlineStr">
         <is>
-          <t>участок приобретён (апрель 2026), проектирование</t>
+          <t>участок приобретён (декабрь 2025), концепция в финальной стадии, старт продаж не объявлен</t>
         </is>
       </c>
       <c r="G25" s="12" t="n">
-        <v>13000</v>
+        <v>20300</v>
       </c>
       <c r="H25" s="12" t="n">
-        <v>8200</v>
+        <v>12400</v>
       </c>
       <c r="I25" s="10" t="n"/>
       <c r="J25" s="10" t="n"/>
@@ -12762,12 +12766,12 @@
       <c r="M25" s="10" t="n"/>
       <c r="N25" s="10" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2025-12-18</t>
         </is>
       </c>
       <c r="O25" s="9" t="inlineStr">
         <is>
-          <t>РИА Недвижимость (также sminex.com, interfax-russia.ru)</t>
+          <t>Московская перспектива (также rbc.ru 18.12.2025, sosedi.life 07.04.2026)</t>
         </is>
       </c>
       <c r="P25" s="13" t="inlineStr">
@@ -12777,19 +12781,19 @@
       </c>
       <c r="Q25" s="9" t="inlineStr">
         <is>
-          <t>Участок 0,5 га (бывшая шёлковая фабрика, 4 здания 5 тыс. м²), продавец KR Properties (А. Клячин), переход прав 23.04.2026. Камерный клубный дом: пентхаусы с видом на Кремль, виллы, двор-сад; фасады по ул. Тимура Фрунзе сохраняются.</t>
+          <t>Участок ~0,6 га у делового квартала «Красная Роза», куплен у структур А. Клячина. Три камерных клубных дома, надземная площадь 20,3 тыс. м², квартиры 12,4 тыс. м². Сохраняется фасад бывшего доходного дома Трындина-Жиро.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="24" customHeight="1">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>Усадьба в Большом Саввинском переулке (клубный дом VSF)</t>
+          <t>Лёвшинский, 19</t>
         </is>
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>Большой Саввинский пер. (усадьба купца Якунина)</t>
+          <t>Большой Лёвшинский пер., 19</t>
         </is>
       </c>
       <c r="C26" s="10" t="inlineStr">
@@ -12804,33 +12808,37 @@
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>ГК «Векторстройфинанс» (VSF)</t>
+          <t>ТСИ Девелопмент (ГК «Трансстройинвест»)</t>
         </is>
       </c>
       <c r="F26" s="9" t="inlineStr">
         <is>
-          <t>анонсирован (приобретение объекта), концепция</t>
-        </is>
-      </c>
-      <c r="G26" s="12" t="n">
-        <v>2500</v>
-      </c>
+          <t>старт бронирования, старт продаж</t>
+        </is>
+      </c>
+      <c r="G26" s="10" t="n"/>
       <c r="H26" s="10" t="n"/>
       <c r="I26" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="J26" s="10" t="n"/>
-      <c r="K26" s="10" t="n"/>
-      <c r="L26" s="10" t="n"/>
+        <v>8</v>
+      </c>
+      <c r="J26" s="12" t="n">
+        <v>16</v>
+      </c>
+      <c r="K26" s="10" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L26" s="10" t="inlineStr">
+        <is>
+          <t>2 кв. 2028</t>
+        </is>
+      </c>
       <c r="M26" s="10" t="n"/>
-      <c r="N26" s="10" t="inlineStr">
-        <is>
-          <t>2025-07-09</t>
-        </is>
-      </c>
-      <c r="O26" s="10" t="inlineStr">
-        <is>
-          <t>elitnoe.ru</t>
+      <c r="N26" s="10" t="n"/>
+      <c r="O26" s="9" t="inlineStr">
+        <is>
+          <t>whitewill.ru (также tehne.com, levshinsky-19.ru)</t>
         </is>
       </c>
       <c r="P26" s="13" t="inlineStr">
@@ -12840,19 +12848,19 @@
       </c>
       <c r="Q26" s="9" t="inlineStr">
         <is>
-          <t>Четырёхэтажное здание 1889 г. и двухэтажное до 1812 г., ~2,5 тыс. м². Оценка инвестиций 3,5–4,5 млрд руб., стоимость объекта до 1,3 млрд руб. Планируется перестройка в элитный клубный дом.</t>
+          <t>Воссоздание фасада доходного дома Духовских (1904, арх. Мейснер), проект HADAA Architects. 16 резиденций 70–239 м², паркинг 18 м/м. Цена от 197,12 млн руб. за лот. Стадия стройки в источниках не подтверждена.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="24" customHeight="1">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>Усачёва, 22</t>
-        </is>
-      </c>
-      <c r="B27" s="10" t="inlineStr">
-        <is>
-          <t>ул. Усачёва, 22</t>
+          <t>Олсуфьевский 10</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>Олсуфьевский пер., 10</t>
         </is>
       </c>
       <c r="C27" s="10" t="inlineStr">
@@ -12865,27 +12873,25 @@
           <t>Хамовники</t>
         </is>
       </c>
-      <c r="E27" s="9" t="inlineStr">
-        <is>
-          <t>Regions Development</t>
+      <c r="E27" s="10" t="inlineStr">
+        <is>
+          <t>Грандор (Grandor)</t>
         </is>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>проект, продажи не начаты</t>
-        </is>
-      </c>
-      <c r="G27" s="12" t="n">
-        <v>24600</v>
-      </c>
+          <t>ГПЗУ получен (апрель 2021), старт продаж ожидается</t>
+        </is>
+      </c>
+      <c r="G27" s="10" t="n"/>
       <c r="H27" s="10" t="n"/>
       <c r="I27" s="12" t="n">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="J27" s="10" t="n"/>
       <c r="K27" s="10" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2026–2027</t>
         </is>
       </c>
       <c r="L27" s="10" t="n"/>
@@ -12893,7 +12899,7 @@
       <c r="N27" s="10" t="n"/>
       <c r="O27" s="9" t="inlineStr">
         <is>
-          <t>novostroev.ru (также usacheva22.ru, sosedi.life)</t>
+          <t>официальный сайт проекта (также novostroy.ru, mskdeluxe.ru/start)</t>
         </is>
       </c>
       <c r="P27" s="13" t="inlineStr">
@@ -12903,19 +12909,19 @@
       </c>
       <c r="Q27" s="9" t="inlineStr">
         <is>
-          <t>Участок ~0,4 га, два корпуса ~14 и 18 этажей, архитектура Arch(e)type, двор без машин. Площадь 24,6 тыс. м² — по обзору делюкс-стартов 2026 novostroev.ru.</t>
+          <t>Участок 0,4 га, семь корпусов 5–8 этажей в индивидуальной архитектуре. В базе делюкс-стартов 2026–2027 mskdeluxe.ru.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="24" customHeight="1">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>Хилков (Хилков переулок, вл. 3)</t>
-        </is>
-      </c>
-      <c r="B28" s="10" t="inlineStr">
-        <is>
-          <t>Хилков пер., вл. 3</t>
+          <t>Премиальный квартал на Лужнецкой набережной, 10А</t>
+        </is>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>Лужнецкая наб., вл. 10А</t>
         </is>
       </c>
       <c r="C28" s="10" t="inlineStr">
@@ -12930,439 +12936,778 @@
       </c>
       <c r="E28" s="10" t="inlineStr">
         <is>
-          <t>Rose Group</t>
+          <t>Sminex</t>
         </is>
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>проектирование (долгосрочный проект), старт продаж ожидается</t>
-        </is>
-      </c>
-      <c r="G28" s="12" t="n">
-        <v>19806</v>
-      </c>
-      <c r="H28" s="12" t="n">
-        <v>8800</v>
-      </c>
-      <c r="I28" s="12" t="n">
-        <v>8</v>
-      </c>
+          <t>проект утверждён (АГР, май 2026), начало строительства 2027</t>
+        </is>
+      </c>
+      <c r="G28" s="10" t="n"/>
+      <c r="H28" s="10" t="n"/>
+      <c r="I28" s="10" t="n"/>
       <c r="J28" s="10" t="n"/>
       <c r="K28" s="10" t="inlineStr">
         <is>
-          <t>2026–2027</t>
+          <t>2027 (стройка)</t>
         </is>
       </c>
       <c r="L28" s="10" t="n"/>
       <c r="M28" s="10" t="n"/>
-      <c r="N28" s="10" t="n"/>
+      <c r="N28" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
       <c r="O28" s="9" t="inlineStr">
         <is>
+          <t>РИА Недвижимость (также anwin.ru)</t>
+        </is>
+      </c>
+      <c r="P28" s="13" t="inlineStr">
+        <is>
+          <t>ссылка</t>
+        </is>
+      </c>
+      <c r="Q28" s="9" t="inlineStr">
+        <is>
+          <t>Два жилых корпуса переменной этажности в неоклассике + эллиптический БЦ 26 тыс. м² («яйцо Фаберже»). Концепция согласована Департаментом градостроительной политики (В. Овчинский). Параметры жилой части не раскрыты.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="24" customHeight="1">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t>Тимура Фрунзе, 11 (клубный дом Sminex)</t>
+        </is>
+      </c>
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>ул. Тимура Фрунзе, 11, стр. 7, 19, 33, 50</t>
+        </is>
+      </c>
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>Хамовники</t>
+        </is>
+      </c>
+      <c r="D29" s="29" t="inlineStr">
+        <is>
+          <t>Хамовники</t>
+        </is>
+      </c>
+      <c r="E29" s="10" t="inlineStr">
+        <is>
+          <t>Sminex</t>
+        </is>
+      </c>
+      <c r="F29" s="9" t="inlineStr">
+        <is>
+          <t>участок приобретён (апрель 2026), проектирование</t>
+        </is>
+      </c>
+      <c r="G29" s="12" t="n">
+        <v>13000</v>
+      </c>
+      <c r="H29" s="12" t="n">
+        <v>8200</v>
+      </c>
+      <c r="I29" s="10" t="n"/>
+      <c r="J29" s="10" t="n"/>
+      <c r="K29" s="10" t="n"/>
+      <c r="L29" s="10" t="n"/>
+      <c r="M29" s="10" t="n"/>
+      <c r="N29" s="10" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="O29" s="9" t="inlineStr">
+        <is>
+          <t>РИА Недвижимость (также sminex.com, interfax-russia.ru)</t>
+        </is>
+      </c>
+      <c r="P29" s="13" t="inlineStr">
+        <is>
+          <t>ссылка</t>
+        </is>
+      </c>
+      <c r="Q29" s="9" t="inlineStr">
+        <is>
+          <t>Участок 0,5 га (бывшая шёлковая фабрика, 4 здания 5 тыс. м²), продавец KR Properties (А. Клячин), переход прав 23.04.2026. Камерный клубный дом: пентхаусы с видом на Кремль, виллы, двор-сад; фасады по ул. Тимура Фрунзе сохраняются.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="24" customHeight="1">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>Усадьба в Большом Саввинском переулке (клубный дом VSF)</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>Большой Саввинский пер. (усадьба купца Якунина)</t>
+        </is>
+      </c>
+      <c r="C30" s="10" t="inlineStr">
+        <is>
+          <t>Хамовники</t>
+        </is>
+      </c>
+      <c r="D30" s="29" t="inlineStr">
+        <is>
+          <t>Хамовники</t>
+        </is>
+      </c>
+      <c r="E30" s="9" t="inlineStr">
+        <is>
+          <t>ГК «Векторстройфинанс» (VSF)</t>
+        </is>
+      </c>
+      <c r="F30" s="9" t="inlineStr">
+        <is>
+          <t>анонсирован (приобретение объекта), концепция</t>
+        </is>
+      </c>
+      <c r="G30" s="12" t="n">
+        <v>2500</v>
+      </c>
+      <c r="H30" s="10" t="n"/>
+      <c r="I30" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="J30" s="10" t="n"/>
+      <c r="K30" s="10" t="n"/>
+      <c r="L30" s="10" t="n"/>
+      <c r="M30" s="10" t="n"/>
+      <c r="N30" s="10" t="inlineStr">
+        <is>
+          <t>2025-07-09</t>
+        </is>
+      </c>
+      <c r="O30" s="10" t="inlineStr">
+        <is>
+          <t>elitnoe.ru</t>
+        </is>
+      </c>
+      <c r="P30" s="13" t="inlineStr">
+        <is>
+          <t>ссылка</t>
+        </is>
+      </c>
+      <c r="Q30" s="9" t="inlineStr">
+        <is>
+          <t>Четырёхэтажное здание 1889 г. и двухэтажное до 1812 г., ~2,5 тыс. м². Оценка инвестиций 3,5–4,5 млрд руб., стоимость объекта до 1,3 млрд руб. Планируется перестройка в элитный клубный дом.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="24" customHeight="1">
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t>Усачёва, 22</t>
+        </is>
+      </c>
+      <c r="B31" s="10" t="inlineStr">
+        <is>
+          <t>ул. Усачёва, 22</t>
+        </is>
+      </c>
+      <c r="C31" s="10" t="inlineStr">
+        <is>
+          <t>Хамовники</t>
+        </is>
+      </c>
+      <c r="D31" s="29" t="inlineStr">
+        <is>
+          <t>Хамовники</t>
+        </is>
+      </c>
+      <c r="E31" s="9" t="inlineStr">
+        <is>
+          <t>Regions Development</t>
+        </is>
+      </c>
+      <c r="F31" s="9" t="inlineStr">
+        <is>
+          <t>проект, продажи не начаты</t>
+        </is>
+      </c>
+      <c r="G31" s="12" t="n">
+        <v>24600</v>
+      </c>
+      <c r="H31" s="10" t="n"/>
+      <c r="I31" s="12" t="n">
+        <v>18</v>
+      </c>
+      <c r="J31" s="10" t="n"/>
+      <c r="K31" s="10" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L31" s="10" t="n"/>
+      <c r="M31" s="10" t="n"/>
+      <c r="N31" s="10" t="n"/>
+      <c r="O31" s="9" t="inlineStr">
+        <is>
+          <t>novostroev.ru (также usacheva22.ru, sosedi.life)</t>
+        </is>
+      </c>
+      <c r="P31" s="13" t="inlineStr">
+        <is>
+          <t>ссылка</t>
+        </is>
+      </c>
+      <c r="Q31" s="9" t="inlineStr">
+        <is>
+          <t>Участок ~0,4 га, два корпуса ~14 и 18 этажей, архитектура Arch(e)type, двор без машин. Площадь 24,6 тыс. м² — по обзору делюкс-стартов 2026 novostroev.ru.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="24" customHeight="1">
+      <c r="A32" s="9" t="inlineStr">
+        <is>
+          <t>Хилков (Хилков переулок, вл. 3)</t>
+        </is>
+      </c>
+      <c r="B32" s="10" t="inlineStr">
+        <is>
+          <t>Хилков пер., вл. 3</t>
+        </is>
+      </c>
+      <c r="C32" s="10" t="inlineStr">
+        <is>
+          <t>Хамовники</t>
+        </is>
+      </c>
+      <c r="D32" s="29" t="inlineStr">
+        <is>
+          <t>Хамовники</t>
+        </is>
+      </c>
+      <c r="E32" s="10" t="inlineStr">
+        <is>
+          <t>Rose Group</t>
+        </is>
+      </c>
+      <c r="F32" s="9" t="inlineStr">
+        <is>
+          <t>проектирование (долгосрочный проект), старт продаж ожидается</t>
+        </is>
+      </c>
+      <c r="G32" s="12" t="n">
+        <v>19806</v>
+      </c>
+      <c r="H32" s="12" t="n">
+        <v>8800</v>
+      </c>
+      <c r="I32" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="J32" s="10" t="n"/>
+      <c r="K32" s="10" t="inlineStr">
+        <is>
+          <t>2026–2027</t>
+        </is>
+      </c>
+      <c r="L32" s="10" t="n"/>
+      <c r="M32" s="10" t="n"/>
+      <c r="N32" s="10" t="n"/>
+      <c r="O32" s="9" t="inlineStr">
+        <is>
           <t>novostroy-m.ru (также mskdeluxe.ru/start)</t>
         </is>
       </c>
-      <c r="P28" s="13" t="inlineStr">
-        <is>
-          <t>ссылка</t>
-        </is>
-      </c>
-      <c r="Q28" s="9" t="inlineStr">
+      <c r="P32" s="13" t="inlineStr">
+        <is>
+          <t>ссылка</t>
+        </is>
+      </c>
+      <c r="Q32" s="9" t="inlineStr">
         <is>
           <t>3–8 этажей, монолит-кирпич, коммерция 1,8 тыс. м², паркинг 170 м/м. Карточка novostroy-m.ru датирована 2016 г.; проект вновь фигурирует в списке делюкс-стартов 2026–2027 на mskdeluxe.ru. Актуальность требует проверки.</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="24" customHeight="1">
-      <c r="A29" s="14" t="inlineStr">
+    <row r="33" ht="24" customHeight="1">
+      <c r="A33" s="14" t="inlineStr">
         <is>
           <t>Aurus Residences / Страна.Сити</t>
         </is>
       </c>
-      <c r="B29" s="14" t="inlineStr">
+      <c r="B33" s="14" t="inlineStr">
         <is>
           <t>2-й Красногвардейский проезд, квартал «Камушки»</t>
         </is>
       </c>
-      <c r="C29" s="15" t="inlineStr">
+      <c r="C33" s="15" t="inlineStr">
         <is>
           <t>Пресненский</t>
         </is>
       </c>
-      <c r="D29" s="30" t="inlineStr">
+      <c r="D33" s="30" t="inlineStr">
         <is>
           <t>Сити</t>
         </is>
       </c>
-      <c r="E29" s="15" t="inlineStr">
+      <c r="E33" s="15" t="inlineStr">
         <is>
           <t>Страна Девелопмент</t>
         </is>
       </c>
-      <c r="F29" s="14" t="inlineStr">
+      <c r="F33" s="14" t="inlineStr">
         <is>
           <t>ГПЗУ получен, подготовка к старту продаж</t>
         </is>
       </c>
-      <c r="G29" s="17" t="n">
+      <c r="G33" s="17" t="n">
         <v>280800</v>
       </c>
-      <c r="H29" s="17" t="n">
+      <c r="H33" s="17" t="n">
         <v>231800</v>
       </c>
-      <c r="I29" s="17" t="n">
+      <c r="I33" s="17" t="n">
         <v>97</v>
       </c>
-      <c r="J29" s="15" t="n"/>
-      <c r="K29" s="15" t="inlineStr">
+      <c r="J33" s="15" t="n"/>
+      <c r="K33" s="15" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="L29" s="15" t="inlineStr">
+      <c r="L33" s="15" t="inlineStr">
         <is>
           <t>2029</t>
         </is>
       </c>
-      <c r="M29" s="15" t="n"/>
-      <c r="N29" s="15" t="inlineStr">
+      <c r="M33" s="15" t="n"/>
+      <c r="N33" s="15" t="inlineStr">
         <is>
           <t>2026-04-07</t>
         </is>
       </c>
-      <c r="O29" s="15" t="inlineStr">
+      <c r="O33" s="15" t="inlineStr">
         <is>
           <t>sosedi.life</t>
         </is>
       </c>
-      <c r="P29" s="18" t="inlineStr">
-        <is>
-          <t>ссылка</t>
-        </is>
-      </c>
-      <c r="Q29" s="14" t="inlineStr">
+      <c r="P33" s="18" t="inlineStr">
+        <is>
+          <t>ссылка</t>
+        </is>
+      </c>
+      <c r="Q33" s="14" t="inlineStr">
         <is>
           <t>Две башни 83 и 97 этажей на шестиярусном стилобате, участок ~1,25 га, архитектура APEX. ГПЗУ получен летом 2024 г., проект проходит согласования. Бизнес/премиум-класс, апартаменты.</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="24" customHeight="1">
-      <c r="A30" s="14" t="inlineStr">
-        <is>
-          <t>Капранова, 3</t>
-        </is>
-      </c>
-      <c r="B30" s="14" t="inlineStr">
-        <is>
-          <t>пер. Капранова, 3 (участки Верхний Предтеченский пер., 11 и Малый Предтеченский пер., 1)</t>
-        </is>
-      </c>
-      <c r="C30" s="15" t="inlineStr">
+    <row r="34" ht="24" customHeight="1">
+      <c r="A34" s="14" t="inlineStr">
+        <is>
+          <t>Жилые башни «Сити-2» (2-й Красногвардейский проезд)</t>
+        </is>
+      </c>
+      <c r="B34" s="14" t="inlineStr">
+        <is>
+          <t>2-й Красногвардейский проезд, Пресненский район (площадка 1,255 га у «Москва-Сити»)</t>
+        </is>
+      </c>
+      <c r="C34" s="15" t="inlineStr">
         <is>
           <t>Пресненский</t>
         </is>
       </c>
-      <c r="D30" s="30" t="inlineStr">
+      <c r="D34" s="30" t="inlineStr">
         <is>
           <t>Сити</t>
         </is>
       </c>
-      <c r="E30" s="15" t="inlineStr">
+      <c r="E34" s="14" t="inlineStr">
+        <is>
+          <t>ГК «Страна Девелопмент» (право застройки получено на торгах города; прежний правообладатель — ООО «Моссититстрой»)</t>
+        </is>
+      </c>
+      <c r="F34" s="14" t="inlineStr">
+        <is>
+          <t>АГР двух жилых башен утвержден (декабрь 2025); старт продаж не объявлен</t>
+        </is>
+      </c>
+      <c r="G34" s="17" t="n">
+        <v>281000</v>
+      </c>
+      <c r="H34" s="17" t="n">
+        <v>232000</v>
+      </c>
+      <c r="I34" s="14" t="inlineStr">
+        <is>
+          <t>две башни, самая высокая — 384 м по утвержденному АГР (ранее заявлялось до 450 м)</t>
+        </is>
+      </c>
+      <c r="J34" s="15" t="n"/>
+      <c r="K34" s="15" t="n"/>
+      <c r="L34" s="15" t="n"/>
+      <c r="M34" s="15" t="n"/>
+      <c r="N34" s="15" t="inlineStr">
+        <is>
+          <t>2025-12-30</t>
+        </is>
+      </c>
+      <c r="O34" s="14" t="inlineStr">
+        <is>
+          <t>72.ru / сеть городских порталов (30.12.2025); IRN.ru (18.04.2024)</t>
+        </is>
+      </c>
+      <c r="P34" s="18" t="inlineStr">
+        <is>
+          <t>ссылка</t>
+        </is>
+      </c>
+      <c r="Q34" s="14" t="inlineStr">
+        <is>
+          <t>~232 тыс. м² жилья и 49 тыс. м² нежилых помещений (IRN.ru, https://www.irn.ru/news/156498.html). Самый высокий жилой комплекс России по утвержденной концепции. Отдельно на Novostroy-M числится «Сити-2» Capital Group (квартал 804, Камушки, три башни до 450 м, ~470 тыс. м², ~385 тыс. м² жилья, «скоро старт») — иная площадка в том же районе, не путать.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="24" customHeight="1">
+      <c r="A35" s="14" t="inlineStr">
+        <is>
+          <t>МФК «На Краснопресненской набережной» (Трёхгорная мануфактура)</t>
+        </is>
+      </c>
+      <c r="B35" s="14" t="inlineStr">
+        <is>
+          <t>Краснопресненская наб., 10</t>
+        </is>
+      </c>
+      <c r="C35" s="15" t="inlineStr">
+        <is>
+          <t>Пресненский</t>
+        </is>
+      </c>
+      <c r="D35" s="30" t="inlineStr">
+        <is>
+          <t>Сити</t>
+        </is>
+      </c>
+      <c r="E35" s="15" t="inlineStr">
+        <is>
+          <t>ГК Ташир</t>
+        </is>
+      </c>
+      <c r="F35" s="14" t="inlineStr">
+        <is>
+          <t>анонсирован, старт продаж ожидается</t>
+        </is>
+      </c>
+      <c r="G35" s="15" t="n"/>
+      <c r="H35" s="15" t="n"/>
+      <c r="I35" s="15" t="n"/>
+      <c r="J35" s="15" t="n"/>
+      <c r="K35" s="15" t="n"/>
+      <c r="L35" s="15" t="inlineStr">
+        <is>
+          <t>2030</t>
+        </is>
+      </c>
+      <c r="M35" s="15" t="n"/>
+      <c r="N35" s="15" t="n"/>
+      <c r="O35" s="15" t="inlineStr">
+        <is>
+          <t>novostroycity.ru</t>
+        </is>
+      </c>
+      <c r="P35" s="18" t="inlineStr">
+        <is>
+          <t>ссылка</t>
+        </is>
+      </c>
+      <c r="Q35" s="14" t="inlineStr">
+        <is>
+          <t>Участок ~1,7 га с ОКН (фабрика Трёхгорной мануфактуры, будет сохранена/реконструирована). Апартаменты премиум-класса + офисы + wellness, подземный паркинг на 750 м/м. Сроки реализации официально не подтверждены; апартаменты, а не квартиры.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="24" customHeight="1">
+      <c r="A36" s="21" t="inlineStr">
+        <is>
+          <t>Клубный дом «Капельский, 5»</t>
+        </is>
+      </c>
+      <c r="B36" s="21" t="inlineStr">
+        <is>
+          <t>Капельский переулок, 5</t>
+        </is>
+      </c>
+      <c r="C36" s="24" t="inlineStr">
+        <is>
+          <t>Мещанский</t>
+        </is>
+      </c>
+      <c r="D36" s="21" t="inlineStr">
+        <is>
+          <t>Мещанский (вне Садового)</t>
+        </is>
+      </c>
+      <c r="E36" s="21" t="inlineStr">
+        <is>
+          <t>не раскрыт (юрлицо на сайте проекта не указано)</t>
+        </is>
+      </c>
+      <c r="F36" s="21" t="inlineStr">
+        <is>
+          <t>проектирование / предстарт продаж (официально: открытие продаж планируется во II–III кв. 2026)</t>
+        </is>
+      </c>
+      <c r="G36" s="24" t="n"/>
+      <c r="H36" s="24" t="n"/>
+      <c r="I36" s="24" t="inlineStr">
+        <is>
+          <t>8–9</t>
+        </is>
+      </c>
+      <c r="J36" s="25" t="n">
+        <v>46</v>
+      </c>
+      <c r="K36" s="21" t="inlineStr">
+        <is>
+          <t>2026 Q2–Q3 (старт продаж)</t>
+        </is>
+      </c>
+      <c r="L36" s="21" t="inlineStr">
+        <is>
+          <t>2029 Q4 (по данным Whitewill)</t>
+        </is>
+      </c>
+      <c r="M36" s="24" t="n"/>
+      <c r="N36" s="24" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="O36" s="21" t="inlineStr">
+        <is>
+          <t>Официальный сайт kapelsky5.ru; Whitewill; Novostroy-M</t>
+        </is>
+      </c>
+      <c r="P36" s="26" t="inlineStr">
+        <is>
+          <t>ссылка</t>
+        </is>
+      </c>
+      <c r="Q36" s="21" t="inlineStr">
+        <is>
+          <t>46 резиденций, переменная этажность, пентхаусы с террасами, приватный сквер, подземный паркинг. ВНИМАНИЕ: локация вне Садового кольца (у м. Проспект Мира, ~1 км севернее), включена по запросу заказчика.; Делюкс/премиум клубный дом; квартиры 54–345 м²; пентхаусы с террасами; двухуровневый паркинг на 56 м/м, 32 кладовые; приватный сад во дворе. Whitewill (https://whitewill.ru/developments/kapelskiy-5) указывает 8 этажей и срок сдачи 4 кв. 2029; Novostroy-M — 9 этажей, «скоро старт». Цены по запросу.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="24" customHeight="1">
+      <c r="A37" s="19" t="inlineStr">
+        <is>
+          <t>Делюкс-комплекс «Капранова, 3» (проект APEX)</t>
+        </is>
+      </c>
+      <c r="B37" s="19" t="inlineStr">
+        <is>
+          <t>переулок Капранова, 3 (БЦ «Премьер Плаза») + Малый Предтеченский пер., 1/2/1, Нововаганьковский пер., 3 стр. 1, Глубокий пер., 7</t>
+        </is>
+      </c>
+      <c r="C37" s="20" t="inlineStr">
+        <is>
+          <t>Пресненский</t>
+        </is>
+      </c>
+      <c r="D37" s="21" t="inlineStr">
+        <is>
+          <t>Пресненский (вне Садового)</t>
+        </is>
+      </c>
+      <c r="E37" s="20" t="inlineStr">
         <is>
           <t>не раскрыт</t>
         </is>
       </c>
-      <c r="F30" s="14" t="inlineStr">
-        <is>
-          <t>анонсирован, старт продаж ожидается</t>
-        </is>
-      </c>
-      <c r="G30" s="15" t="n"/>
-      <c r="H30" s="15" t="n"/>
-      <c r="I30" s="17" t="n">
-        <v>12</v>
-      </c>
-      <c r="J30" s="15" t="n"/>
-      <c r="K30" s="15" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="L30" s="15" t="n"/>
-      <c r="M30" s="15" t="n"/>
-      <c r="N30" s="15" t="n"/>
-      <c r="O30" s="14" t="inlineStr">
-        <is>
-          <t>mskdeluxe.ru (также smart-lab.ru обзор стартов на Пресне)</t>
-        </is>
-      </c>
-      <c r="P30" s="18" t="inlineStr">
-        <is>
-          <t>ссылка</t>
-        </is>
-      </c>
-      <c r="Q30" s="14" t="inlineStr">
-        <is>
-          <t>Делюкс-проект в базе перспективных стартов 2026–2027 (mskdeluxe.ru, цены «от 60 млн руб.»). Обзор smart-lab.ru/blog/1231916.php указывает старт продаж в 2026 г., 12 этажей, двор без машин. Застройщик и параметры в открытых источниках не подтверждены. ~400 м от м. Краснопресненская, вне Садового кольца.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="24" customHeight="1">
-      <c r="A31" s="14" t="inlineStr">
-        <is>
-          <t>МФК «На Краснопресненской набережной» (Трёхгорная мануфактура)</t>
-        </is>
-      </c>
-      <c r="B31" s="14" t="inlineStr">
-        <is>
-          <t>Краснопресненская наб., 10</t>
-        </is>
-      </c>
-      <c r="C31" s="15" t="inlineStr">
+      <c r="F37" s="19" t="inlineStr">
+        <is>
+          <t>визуализации направлены на согласование в город (ноябрь 2025); предстарт, старт продаж заявлен на 2026</t>
+        </is>
+      </c>
+      <c r="G37" s="20" t="n"/>
+      <c r="H37" s="20" t="n"/>
+      <c r="I37" s="19" t="inlineStr">
+        <is>
+          <t>9–23 (шесть корпусов)</t>
+        </is>
+      </c>
+      <c r="J37" s="22" t="n">
+        <v>255</v>
+      </c>
+      <c r="K37" s="19" t="inlineStr">
+        <is>
+          <t>2026 (старт продаж)</t>
+        </is>
+      </c>
+      <c r="L37" s="20" t="n"/>
+      <c r="M37" s="20" t="n"/>
+      <c r="N37" s="20" t="inlineStr">
+        <is>
+          <t>2025-11-19</t>
+        </is>
+      </c>
+      <c r="O37" s="19" t="inlineStr">
+        <is>
+          <t>Москвич Mag (19.11.2025); sosedi.life (07.04.2026)</t>
+        </is>
+      </c>
+      <c r="P37" s="23" t="inlineStr">
+        <is>
+          <t>ссылка</t>
+        </is>
+      </c>
+      <c r="Q37" s="19" t="inlineStr">
+        <is>
+          <t>Делюкс-проект в базе перспективных стартов 2026–2027 (mskdeluxe.ru, цены «от 60 млн руб.»). Обзор smart-lab.ru/blog/1231916.php указывает старт продаж в 2026 г., 12 этажей, двор без машин. Застройщик и параметры в открытых источниках не подтверждены. ~400 м от м. Краснопресненская, вне Садового кольца.; Единая застройка нескольких участков за Домом Правительства у Пресненского детского парка; башни с «волнообразными» фасадами, снос БЦ «Премьер Плаза», сохранение усадьбы Резанова. По sosedi.life (https://sosedi.life/news/zhk-kapranova-3/): участок &gt;2,5 га, 6 корпусов 9–23 этажа, 255 квартир, двор 7 039,6 м², лобби Balcon, 2–5 квартир на этаже. Указанные в запросе «12 этажей» источниками не подтверждаются. В списке делюкс-стартов mskdeluxe.ru.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="24" customHeight="1">
+      <c r="A38" s="21" t="inlineStr">
+        <is>
+          <t>КРТ вдоль Звенигородского шоссе (три участка, 73,62 га)</t>
+        </is>
+      </c>
+      <c r="B38" s="21" t="inlineStr">
+        <is>
+          <t>Вдоль Звенигородского шоссе между 3-й Магистральной улицей и ТТК (Пресненский / Хорошёвский районы)</t>
+        </is>
+      </c>
+      <c r="C38" s="21" t="inlineStr">
+        <is>
+          <t>Пресненский / Хорошёвский</t>
+        </is>
+      </c>
+      <c r="D38" s="21" t="inlineStr">
+        <is>
+          <t>Пресненский (вне Садового)</t>
+        </is>
+      </c>
+      <c r="E38" s="21" t="inlineStr">
+        <is>
+          <t>не раскрыт (оператор/инвестор не назван; в числе 9 проектов КРТ, утвержденных в августе 2026)</t>
+        </is>
+      </c>
+      <c r="F38" s="21" t="inlineStr">
+        <is>
+          <t>решение о КРТ принято (август 2026); оператор/торги не объявлены</t>
+        </is>
+      </c>
+      <c r="G38" s="25" t="n">
+        <v>3200000</v>
+      </c>
+      <c r="H38" s="24" t="n"/>
+      <c r="I38" s="24" t="n"/>
+      <c r="J38" s="24" t="n"/>
+      <c r="K38" s="24" t="n"/>
+      <c r="L38" s="24" t="n"/>
+      <c r="M38" s="24" t="n"/>
+      <c r="N38" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="O38" s="21" t="inlineStr">
+        <is>
+          <t>Интерфакс-Россия; Ведомости.Город (02.09.2026)</t>
+        </is>
+      </c>
+      <c r="P38" s="26" t="inlineStr">
+        <is>
+          <t>ссылка</t>
+        </is>
+      </c>
+      <c r="Q38" s="21" t="inlineStr">
+        <is>
+          <t>Три участка нежилой застройки общей площадью 73,62 га; &gt;3,2 млн м² недвижимости (жильё + общественно-деловые объекты, школы на 4050 мест, детсады на 1775 мест), 35,5 тыс. рабочих мест. Часть «Большого Сити» (Шелепиха/Магистральные улицы), класс жилья не заявлен — не обязательно премиум.; Три участка нежилой застройки (старые склады, админздания) общей площадью 73,62 га; свыше 3,2 млн м² — жилье, общественно-деловые и социальные объекты; строительство/реконструкция дорог ~6,5 км; здание конечной станции наземного транспорта с отстойно-разворотной площадкой (Ведомости, https://www.vedomosti.ru/gorod/ourcity/articles/gorodskoi-kvartal). Жилая премиальная часть отдельно не выделена; класс жилья не указан. Оператор (Московский фонд реновации / КРТ 21 / инвестор по торгам) не объявлен.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="24" customHeight="1">
+      <c r="A39" s="19" t="inlineStr">
+        <is>
+          <t>Участок КРТ «Большой Тишинский переулок, 8»</t>
+        </is>
+      </c>
+      <c r="B39" s="19" t="inlineStr">
+        <is>
+          <t>Большой Тишинский переулок, 8 (стр. 1, 2)</t>
+        </is>
+      </c>
+      <c r="C39" s="20" t="inlineStr">
         <is>
           <t>Пресненский</t>
         </is>
       </c>
-      <c r="D31" s="30" t="inlineStr">
-        <is>
-          <t>Сити</t>
-        </is>
-      </c>
-      <c r="E31" s="15" t="inlineStr">
-        <is>
-          <t>ГК Ташир</t>
-        </is>
-      </c>
-      <c r="F31" s="14" t="inlineStr">
-        <is>
-          <t>анонсирован, старт продаж ожидается</t>
-        </is>
-      </c>
-      <c r="G31" s="15" t="n"/>
-      <c r="H31" s="15" t="n"/>
-      <c r="I31" s="15" t="n"/>
-      <c r="J31" s="15" t="n"/>
-      <c r="K31" s="15" t="n"/>
-      <c r="L31" s="15" t="inlineStr">
-        <is>
-          <t>2030</t>
-        </is>
-      </c>
-      <c r="M31" s="15" t="n"/>
-      <c r="N31" s="15" t="n"/>
-      <c r="O31" s="15" t="inlineStr">
-        <is>
-          <t>novostroycity.ru</t>
-        </is>
-      </c>
-      <c r="P31" s="18" t="inlineStr">
-        <is>
-          <t>ссылка</t>
-        </is>
-      </c>
-      <c r="Q31" s="14" t="inlineStr">
-        <is>
-          <t>Участок ~1,7 га с ОКН (фабрика Трёхгорной мануфактуры, будет сохранена/реконструирована). Апартаменты премиум-класса + офисы + wellness, подземный паркинг на 750 м/м. Сроки реализации официально не подтверждены; апартаменты, а не квартиры.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="24" customHeight="1">
-      <c r="A32" s="21" t="inlineStr">
-        <is>
-          <t>Капельский, 5</t>
-        </is>
-      </c>
-      <c r="B32" s="24" t="inlineStr">
-        <is>
-          <t>Капельский пер., 5</t>
-        </is>
-      </c>
-      <c r="C32" s="24" t="inlineStr">
-        <is>
-          <t>Мещанский</t>
-        </is>
-      </c>
-      <c r="D32" s="21" t="inlineStr">
-        <is>
-          <t>Мещанский (вне Садового)</t>
-        </is>
-      </c>
-      <c r="E32" s="24" t="inlineStr">
+      <c r="D39" s="21" t="inlineStr">
+        <is>
+          <t>Пресненский (вне Садового)</t>
+        </is>
+      </c>
+      <c r="E39" s="20" t="inlineStr">
         <is>
           <t>не раскрыт</t>
         </is>
       </c>
-      <c r="F32" s="21" t="inlineStr">
-        <is>
-          <t>проектирование, старт продаж ожидается во II–III кв. 2026 после проектной декларации</t>
-        </is>
-      </c>
-      <c r="G32" s="24" t="n"/>
-      <c r="H32" s="24" t="n"/>
-      <c r="I32" s="24" t="n"/>
-      <c r="J32" s="25" t="n">
-        <v>46</v>
-      </c>
-      <c r="K32" s="24" t="inlineStr">
-        <is>
-          <t>2026 (II–III кв.)</t>
-        </is>
-      </c>
-      <c r="L32" s="24" t="n"/>
-      <c r="M32" s="24" t="n"/>
-      <c r="N32" s="24" t="n"/>
-      <c r="O32" s="21" t="inlineStr">
-        <is>
-          <t>официальный сайт проекта (также kvartiravmoskve.ru, whitewill.ru)</t>
-        </is>
-      </c>
-      <c r="P32" s="26" t="inlineStr">
-        <is>
-          <t>ссылка</t>
-        </is>
-      </c>
-      <c r="Q32" s="21" t="inlineStr">
-        <is>
-          <t>46 резиденций, переменная этажность, пентхаусы с террасами, приватный сквер, подземный паркинг. ВНИМАНИЕ: локация вне Садового кольца (у м. Проспект Мира, ~1 км севернее), включена по запросу заказчика.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="24" customHeight="1">
-      <c r="A33" s="19" t="inlineStr">
-        <is>
-          <t>КРТ вдоль Звенигородского шоссе (Пресненский / Хорошёвский)</t>
-        </is>
-      </c>
-      <c r="B33" s="19" t="inlineStr">
-        <is>
-          <t>Звенигородское шоссе, между 3-й Магистральной ул. и ТТК (1-я Магистральная, 25 и др.)</t>
-        </is>
-      </c>
-      <c r="C33" s="20" t="inlineStr">
-        <is>
-          <t>Пресненский</t>
-        </is>
-      </c>
-      <c r="D33" s="21" t="inlineStr">
-        <is>
-          <t>Пресненский (вне Садового)</t>
-        </is>
-      </c>
-      <c r="E33" s="20" t="inlineStr">
-        <is>
-          <t>не раскрыт</t>
-        </is>
-      </c>
-      <c r="F33" s="20" t="inlineStr">
-        <is>
-          <t>ЗУ/КРТ утверждён</t>
-        </is>
-      </c>
-      <c r="G33" s="22" t="n">
-        <v>3200000</v>
-      </c>
-      <c r="H33" s="20" t="n"/>
-      <c r="I33" s="20" t="n"/>
-      <c r="J33" s="20" t="n"/>
-      <c r="K33" s="20" t="n"/>
-      <c r="L33" s="20" t="n"/>
-      <c r="M33" s="20" t="n"/>
-      <c r="N33" s="20" t="inlineStr">
-        <is>
-          <t>2025-09-02</t>
-        </is>
-      </c>
-      <c r="O33" s="20" t="inlineStr">
-        <is>
-          <t>Агентство «Москва»</t>
-        </is>
-      </c>
-      <c r="P33" s="23" t="inlineStr">
-        <is>
-          <t>ссылка</t>
-        </is>
-      </c>
-      <c r="Q33" s="19" t="inlineStr">
-        <is>
-          <t>Три участка нежилой застройки общей площадью 73,62 га; &gt;3,2 млн м² недвижимости (жильё + общественно-деловые объекты, школы на 4050 мест, детсады на 1775 мест), 35,5 тыс. рабочих мест. Часть «Большого Сити» (Шелепиха/Магистральные улицы), класс жилья не заявлен — не обязательно премиум.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="24" customHeight="1">
-      <c r="A34" s="21" t="inlineStr">
-        <is>
-          <t>Участок КРТ «Большой Тишинский переулок, 8»</t>
-        </is>
-      </c>
-      <c r="B34" s="21" t="inlineStr">
-        <is>
-          <t>Большой Тишинский пер., 8 (два административных здания 1909–1915 гг.)</t>
-        </is>
-      </c>
-      <c r="C34" s="24" t="inlineStr">
-        <is>
-          <t>Пресненский</t>
-        </is>
-      </c>
-      <c r="D34" s="21" t="inlineStr">
-        <is>
-          <t>Пресненский (вне Садового)</t>
-        </is>
-      </c>
-      <c r="E34" s="24" t="inlineStr">
-        <is>
-          <t>не раскрыт</t>
-        </is>
-      </c>
-      <c r="F34" s="24" t="inlineStr">
-        <is>
-          <t>ЗУ/КРТ утверждён</t>
-        </is>
-      </c>
-      <c r="G34" s="25" t="n">
+      <c r="F39" s="19" t="inlineStr">
+        <is>
+          <t>решение о КРТ (по данным заказчика — август 2026); оператор/правообладатель и торги в открытых источниках не найдены</t>
+        </is>
+      </c>
+      <c r="G39" s="22" t="n">
         <v>10000</v>
       </c>
-      <c r="H34" s="25" t="n">
+      <c r="H39" s="22" t="n">
         <v>6000</v>
       </c>
-      <c r="I34" s="24" t="n"/>
-      <c r="J34" s="24" t="n"/>
-      <c r="K34" s="24" t="n"/>
-      <c r="L34" s="24" t="n"/>
-      <c r="M34" s="24" t="n"/>
-      <c r="N34" s="24" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="O34" s="24" t="inlineStr">
-        <is>
-          <t>АСН-инфо</t>
-        </is>
-      </c>
-      <c r="P34" s="26" t="inlineStr">
-        <is>
-          <t>ссылка</t>
-        </is>
-      </c>
-      <c r="Q34" s="21" t="inlineStr">
-        <is>
-          <t>Участок ~0,3 га включён в программу КРТ решением властей Москвы. Существующие здания реконструированы в 2004 г., в 2020 г. переоборудованы под хостелы. Оператор/девелопер в публикации не назван; в других открытых источниках на 07.09.2026 не найден. Локация — Пресненский район вне Садового кольца, между Б. Грузинской и Пресненским Валом (условно отнесено к зоне Пресня/Сити).</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="30" customHeight="1">
-      <c r="A36" s="27" t="inlineStr">
+      <c r="I39" s="20" t="n"/>
+      <c r="J39" s="20" t="n"/>
+      <c r="K39" s="20" t="n"/>
+      <c r="L39" s="20" t="n"/>
+      <c r="M39" s="20" t="n"/>
+      <c r="N39" s="20" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="O39" s="19" t="inlineStr">
+        <is>
+          <t>krt.mos.ru (реестр проектов КРТ Москвы)</t>
+        </is>
+      </c>
+      <c r="P39" s="23" t="inlineStr">
+        <is>
+          <t>ссылка</t>
+        </is>
+      </c>
+      <c r="Q39" s="19" t="inlineStr">
+        <is>
+          <t>Участок ~0,3 га включён в программу КРТ решением властей Москвы. Существующие здания реконструированы в 2004 г., в 2020 г. переоборудованы под хостелы. Оператор/девелопер в публикации не назван; в других открытых источниках на 07.09.2026 не найден. Локация — Пресненский район вне Садового кольца, между Б. Грузинской и Пресненским Валом (условно отнесено к зоне Пресня/Сити).; Поиск по mos.ru, krt.mos.ru, stroi.mos.ru, Ведомости, РБК, Интерфакс, М24, Известия (август–сентябрь 2026) не выявил отдельной публикации по этому участку: новости августа 2026 о КРТ (250 проектов, 63 договора с начала года) даются агрегированно. Ближайший крупный проект — квартал «Тишинский бульвар» Sminex (Электрический пер., 1), связь с участком №8 не подтверждена. Площадь 0,3 га / ~10 000 м² — из исходных данных запроса, независимого подтверждения нет.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="30" customHeight="1">
+      <c r="A41" s="27" t="inlineStr">
         <is>
           <t>Источники: открытые публикации 2025–2026 (stroi.mos.ru, mos.ru, отраслевые СМИ, публичные Telegram-каналы). Закрытый канал t.me/c/3370602239 недоступен без членства — пост №1364 про ЗУ «Большой Тишинский, 8» подтверждён по открытым источникам.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:Q34"/>
+  <autoFilter ref="A3:Q39"/>
   <mergeCells count="3">
     <mergeCell ref="A2:Q2"/>
     <mergeCell ref="A1:Q1"/>
-    <mergeCell ref="A36:Q36"/>
+    <mergeCell ref="A41:Q41"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P4" r:id="rId1"/>
@@ -13396,6 +13741,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P32" r:id="rId29"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P33" r:id="rId30"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P34" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P35" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P36" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P37" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P38" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P39" r:id="rId36"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.2" footer="0.2"/>

</xml_diff>

<commit_message>
Deduplicate planning entries against sheet 2
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Bv8NELxW2W7udnb3XUFGS2
</commit_message>
<xml_diff>
--- a/docs/premium-cao/premium-zhk-cao.xlsx
+++ b/docs/premium-cao/premium-zhk-cao.xlsx
@@ -18,9 +18,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2. Строится'!$A$3:$P$51</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'2. Строится'!$3:$3</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'2. Строится'!$A$1:$P$53</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'3. Проектирование'!$A$3:$Q$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'3. Проектирование'!$A$3:$Q$36</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'3. Проектирование'!$3:$3</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'3. Проектирование'!$A$1:$Q$41</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'3. Проектирование'!$A$1:$Q$38</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -8906,7 +8906,7 @@
       </c>
       <c r="P19" s="4" t="inlineStr"/>
     </row>
-    <row r="20" ht="15" customHeight="1">
+    <row r="20" ht="24" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Клубный дом DUO (Дуо)</t>
@@ -8972,7 +8972,7 @@
       </c>
       <c r="P20" s="4" t="inlineStr">
         <is>
-          <t>инвестор V2Group; юрлицо СЗ Суплекс Технолоджис; cian: 2028</t>
+          <t>Софийская наб., усадьба Кокорева; в июне 2026 fee-девелопер Hutton вышел из проекта, площадка у V2 Group (Коммерсантъ); инвестор V2Group; юрлицо СЗ Суплекс Технолоджис; cian: 2028</t>
         </is>
       </c>
     </row>
@@ -11252,7 +11252,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q41"/>
+  <dimension ref="A1:Q38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -11711,17 +11711,17 @@
     <row r="9" ht="24" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Клубный дом Duo (Софийская набережная, усадьба Кокорева)</t>
+          <t>Клубный дом «Большая Никитская, 16» (R4S)</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Софийская набережная (бывшая усадьба Кокорева), напротив Кремля</t>
+          <t>Большая Никитская улица, 16 (реконструкция доходного дома, объект культурного наследия)</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Якиманка</t>
+          <t>Пресненский</t>
         </is>
       </c>
       <c r="D9" s="28" t="inlineStr">
@@ -11731,35 +11731,41 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>V2 Group (владелец площадки; fee-девелопер Hutton вышел из проекта в июне 2026)</t>
+          <t>R4S Group (генподрядчик — Спецжилремонт)</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>строительство завершается; сдача II кв. 2026, выдача ключей до конца декабря 2026; продано ~27%; ищется новый партнер</t>
-        </is>
-      </c>
-      <c r="G9" s="7" t="n">
-        <v>18700</v>
-      </c>
+          <t>реконструкция; старт продаж I кв. 2026; ввод III кв. 2026</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="n"/>
       <c r="H9" s="5" t="n"/>
-      <c r="I9" s="5" t="n"/>
-      <c r="J9" s="5" t="n"/>
-      <c r="K9" s="5" t="n"/>
-      <c r="L9" s="4" t="inlineStr">
-        <is>
-          <t>2026 Q2 (ключи — декабрь 2026)</t>
+      <c r="I9" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="J9" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t>2026 Q1 (старт продаж)</t>
+        </is>
+      </c>
+      <c r="L9" s="5" t="inlineStr">
+        <is>
+          <t>2026 Q3</t>
         </is>
       </c>
       <c r="M9" s="5" t="n"/>
       <c r="N9" s="5" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="O9" s="4" t="inlineStr">
         <is>
-          <t>Коммерсантъ (17.06.2026)</t>
+          <t>Novostroev.ru (19.01.2026); sosedi.life</t>
         </is>
       </c>
       <c r="P9" s="8" t="inlineStr">
@@ -11769,19 +11775,19 @@
       </c>
       <c r="Q9" s="4" t="inlineStr">
         <is>
-          <t>Не новая очередь Golden Island, а смена управляющего девелопера на Софийской набережной: Hutton (И. Давыдик, А. Антонов) вышел из проекта; собственник V2 Group (В. Фоминых, В. Грознов) купил площадку у MR Group в 2023 за ~4,5–5 млрд руб. Новых очередей «Золотого острова» (Capital Group, ЖК «Золотой») в 2025–2026 не анонсировано.</t>
+          <t>Единственная публичная новинка на Большой Никитской в 2025–2026: 4 квартиры 139,4 / 141,4 / 151 / 234 м². Другие участки на Большой Никитской в открытых анонсах не найдены.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Клубный дом «Большая Никитская, 16» (R4S)</t>
+          <t>Клубный дом «Малая Никитская, 27»</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Большая Никитская улица, 16 (реконструкция доходного дома, объект культурного наследия)</t>
+          <t>Малая Никитская улица, 27 (два двухэтажных особняка 1861 г., бывший «Клуб 27»)</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -11796,41 +11802,31 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>R4S Group (генподрядчик — Спецжилремонт)</t>
+          <t>не раскрыт (по данным форума pronovostroy.ru — Mono/ПИК; официально не подтверждено)</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>реконструкция; старт продаж I кв. 2026; ввод III кв. 2026</t>
+          <t>проект на согласовании (высотность 33 м); продажи не открыты</t>
         </is>
       </c>
       <c r="G10" s="5" t="n"/>
       <c r="H10" s="5" t="n"/>
-      <c r="I10" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="J10" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="K10" s="4" t="inlineStr">
-        <is>
-          <t>2026 Q1 (старт продаж)</t>
-        </is>
-      </c>
-      <c r="L10" s="5" t="inlineStr">
-        <is>
-          <t>2026 Q3</t>
-        </is>
-      </c>
-      <c r="M10" s="5" t="n"/>
+      <c r="I10" s="5" t="n"/>
+      <c r="J10" s="5" t="n"/>
+      <c r="K10" s="5" t="n"/>
+      <c r="L10" s="5" t="n"/>
+      <c r="M10" s="7" t="n">
+        <v>3000000</v>
+      </c>
       <c r="N10" s="5" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2024-03-31</t>
         </is>
       </c>
       <c r="O10" s="4" t="inlineStr">
         <is>
-          <t>Novostroev.ru (19.01.2026); sosedi.life</t>
+          <t>Москвич Mag (31.03.2024); sosedi.life (07.04.2026); pronovostroy.ru</t>
         </is>
       </c>
       <c r="P10" s="8" t="inlineStr">
@@ -11840,24 +11836,24 @@
       </c>
       <c r="Q10" s="4" t="inlineStr">
         <is>
-          <t>Единственная публичная новинка на Большой Никитской в 2025–2026: 4 квартиры 139,4 / 141,4 / 151 / 234 м². Другие участки на Большой Никитской в открытых анонсах не найдены.</t>
+          <t>Клубный дом высотой 33 м по проекту бюро WALL на месте двух двухэтажных особняков (бывший отель Club 27). Ориентировочная цена «от ~3 млн руб./м²» — оценка источника, не подтверждена застройщиком. В базе mskdeluxe.ru фигурирует как «Малая Никитская, 29-31».; Архитектура — бюро WALL (ярусные объемы, черно-белые фасады). Существующие здания ~4 000 м² сносятся. Цена ~3 млн руб./м² — предварительное рыночное ожидание (sosedi.life, https://sosedi.life/news/zhk-malaya-nikitskaya-27/), не оферта. Restate.ru (2025–2026) отмечал неопределенность со стартом: возможна продажа площадки вместо запуска.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Клубный дом «Малая Никитская, 27»</t>
+          <t>Малая Дмитровка, 5/9</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Малая Никитская улица, 27 (два двухэтажных особняка 1861 г., бывший «Клуб 27»)</t>
+          <t>ул. Малая Дмитровка, 5/9</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Пресненский</t>
+          <t>Тверской</t>
         </is>
       </c>
       <c r="D11" s="28" t="inlineStr">
@@ -11865,33 +11861,35 @@
           <t>Садовое кольцо</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>не раскрыт (по данным форума pronovostroy.ru — Mono/ПИК; официально не подтверждено)</t>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Группа «Эталон»</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>проект на согласовании (высотность 33 м); продажи не открыты</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="n"/>
+          <t>анонсирован, старт продаж ожидается в 2026 г.</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="n">
+        <v>12000</v>
+      </c>
       <c r="H11" s="5" t="n"/>
-      <c r="I11" s="5" t="n"/>
+      <c r="I11" s="7" t="n">
+        <v>9</v>
+      </c>
       <c r="J11" s="5" t="n"/>
-      <c r="K11" s="5" t="n"/>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
       <c r="L11" s="5" t="n"/>
-      <c r="M11" s="7" t="n">
-        <v>3000000</v>
-      </c>
-      <c r="N11" s="5" t="inlineStr">
-        <is>
-          <t>2024-03-31</t>
-        </is>
-      </c>
+      <c r="M11" s="5" t="n"/>
+      <c r="N11" s="5" t="n"/>
       <c r="O11" s="4" t="inlineStr">
         <is>
-          <t>Москвич Mag (31.03.2024); sosedi.life (07.04.2026); pronovostroy.ru</t>
+          <t>sosedi.life (также mskdeluxe.ru/start, anwin.ru)</t>
         </is>
       </c>
       <c r="P11" s="8" t="inlineStr">
@@ -11901,24 +11899,24 @@
       </c>
       <c r="Q11" s="4" t="inlineStr">
         <is>
-          <t>Клубный дом высотой 33 м по проекту бюро WALL на месте двух двухэтажных особняков (бывший отель Club 27). Ориентировочная цена «от ~3 млн руб./м²» — оценка источника, не подтверждена застройщиком. В базе mskdeluxe.ru фигурирует как «Малая Никитская, 29-31».; Архитектура — бюро WALL (ярусные объемы, черно-белые фасады). Существующие здания ~4 000 м² сносятся. Цена ~3 млн руб./м² — предварительное рыночное ожидание (sosedi.life, https://sosedi.life/news/zhk-malaya-nikitskaya-27/), не оферта. Restate.ru (2025–2026) отмечал неопределенность со стартом: возможна продажа площадки вместо запуска.</t>
+          <t>Участок ~0,4 га у сада «Эрмитаж», 2 корпуса 7–9 этажей, волнообразные фасады, делюкс-класс.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="24" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Малая Дмитровка, 5/9</t>
+          <t>Малая Никитская, 29–31 (ожидаемый делюкс-старт)</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>ул. Малая Дмитровка, 5/9</t>
+          <t>Малая Никитская улица, 29–31</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Тверской</t>
+          <t>Пресненский</t>
         </is>
       </c>
       <c r="D12" s="28" t="inlineStr">
@@ -11928,33 +11926,25 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Группа «Эталон»</t>
+          <t>не раскрыт</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>анонсирован, старт продаж ожидается в 2026 г.</t>
-        </is>
-      </c>
-      <c r="G12" s="7" t="n">
-        <v>12000</v>
-      </c>
+          <t>в списке ожидаемых стартов делюкс-класса 2026 (агрегатор); подробностей нет</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="n"/>
       <c r="H12" s="5" t="n"/>
-      <c r="I12" s="7" t="n">
-        <v>9</v>
-      </c>
+      <c r="I12" s="5" t="n"/>
       <c r="J12" s="5" t="n"/>
-      <c r="K12" s="5" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
+      <c r="K12" s="5" t="n"/>
       <c r="L12" s="5" t="n"/>
       <c r="M12" s="5" t="n"/>
       <c r="N12" s="5" t="n"/>
       <c r="O12" s="4" t="inlineStr">
         <is>
-          <t>sosedi.life (также mskdeluxe.ru/start, anwin.ru)</t>
+          <t>mskdeluxe.ru (список стартов делюкс 2026)</t>
         </is>
       </c>
       <c r="P12" s="8" t="inlineStr">
@@ -11964,24 +11954,24 @@
       </c>
       <c r="Q12" s="4" t="inlineStr">
         <is>
-          <t>Участок ~0,4 га у сада «Эрмитаж», 2 корпуса 7–9 этажей, волнообразные фасады, делюкс-класс.</t>
+          <t>В том же списке mskdeluxe.ru: М. Дмитровка 5/9, Льва Толстого 14, Хилков 3, Б. Пироговская 51, Б. Харитоньевский 13, Олсуфьевский 10, Большая Ордынка 25, Воздвиженка 7/6, Малая Полянка 3 — без параметров и девелоперов.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="24" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Малая Дмитровка, 5/9 (ожидаемый делюкс-старт)</t>
+          <t>Малая Ордынка, 14/1</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Малая Дмитровка, 5/9</t>
+          <t>ул. Малая Ордынка, 14/1</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Тверской</t>
+          <t>Замоскворечье</t>
         </is>
       </c>
       <c r="D13" s="28" t="inlineStr">
@@ -11991,25 +11981,39 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>не раскрыт</t>
+          <t>Гута-Девелопмент</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>в списке ожидаемых стартов делюкс-класса 2026 (агрегатор); подробностей нет</t>
-        </is>
-      </c>
-      <c r="G13" s="5" t="n"/>
+          <t>старт продаж 06.04.2026</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="n">
+        <v>3000</v>
+      </c>
       <c r="H13" s="5" t="n"/>
-      <c r="I13" s="5" t="n"/>
-      <c r="J13" s="5" t="n"/>
-      <c r="K13" s="5" t="n"/>
+      <c r="I13" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="J13" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
       <c r="L13" s="5" t="n"/>
       <c r="M13" s="5" t="n"/>
-      <c r="N13" s="5" t="n"/>
+      <c r="N13" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
       <c r="O13" s="4" t="inlineStr">
         <is>
-          <t>mskdeluxe.ru (список стартов делюкс 2026)</t>
+          <t>sosedi.life (также novostroev.ru обзор делюкс-стартов 2026)</t>
         </is>
       </c>
       <c r="P13" s="8" t="inlineStr">
@@ -12019,24 +12023,24 @@
       </c>
       <c r="Q13" s="4" t="inlineStr">
         <is>
-          <t>Единственное упоминание новой площадки в зоне Петровка/Дмитровка; по Петровке и Большой Дмитровке в 2025–2026 новых анонсов не найдено (только реализуемые «Советник» (Insigma) и Petrovsky).</t>
+          <t>Участок 0,1 га, 11 квартир, 14 подземных м/м, архитектура A2M. Делюкс.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Малая Никитская, 29–31 (ожидаемый делюкс-старт)</t>
+          <t>Палашёвский 11 (Большой Палашёвский, 11–13/15)</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Малая Никитская улица, 29–31</t>
+          <t>Большой Палашёвский пер., 11–13</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Пресненский</t>
+          <t>Тверской</t>
         </is>
       </c>
       <c r="D14" s="28" t="inlineStr">
@@ -12044,27 +12048,47 @@
           <t>Садовое кольцо</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>не раскрыт</t>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Sminex (СЗ «Смайнэкс Палашёвский 11»)</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>в списке ожидаемых стартов делюкс-класса 2026 (агрегатор); подробностей нет</t>
-        </is>
-      </c>
-      <c r="G14" s="5" t="n"/>
+          <t>старт продаж без стройки (закрытый старт 22.04.2026)</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="n">
+        <v>15600</v>
+      </c>
       <c r="H14" s="5" t="n"/>
-      <c r="I14" s="5" t="n"/>
-      <c r="J14" s="5" t="n"/>
-      <c r="K14" s="5" t="n"/>
-      <c r="L14" s="5" t="n"/>
-      <c r="M14" s="5" t="n"/>
-      <c r="N14" s="5" t="n"/>
-      <c r="O14" s="4" t="inlineStr">
-        <is>
-          <t>mskdeluxe.ru (список стартов делюкс 2026)</t>
+      <c r="I14" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="J14" s="7" t="n">
+        <v>43</v>
+      </c>
+      <c r="K14" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="L14" s="5" t="inlineStr">
+        <is>
+          <t>1 кв. 2030</t>
+        </is>
+      </c>
+      <c r="M14" s="7" t="n">
+        <v>3500000</v>
+      </c>
+      <c r="N14" s="5" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="O14" s="5" t="inlineStr">
+        <is>
+          <t>novostroev.ru</t>
         </is>
       </c>
       <c r="P14" s="8" t="inlineStr">
@@ -12074,24 +12098,24 @@
       </c>
       <c r="Q14" s="4" t="inlineStr">
         <is>
-          <t>В том же списке mskdeluxe.ru: М. Дмитровка 5/9, Льва Толстого 14, Хилков 3, Б. Пироговская 51, Б. Харитоньевский 13, Олсуфьевский 10, Большая Ордынка 25, Воздвиженка 7/6, Малая Полянка 3 — без параметров и девелоперов.</t>
+          <t>Три корпуса 8–9 этажей с контрастными фасадами у Патриарших. Старт продаж 22.04.2026, лоты от 222,4 млн руб. (nngm.ru), от ~3,5 млн руб./м². Сдача 1 кв. 2030 (novostroev.ru, обзор делюкс-стартов 2026).</t>
         </is>
       </c>
     </row>
     <row r="15" ht="24" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Малая Ордынка, 14/1</t>
+          <t>Полянка-3</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>ул. Малая Ордынка, 14/1</t>
+          <t>ул. Малая Полянка, 3</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Замоскворечье</t>
+          <t>Якиманка</t>
         </is>
       </c>
       <c r="D15" s="28" t="inlineStr">
@@ -12099,41 +12123,35 @@
           <t>Садовое кольцо</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>Гута-Девелопмент</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>старт продаж 06.04.2026</t>
-        </is>
-      </c>
-      <c r="G15" s="7" t="n">
-        <v>3000</v>
-      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Aurix Development (Группа «Эталон»)</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>старт продаж 2026</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="n"/>
       <c r="H15" s="5" t="n"/>
       <c r="I15" s="7" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="K15" s="5" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="L15" s="5" t="n"/>
       <c r="M15" s="5" t="n"/>
-      <c r="N15" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-06</t>
-        </is>
-      </c>
+      <c r="N15" s="5" t="n"/>
       <c r="O15" s="4" t="inlineStr">
         <is>
-          <t>sosedi.life (также novostroev.ru обзор делюкс-стартов 2026)</t>
+          <t>официальный сайт проекта (также mskdeluxe.ru/start)</t>
         </is>
       </c>
       <c r="P15" s="8" t="inlineStr">
@@ -12143,24 +12161,24 @@
       </c>
       <c r="Q15" s="4" t="inlineStr">
         <is>
-          <t>Участок 0,1 га, 11 квартир, 14 подземных м/м, архитектура A2M. Делюкс.</t>
+          <t>9 этажей, 34 квартиры, паркинг на 36 м/м, проект Etalon Project. Продажи открыты в 2026 г.; стадия строительства в открытых источниках не уточнена.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Палашёвский 11 (Большой Палашёвский, 11–13/15)</t>
+          <t>Роден (ранее анонсировался как Veil)</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Большой Палашёвский пер., 11–13</t>
+          <t>Большой Харитоньевский пер., 13А</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Тверской</t>
+          <t>Басманный</t>
         </is>
       </c>
       <c r="D16" s="28" t="inlineStr">
@@ -12168,47 +12186,37 @@
           <t>Садовое кольцо</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>Sminex (СЗ «Смайнэкс Палашёвский 11»)</t>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>MR Group</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>старт продаж без стройки (закрытый старт 22.04.2026)</t>
-        </is>
-      </c>
-      <c r="G16" s="7" t="n">
-        <v>15600</v>
-      </c>
+          <t>старт продаж июль–август 2026</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="n"/>
       <c r="H16" s="5" t="n"/>
       <c r="I16" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="J16" s="7" t="n">
-        <v>43</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="J16" s="5" t="n"/>
       <c r="K16" s="5" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
-        </is>
-      </c>
-      <c r="L16" s="5" t="inlineStr">
-        <is>
-          <t>1 кв. 2030</t>
-        </is>
-      </c>
-      <c r="M16" s="7" t="n">
-        <v>3500000</v>
-      </c>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="L16" s="5" t="n"/>
+      <c r="M16" s="5" t="n"/>
       <c r="N16" s="5" t="inlineStr">
         <is>
-          <t>2026-04</t>
-        </is>
-      </c>
-      <c r="O16" s="5" t="inlineStr">
-        <is>
-          <t>novostroev.ru</t>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="O16" s="4" t="inlineStr">
+        <is>
+          <t>novostroev.ru (также roden.moscow)</t>
         </is>
       </c>
       <c r="P16" s="8" t="inlineStr">
@@ -12218,24 +12226,24 @@
       </c>
       <c r="Q16" s="4" t="inlineStr">
         <is>
-          <t>Три корпуса 8–9 этажей с контрастными фасадами у Патриарших. Старт продаж 22.04.2026, лоты от 222,4 млн руб. (nngm.ru), от ~3,5 млн руб./м². Сдача 1 кв. 2030 (novostroev.ru, обзор делюкс-стартов 2026).</t>
+          <t>Клубный дом делюкс-класса у Чистых прудов, 1 монолитный корпус 7 этажей, архитектура WALL. В обзоре делюкс-стартов 2026 novostroev.ru фигурировал как Veil, 9 этажей.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Полянка-3</t>
+          <t>Рождественка 8</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>ул. Малая Полянка, 3</t>
+          <t>ул. Рождественка / Кузнецкий Мост / Варсонофьевский пер.</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Якиманка</t>
+          <t>Мещанский</t>
         </is>
       </c>
       <c r="D17" s="28" t="inlineStr">
@@ -12245,33 +12253,37 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Aurix Development (Группа «Эталон»)</t>
-        </is>
-      </c>
-      <c r="F17" s="5" t="inlineStr">
-        <is>
-          <t>старт продаж 2026</t>
-        </is>
-      </c>
-      <c r="G17" s="5" t="n"/>
-      <c r="H17" s="5" t="n"/>
+          <t>Sminex (проект выкуплен у «Галс-Девелопмент»)</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>проект приобретён, старт продаж ожидается</t>
+        </is>
+      </c>
+      <c r="G17" s="7" t="n">
+        <v>36400</v>
+      </c>
+      <c r="H17" s="7" t="n">
+        <v>18000</v>
+      </c>
       <c r="I17" s="7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>34</v>
-      </c>
-      <c r="K17" s="5" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
+        <v>115</v>
+      </c>
+      <c r="K17" s="5" t="n"/>
       <c r="L17" s="5" t="n"/>
       <c r="M17" s="5" t="n"/>
-      <c r="N17" s="5" t="n"/>
+      <c r="N17" s="5" t="inlineStr">
+        <is>
+          <t>2025-12-12</t>
+        </is>
+      </c>
       <c r="O17" s="4" t="inlineStr">
         <is>
-          <t>официальный сайт проекта (также mskdeluxe.ru/start)</t>
+          <t>РИА Недвижимость (также kommersant.ru/doc/8291907, cre.ru)</t>
         </is>
       </c>
       <c r="P17" s="8" t="inlineStr">
@@ -12281,24 +12293,24 @@
       </c>
       <c r="Q17" s="4" t="inlineStr">
         <is>
-          <t>9 этажей, 34 квартиры, паркинг на 36 м/м, проект Etalon Project. Продажи открыты в 2026 г.; стадия строительства в открытых источниках не уточнена.</t>
+          <t>Семь корпусов 2–10 этажей, 115 квартир 61–426 м², таунхаусы и пентхаусы, двор-парк Scape, реставрация особняка конца XIX в. Сделка 12.12.2025.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Роден (ранее анонсировался как Veil)</t>
+          <t>Типография Сытина (Пятницкая, 71/5)</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Большой Харитоньевский пер., 13А</t>
+          <t>ул. Пятницкая, 71/5 (2-й Монетчиковский пер., 5)</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Басманный</t>
+          <t>Замоскворечье</t>
         </is>
       </c>
       <c r="D18" s="28" t="inlineStr">
@@ -12308,35 +12320,29 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>MR Group</t>
+          <t>Sminex</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>старт продаж июль–август 2026</t>
+          <t>участок приобретён (март 2026), проектирование</t>
         </is>
       </c>
       <c r="G18" s="5" t="n"/>
       <c r="H18" s="5" t="n"/>
-      <c r="I18" s="7" t="n">
-        <v>7</v>
-      </c>
+      <c r="I18" s="5" t="n"/>
       <c r="J18" s="5" t="n"/>
-      <c r="K18" s="5" t="inlineStr">
-        <is>
-          <t>2026-07</t>
-        </is>
-      </c>
+      <c r="K18" s="5" t="n"/>
       <c r="L18" s="5" t="n"/>
       <c r="M18" s="5" t="n"/>
       <c r="N18" s="5" t="inlineStr">
         <is>
-          <t>2026-07</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="O18" s="4" t="inlineStr">
         <is>
-          <t>novostroev.ru (также roden.moscow)</t>
+          <t>РИА Недвижимость (также sminex.com, mperspektiva.ru)</t>
         </is>
       </c>
       <c r="P18" s="8" t="inlineStr">
@@ -12346,145 +12352,141 @@
       </c>
       <c r="Q18" s="4" t="inlineStr">
         <is>
-          <t>Клубный дом делюкс-класса у Чистых прудов, 1 монолитный корпус 7 этажей, архитектура WALL. В обзоре делюкс-стартов 2026 novostroev.ru фигурировал как Veil, 9 этажей.</t>
+          <t>Участок 1,8 га, 8 зданий 38,5 тыс. м², в т.ч. 3 корпуса типографии Сытина (ОКН, арх. Эрихсон/Шухов). Продавец — В. Погребенко, оценка сделки 12–14 млрд руб., инвестиции 25–30 млрд руб. План: реставрация + новые элитные клубные дома. Участок у Садового кольца (Валовая ул.).</t>
         </is>
       </c>
     </row>
     <row r="19" ht="24" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>Рождественка 8</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>ул. Рождественка / Кузнецкий Мост / Варсонофьевский пер.</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>Мещанский</t>
-        </is>
-      </c>
-      <c r="D19" s="28" t="inlineStr">
-        <is>
-          <t>Садовое кольцо</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>Sminex (проект выкуплен у «Галс-Девелопмент»)</t>
-        </is>
-      </c>
-      <c r="F19" s="4" t="inlineStr">
-        <is>
-          <t>проект приобретён, старт продаж ожидается</t>
-        </is>
-      </c>
-      <c r="G19" s="7" t="n">
-        <v>36400</v>
-      </c>
-      <c r="H19" s="7" t="n">
-        <v>18000</v>
-      </c>
-      <c r="I19" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="J19" s="7" t="n">
-        <v>115</v>
-      </c>
-      <c r="K19" s="5" t="n"/>
-      <c r="L19" s="5" t="n"/>
-      <c r="M19" s="5" t="n"/>
-      <c r="N19" s="5" t="inlineStr">
-        <is>
-          <t>2025-12-12</t>
-        </is>
-      </c>
-      <c r="O19" s="4" t="inlineStr">
-        <is>
-          <t>РИА Недвижимость (также kommersant.ru/doc/8291907, cre.ru)</t>
-        </is>
-      </c>
-      <c r="P19" s="8" t="inlineStr">
-        <is>
-          <t>ссылка</t>
-        </is>
-      </c>
-      <c r="Q19" s="4" t="inlineStr">
-        <is>
-          <t>Семь корпусов 2–10 этажей, 115 квартир 61–426 м², таунхаусы и пентхаусы, двор-парк Scape, реставрация особняка конца XIX в. Сделка 12.12.2025.</t>
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>Большая Пироговская, 51 (общежития Института красной профессуры)</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>ул. Большая Пироговская, 51</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>Хамовники</t>
+        </is>
+      </c>
+      <c r="D19" s="29" t="inlineStr">
+        <is>
+          <t>Хамовники</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>Vesper (fee-девелопер) / собственник Capital Group</t>
+        </is>
+      </c>
+      <c r="F19" s="9" t="inlineStr">
+        <is>
+          <t>анонсирован (fee-development), концепция</t>
+        </is>
+      </c>
+      <c r="G19" s="12" t="n">
+        <v>46700</v>
+      </c>
+      <c r="H19" s="10" t="n"/>
+      <c r="I19" s="10" t="n"/>
+      <c r="J19" s="10" t="n"/>
+      <c r="K19" s="10" t="n"/>
+      <c r="L19" s="10" t="n"/>
+      <c r="M19" s="10" t="n"/>
+      <c r="N19" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="O19" s="9" t="inlineStr">
+        <is>
+          <t>РИА Недвижимость (также vedomosti.ru 18.06.2026)</t>
+        </is>
+      </c>
+      <c r="P19" s="13" t="inlineStr">
+        <is>
+          <t>ссылка</t>
+        </is>
+      </c>
+      <c r="Q19" s="9" t="inlineStr">
+        <is>
+          <t>Участок 1,5 га, ансамбль восьми 6-этажных корпусов 1929–32 гг. (арх. Осипов, Рухлядев; статус памятника утрачен в 2000-х). Планируемая площадь выросла с 39 до 46,7 тыс. м². Vesper — концепция, продукт и управление реализацией. В базе mskdeluxe.ru — «Б.Пироговская, 51».</t>
         </is>
       </c>
     </row>
     <row r="20" ht="24" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>Типография Сытина (Пятницкая, 71/5)</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>ул. Пятницкая, 71/5 (2-й Монетчиковский пер., 5)</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>Замоскворечье</t>
-        </is>
-      </c>
-      <c r="D20" s="28" t="inlineStr">
-        <is>
-          <t>Садовое кольцо</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="inlineStr">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>Квартал на Савинской набережной («Московский шёлк»)</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>Савинская наб. (территория БЦ «Московский шёлк»)</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>Хамовники</t>
+        </is>
+      </c>
+      <c r="D20" s="29" t="inlineStr">
+        <is>
+          <t>Хамовники</t>
+        </is>
+      </c>
+      <c r="E20" s="10" t="inlineStr">
         <is>
           <t>Sminex</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr">
-        <is>
-          <t>участок приобретён (март 2026), проектирование</t>
-        </is>
-      </c>
-      <c r="G20" s="5" t="n"/>
-      <c r="H20" s="5" t="n"/>
-      <c r="I20" s="5" t="n"/>
-      <c r="J20" s="5" t="n"/>
-      <c r="K20" s="5" t="n"/>
-      <c r="L20" s="5" t="n"/>
-      <c r="M20" s="5" t="n"/>
-      <c r="N20" s="5" t="inlineStr">
-        <is>
-          <t>2026-03-17</t>
-        </is>
-      </c>
-      <c r="O20" s="4" t="inlineStr">
-        <is>
-          <t>РИА Недвижимость (также sminex.com, mperspektiva.ru)</t>
-        </is>
-      </c>
-      <c r="P20" s="8" t="inlineStr">
-        <is>
-          <t>ссылка</t>
-        </is>
-      </c>
-      <c r="Q20" s="4" t="inlineStr">
-        <is>
-          <t>Участок 1,8 га, 8 зданий 38,5 тыс. м², в т.ч. 3 корпуса типографии Сытина (ОКН, арх. Эрихсон/Шухов). Продавец — В. Погребенко, оценка сделки 12–14 млрд руб., инвестиции 25–30 млрд руб. План: реставрация + новые элитные клубные дома. Участок у Садового кольца (Валовая ул.).</t>
+      <c r="F20" s="10" t="inlineStr">
+        <is>
+          <t>проектирование</t>
+        </is>
+      </c>
+      <c r="G20" s="12" t="n">
+        <v>125000</v>
+      </c>
+      <c r="H20" s="10" t="n"/>
+      <c r="I20" s="10" t="n"/>
+      <c r="J20" s="10" t="n"/>
+      <c r="K20" s="10" t="n"/>
+      <c r="L20" s="10" t="n"/>
+      <c r="M20" s="10" t="n"/>
+      <c r="N20" s="10" t="inlineStr">
+        <is>
+          <t>2024-03-12</t>
+        </is>
+      </c>
+      <c r="O20" s="9" t="inlineStr">
+        <is>
+          <t>РИА Недвижимость (стадия подтверждена mperspektiva.ru 18.12.2025)</t>
+        </is>
+      </c>
+      <c r="P20" s="13" t="inlineStr">
+        <is>
+          <t>ссылка</t>
+        </is>
+      </c>
+      <c r="Q20" s="9" t="inlineStr">
+        <is>
+          <t>ЖК ~125 тыс. м² на территории делового квартала «Московский шёлк». По данным Sminex на декабрь 2025 г. находится в стадии проектирования (вместе с Лужнецкой).</t>
         </is>
       </c>
     </row>
     <row r="21" ht="24" customHeight="1">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>Большая Пироговская, 51 (общежития Института красной профессуры)</t>
+          <t>Клубный дом «Земледельческий, 15»</t>
         </is>
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>ул. Большая Пироговская, 51</t>
+          <t>Земледельческий переулок, 15 (на месте административного здания 1975 г., 5 этажей, 5 744 м²)</t>
         </is>
       </c>
       <c r="C21" s="10" t="inlineStr">
@@ -12497,33 +12499,39 @@
           <t>Хамовники</t>
         </is>
       </c>
-      <c r="E21" s="9" t="inlineStr">
-        <is>
-          <t>Vesper (fee-девелопер) / собственник Capital Group</t>
+      <c r="E21" s="10" t="inlineStr">
+        <is>
+          <t>не раскрыт</t>
         </is>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
-          <t>анонсирован (fee-development), концепция</t>
+          <t>проектирование (агрегаторы; в списке ожидаемых стартов делюкс-класса 2026 на mskdeluxe.ru)</t>
         </is>
       </c>
       <c r="G21" s="12" t="n">
-        <v>46700</v>
+        <v>8000</v>
       </c>
       <c r="H21" s="10" t="n"/>
       <c r="I21" s="10" t="n"/>
-      <c r="J21" s="10" t="n"/>
-      <c r="K21" s="10" t="n"/>
+      <c r="J21" s="12" t="n">
+        <v>77</v>
+      </c>
+      <c r="K21" s="10" t="inlineStr">
+        <is>
+          <t>2026–2027</t>
+        </is>
+      </c>
       <c r="L21" s="10" t="n"/>
       <c r="M21" s="10" t="n"/>
       <c r="N21" s="10" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="O21" s="9" t="inlineStr">
         <is>
-          <t>РИА Недвижимость (также vedomosti.ru 18.06.2026)</t>
+          <t>kvartiravmoskve.ru (обновлено 21.06.2026); mskdeluxe.ru/start</t>
         </is>
       </c>
       <c r="P21" s="13" t="inlineStr">
@@ -12533,58 +12541,54 @@
       </c>
       <c r="Q21" s="9" t="inlineStr">
         <is>
-          <t>Участок 1,5 га, ансамбль восьми 6-этажных корпусов 1929–32 гг. (арх. Осипов, Рухлядев; статус памятника утрачен в 2000-х). Планируемая площадь выросла с 39 до 46,7 тыс. м². Vesper — концепция, продукт и управление реализацией. В базе mskdeluxe.ru — «Б.Пироговская, 51».</t>
+          <t>Участок 0,3 га (сейчас административное здание 1975 г., 5 эт., 5,7 тыс. м²), клубный дом ~8 тыс. м², 77 квартир, коммерция, подземный паркинг. Делюкс.; Участок 0,3 га; делюкс; 77 квартир + коммерческая часть; подземный паркинг; монолит-кирпич; 1 км до м. Смоленская. Сделок по продаже БЦ и решений Москомархитектуры в открытых источниках не найдено.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="24" customHeight="1">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>Квартал на Савинской набережной («Московский шёлк»)</t>
+          <t>Клубный дом на Курсовом переулке, 15 (проект бюро Дмитрия Великовского)</t>
         </is>
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>Савинская наб. (территория БЦ «Московский шёлк»)</t>
-        </is>
-      </c>
-      <c r="C22" s="10" t="inlineStr">
+          <t>Курсовой переулок, 15</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>Хамовники (Остоженка)</t>
+        </is>
+      </c>
+      <c r="D22" s="29" t="inlineStr">
         <is>
           <t>Хамовники</t>
         </is>
       </c>
-      <c r="D22" s="29" t="inlineStr">
-        <is>
-          <t>Хамовники</t>
-        </is>
-      </c>
-      <c r="E22" s="10" t="inlineStr">
-        <is>
-          <t>Sminex</t>
-        </is>
-      </c>
-      <c r="F22" s="10" t="inlineStr">
-        <is>
-          <t>проектирование</t>
-        </is>
-      </c>
-      <c r="G22" s="12" t="n">
-        <v>125000</v>
-      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>не раскрыт (проект бюро Дмитрия Великовского)</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>проект / предстарт; в открытых источниках только страница агрегатора</t>
+        </is>
+      </c>
+      <c r="G22" s="10" t="n"/>
       <c r="H22" s="10" t="n"/>
-      <c r="I22" s="10" t="n"/>
+      <c r="I22" s="12" t="n">
+        <v>6</v>
+      </c>
       <c r="J22" s="10" t="n"/>
       <c r="K22" s="10" t="n"/>
       <c r="L22" s="10" t="n"/>
       <c r="M22" s="10" t="n"/>
-      <c r="N22" s="10" t="inlineStr">
-        <is>
-          <t>2024-03-12</t>
-        </is>
-      </c>
+      <c r="N22" s="10" t="n"/>
       <c r="O22" s="9" t="inlineStr">
         <is>
-          <t>РИА Недвижимость (стадия подтверждена mperspektiva.ru 18.12.2025)</t>
+          <t>Anwin (агрегатор элитной недвижимости)</t>
         </is>
       </c>
       <c r="P22" s="13" t="inlineStr">
@@ -12594,19 +12598,19 @@
       </c>
       <c r="Q22" s="9" t="inlineStr">
         <is>
-          <t>ЖК ~125 тыс. м² на территории делового квартала «Московский шёлк». По данным Sminex на декабрь 2025 г. находится в стадии проектирования (вместе с Лужнецкой).</t>
+          <t>«Золотая миля», 6 этажей, камерный клубный дом. Подробные параметры и застройщик в открытых источниках не раскрыты.; По описанию агрегатора: 6-этажный дом по проекту бюро Дмитрия Великовского, панорамное остекление, локация «Золотой мили» рядом с Зачатьевским монастырем. Сейчас по адресу — детский клуб-студия «Пречистенские ворота». Пресса (Коммерсант, РБК, Ведомости, Москвич Mag) и Москомархитектура публикаций по площадке не имеют; девелопер и параметры не подтверждены.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="24" customHeight="1">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>Клубный дом «Земледельческий, 15»</t>
+          <t>Льва Толстого, 14–16 (три клубных дома Sminex)</t>
         </is>
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>Земледельческий переулок, 15 (на месте административного здания 1975 г., 5 этажей, 5 744 м²)</t>
+          <t>ул. Льва Толстого, 14</t>
         </is>
       </c>
       <c r="C23" s="10" t="inlineStr">
@@ -12621,37 +12625,33 @@
       </c>
       <c r="E23" s="10" t="inlineStr">
         <is>
-          <t>не раскрыт</t>
+          <t>Sminex</t>
         </is>
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
-          <t>проектирование (агрегаторы; в списке ожидаемых стартов делюкс-класса 2026 на mskdeluxe.ru)</t>
+          <t>участок приобретён (декабрь 2025), концепция в финальной стадии, старт продаж не объявлен</t>
         </is>
       </c>
       <c r="G23" s="12" t="n">
-        <v>8000</v>
-      </c>
-      <c r="H23" s="10" t="n"/>
+        <v>20300</v>
+      </c>
+      <c r="H23" s="12" t="n">
+        <v>12400</v>
+      </c>
       <c r="I23" s="10" t="n"/>
-      <c r="J23" s="12" t="n">
-        <v>77</v>
-      </c>
-      <c r="K23" s="10" t="inlineStr">
-        <is>
-          <t>2026–2027</t>
-        </is>
-      </c>
+      <c r="J23" s="10" t="n"/>
+      <c r="K23" s="10" t="n"/>
       <c r="L23" s="10" t="n"/>
       <c r="M23" s="10" t="n"/>
       <c r="N23" s="10" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2025-12-18</t>
         </is>
       </c>
       <c r="O23" s="9" t="inlineStr">
         <is>
-          <t>kvartiravmoskve.ru (обновлено 21.06.2026); mskdeluxe.ru/start</t>
+          <t>Московская перспектива (также rbc.ru 18.12.2025, sosedi.life 07.04.2026)</t>
         </is>
       </c>
       <c r="P23" s="13" t="inlineStr">
@@ -12661,24 +12661,24 @@
       </c>
       <c r="Q23" s="9" t="inlineStr">
         <is>
-          <t>Участок 0,3 га (сейчас административное здание 1975 г., 5 эт., 5,7 тыс. м²), клубный дом ~8 тыс. м², 77 квартир, коммерция, подземный паркинг. Делюкс.; Участок 0,3 га; делюкс; 77 квартир + коммерческая часть; подземный паркинг; монолит-кирпич; 1 км до м. Смоленская. Сделок по продаже БЦ и решений Москомархитектуры в открытых источниках не найдено.</t>
+          <t>Участок ~0,6 га у делового квартала «Красная Роза», куплен у структур А. Клячина. Три камерных клубных дома, надземная площадь 20,3 тыс. м², квартиры 12,4 тыс. м². Сохраняется фасад бывшего доходного дома Трындина-Жиро.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="24" customHeight="1">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>Клубный дом на Курсовом переулке, 15 (проект бюро Дмитрия Великовского)</t>
+          <t>Лёвшинский, 19</t>
         </is>
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>Курсовой переулок, 15</t>
-        </is>
-      </c>
-      <c r="C24" s="9" t="inlineStr">
-        <is>
-          <t>Хамовники (Остоженка)</t>
+          <t>Большой Лёвшинский пер., 19</t>
+        </is>
+      </c>
+      <c r="C24" s="10" t="inlineStr">
+        <is>
+          <t>Хамовники</t>
         </is>
       </c>
       <c r="D24" s="29" t="inlineStr">
@@ -12688,27 +12688,37 @@
       </c>
       <c r="E24" s="9" t="inlineStr">
         <is>
-          <t>не раскрыт (проект бюро Дмитрия Великовского)</t>
+          <t>ТСИ Девелопмент (ГК «Трансстройинвест»)</t>
         </is>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
-          <t>проект / предстарт; в открытых источниках только страница агрегатора</t>
+          <t>старт бронирования, старт продаж</t>
         </is>
       </c>
       <c r="G24" s="10" t="n"/>
       <c r="H24" s="10" t="n"/>
       <c r="I24" s="12" t="n">
-        <v>6</v>
-      </c>
-      <c r="J24" s="10" t="n"/>
-      <c r="K24" s="10" t="n"/>
-      <c r="L24" s="10" t="n"/>
+        <v>8</v>
+      </c>
+      <c r="J24" s="12" t="n">
+        <v>16</v>
+      </c>
+      <c r="K24" s="10" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L24" s="10" t="inlineStr">
+        <is>
+          <t>2 кв. 2028</t>
+        </is>
+      </c>
       <c r="M24" s="10" t="n"/>
       <c r="N24" s="10" t="n"/>
       <c r="O24" s="9" t="inlineStr">
         <is>
-          <t>Anwin (агрегатор элитной недвижимости)</t>
+          <t>whitewill.ru (также tehne.com, levshinsky-19.ru)</t>
         </is>
       </c>
       <c r="P24" s="13" t="inlineStr">
@@ -12718,19 +12728,19 @@
       </c>
       <c r="Q24" s="9" t="inlineStr">
         <is>
-          <t>«Золотая миля», 6 этажей, камерный клубный дом. Подробные параметры и застройщик в открытых источниках не раскрыты.; По описанию агрегатора: 6-этажный дом по проекту бюро Дмитрия Великовского, панорамное остекление, локация «Золотой мили» рядом с Зачатьевским монастырем. Сейчас по адресу — детский клуб-студия «Пречистенские ворота». Пресса (Коммерсант, РБК, Ведомости, Москвич Mag) и Москомархитектура публикаций по площадке не имеют; девелопер и параметры не подтверждены.</t>
+          <t>Воссоздание фасада доходного дома Духовских (1904, арх. Мейснер), проект HADAA Architects. 16 резиденций 70–239 м², паркинг 18 м/м. Цена от 197,12 млн руб. за лот. Стадия стройки в источниках не подтверждена.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="24" customHeight="1">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t>Льва Толстого, 14–16 (три клубных дома Sminex)</t>
+          <t>Олсуфьевский 10</t>
         </is>
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>ул. Льва Толстого, 14</t>
+          <t>Олсуфьевский пер., 10</t>
         </is>
       </c>
       <c r="C25" s="10" t="inlineStr">
@@ -12745,33 +12755,31 @@
       </c>
       <c r="E25" s="10" t="inlineStr">
         <is>
-          <t>Sminex</t>
+          <t>Грандор (Grandor)</t>
         </is>
       </c>
       <c r="F25" s="9" t="inlineStr">
         <is>
-          <t>участок приобретён (декабрь 2025), концепция в финальной стадии, старт продаж не объявлен</t>
-        </is>
-      </c>
-      <c r="G25" s="12" t="n">
-        <v>20300</v>
-      </c>
-      <c r="H25" s="12" t="n">
-        <v>12400</v>
-      </c>
-      <c r="I25" s="10" t="n"/>
+          <t>ГПЗУ получен (апрель 2021), старт продаж ожидается</t>
+        </is>
+      </c>
+      <c r="G25" s="10" t="n"/>
+      <c r="H25" s="10" t="n"/>
+      <c r="I25" s="12" t="n">
+        <v>8</v>
+      </c>
       <c r="J25" s="10" t="n"/>
-      <c r="K25" s="10" t="n"/>
+      <c r="K25" s="10" t="inlineStr">
+        <is>
+          <t>2026–2027</t>
+        </is>
+      </c>
       <c r="L25" s="10" t="n"/>
       <c r="M25" s="10" t="n"/>
-      <c r="N25" s="10" t="inlineStr">
-        <is>
-          <t>2025-12-18</t>
-        </is>
-      </c>
+      <c r="N25" s="10" t="n"/>
       <c r="O25" s="9" t="inlineStr">
         <is>
-          <t>Московская перспектива (также rbc.ru 18.12.2025, sosedi.life 07.04.2026)</t>
+          <t>официальный сайт проекта (также novostroy.ru, mskdeluxe.ru/start)</t>
         </is>
       </c>
       <c r="P25" s="13" t="inlineStr">
@@ -12781,19 +12789,19 @@
       </c>
       <c r="Q25" s="9" t="inlineStr">
         <is>
-          <t>Участок ~0,6 га у делового квартала «Красная Роза», куплен у структур А. Клячина. Три камерных клубных дома, надземная площадь 20,3 тыс. м², квартиры 12,4 тыс. м². Сохраняется фасад бывшего доходного дома Трындина-Жиро.</t>
+          <t>Участок 0,4 га, семь корпусов 5–8 этажей в индивидуальной архитектуре. В базе делюкс-стартов 2026–2027 mskdeluxe.ru.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="24" customHeight="1">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>Лёвшинский, 19</t>
+          <t>Премиальный квартал на Лужнецкой набережной, 10А</t>
         </is>
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>Большой Лёвшинский пер., 19</t>
+          <t>Лужнецкая наб., вл. 10А</t>
         </is>
       </c>
       <c r="C26" s="10" t="inlineStr">
@@ -12806,39 +12814,35 @@
           <t>Хамовники</t>
         </is>
       </c>
-      <c r="E26" s="9" t="inlineStr">
-        <is>
-          <t>ТСИ Девелопмент (ГК «Трансстройинвест»)</t>
+      <c r="E26" s="10" t="inlineStr">
+        <is>
+          <t>Sminex</t>
         </is>
       </c>
       <c r="F26" s="9" t="inlineStr">
         <is>
-          <t>старт бронирования, старт продаж</t>
+          <t>проект утверждён (АГР, май 2026), начало строительства 2027</t>
         </is>
       </c>
       <c r="G26" s="10" t="n"/>
       <c r="H26" s="10" t="n"/>
-      <c r="I26" s="12" t="n">
-        <v>8</v>
-      </c>
-      <c r="J26" s="12" t="n">
-        <v>16</v>
-      </c>
+      <c r="I26" s="10" t="n"/>
+      <c r="J26" s="10" t="n"/>
       <c r="K26" s="10" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="L26" s="10" t="inlineStr">
-        <is>
-          <t>2 кв. 2028</t>
-        </is>
-      </c>
+          <t>2027 (стройка)</t>
+        </is>
+      </c>
+      <c r="L26" s="10" t="n"/>
       <c r="M26" s="10" t="n"/>
-      <c r="N26" s="10" t="n"/>
+      <c r="N26" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
       <c r="O26" s="9" t="inlineStr">
         <is>
-          <t>whitewill.ru (также tehne.com, levshinsky-19.ru)</t>
+          <t>РИА Недвижимость (также anwin.ru)</t>
         </is>
       </c>
       <c r="P26" s="13" t="inlineStr">
@@ -12848,19 +12852,19 @@
       </c>
       <c r="Q26" s="9" t="inlineStr">
         <is>
-          <t>Воссоздание фасада доходного дома Духовских (1904, арх. Мейснер), проект HADAA Architects. 16 резиденций 70–239 м², паркинг 18 м/м. Цена от 197,12 млн руб. за лот. Стадия стройки в источниках не подтверждена.</t>
+          <t>Два жилых корпуса переменной этажности в неоклассике + эллиптический БЦ 26 тыс. м² («яйцо Фаберже»). Концепция согласована Департаментом градостроительной политики (В. Овчинский). Параметры жилой части не раскрыты.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="24" customHeight="1">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>Олсуфьевский 10</t>
+          <t>Тимура Фрунзе, 11 (клубный дом Sminex)</t>
         </is>
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>Олсуфьевский пер., 10</t>
+          <t>ул. Тимура Фрунзе, 11, стр. 7, 19, 33, 50</t>
         </is>
       </c>
       <c r="C27" s="10" t="inlineStr">
@@ -12875,31 +12879,33 @@
       </c>
       <c r="E27" s="10" t="inlineStr">
         <is>
-          <t>Грандор (Grandor)</t>
+          <t>Sminex</t>
         </is>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>ГПЗУ получен (апрель 2021), старт продаж ожидается</t>
-        </is>
-      </c>
-      <c r="G27" s="10" t="n"/>
-      <c r="H27" s="10" t="n"/>
-      <c r="I27" s="12" t="n">
-        <v>8</v>
-      </c>
+          <t>участок приобретён (апрель 2026), проектирование</t>
+        </is>
+      </c>
+      <c r="G27" s="12" t="n">
+        <v>13000</v>
+      </c>
+      <c r="H27" s="12" t="n">
+        <v>8200</v>
+      </c>
+      <c r="I27" s="10" t="n"/>
       <c r="J27" s="10" t="n"/>
-      <c r="K27" s="10" t="inlineStr">
-        <is>
-          <t>2026–2027</t>
-        </is>
-      </c>
+      <c r="K27" s="10" t="n"/>
       <c r="L27" s="10" t="n"/>
       <c r="M27" s="10" t="n"/>
-      <c r="N27" s="10" t="n"/>
+      <c r="N27" s="10" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
       <c r="O27" s="9" t="inlineStr">
         <is>
-          <t>официальный сайт проекта (также novostroy.ru, mskdeluxe.ru/start)</t>
+          <t>РИА Недвижимость (также sminex.com, interfax-russia.ru)</t>
         </is>
       </c>
       <c r="P27" s="13" t="inlineStr">
@@ -12909,19 +12915,19 @@
       </c>
       <c r="Q27" s="9" t="inlineStr">
         <is>
-          <t>Участок 0,4 га, семь корпусов 5–8 этажей в индивидуальной архитектуре. В базе делюкс-стартов 2026–2027 mskdeluxe.ru.</t>
+          <t>Участок 0,5 га (бывшая шёлковая фабрика, 4 здания 5 тыс. м²), продавец KR Properties (А. Клячин), переход прав 23.04.2026. Камерный клубный дом: пентхаусы с видом на Кремль, виллы, двор-сад; фасады по ул. Тимура Фрунзе сохраняются.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="24" customHeight="1">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>Премиальный квартал на Лужнецкой набережной, 10А</t>
+          <t>Усадьба в Большом Саввинском переулке (клубный дом VSF)</t>
         </is>
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>Лужнецкая наб., вл. 10А</t>
+          <t>Большой Саввинский пер. (усадьба купца Якунина)</t>
         </is>
       </c>
       <c r="C28" s="10" t="inlineStr">
@@ -12934,35 +12940,35 @@
           <t>Хамовники</t>
         </is>
       </c>
-      <c r="E28" s="10" t="inlineStr">
-        <is>
-          <t>Sminex</t>
+      <c r="E28" s="9" t="inlineStr">
+        <is>
+          <t>ГК «Векторстройфинанс» (VSF)</t>
         </is>
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>проект утверждён (АГР, май 2026), начало строительства 2027</t>
-        </is>
-      </c>
-      <c r="G28" s="10" t="n"/>
+          <t>анонсирован (приобретение объекта), концепция</t>
+        </is>
+      </c>
+      <c r="G28" s="12" t="n">
+        <v>2500</v>
+      </c>
       <c r="H28" s="10" t="n"/>
-      <c r="I28" s="10" t="n"/>
+      <c r="I28" s="12" t="n">
+        <v>4</v>
+      </c>
       <c r="J28" s="10" t="n"/>
-      <c r="K28" s="10" t="inlineStr">
-        <is>
-          <t>2027 (стройка)</t>
-        </is>
-      </c>
+      <c r="K28" s="10" t="n"/>
       <c r="L28" s="10" t="n"/>
       <c r="M28" s="10" t="n"/>
       <c r="N28" s="10" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="O28" s="9" t="inlineStr">
-        <is>
-          <t>РИА Недвижимость (также anwin.ru)</t>
+          <t>2025-07-09</t>
+        </is>
+      </c>
+      <c r="O28" s="10" t="inlineStr">
+        <is>
+          <t>elitnoe.ru</t>
         </is>
       </c>
       <c r="P28" s="13" t="inlineStr">
@@ -12972,19 +12978,19 @@
       </c>
       <c r="Q28" s="9" t="inlineStr">
         <is>
-          <t>Два жилых корпуса переменной этажности в неоклассике + эллиптический БЦ 26 тыс. м² («яйцо Фаберже»). Концепция согласована Департаментом градостроительной политики (В. Овчинский). Параметры жилой части не раскрыты.</t>
+          <t>Четырёхэтажное здание 1889 г. и двухэтажное до 1812 г., ~2,5 тыс. м². Оценка инвестиций 3,5–4,5 млрд руб., стоимость объекта до 1,3 млрд руб. Планируется перестройка в элитный клубный дом.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="24" customHeight="1">
       <c r="A29" s="9" t="inlineStr">
         <is>
-          <t>Тимура Фрунзе, 11 (клубный дом Sminex)</t>
-        </is>
-      </c>
-      <c r="B29" s="9" t="inlineStr">
-        <is>
-          <t>ул. Тимура Фрунзе, 11, стр. 7, 19, 33, 50</t>
+          <t>Усачёва, 22</t>
+        </is>
+      </c>
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>ул. Усачёва, 22</t>
         </is>
       </c>
       <c r="C29" s="10" t="inlineStr">
@@ -12997,35 +13003,35 @@
           <t>Хамовники</t>
         </is>
       </c>
-      <c r="E29" s="10" t="inlineStr">
-        <is>
-          <t>Sminex</t>
+      <c r="E29" s="9" t="inlineStr">
+        <is>
+          <t>Regions Development</t>
         </is>
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>участок приобретён (апрель 2026), проектирование</t>
+          <t>проект, продажи не начаты</t>
         </is>
       </c>
       <c r="G29" s="12" t="n">
-        <v>13000</v>
-      </c>
-      <c r="H29" s="12" t="n">
-        <v>8200</v>
-      </c>
-      <c r="I29" s="10" t="n"/>
+        <v>24600</v>
+      </c>
+      <c r="H29" s="10" t="n"/>
+      <c r="I29" s="12" t="n">
+        <v>18</v>
+      </c>
       <c r="J29" s="10" t="n"/>
-      <c r="K29" s="10" t="n"/>
+      <c r="K29" s="10" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
       <c r="L29" s="10" t="n"/>
       <c r="M29" s="10" t="n"/>
-      <c r="N29" s="10" t="inlineStr">
-        <is>
-          <t>2026-04-24</t>
-        </is>
-      </c>
+      <c r="N29" s="10" t="n"/>
       <c r="O29" s="9" t="inlineStr">
         <is>
-          <t>РИА Недвижимость (также sminex.com, interfax-russia.ru)</t>
+          <t>novostroev.ru (также usacheva22.ru, sosedi.life)</t>
         </is>
       </c>
       <c r="P29" s="13" t="inlineStr">
@@ -13035,19 +13041,19 @@
       </c>
       <c r="Q29" s="9" t="inlineStr">
         <is>
-          <t>Участок 0,5 га (бывшая шёлковая фабрика, 4 здания 5 тыс. м²), продавец KR Properties (А. Клячин), переход прав 23.04.2026. Камерный клубный дом: пентхаусы с видом на Кремль, виллы, двор-сад; фасады по ул. Тимура Фрунзе сохраняются.</t>
+          <t>Участок ~0,4 га, два корпуса ~14 и 18 этажей, архитектура Arch(e)type, двор без машин. Площадь 24,6 тыс. м² — по обзору делюкс-стартов 2026 novostroev.ru.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="24" customHeight="1">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>Усадьба в Большом Саввинском переулке (клубный дом VSF)</t>
-        </is>
-      </c>
-      <c r="B30" s="9" t="inlineStr">
-        <is>
-          <t>Большой Саввинский пер. (усадьба купца Якунина)</t>
+          <t>Хилков (Хилков переулок, вл. 3)</t>
+        </is>
+      </c>
+      <c r="B30" s="10" t="inlineStr">
+        <is>
+          <t>Хилков пер., вл. 3</t>
         </is>
       </c>
       <c r="C30" s="10" t="inlineStr">
@@ -13060,35 +13066,37 @@
           <t>Хамовники</t>
         </is>
       </c>
-      <c r="E30" s="9" t="inlineStr">
-        <is>
-          <t>ГК «Векторстройфинанс» (VSF)</t>
+      <c r="E30" s="10" t="inlineStr">
+        <is>
+          <t>Rose Group</t>
         </is>
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
-          <t>анонсирован (приобретение объекта), концепция</t>
+          <t>проектирование (долгосрочный проект), старт продаж ожидается</t>
         </is>
       </c>
       <c r="G30" s="12" t="n">
-        <v>2500</v>
-      </c>
-      <c r="H30" s="10" t="n"/>
+        <v>19806</v>
+      </c>
+      <c r="H30" s="12" t="n">
+        <v>8800</v>
+      </c>
       <c r="I30" s="12" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="J30" s="10" t="n"/>
-      <c r="K30" s="10" t="n"/>
+      <c r="K30" s="10" t="inlineStr">
+        <is>
+          <t>2026–2027</t>
+        </is>
+      </c>
       <c r="L30" s="10" t="n"/>
       <c r="M30" s="10" t="n"/>
-      <c r="N30" s="10" t="inlineStr">
-        <is>
-          <t>2025-07-09</t>
-        </is>
-      </c>
-      <c r="O30" s="10" t="inlineStr">
-        <is>
-          <t>elitnoe.ru</t>
+      <c r="N30" s="10" t="n"/>
+      <c r="O30" s="9" t="inlineStr">
+        <is>
+          <t>novostroy-m.ru (также mskdeluxe.ru/start)</t>
         </is>
       </c>
       <c r="P30" s="13" t="inlineStr">
@@ -13098,397 +13106,395 @@
       </c>
       <c r="Q30" s="9" t="inlineStr">
         <is>
-          <t>Четырёхэтажное здание 1889 г. и двухэтажное до 1812 г., ~2,5 тыс. м². Оценка инвестиций 3,5–4,5 млрд руб., стоимость объекта до 1,3 млрд руб. Планируется перестройка в элитный клубный дом.</t>
+          <t>3–8 этажей, монолит-кирпич, коммерция 1,8 тыс. м², паркинг 170 м/м. Карточка novostroy-m.ru датирована 2016 г.; проект вновь фигурирует в списке делюкс-стартов 2026–2027 на mskdeluxe.ru. Актуальность требует проверки.</t>
         </is>
       </c>
     </row>
     <row r="31" ht="24" customHeight="1">
-      <c r="A31" s="9" t="inlineStr">
-        <is>
-          <t>Усачёва, 22</t>
-        </is>
-      </c>
-      <c r="B31" s="10" t="inlineStr">
-        <is>
-          <t>ул. Усачёва, 22</t>
-        </is>
-      </c>
-      <c r="C31" s="10" t="inlineStr">
-        <is>
-          <t>Хамовники</t>
-        </is>
-      </c>
-      <c r="D31" s="29" t="inlineStr">
-        <is>
-          <t>Хамовники</t>
-        </is>
-      </c>
-      <c r="E31" s="9" t="inlineStr">
-        <is>
-          <t>Regions Development</t>
-        </is>
-      </c>
-      <c r="F31" s="9" t="inlineStr">
-        <is>
-          <t>проект, продажи не начаты</t>
-        </is>
-      </c>
-      <c r="G31" s="12" t="n">
-        <v>24600</v>
-      </c>
-      <c r="H31" s="10" t="n"/>
-      <c r="I31" s="12" t="n">
-        <v>18</v>
-      </c>
-      <c r="J31" s="10" t="n"/>
-      <c r="K31" s="10" t="inlineStr">
+      <c r="A31" s="14" t="inlineStr">
+        <is>
+          <t>Aurus Residences / Страна.Сити</t>
+        </is>
+      </c>
+      <c r="B31" s="14" t="inlineStr">
+        <is>
+          <t>2-й Красногвардейский проезд, квартал «Камушки»</t>
+        </is>
+      </c>
+      <c r="C31" s="15" t="inlineStr">
+        <is>
+          <t>Пресненский</t>
+        </is>
+      </c>
+      <c r="D31" s="30" t="inlineStr">
+        <is>
+          <t>Сити</t>
+        </is>
+      </c>
+      <c r="E31" s="15" t="inlineStr">
+        <is>
+          <t>Страна Девелопмент</t>
+        </is>
+      </c>
+      <c r="F31" s="14" t="inlineStr">
+        <is>
+          <t>ГПЗУ получен, подготовка к старту продаж</t>
+        </is>
+      </c>
+      <c r="G31" s="17" t="n">
+        <v>280800</v>
+      </c>
+      <c r="H31" s="17" t="n">
+        <v>231800</v>
+      </c>
+      <c r="I31" s="17" t="n">
+        <v>97</v>
+      </c>
+      <c r="J31" s="15" t="n"/>
+      <c r="K31" s="15" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="L31" s="10" t="n"/>
-      <c r="M31" s="10" t="n"/>
-      <c r="N31" s="10" t="n"/>
-      <c r="O31" s="9" t="inlineStr">
-        <is>
-          <t>novostroev.ru (также usacheva22.ru, sosedi.life)</t>
-        </is>
-      </c>
-      <c r="P31" s="13" t="inlineStr">
-        <is>
-          <t>ссылка</t>
-        </is>
-      </c>
-      <c r="Q31" s="9" t="inlineStr">
-        <is>
-          <t>Участок ~0,4 га, два корпуса ~14 и 18 этажей, архитектура Arch(e)type, двор без машин. Площадь 24,6 тыс. м² — по обзору делюкс-стартов 2026 novostroev.ru.</t>
+      <c r="L31" s="15" t="inlineStr">
+        <is>
+          <t>2029</t>
+        </is>
+      </c>
+      <c r="M31" s="15" t="n"/>
+      <c r="N31" s="15" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="O31" s="15" t="inlineStr">
+        <is>
+          <t>sosedi.life</t>
+        </is>
+      </c>
+      <c r="P31" s="18" t="inlineStr">
+        <is>
+          <t>ссылка</t>
+        </is>
+      </c>
+      <c r="Q31" s="14" t="inlineStr">
+        <is>
+          <t>Две башни 83 и 97 этажей на шестиярусном стилобате, участок ~1,25 га, архитектура APEX. ГПЗУ получен летом 2024 г., проект проходит согласования. Бизнес/премиум-класс, апартаменты.; АГР утверждён в декабре 2025, ~232 тыс. м² жилья (Москомархитектура); https://72.ru/text/gorod/2025/12/30/76197016/</t>
         </is>
       </c>
     </row>
     <row r="32" ht="24" customHeight="1">
-      <c r="A32" s="9" t="inlineStr">
-        <is>
-          <t>Хилков (Хилков переулок, вл. 3)</t>
-        </is>
-      </c>
-      <c r="B32" s="10" t="inlineStr">
-        <is>
-          <t>Хилков пер., вл. 3</t>
-        </is>
-      </c>
-      <c r="C32" s="10" t="inlineStr">
-        <is>
-          <t>Хамовники</t>
-        </is>
-      </c>
-      <c r="D32" s="29" t="inlineStr">
-        <is>
-          <t>Хамовники</t>
-        </is>
-      </c>
-      <c r="E32" s="10" t="inlineStr">
-        <is>
-          <t>Rose Group</t>
-        </is>
-      </c>
-      <c r="F32" s="9" t="inlineStr">
-        <is>
-          <t>проектирование (долгосрочный проект), старт продаж ожидается</t>
-        </is>
-      </c>
-      <c r="G32" s="12" t="n">
-        <v>19806</v>
-      </c>
-      <c r="H32" s="12" t="n">
-        <v>8800</v>
-      </c>
-      <c r="I32" s="12" t="n">
-        <v>8</v>
-      </c>
-      <c r="J32" s="10" t="n"/>
-      <c r="K32" s="10" t="inlineStr">
-        <is>
-          <t>2026–2027</t>
-        </is>
-      </c>
-      <c r="L32" s="10" t="n"/>
-      <c r="M32" s="10" t="n"/>
-      <c r="N32" s="10" t="n"/>
-      <c r="O32" s="9" t="inlineStr">
-        <is>
-          <t>novostroy-m.ru (также mskdeluxe.ru/start)</t>
-        </is>
-      </c>
-      <c r="P32" s="13" t="inlineStr">
-        <is>
-          <t>ссылка</t>
-        </is>
-      </c>
-      <c r="Q32" s="9" t="inlineStr">
-        <is>
-          <t>3–8 этажей, монолит-кирпич, коммерция 1,8 тыс. м², паркинг 170 м/м. Карточка novostroy-m.ru датирована 2016 г.; проект вновь фигурирует в списке делюкс-стартов 2026–2027 на mskdeluxe.ru. Актуальность требует проверки.</t>
+      <c r="A32" s="14" t="inlineStr">
+        <is>
+          <t>МФК «На Краснопресненской набережной» (Трёхгорная мануфактура)</t>
+        </is>
+      </c>
+      <c r="B32" s="14" t="inlineStr">
+        <is>
+          <t>Краснопресненская наб., 10</t>
+        </is>
+      </c>
+      <c r="C32" s="15" t="inlineStr">
+        <is>
+          <t>Пресненский</t>
+        </is>
+      </c>
+      <c r="D32" s="30" t="inlineStr">
+        <is>
+          <t>Сити</t>
+        </is>
+      </c>
+      <c r="E32" s="15" t="inlineStr">
+        <is>
+          <t>ГК Ташир</t>
+        </is>
+      </c>
+      <c r="F32" s="14" t="inlineStr">
+        <is>
+          <t>анонсирован, старт продаж ожидается</t>
+        </is>
+      </c>
+      <c r="G32" s="15" t="n"/>
+      <c r="H32" s="15" t="n"/>
+      <c r="I32" s="15" t="n"/>
+      <c r="J32" s="15" t="n"/>
+      <c r="K32" s="15" t="n"/>
+      <c r="L32" s="15" t="inlineStr">
+        <is>
+          <t>2030</t>
+        </is>
+      </c>
+      <c r="M32" s="15" t="n"/>
+      <c r="N32" s="15" t="n"/>
+      <c r="O32" s="15" t="inlineStr">
+        <is>
+          <t>novostroycity.ru</t>
+        </is>
+      </c>
+      <c r="P32" s="18" t="inlineStr">
+        <is>
+          <t>ссылка</t>
+        </is>
+      </c>
+      <c r="Q32" s="14" t="inlineStr">
+        <is>
+          <t>Участок ~1,7 га с ОКН (фабрика Трёхгорной мануфактуры, будет сохранена/реконструирована). Апартаменты премиум-класса + офисы + wellness, подземный паркинг на 750 м/м. Сроки реализации официально не подтверждены; апартаменты, а не квартиры.</t>
         </is>
       </c>
     </row>
     <row r="33" ht="24" customHeight="1">
-      <c r="A33" s="14" t="inlineStr">
-        <is>
-          <t>Aurus Residences / Страна.Сити</t>
-        </is>
-      </c>
-      <c r="B33" s="14" t="inlineStr">
-        <is>
-          <t>2-й Красногвардейский проезд, квартал «Камушки»</t>
-        </is>
-      </c>
-      <c r="C33" s="15" t="inlineStr">
+      <c r="A33" s="19" t="inlineStr">
+        <is>
+          <t>Клубный дом «Капельский, 5»</t>
+        </is>
+      </c>
+      <c r="B33" s="19" t="inlineStr">
+        <is>
+          <t>Капельский переулок, 5</t>
+        </is>
+      </c>
+      <c r="C33" s="20" t="inlineStr">
+        <is>
+          <t>Мещанский</t>
+        </is>
+      </c>
+      <c r="D33" s="21" t="inlineStr">
+        <is>
+          <t>Мещанский (вне Садового)</t>
+        </is>
+      </c>
+      <c r="E33" s="19" t="inlineStr">
+        <is>
+          <t>не раскрыт (юрлицо на сайте проекта не указано)</t>
+        </is>
+      </c>
+      <c r="F33" s="19" t="inlineStr">
+        <is>
+          <t>проектирование / предстарт продаж (официально: открытие продаж планируется во II–III кв. 2026)</t>
+        </is>
+      </c>
+      <c r="G33" s="20" t="n"/>
+      <c r="H33" s="20" t="n"/>
+      <c r="I33" s="20" t="inlineStr">
+        <is>
+          <t>8–9</t>
+        </is>
+      </c>
+      <c r="J33" s="22" t="n">
+        <v>46</v>
+      </c>
+      <c r="K33" s="19" t="inlineStr">
+        <is>
+          <t>2026 Q2–Q3 (старт продаж)</t>
+        </is>
+      </c>
+      <c r="L33" s="19" t="inlineStr">
+        <is>
+          <t>2029 Q4 (по данным Whitewill)</t>
+        </is>
+      </c>
+      <c r="M33" s="20" t="n"/>
+      <c r="N33" s="20" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="O33" s="19" t="inlineStr">
+        <is>
+          <t>Официальный сайт kapelsky5.ru; Whitewill; Novostroy-M</t>
+        </is>
+      </c>
+      <c r="P33" s="23" t="inlineStr">
+        <is>
+          <t>ссылка</t>
+        </is>
+      </c>
+      <c r="Q33" s="19" t="inlineStr">
+        <is>
+          <t>46 резиденций, переменная этажность, пентхаусы с террасами, приватный сквер, подземный паркинг. ВНИМАНИЕ: локация вне Садового кольца (у м. Проспект Мира, ~1 км севернее), включена по запросу заказчика.; Делюкс/премиум клубный дом; квартиры 54–345 м²; пентхаусы с террасами; двухуровневый паркинг на 56 м/м, 32 кладовые; приватный сад во дворе. Whitewill (https://whitewill.ru/developments/kapelskiy-5) указывает 8 этажей и срок сдачи 4 кв. 2029; Novostroy-M — 9 этажей, «скоро старт». Цены по запросу.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="24" customHeight="1">
+      <c r="A34" s="21" t="inlineStr">
+        <is>
+          <t>Делюкс-комплекс «Капранова, 3» (проект APEX)</t>
+        </is>
+      </c>
+      <c r="B34" s="21" t="inlineStr">
+        <is>
+          <t>переулок Капранова, 3 (БЦ «Премьер Плаза») + Малый Предтеченский пер., 1/2/1, Нововаганьковский пер., 3 стр. 1, Глубокий пер., 7</t>
+        </is>
+      </c>
+      <c r="C34" s="24" t="inlineStr">
         <is>
           <t>Пресненский</t>
         </is>
       </c>
-      <c r="D33" s="30" t="inlineStr">
-        <is>
-          <t>Сити</t>
-        </is>
-      </c>
-      <c r="E33" s="15" t="inlineStr">
-        <is>
-          <t>Страна Девелопмент</t>
-        </is>
-      </c>
-      <c r="F33" s="14" t="inlineStr">
-        <is>
-          <t>ГПЗУ получен, подготовка к старту продаж</t>
-        </is>
-      </c>
-      <c r="G33" s="17" t="n">
-        <v>280800</v>
-      </c>
-      <c r="H33" s="17" t="n">
-        <v>231800</v>
-      </c>
-      <c r="I33" s="17" t="n">
-        <v>97</v>
-      </c>
-      <c r="J33" s="15" t="n"/>
-      <c r="K33" s="15" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="L33" s="15" t="inlineStr">
-        <is>
-          <t>2029</t>
-        </is>
-      </c>
-      <c r="M33" s="15" t="n"/>
-      <c r="N33" s="15" t="inlineStr">
-        <is>
-          <t>2026-04-07</t>
-        </is>
-      </c>
-      <c r="O33" s="15" t="inlineStr">
-        <is>
-          <t>sosedi.life</t>
-        </is>
-      </c>
-      <c r="P33" s="18" t="inlineStr">
-        <is>
-          <t>ссылка</t>
-        </is>
-      </c>
-      <c r="Q33" s="14" t="inlineStr">
-        <is>
-          <t>Две башни 83 и 97 этажей на шестиярусном стилобате, участок ~1,25 га, архитектура APEX. ГПЗУ получен летом 2024 г., проект проходит согласования. Бизнес/премиум-класс, апартаменты.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="24" customHeight="1">
-      <c r="A34" s="14" t="inlineStr">
-        <is>
-          <t>Жилые башни «Сити-2» (2-й Красногвардейский проезд)</t>
-        </is>
-      </c>
-      <c r="B34" s="14" t="inlineStr">
-        <is>
-          <t>2-й Красногвардейский проезд, Пресненский район (площадка 1,255 га у «Москва-Сити»)</t>
-        </is>
-      </c>
-      <c r="C34" s="15" t="inlineStr">
-        <is>
-          <t>Пресненский</t>
-        </is>
-      </c>
-      <c r="D34" s="30" t="inlineStr">
-        <is>
-          <t>Сити</t>
-        </is>
-      </c>
-      <c r="E34" s="14" t="inlineStr">
-        <is>
-          <t>ГК «Страна Девелопмент» (право застройки получено на торгах города; прежний правообладатель — ООО «Моссититстрой»)</t>
-        </is>
-      </c>
-      <c r="F34" s="14" t="inlineStr">
-        <is>
-          <t>АГР двух жилых башен утвержден (декабрь 2025); старт продаж не объявлен</t>
-        </is>
-      </c>
-      <c r="G34" s="17" t="n">
-        <v>281000</v>
-      </c>
-      <c r="H34" s="17" t="n">
-        <v>232000</v>
-      </c>
-      <c r="I34" s="14" t="inlineStr">
-        <is>
-          <t>две башни, самая высокая — 384 м по утвержденному АГР (ранее заявлялось до 450 м)</t>
-        </is>
-      </c>
-      <c r="J34" s="15" t="n"/>
-      <c r="K34" s="15" t="n"/>
-      <c r="L34" s="15" t="n"/>
-      <c r="M34" s="15" t="n"/>
-      <c r="N34" s="15" t="inlineStr">
-        <is>
-          <t>2025-12-30</t>
-        </is>
-      </c>
-      <c r="O34" s="14" t="inlineStr">
-        <is>
-          <t>72.ru / сеть городских порталов (30.12.2025); IRN.ru (18.04.2024)</t>
-        </is>
-      </c>
-      <c r="P34" s="18" t="inlineStr">
-        <is>
-          <t>ссылка</t>
-        </is>
-      </c>
-      <c r="Q34" s="14" t="inlineStr">
-        <is>
-          <t>~232 тыс. м² жилья и 49 тыс. м² нежилых помещений (IRN.ru, https://www.irn.ru/news/156498.html). Самый высокий жилой комплекс России по утвержденной концепции. Отдельно на Novostroy-M числится «Сити-2» Capital Group (квартал 804, Камушки, три башни до 450 м, ~470 тыс. м², ~385 тыс. м² жилья, «скоро старт») — иная площадка в том же районе, не путать.</t>
+      <c r="D34" s="21" t="inlineStr">
+        <is>
+          <t>Пресненский (вне Садового)</t>
+        </is>
+      </c>
+      <c r="E34" s="24" t="inlineStr">
+        <is>
+          <t>не раскрыт</t>
+        </is>
+      </c>
+      <c r="F34" s="21" t="inlineStr">
+        <is>
+          <t>визуализации направлены на согласование в город (ноябрь 2025); предстарт, старт продаж заявлен на 2026</t>
+        </is>
+      </c>
+      <c r="G34" s="24" t="n"/>
+      <c r="H34" s="24" t="n"/>
+      <c r="I34" s="21" t="inlineStr">
+        <is>
+          <t>9–23 (шесть корпусов)</t>
+        </is>
+      </c>
+      <c r="J34" s="25" t="n">
+        <v>255</v>
+      </c>
+      <c r="K34" s="21" t="inlineStr">
+        <is>
+          <t>2026 (старт продаж)</t>
+        </is>
+      </c>
+      <c r="L34" s="24" t="n"/>
+      <c r="M34" s="24" t="n"/>
+      <c r="N34" s="24" t="inlineStr">
+        <is>
+          <t>2025-11-19</t>
+        </is>
+      </c>
+      <c r="O34" s="21" t="inlineStr">
+        <is>
+          <t>Москвич Mag (19.11.2025); sosedi.life (07.04.2026)</t>
+        </is>
+      </c>
+      <c r="P34" s="26" t="inlineStr">
+        <is>
+          <t>ссылка</t>
+        </is>
+      </c>
+      <c r="Q34" s="21" t="inlineStr">
+        <is>
+          <t>Делюкс-проект в базе перспективных стартов 2026–2027 (mskdeluxe.ru, цены «от 60 млн руб.»). Обзор smart-lab.ru/blog/1231916.php указывает старт продаж в 2026 г., 12 этажей, двор без машин. Застройщик и параметры в открытых источниках не подтверждены. ~400 м от м. Краснопресненская, вне Садового кольца.; Единая застройка нескольких участков за Домом Правительства у Пресненского детского парка; башни с «волнообразными» фасадами, снос БЦ «Премьер Плаза», сохранение усадьбы Резанова. По sosedi.life (https://sosedi.life/news/zhk-kapranova-3/): участок &gt;2,5 га, 6 корпусов 9–23 этажа, 255 квартир, двор 7 039,6 м², лобби Balcon, 2–5 квартир на этаже. Указанные в запросе «12 этажей» источниками не подтверждаются. В списке делюкс-стартов mskdeluxe.ru.</t>
         </is>
       </c>
     </row>
     <row r="35" ht="24" customHeight="1">
-      <c r="A35" s="14" t="inlineStr">
-        <is>
-          <t>МФК «На Краснопресненской набережной» (Трёхгорная мануфактура)</t>
-        </is>
-      </c>
-      <c r="B35" s="14" t="inlineStr">
-        <is>
-          <t>Краснопресненская наб., 10</t>
-        </is>
-      </c>
-      <c r="C35" s="15" t="inlineStr">
-        <is>
-          <t>Пресненский</t>
-        </is>
-      </c>
-      <c r="D35" s="30" t="inlineStr">
-        <is>
-          <t>Сити</t>
-        </is>
-      </c>
-      <c r="E35" s="15" t="inlineStr">
-        <is>
-          <t>ГК Ташир</t>
-        </is>
-      </c>
-      <c r="F35" s="14" t="inlineStr">
-        <is>
-          <t>анонсирован, старт продаж ожидается</t>
-        </is>
-      </c>
-      <c r="G35" s="15" t="n"/>
-      <c r="H35" s="15" t="n"/>
-      <c r="I35" s="15" t="n"/>
-      <c r="J35" s="15" t="n"/>
-      <c r="K35" s="15" t="n"/>
-      <c r="L35" s="15" t="inlineStr">
-        <is>
-          <t>2030</t>
-        </is>
-      </c>
-      <c r="M35" s="15" t="n"/>
-      <c r="N35" s="15" t="n"/>
-      <c r="O35" s="15" t="inlineStr">
-        <is>
-          <t>novostroycity.ru</t>
-        </is>
-      </c>
-      <c r="P35" s="18" t="inlineStr">
-        <is>
-          <t>ссылка</t>
-        </is>
-      </c>
-      <c r="Q35" s="14" t="inlineStr">
-        <is>
-          <t>Участок ~1,7 га с ОКН (фабрика Трёхгорной мануфактуры, будет сохранена/реконструирована). Апартаменты премиум-класса + офисы + wellness, подземный паркинг на 750 м/м. Сроки реализации официально не подтверждены; апартаменты, а не квартиры.</t>
+      <c r="A35" s="19" t="inlineStr">
+        <is>
+          <t>КРТ вдоль Звенигородского шоссе (три участка, 73,62 га)</t>
+        </is>
+      </c>
+      <c r="B35" s="19" t="inlineStr">
+        <is>
+          <t>Вдоль Звенигородского шоссе между 3-й Магистральной улицей и ТТК (Пресненский / Хорошёвский районы)</t>
+        </is>
+      </c>
+      <c r="C35" s="19" t="inlineStr">
+        <is>
+          <t>Пресненский / Хорошёвский</t>
+        </is>
+      </c>
+      <c r="D35" s="21" t="inlineStr">
+        <is>
+          <t>Пресненский (вне Садового)</t>
+        </is>
+      </c>
+      <c r="E35" s="19" t="inlineStr">
+        <is>
+          <t>не раскрыт (оператор/инвестор не назван; в числе 9 проектов КРТ, утвержденных в августе 2026)</t>
+        </is>
+      </c>
+      <c r="F35" s="19" t="inlineStr">
+        <is>
+          <t>решение о КРТ принято (август 2026); оператор/торги не объявлены</t>
+        </is>
+      </c>
+      <c r="G35" s="22" t="n">
+        <v>3200000</v>
+      </c>
+      <c r="H35" s="20" t="n"/>
+      <c r="I35" s="20" t="n"/>
+      <c r="J35" s="20" t="n"/>
+      <c r="K35" s="20" t="n"/>
+      <c r="L35" s="20" t="n"/>
+      <c r="M35" s="20" t="n"/>
+      <c r="N35" s="20" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="O35" s="19" t="inlineStr">
+        <is>
+          <t>Интерфакс-Россия; Ведомости.Город (02.09.2026)</t>
+        </is>
+      </c>
+      <c r="P35" s="23" t="inlineStr">
+        <is>
+          <t>ссылка</t>
+        </is>
+      </c>
+      <c r="Q35" s="19" t="inlineStr">
+        <is>
+          <t>Три участка нежилой застройки общей площадью 73,62 га; &gt;3,2 млн м² недвижимости (жильё + общественно-деловые объекты, школы на 4050 мест, детсады на 1775 мест), 35,5 тыс. рабочих мест. Часть «Большого Сити» (Шелепиха/Магистральные улицы), класс жилья не заявлен — не обязательно премиум.; Три участка нежилой застройки (старые склады, админздания) общей площадью 73,62 га; свыше 3,2 млн м² — жилье, общественно-деловые и социальные объекты; строительство/реконструкция дорог ~6,5 км; здание конечной станции наземного транспорта с отстойно-разворотной площадкой (Ведомости, https://www.vedomosti.ru/gorod/ourcity/articles/gorodskoi-kvartal). Жилая премиальная часть отдельно не выделена; класс жилья не указан. Оператор (Московский фонд реновации / КРТ 21 / инвестор по торгам) не объявлен.</t>
         </is>
       </c>
     </row>
     <row r="36" ht="24" customHeight="1">
       <c r="A36" s="21" t="inlineStr">
         <is>
-          <t>Клубный дом «Капельский, 5»</t>
+          <t>Участок КРТ «Большой Тишинский переулок, 8»</t>
         </is>
       </c>
       <c r="B36" s="21" t="inlineStr">
         <is>
-          <t>Капельский переулок, 5</t>
+          <t>Большой Тишинский переулок, 8 (стр. 1, 2)</t>
         </is>
       </c>
       <c r="C36" s="24" t="inlineStr">
         <is>
-          <t>Мещанский</t>
+          <t>Пресненский</t>
         </is>
       </c>
       <c r="D36" s="21" t="inlineStr">
         <is>
-          <t>Мещанский (вне Садового)</t>
-        </is>
-      </c>
-      <c r="E36" s="21" t="inlineStr">
-        <is>
-          <t>не раскрыт (юрлицо на сайте проекта не указано)</t>
+          <t>Пресненский (вне Садового)</t>
+        </is>
+      </c>
+      <c r="E36" s="24" t="inlineStr">
+        <is>
+          <t>не раскрыт</t>
         </is>
       </c>
       <c r="F36" s="21" t="inlineStr">
         <is>
-          <t>проектирование / предстарт продаж (официально: открытие продаж планируется во II–III кв. 2026)</t>
-        </is>
-      </c>
-      <c r="G36" s="24" t="n"/>
-      <c r="H36" s="24" t="n"/>
-      <c r="I36" s="24" t="inlineStr">
-        <is>
-          <t>8–9</t>
-        </is>
-      </c>
-      <c r="J36" s="25" t="n">
-        <v>46</v>
-      </c>
-      <c r="K36" s="21" t="inlineStr">
-        <is>
-          <t>2026 Q2–Q3 (старт продаж)</t>
-        </is>
-      </c>
-      <c r="L36" s="21" t="inlineStr">
-        <is>
-          <t>2029 Q4 (по данным Whitewill)</t>
-        </is>
-      </c>
+          <t>решение о КРТ (по данным заказчика — август 2026); оператор/правообладатель и торги в открытых источниках не найдены</t>
+        </is>
+      </c>
+      <c r="G36" s="25" t="n">
+        <v>10000</v>
+      </c>
+      <c r="H36" s="25" t="n">
+        <v>6000</v>
+      </c>
+      <c r="I36" s="24" t="n"/>
+      <c r="J36" s="24" t="n"/>
+      <c r="K36" s="24" t="n"/>
+      <c r="L36" s="24" t="n"/>
       <c r="M36" s="24" t="n"/>
       <c r="N36" s="24" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="O36" s="21" t="inlineStr">
         <is>
-          <t>Официальный сайт kapelsky5.ru; Whitewill; Novostroy-M</t>
+          <t>krt.mos.ru (реестр проектов КРТ Москвы)</t>
         </is>
       </c>
       <c r="P36" s="26" t="inlineStr">
@@ -13498,216 +13504,23 @@
       </c>
       <c r="Q36" s="21" t="inlineStr">
         <is>
-          <t>46 резиденций, переменная этажность, пентхаусы с террасами, приватный сквер, подземный паркинг. ВНИМАНИЕ: локация вне Садового кольца (у м. Проспект Мира, ~1 км севернее), включена по запросу заказчика.; Делюкс/премиум клубный дом; квартиры 54–345 м²; пентхаусы с террасами; двухуровневый паркинг на 56 м/м, 32 кладовые; приватный сад во дворе. Whitewill (https://whitewill.ru/developments/kapelskiy-5) указывает 8 этажей и срок сдачи 4 кв. 2029; Novostroy-M — 9 этажей, «скоро старт». Цены по запросу.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="24" customHeight="1">
-      <c r="A37" s="19" t="inlineStr">
-        <is>
-          <t>Делюкс-комплекс «Капранова, 3» (проект APEX)</t>
-        </is>
-      </c>
-      <c r="B37" s="19" t="inlineStr">
-        <is>
-          <t>переулок Капранова, 3 (БЦ «Премьер Плаза») + Малый Предтеченский пер., 1/2/1, Нововаганьковский пер., 3 стр. 1, Глубокий пер., 7</t>
-        </is>
-      </c>
-      <c r="C37" s="20" t="inlineStr">
-        <is>
-          <t>Пресненский</t>
-        </is>
-      </c>
-      <c r="D37" s="21" t="inlineStr">
-        <is>
-          <t>Пресненский (вне Садового)</t>
-        </is>
-      </c>
-      <c r="E37" s="20" t="inlineStr">
-        <is>
-          <t>не раскрыт</t>
-        </is>
-      </c>
-      <c r="F37" s="19" t="inlineStr">
-        <is>
-          <t>визуализации направлены на согласование в город (ноябрь 2025); предстарт, старт продаж заявлен на 2026</t>
-        </is>
-      </c>
-      <c r="G37" s="20" t="n"/>
-      <c r="H37" s="20" t="n"/>
-      <c r="I37" s="19" t="inlineStr">
-        <is>
-          <t>9–23 (шесть корпусов)</t>
-        </is>
-      </c>
-      <c r="J37" s="22" t="n">
-        <v>255</v>
-      </c>
-      <c r="K37" s="19" t="inlineStr">
-        <is>
-          <t>2026 (старт продаж)</t>
-        </is>
-      </c>
-      <c r="L37" s="20" t="n"/>
-      <c r="M37" s="20" t="n"/>
-      <c r="N37" s="20" t="inlineStr">
-        <is>
-          <t>2025-11-19</t>
-        </is>
-      </c>
-      <c r="O37" s="19" t="inlineStr">
-        <is>
-          <t>Москвич Mag (19.11.2025); sosedi.life (07.04.2026)</t>
-        </is>
-      </c>
-      <c r="P37" s="23" t="inlineStr">
-        <is>
-          <t>ссылка</t>
-        </is>
-      </c>
-      <c r="Q37" s="19" t="inlineStr">
-        <is>
-          <t>Делюкс-проект в базе перспективных стартов 2026–2027 (mskdeluxe.ru, цены «от 60 млн руб.»). Обзор smart-lab.ru/blog/1231916.php указывает старт продаж в 2026 г., 12 этажей, двор без машин. Застройщик и параметры в открытых источниках не подтверждены. ~400 м от м. Краснопресненская, вне Садового кольца.; Единая застройка нескольких участков за Домом Правительства у Пресненского детского парка; башни с «волнообразными» фасадами, снос БЦ «Премьер Плаза», сохранение усадьбы Резанова. По sosedi.life (https://sosedi.life/news/zhk-kapranova-3/): участок &gt;2,5 га, 6 корпусов 9–23 этажа, 255 квартир, двор 7 039,6 м², лобби Balcon, 2–5 квартир на этаже. Указанные в запросе «12 этажей» источниками не подтверждаются. В списке делюкс-стартов mskdeluxe.ru.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="24" customHeight="1">
-      <c r="A38" s="21" t="inlineStr">
-        <is>
-          <t>КРТ вдоль Звенигородского шоссе (три участка, 73,62 га)</t>
-        </is>
-      </c>
-      <c r="B38" s="21" t="inlineStr">
-        <is>
-          <t>Вдоль Звенигородского шоссе между 3-й Магистральной улицей и ТТК (Пресненский / Хорошёвский районы)</t>
-        </is>
-      </c>
-      <c r="C38" s="21" t="inlineStr">
-        <is>
-          <t>Пресненский / Хорошёвский</t>
-        </is>
-      </c>
-      <c r="D38" s="21" t="inlineStr">
-        <is>
-          <t>Пресненский (вне Садового)</t>
-        </is>
-      </c>
-      <c r="E38" s="21" t="inlineStr">
-        <is>
-          <t>не раскрыт (оператор/инвестор не назван; в числе 9 проектов КРТ, утвержденных в августе 2026)</t>
-        </is>
-      </c>
-      <c r="F38" s="21" t="inlineStr">
-        <is>
-          <t>решение о КРТ принято (август 2026); оператор/торги не объявлены</t>
-        </is>
-      </c>
-      <c r="G38" s="25" t="n">
-        <v>3200000</v>
-      </c>
-      <c r="H38" s="24" t="n"/>
-      <c r="I38" s="24" t="n"/>
-      <c r="J38" s="24" t="n"/>
-      <c r="K38" s="24" t="n"/>
-      <c r="L38" s="24" t="n"/>
-      <c r="M38" s="24" t="n"/>
-      <c r="N38" s="24" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="O38" s="21" t="inlineStr">
-        <is>
-          <t>Интерфакс-Россия; Ведомости.Город (02.09.2026)</t>
-        </is>
-      </c>
-      <c r="P38" s="26" t="inlineStr">
-        <is>
-          <t>ссылка</t>
-        </is>
-      </c>
-      <c r="Q38" s="21" t="inlineStr">
-        <is>
-          <t>Три участка нежилой застройки общей площадью 73,62 га; &gt;3,2 млн м² недвижимости (жильё + общественно-деловые объекты, школы на 4050 мест, детсады на 1775 мест), 35,5 тыс. рабочих мест. Часть «Большого Сити» (Шелепиха/Магистральные улицы), класс жилья не заявлен — не обязательно премиум.; Три участка нежилой застройки (старые склады, админздания) общей площадью 73,62 га; свыше 3,2 млн м² — жилье, общественно-деловые и социальные объекты; строительство/реконструкция дорог ~6,5 км; здание конечной станции наземного транспорта с отстойно-разворотной площадкой (Ведомости, https://www.vedomosti.ru/gorod/ourcity/articles/gorodskoi-kvartal). Жилая премиальная часть отдельно не выделена; класс жилья не указан. Оператор (Московский фонд реновации / КРТ 21 / инвестор по торгам) не объявлен.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="24" customHeight="1">
-      <c r="A39" s="19" t="inlineStr">
-        <is>
-          <t>Участок КРТ «Большой Тишинский переулок, 8»</t>
-        </is>
-      </c>
-      <c r="B39" s="19" t="inlineStr">
-        <is>
-          <t>Большой Тишинский переулок, 8 (стр. 1, 2)</t>
-        </is>
-      </c>
-      <c r="C39" s="20" t="inlineStr">
-        <is>
-          <t>Пресненский</t>
-        </is>
-      </c>
-      <c r="D39" s="21" t="inlineStr">
-        <is>
-          <t>Пресненский (вне Садового)</t>
-        </is>
-      </c>
-      <c r="E39" s="20" t="inlineStr">
-        <is>
-          <t>не раскрыт</t>
-        </is>
-      </c>
-      <c r="F39" s="19" t="inlineStr">
-        <is>
-          <t>решение о КРТ (по данным заказчика — август 2026); оператор/правообладатель и торги в открытых источниках не найдены</t>
-        </is>
-      </c>
-      <c r="G39" s="22" t="n">
-        <v>10000</v>
-      </c>
-      <c r="H39" s="22" t="n">
-        <v>6000</v>
-      </c>
-      <c r="I39" s="20" t="n"/>
-      <c r="J39" s="20" t="n"/>
-      <c r="K39" s="20" t="n"/>
-      <c r="L39" s="20" t="n"/>
-      <c r="M39" s="20" t="n"/>
-      <c r="N39" s="20" t="inlineStr">
-        <is>
-          <t>2026-08</t>
-        </is>
-      </c>
-      <c r="O39" s="19" t="inlineStr">
-        <is>
-          <t>krt.mos.ru (реестр проектов КРТ Москвы)</t>
-        </is>
-      </c>
-      <c r="P39" s="23" t="inlineStr">
-        <is>
-          <t>ссылка</t>
-        </is>
-      </c>
-      <c r="Q39" s="19" t="inlineStr">
-        <is>
           <t>Участок ~0,3 га включён в программу КРТ решением властей Москвы. Существующие здания реконструированы в 2004 г., в 2020 г. переоборудованы под хостелы. Оператор/девелопер в публикации не назван; в других открытых источниках на 07.09.2026 не найден. Локация — Пресненский район вне Садового кольца, между Б. Грузинской и Пресненским Валом (условно отнесено к зоне Пресня/Сити).; Поиск по mos.ru, krt.mos.ru, stroi.mos.ru, Ведомости, РБК, Интерфакс, М24, Известия (август–сентябрь 2026) не выявил отдельной публикации по этому участку: новости августа 2026 о КРТ (250 проектов, 63 договора с начала года) даются агрегированно. Ближайший крупный проект — квартал «Тишинский бульвар» Sminex (Электрический пер., 1), связь с участком №8 не подтверждена. Площадь 0,3 га / ~10 000 м² — из исходных данных запроса, независимого подтверждения нет.</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="30" customHeight="1">
-      <c r="A41" s="27" t="inlineStr">
+    <row r="38" ht="30" customHeight="1">
+      <c r="A38" s="27" t="inlineStr">
         <is>
           <t>Источники: открытые публикации 2025–2026 (stroi.mos.ru, mos.ru, отраслевые СМИ, публичные Telegram-каналы). Закрытый канал t.me/c/3370602239 недоступен без членства — пост №1364 про ЗУ «Большой Тишинский, 8» подтверждён по открытым источникам.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:Q39"/>
+  <autoFilter ref="A3:Q36"/>
   <mergeCells count="3">
+    <mergeCell ref="A38:Q38"/>
     <mergeCell ref="A2:Q2"/>
     <mergeCell ref="A1:Q1"/>
-    <mergeCell ref="A41:Q41"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P4" r:id="rId1"/>
@@ -13743,9 +13556,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P34" r:id="rId31"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P35" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P36" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P37" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P38" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P39" r:id="rId36"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.2" footer="0.2"/>

</xml_diff>

<commit_message>
Rebuild premium ЦАО workbook
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Bv8NELxW2W7udnb3XUFGS2
</commit_message>
<xml_diff>
--- a/docs/premium-cao/premium-zhk-cao.xlsx
+++ b/docs/premium-cao/premium-zhk-cao.xlsx
@@ -729,7 +729,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1">
+    <row r="4" ht="24" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Резиденция Тверская</t>
@@ -810,7 +810,7 @@
       </c>
       <c r="S4" s="4" t="inlineStr">
         <is>
-          <t>апарт-отель; юрлицо Техноком Трейд</t>
+          <t>апарт-отель; юрлицо Техноком Трейд; карточка ЖК на Циан не найдена, год по объявлениям</t>
         </is>
       </c>
     </row>
@@ -887,7 +887,11 @@
         </is>
       </c>
       <c r="R5" s="11" t="inlineStr"/>
-      <c r="S5" s="10" t="inlineStr"/>
+      <c r="S5" s="10" t="inlineStr">
+        <is>
+          <t>карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="24" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
@@ -970,7 +974,7 @@
       </c>
       <c r="S6" s="4" t="inlineStr">
         <is>
-          <t>24 квартиры + 3 особняка + 9 таунхаусов; юрлицо Торгпродуктсервис; арх. Илья Уткин</t>
+          <t>24 квартиры + 3 особняка + 9 таунхаусов; юрлицо Торгпродуктсервис; арх. Илья Уткин; карточка ЖК на Циан не найдена, год по объявлениям</t>
         </is>
       </c>
     </row>
@@ -1047,7 +1051,11 @@
         </is>
       </c>
       <c r="R7" s="11" t="inlineStr"/>
-      <c r="S7" s="10" t="inlineStr"/>
+      <c r="S7" s="10" t="inlineStr">
+        <is>
+          <t>карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
@@ -1122,7 +1130,11 @@
         </is>
       </c>
       <c r="R8" s="5" t="inlineStr"/>
-      <c r="S8" s="4" t="inlineStr"/>
+      <c r="S8" s="4" t="inlineStr">
+        <is>
+          <t>карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
@@ -1197,9 +1209,13 @@
         </is>
       </c>
       <c r="R9" s="11" t="inlineStr"/>
-      <c r="S9" s="10" t="inlineStr"/>
-    </row>
-    <row r="10" ht="15" customHeight="1">
+      <c r="S9" s="10" t="inlineStr">
+        <is>
+          <t>карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Sinatra (Синатра)</t>
@@ -1278,7 +1294,7 @@
       </c>
       <c r="S10" s="4" t="inlineStr">
         <is>
-          <t>реконструкция; cian years 2018/2020</t>
+          <t>реконструкция; cian years 2018/2020; карточка ЖК на Циан не найдена, год по объявлениям</t>
         </is>
       </c>
     </row>
@@ -1355,9 +1371,13 @@
         </is>
       </c>
       <c r="R11" s="11" t="inlineStr"/>
-      <c r="S11" s="10" t="inlineStr"/>
-    </row>
-    <row r="12" ht="15" customHeight="1">
+      <c r="S11" s="10" t="inlineStr">
+        <is>
+          <t>карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="24" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Уланский, 13</t>
@@ -1438,11 +1458,11 @@
       </c>
       <c r="S12" s="4" t="inlineStr">
         <is>
-          <t>реконструкция особняка 1886 г.; апартаменты</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="15" customHeight="1">
+          <t>реконструкция особняка 1886 г.; апартаменты; карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="24" customHeight="1">
       <c r="A13" s="10" t="inlineStr">
         <is>
           <t>Современник</t>
@@ -1521,7 +1541,7 @@
       </c>
       <c r="S13" s="10" t="inlineStr">
         <is>
-          <t>реновация здания XIX в.</t>
+          <t>реновация здания XIX в.; карточка ЖК на Циан не найдена, год по объявлениям</t>
         </is>
       </c>
     </row>
@@ -1604,9 +1624,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="S14" s="4" t="inlineStr"/>
-    </row>
-    <row r="15" ht="15" customHeight="1">
+      <c r="S14" s="4" t="inlineStr">
+        <is>
+          <t>карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1">
       <c r="A15" s="10" t="inlineStr">
         <is>
           <t>SkyView</t>
@@ -1685,11 +1709,11 @@
       </c>
       <c r="S15" s="10" t="inlineStr">
         <is>
-          <t>4 башни на месте Киноцентра</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="15" customHeight="1">
+          <t>4 башни на месте Киноцентра; карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="24" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Полянка/44</t>
@@ -1768,7 +1792,7 @@
       </c>
       <c r="S16" s="4" t="inlineStr">
         <is>
-          <t>7 корпусов сданы март 2019; cian: застройщик ТЕЛЕКОМ</t>
+          <t>7 корпусов сданы март 2019; cian: застройщик ТЕЛЕКОМ; карточка ЖК на Циан не найдена, год по объявлениям</t>
         </is>
       </c>
     </row>
@@ -1851,11 +1875,11 @@
       </c>
       <c r="S17" s="10" t="inlineStr">
         <is>
-          <t>cian years 2021 (первая очередь)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="15" customHeight="1">
+          <t>cian years 2021 (первая очередь); карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="24" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Bogenhouse (Богенхаус)</t>
@@ -1936,11 +1960,11 @@
       </c>
       <c r="S18" s="4" t="inlineStr">
         <is>
-          <t>апартаменты; также ГК Дельта</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="15" customHeight="1">
+          <t>апартаменты; также ГК Дельта; карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="24" customHeight="1">
       <c r="A19" s="10" t="inlineStr">
         <is>
           <t>BALCHUG VIEWPOINT (Балчуг Вьюпоинт)</t>
@@ -2019,7 +2043,7 @@
       </c>
       <c r="S19" s="10" t="inlineStr">
         <is>
-          <t>апартаменты</t>
+          <t>апартаменты; карточка ЖК на Циан не найдена, год по объявлениям</t>
         </is>
       </c>
     </row>
@@ -2096,7 +2120,11 @@
         </is>
       </c>
       <c r="R20" s="5" t="inlineStr"/>
-      <c r="S20" s="4" t="inlineStr"/>
+      <c r="S20" s="4" t="inlineStr">
+        <is>
+          <t>карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="15" customHeight="1">
       <c r="A21" s="10" t="inlineStr">
@@ -2177,9 +2205,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="S21" s="10" t="inlineStr"/>
-    </row>
-    <row r="22" ht="15" customHeight="1">
+      <c r="S21" s="10" t="inlineStr">
+        <is>
+          <t>карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="24" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Клубный дом ЦВЕТ32</t>
@@ -2260,11 +2292,11 @@
       </c>
       <c r="S22" s="4" t="inlineStr">
         <is>
-          <t>введён 28.08.2019; апартаменты</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="15" customHeight="1">
+          <t>введён 28.08.2019; апартаменты; карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="24" customHeight="1">
       <c r="A23" s="10" t="inlineStr">
         <is>
           <t>A.Residence (А Резиденс)</t>
@@ -2345,11 +2377,11 @@
       </c>
       <c r="S23" s="10" t="inlineStr">
         <is>
-          <t>арх. Цимайло Ляшенко и Партнеры</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="15" customHeight="1">
+          <t>арх. Цимайло Ляшенко и Партнеры; карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="24" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
           <t>Edison House (Эдисон Хаус)</t>
@@ -2428,7 +2460,7 @@
       </c>
       <c r="S24" s="4" t="inlineStr">
         <is>
-          <t>cian years 2018; источники: 3 кв. 2019</t>
+          <t>cian years 2018; источники: 3 кв. 2019; карточка ЖК на Циан не найдена, год по объявлениям</t>
         </is>
       </c>
     </row>
@@ -2505,7 +2537,11 @@
         </is>
       </c>
       <c r="R25" s="11" t="inlineStr"/>
-      <c r="S25" s="10" t="inlineStr"/>
+      <c r="S25" s="10" t="inlineStr">
+        <is>
+          <t>карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="15" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
@@ -2586,9 +2622,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="S26" s="4" t="inlineStr"/>
-    </row>
-    <row r="27" ht="15" customHeight="1">
+      <c r="S26" s="4" t="inlineStr">
+        <is>
+          <t>карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="24" customHeight="1">
       <c r="A27" s="10" t="inlineStr">
         <is>
           <t>Дом NV/9</t>
@@ -2667,7 +2707,7 @@
       </c>
       <c r="S27" s="10" t="inlineStr">
         <is>
-          <t>NV/9 ARTKVARTAL; юрлицо Стрелецкая Слобода</t>
+          <t>NV/9 ARTKVARTAL; юрлицо Стрелецкая Слобода; карточка ЖК на Циан не найдена, год по объявлениям</t>
         </is>
       </c>
     </row>
@@ -2752,11 +2792,11 @@
       </c>
       <c r="S28" s="4" t="inlineStr">
         <is>
-          <t>21 квартира + 4 резиденции + 3 пентхауса; арх. Цимайло Ляшенко</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="15" customHeight="1">
+          <t>21 квартира + 4 резиденции + 3 пентхауса; арх. Цимайло Ляшенко; карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="24" customHeight="1">
       <c r="A29" s="10" t="inlineStr">
         <is>
           <t>Клубный дом Космо 4/22</t>
@@ -2837,11 +2877,11 @@
       </c>
       <c r="S29" s="10" t="inlineStr">
         <is>
-          <t>апартаменты</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="15" customHeight="1">
+          <t>апартаменты; карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="24" customHeight="1">
       <c r="A30" s="4" t="inlineStr">
         <is>
           <t>Софийский</t>
@@ -2920,11 +2960,11 @@
       </c>
       <c r="S30" s="4" t="inlineStr">
         <is>
-          <t>апартаменты; введён январь 2019</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="15" customHeight="1">
+          <t>апартаменты; введён январь 2019; карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="24" customHeight="1">
       <c r="A31" s="10" t="inlineStr">
         <is>
           <t>Дом на Тишинке</t>
@@ -3003,11 +3043,11 @@
       </c>
       <c r="S31" s="10" t="inlineStr">
         <is>
-          <t>арх. Павел Андреев</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="15" customHeight="1">
+          <t>арх. Павел Андреев; карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="24" customHeight="1">
       <c r="A32" s="4" t="inlineStr">
         <is>
           <t>Резиденция 1864</t>
@@ -3088,11 +3128,11 @@
       </c>
       <c r="S32" s="4" t="inlineStr">
         <is>
-          <t>апартаменты; бывший Царев сад</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="15" customHeight="1">
+          <t>апартаменты; бывший Царев сад; карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="24" customHeight="1">
       <c r="A33" s="10" t="inlineStr">
         <is>
           <t>Тессинский, 1</t>
@@ -3171,7 +3211,7 @@
       </c>
       <c r="S33" s="10" t="inlineStr">
         <is>
-          <t>ввод август 2023</t>
+          <t>ввод август 2023; карточка ЖК на Циан не найдена, год по объявлениям</t>
         </is>
       </c>
     </row>
@@ -3248,9 +3288,13 @@
         </is>
       </c>
       <c r="R34" s="5" t="inlineStr"/>
-      <c r="S34" s="4" t="inlineStr"/>
-    </row>
-    <row r="35" ht="15" customHeight="1">
+      <c r="S34" s="4" t="inlineStr">
+        <is>
+          <t>карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="24" customHeight="1">
       <c r="A35" s="10" t="inlineStr">
         <is>
           <t>Artisan (Артисан)</t>
@@ -3329,11 +3373,11 @@
       </c>
       <c r="S35" s="10" t="inlineStr">
         <is>
-          <t>также указывается Era One Holding</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="15" customHeight="1">
+          <t>также указывается Era One Holding; карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="24" customHeight="1">
       <c r="A36" s="4" t="inlineStr">
         <is>
           <t>Абрикосов</t>
@@ -3414,11 +3458,11 @@
       </c>
       <c r="S36" s="4" t="inlineStr">
         <is>
-          <t>реставрация усадьбы Абрикосовых</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="15" customHeight="1">
+          <t>реставрация усадьбы Абрикосовых; карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="24" customHeight="1">
       <c r="A37" s="10" t="inlineStr">
         <is>
           <t>Клубный дом CULT (Клубный дом Культ)</t>
@@ -3497,11 +3541,11 @@
       </c>
       <c r="S37" s="10" t="inlineStr">
         <is>
-          <t>реконструкция гостиницы Варшава; арх. SPEECH</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="15" customHeight="1">
+          <t>реконструкция гостиницы Варшава; арх. SPEECH; карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="24" customHeight="1">
       <c r="A38" s="4" t="inlineStr">
         <is>
           <t>SAVVIN RIVER RESIDENCE (Саввин Ривер Резиденс)</t>
@@ -3582,11 +3626,11 @@
       </c>
       <c r="S38" s="4" t="inlineStr">
         <is>
-          <t>арх. Цимайло Ляшенко и Партнеры</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="15" customHeight="1">
+          <t>арх. Цимайло Ляшенко и Партнеры; карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="24" customHeight="1">
       <c r="A39" s="10" t="inlineStr">
         <is>
           <t>Рахманинов</t>
@@ -3667,11 +3711,11 @@
       </c>
       <c r="S39" s="10" t="inlineStr">
         <is>
-          <t>реконструкция; также АгроСервисСтрой</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="15" customHeight="1">
+          <t>реконструкция; также АгроСервисСтрой; карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="24" customHeight="1">
       <c r="A40" s="4" t="inlineStr">
         <is>
           <t>Пироговская 14</t>
@@ -3752,7 +3796,7 @@
       </c>
       <c r="S40" s="4" t="inlineStr">
         <is>
-          <t>апартаменты; генподрядчик STRABAG</t>
+          <t>апартаменты; генподрядчик STRABAG; карточка ЖК на Циан не найдена, год по объявлениям</t>
         </is>
       </c>
     </row>
@@ -3835,7 +3879,11 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="S41" s="10" t="inlineStr"/>
+      <c r="S41" s="10" t="inlineStr">
+        <is>
+          <t>карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="15" customHeight="1">
       <c r="A42" s="4" t="inlineStr">
@@ -3916,11 +3964,11 @@
       </c>
       <c r="S42" s="4" t="inlineStr">
         <is>
-          <t>4 секции</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="15" customHeight="1">
+          <t>4 секции; карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="24" customHeight="1">
       <c r="A43" s="10" t="inlineStr">
         <is>
           <t>Садовые кварталы</t>
@@ -3995,11 +4043,11 @@
       <c r="R43" s="11" t="inlineStr"/>
       <c r="S43" s="10" t="inlineStr">
         <is>
-          <t>очереди 2012–2023; в выборку попали корпуса 2018+</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="15" customHeight="1">
+          <t>очереди 2012–2023; в выборку попали корпуса 2018+; карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="24" customHeight="1">
       <c r="A44" s="4" t="inlineStr">
         <is>
           <t>Малая Ордынка 19</t>
@@ -4080,11 +4128,11 @@
       </c>
       <c r="S44" s="4" t="inlineStr">
         <is>
-          <t>завершён сентябрь 2019</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="15" customHeight="1">
+          <t>завершён сентябрь 2019; карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="24" customHeight="1">
       <c r="A45" s="10" t="inlineStr">
         <is>
           <t>Дом в Газетном</t>
@@ -4163,7 +4211,7 @@
       </c>
       <c r="S45" s="10" t="inlineStr">
         <is>
-          <t>реконструкция</t>
+          <t>реконструкция; карточка ЖК на Циан не найдена, год по объявлениям</t>
         </is>
       </c>
     </row>
@@ -4246,7 +4294,11 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="S46" s="4" t="inlineStr"/>
+      <c r="S46" s="4" t="inlineStr">
+        <is>
+          <t>карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="15" customHeight="1">
       <c r="A47" s="10" t="inlineStr">
@@ -4321,9 +4373,13 @@
         </is>
       </c>
       <c r="R47" s="11" t="inlineStr"/>
-      <c r="S47" s="10" t="inlineStr"/>
-    </row>
-    <row r="48" ht="15" customHeight="1">
+      <c r="S47" s="10" t="inlineStr">
+        <is>
+          <t>карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="24" customHeight="1">
       <c r="A48" s="4" t="inlineStr">
         <is>
           <t>Золотой, жилой квартал</t>
@@ -4404,11 +4460,11 @@
       </c>
       <c r="S48" s="4" t="inlineStr">
         <is>
-          <t>126 квартир + 19 двухуровневых; арх. SPEECH</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="15" customHeight="1">
+          <t>126 квартир + 19 двухуровневых; арх. SPEECH; карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="24" customHeight="1">
       <c r="A49" s="10" t="inlineStr">
         <is>
           <t>Саввинская 17</t>
@@ -4489,7 +4545,7 @@
       </c>
       <c r="S49" s="10" t="inlineStr">
         <is>
-          <t>потолки 6.4-7 м; арх. AI Studio</t>
+          <t>потолки 6.4-7 м; арх. AI Studio; карточка ЖК на Циан не найдена, год по объявлениям</t>
         </is>
       </c>
     </row>
@@ -4574,11 +4630,11 @@
       </c>
       <c r="S50" s="4" t="inlineStr">
         <is>
-          <t>сдан в 2026, продажи от застройщика; реконструкция дома 1915 г.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="15" customHeight="1">
+          <t>сдан в 2026, продажи от застройщика; реконструкция дома 1915 г.; карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="24" customHeight="1">
       <c r="A51" s="10" t="inlineStr">
         <is>
           <t>Magnum (Магнум)</t>
@@ -4657,11 +4713,11 @@
       </c>
       <c r="S51" s="10" t="inlineStr">
         <is>
-          <t>арх. бюро VOSTOK</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="15" customHeight="1">
+          <t>арх. бюро VOSTOK; карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="24" customHeight="1">
       <c r="A52" s="4" t="inlineStr">
         <is>
           <t>Дом Бакст на Патриарших</t>
@@ -4740,11 +4796,11 @@
       </c>
       <c r="S52" s="4" t="inlineStr">
         <is>
-          <t>также указывается АСН-Инвест; арх. Павел Андреев</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="15" customHeight="1">
+          <t>также указывается АСН-Инвест; арх. Павел Андреев; карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="24" customHeight="1">
       <c r="A53" s="10" t="inlineStr">
         <is>
           <t>Клубный дом TURGENEV (Тургенев)</t>
@@ -4825,11 +4881,11 @@
       </c>
       <c r="S53" s="10" t="inlineStr">
         <is>
-          <t>5 секций; арх. Squire &amp; Partners</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="15" customHeight="1">
+          <t>5 секций; арх. Squire &amp; Partners; карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="24" customHeight="1">
       <c r="A54" s="4" t="inlineStr">
         <is>
           <t>Villa Grace (Вилла Грейс)</t>
@@ -4910,7 +4966,7 @@
       </c>
       <c r="S54" s="4" t="inlineStr">
         <is>
-          <t>ввод 3 кв. 2020; часть источников 4 кв. 2022</t>
+          <t>ввод 3 кв. 2020; часть источников 4 кв. 2022; карточка ЖК на Циан не найдена, год по объявлениям</t>
         </is>
       </c>
     </row>
@@ -4987,7 +5043,11 @@
         </is>
       </c>
       <c r="R55" s="11" t="inlineStr"/>
-      <c r="S55" s="10" t="inlineStr"/>
+      <c r="S55" s="10" t="inlineStr">
+        <is>
+          <t>карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="15" customHeight="1">
       <c r="A56" s="4" t="inlineStr">
@@ -5068,7 +5128,11 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="S56" s="4" t="inlineStr"/>
+      <c r="S56" s="4" t="inlineStr">
+        <is>
+          <t>карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="15" customHeight="1">
       <c r="A57" s="10" t="inlineStr">
@@ -5143,9 +5207,13 @@
         </is>
       </c>
       <c r="R57" s="11" t="inlineStr"/>
-      <c r="S57" s="10" t="inlineStr"/>
-    </row>
-    <row r="58" ht="15" customHeight="1">
+      <c r="S57" s="10" t="inlineStr">
+        <is>
+          <t>карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="24" customHeight="1">
       <c r="A58" s="4" t="inlineStr">
         <is>
           <t>Саввинская 27</t>
@@ -5226,7 +5294,7 @@
       </c>
       <c r="S58" s="4" t="inlineStr">
         <is>
-          <t>апартаменты</t>
+          <t>апартаменты; карточка ЖК на Циан не найдена, год по объявлениям</t>
         </is>
       </c>
     </row>
@@ -5303,9 +5371,13 @@
         </is>
       </c>
       <c r="R59" s="11" t="inlineStr"/>
-      <c r="S59" s="10" t="inlineStr"/>
-    </row>
-    <row r="60" ht="15" customHeight="1">
+      <c r="S59" s="10" t="inlineStr">
+        <is>
+          <t>карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="24" customHeight="1">
       <c r="A60" s="4" t="inlineStr">
         <is>
           <t>Хамовники 12</t>
@@ -5386,7 +5458,7 @@
       </c>
       <c r="S60" s="4" t="inlineStr">
         <is>
-          <t>арх. Евгений Герасимов</t>
+          <t>арх. Евгений Герасимов; карточка ЖК на Циан не найдена, год по объявлениям</t>
         </is>
       </c>
     </row>
@@ -5463,7 +5535,11 @@
         </is>
       </c>
       <c r="R61" s="11" t="inlineStr"/>
-      <c r="S61" s="10" t="inlineStr"/>
+      <c r="S61" s="10" t="inlineStr">
+        <is>
+          <t>карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="15" customHeight="1">
       <c r="A62" s="4" t="inlineStr">
@@ -5538,7 +5614,11 @@
         </is>
       </c>
       <c r="R62" s="5" t="inlineStr"/>
-      <c r="S62" s="4" t="inlineStr"/>
+      <c r="S62" s="4" t="inlineStr">
+        <is>
+          <t>карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="24" customHeight="1">
       <c r="A63" s="10" t="inlineStr">
@@ -5613,7 +5693,11 @@
         </is>
       </c>
       <c r="R63" s="11" t="inlineStr"/>
-      <c r="S63" s="10" t="inlineStr"/>
+      <c r="S63" s="10" t="inlineStr">
+        <is>
+          <t>карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="15" customHeight="1">
       <c r="A64" s="4" t="inlineStr">
@@ -5688,7 +5772,11 @@
         </is>
       </c>
       <c r="R64" s="5" t="inlineStr"/>
-      <c r="S64" s="4" t="inlineStr"/>
+      <c r="S64" s="4" t="inlineStr">
+        <is>
+          <t>карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="24" customHeight="1">
       <c r="A65" s="10" t="inlineStr">
@@ -5769,11 +5857,11 @@
       </c>
       <c r="S65" s="10" t="inlineStr">
         <is>
-          <t>введён июль 2024; арх. John McAslan + Partners</t>
-        </is>
-      </c>
-    </row>
-    <row r="66" ht="15" customHeight="1">
+          <t>введён июль 2024; арх. John McAslan + Partners; карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="24" customHeight="1">
       <c r="A66" s="4" t="inlineStr">
         <is>
           <t>Малая Бронная 15</t>
@@ -5854,7 +5942,7 @@
       </c>
       <c r="S66" s="4" t="inlineStr">
         <is>
-          <t>акт ввода 31.07.2019</t>
+          <t>акт ввода 31.07.2019; карточка ЖК на Циан не найдена, год по объявлениям</t>
         </is>
       </c>
     </row>
@@ -5931,7 +6019,11 @@
         </is>
       </c>
       <c r="R67" s="11" t="inlineStr"/>
-      <c r="S67" s="10" t="inlineStr"/>
+      <c r="S67" s="10" t="inlineStr">
+        <is>
+          <t>карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="30" customHeight="1">
       <c r="A69" s="18" t="inlineStr">
@@ -6664,7 +6756,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1">
+    <row r="10" ht="24" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Тессинский V</t>
@@ -6733,7 +6825,7 @@
       </c>
       <c r="Q10" s="4" t="inlineStr">
         <is>
-          <t>старт продаж апрель 2026, котлован</t>
+          <t>старт продаж апрель 2026, котлован; карточка ЖК на Циан не найдена, год по объявлениям</t>
         </is>
       </c>
     </row>
@@ -6960,7 +7052,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1">
+    <row r="14" ht="24" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve"> Клубный дом «Резиденции Воронцова»</t>
@@ -7029,7 +7121,7 @@
       </c>
       <c r="Q14" s="4" t="inlineStr">
         <is>
-          <t>ранее Sun Development; арх. Blank Architects</t>
+          <t>ранее Sun Development; арх. Blank Architects; карточка ЖК на Циан не найдена, год по объявлениям</t>
         </is>
       </c>
     </row>
@@ -7333,7 +7425,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="15" customHeight="1">
+    <row r="19" ht="24" customHeight="1">
       <c r="A19" s="10" t="inlineStr">
         <is>
           <t>Казачий</t>
@@ -7402,7 +7494,7 @@
       </c>
       <c r="Q19" s="10" t="inlineStr">
         <is>
-          <t>76 квартир + 4 пентхауса; арх. WALL</t>
+          <t>76 квартир + 4 пентхауса; арх. WALL; карточка ЖК на Циан не найдена, год по объявлениям</t>
         </is>
       </c>
     </row>
@@ -7623,7 +7715,11 @@
           <t>Циан 2026-09-07</t>
         </is>
       </c>
-      <c r="Q22" s="4" t="inlineStr"/>
+      <c r="Q22" s="4" t="inlineStr">
+        <is>
+          <t>карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="15" customHeight="1">
       <c r="A23" s="10" t="inlineStr">
@@ -7692,9 +7788,13 @@
           <t>Циан 2026-09-07</t>
         </is>
       </c>
-      <c r="Q23" s="10" t="inlineStr"/>
-    </row>
-    <row r="24" ht="15" customHeight="1">
+      <c r="Q23" s="10" t="inlineStr">
+        <is>
+          <t>карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="24" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
           <t>ТИТУЛ Империал</t>
@@ -7763,7 +7863,7 @@
       </c>
       <c r="Q24" s="4" t="inlineStr">
         <is>
-          <t>12 лотов 83-131 м², не более 3 квартир на этаже</t>
+          <t>12 лотов 83-131 м², не более 3 квартир на этаже; карточка ЖК на Циан не найдена, год по объявлениям</t>
         </is>
       </c>
     </row>
@@ -7836,11 +7936,11 @@
       </c>
       <c r="Q25" s="10" t="inlineStr">
         <is>
-          <t>Софийская наб., усадьба Кокорева; в июне 2026 fee-девелопер Hutton вышел из проекта, площадка у V2 Group (Коммерсантъ); инвестор V2Group; юрлицо СЗ Суплекс Технолоджис; cian: 2028</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="15" customHeight="1">
+          <t>Софийская наб., усадьба Кокорева; в июне 2026 fee-девелопер Hutton вышел из проекта, площадка у V2 Group (Коммерсантъ); инвестор V2Group; юрлицо СЗ Суплекс Технолоджис; cian: 2028; карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="24" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
         <is>
           <t>Дом Спорта</t>
@@ -7909,7 +8009,7 @@
       </c>
       <c r="Q26" s="4" t="inlineStr">
         <is>
-          <t>старт продаж 2026, стройка начата (Ведомости)</t>
+          <t>старт продаж 2026, стройка начата (Ведомости); карточка ЖК на Циан не найдена, год по объявлениям</t>
         </is>
       </c>
     </row>
@@ -8363,7 +8463,7 @@
       </c>
       <c r="Q32" s="4" t="inlineStr"/>
     </row>
-    <row r="33" ht="15" customHeight="1">
+    <row r="33" ht="24" customHeight="1">
       <c r="A33" s="10" t="inlineStr">
         <is>
           <t>Kuznetsky Most 12 by Lalique (Кузнецкий Мост 12)</t>
@@ -8432,11 +8532,11 @@
       </c>
       <c r="Q33" s="10" t="inlineStr">
         <is>
-          <t>реконструкция; коллаборация с Lalique</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="15" customHeight="1">
+          <t>реконструкция; коллаборация с Lalique; карточка ЖК на Циан не найдена, год по объявлениям</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="24" customHeight="1">
       <c r="A34" s="4" t="inlineStr">
         <is>
           <t>ДОМ XXII</t>
@@ -8505,7 +8605,7 @@
       </c>
       <c r="Q34" s="4" t="inlineStr">
         <is>
-          <t>арх. Сергей Киселев и Партнеры</t>
+          <t>арх. Сергей Киселев и Партнеры; карточка ЖК на Циан не найдена, год по объявлениям</t>
         </is>
       </c>
     </row>
@@ -9032,7 +9132,7 @@
       </c>
       <c r="Q41" s="10" t="inlineStr">
         <is>
-          <t>Le Dôme; СЗ Соймоновский 3; арх. Paris Classical Architecture</t>
+          <t>Le Dôme; СЗ Соймоновский 3; арх. Paris Classical Architecture; карточка ЖК на Циан не найдена, год по объявлениям</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Workbook: 10pt body font, tighter planning widths
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Bv8NELxW2W7udnb3XUFGS2
</commit_message>
<xml_diff>
--- a/docs/premium-cao/premium-zhk-cao.xlsx
+++ b/docs/premium-cao/premium-zhk-cao.xlsx
@@ -29,7 +29,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -57,18 +57,23 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <sz val="9"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
       <sz val="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="000563C1"/>
-      <sz val="9"/>
-      <u val="single"/>
     </font>
   </fonts>
   <fills count="9">
@@ -175,7 +180,7 @@
     <xf numFmtId="3" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -193,7 +198,7 @@
     <xf numFmtId="3" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="7" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -211,13 +216,13 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -6472,7 +6477,7 @@
       </c>
       <c r="P30" s="4" t="inlineStr"/>
     </row>
-    <row r="31" ht="15" customHeight="1">
+    <row r="31" ht="26" customHeight="1">
       <c r="A31" s="10" t="inlineStr">
         <is>
           <t>Клубный дом DUO (Дуо)</t>
@@ -6485,7 +6490,7 @@
       </c>
       <c r="C31" s="11" t="inlineStr">
         <is>
-          <t>2028</t>
+          <t>1 кв. 2028</t>
         </is>
       </c>
       <c r="D31" s="10" t="inlineStr">
@@ -6533,7 +6538,11 @@
           <t>бетон</t>
         </is>
       </c>
-      <c r="O31" s="11" t="inlineStr"/>
+      <c r="O31" s="15" t="inlineStr">
+        <is>
+          <t>ссылка</t>
+        </is>
+      </c>
       <c r="P31" s="10" t="inlineStr"/>
     </row>
     <row r="32" ht="15" customHeight="1">
@@ -6549,7 +6558,7 @@
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>2029</t>
+          <t>1 кв. 2029</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
@@ -6597,7 +6606,11 @@
           <t>бетон</t>
         </is>
       </c>
-      <c r="O32" s="5" t="inlineStr"/>
+      <c r="O32" s="9" t="inlineStr">
+        <is>
+          <t>ссылка</t>
+        </is>
+      </c>
       <c r="P32" s="4" t="inlineStr"/>
     </row>
     <row r="33" ht="26" customHeight="1">
@@ -7865,23 +7878,25 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId45"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.35" bottom="0.35" header="0.2" footer="0.2"/>
@@ -7906,22 +7921,22 @@
   <dimension ref="A1:P32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="9" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
     <col width="10" customWidth="1" min="13" max="13"/>
     <col width="10" customWidth="1" min="14" max="14"/>
     <col width="7" customWidth="1" min="15" max="15"/>
-    <col width="60" customWidth="1" min="16" max="16"/>
+    <col width="52" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">

</xml_diff>

<commit_message>
Add sheet-1 project descriptions
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Bv8NELxW2W7udnb3XUFGS2
</commit_message>
<xml_diff>
--- a/docs/premium-cao/premium-zhk-cao.xlsx
+++ b/docs/premium-cao/premium-zhk-cao.xlsx
@@ -787,9 +787,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q4" s="4" t="inlineStr"/>
-    </row>
-    <row r="5" ht="15" customHeight="1">
+      <c r="Q4" s="4" t="inlineStr">
+        <is>
+          <t>Клубный дом 12 эт. на 190 апартаментов с отель-сервисом и отделкой, у Белорусской и Маяковской</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="26" customHeight="1">
       <c r="A5" s="10" t="inlineStr">
         <is>
           <t>NEVA TOWERS (Нева Тауэрс)</t>
@@ -860,9 +864,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q5" s="10" t="inlineStr"/>
-    </row>
-    <row r="6" ht="15" customHeight="1">
+      <c r="Q5" s="10" t="inlineStr">
+        <is>
+          <t>Две башни 63 и 77 эт. в Сити на общем стилобате, апартаменты, панорамные окна, бассейн на крыше</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="26" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Sinatra (Синатра)</t>
@@ -933,9 +941,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q6" s="4" t="inlineStr"/>
-    </row>
-    <row r="7" ht="15" customHeight="1">
+      <c r="Q6" s="4" t="inlineStr">
+        <is>
+          <t>Клубный дом 7 эт. на 82 апартамента и пентхауса с потолками до 5,5 м, Тишинка у Белорусской</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="26" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
           <t>LUMIN (ЛЮМИН)</t>
@@ -1006,9 +1018,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q7" s="10" t="inlineStr"/>
-    </row>
-    <row r="8" ht="15" customHeight="1">
+      <c r="Q7" s="10" t="inlineStr">
+        <is>
+          <t>Клубный дом 8 эт. на 58 лотов, стеклянные фасады (ЦЛП), терраса на крыше, 250 м от Зарядья</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="26" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Уланский, 13</t>
@@ -1079,9 +1095,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q8" s="4" t="inlineStr"/>
-    </row>
-    <row r="9" ht="15" customHeight="1">
+      <c r="Q8" s="4" t="inlineStr">
+        <is>
+          <t>Реконструкция доходного дома 1886 г., 4 эт., 10 квартир и 2 пентхауса, у Чистых прудов</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="26" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
         <is>
           <t>Современник</t>
@@ -1152,9 +1172,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q9" s="10" t="inlineStr"/>
-    </row>
-    <row r="10" ht="15" customHeight="1">
+      <c r="Q9" s="10" t="inlineStr">
+        <is>
+          <t>Реконструкция дома XIX в. с надстройкой, 5 эт., 86 квартир, у Чистых прудов и Красных Ворот</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="26" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Репаблик</t>
@@ -1225,9 +1249,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q10" s="4" t="inlineStr"/>
-    </row>
-    <row r="11" ht="15" customHeight="1">
+      <c r="Q10" s="4" t="inlineStr">
+        <is>
+          <t>Квартал из 10 башен 26–33 эт. на месте вагонных мастерских, лобби до 7 м, у Белорусской</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="26" customHeight="1">
       <c r="A11" s="10" t="inlineStr">
         <is>
           <t>City Park (Сити Парк)</t>
@@ -1298,9 +1326,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q11" s="10" t="inlineStr"/>
-    </row>
-    <row r="12" ht="15" customHeight="1">
+      <c r="Q11" s="10" t="inlineStr">
+        <is>
+          <t>Квартал из 6 корпусов 6–20 эт., 1220 квартир, двор-парк, рядом с Сити и парком Красная Пресня</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="26" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t>SkyView</t>
@@ -1371,9 +1403,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q12" s="4" t="inlineStr"/>
-    </row>
-    <row r="13" ht="15" customHeight="1">
+      <c r="Q12" s="4" t="inlineStr">
+        <is>
+          <t>Четыре 20-эт. башни на 304 апартамента у Белого дома, панорамные виды, парк Пресня рядом</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="26" customHeight="1">
       <c r="A13" s="10" t="inlineStr">
         <is>
           <t>Полянка/44</t>
@@ -1444,7 +1480,11 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q13" s="10" t="inlineStr"/>
+      <c r="Q13" s="10" t="inlineStr">
+        <is>
+          <t>Квартал из 8 особняков (3 исторических) по 22–24 квартиры, сад с ручьём, паркинг, у Полянки</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="26" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
@@ -1517,9 +1557,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q14" s="4" t="inlineStr"/>
-    </row>
-    <row r="15" ht="15" customHeight="1">
+      <c r="Q14" s="4" t="inlineStr">
+        <is>
+          <t>Квартал из 8 домов-особняков 7–9 эт., 59 лотов, фасады из юрского мрамора, 1,5 км до Зарядья</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="26" customHeight="1">
       <c r="A15" s="10" t="inlineStr">
         <is>
           <t>Bogenhouse (Богенхаус)</t>
@@ -1590,9 +1634,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q15" s="10" t="inlineStr"/>
-    </row>
-    <row r="16" ht="15" customHeight="1">
+      <c r="Q15" s="10" t="inlineStr">
+        <is>
+          <t>Клубный дом 5 эт. на 43 апартамента и 5 пентхаусов на Озерковской наб., Замоскворечье</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="26" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Capital Towers (Капитал Тауэрс)</t>
@@ -1663,9 +1711,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q16" s="4" t="inlineStr"/>
-    </row>
-    <row r="17" ht="15" customHeight="1">
+      <c r="Q16" s="4" t="inlineStr">
+        <is>
+          <t>Три башни 61–65 эт. на стилобате у Сити, 787 квартир, виды на реку и парк Красная Пресня</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="26" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
           <t>BALCHUG VIEWPOINT (Балчуг Вьюпоинт)</t>
@@ -1736,7 +1788,11 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q17" s="10" t="inlineStr"/>
+      <c r="Q17" s="10" t="inlineStr">
+        <is>
+          <t>Апарт-комплекс 9 эт. на 116 резиденций на Садовнической наб., панорамные окна, 10 мин до Кремля</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="26" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
@@ -1809,7 +1865,11 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q18" s="4" t="inlineStr"/>
+      <c r="Q18" s="4" t="inlineStr">
+        <is>
+          <t>Клубный дом 6 эт. на 18 квартир с потолками 3,5 м, 2 пентхауса, 200 м от м. Полянка</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="26" customHeight="1">
       <c r="A19" s="10" t="inlineStr">
@@ -1882,9 +1942,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q19" s="10" t="inlineStr"/>
-    </row>
-    <row r="20" ht="15" customHeight="1">
+      <c r="Q19" s="10" t="inlineStr">
+        <is>
+          <t>Клубный дом 8 эт. на 47 апартаментов, фасады из травертина (ЦЛП), у Цветного бульвара</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="26" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
           <t>A.Residence (А Резиденс)</t>
@@ -1955,9 +2019,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q20" s="4" t="inlineStr"/>
-    </row>
-    <row r="21" ht="15" customHeight="1">
+      <c r="Q20" s="4" t="inlineStr">
+        <is>
+          <t>Пять корпусов 5–9 эт., 190 апартаментов и пентхаусов, фасады из камня (ЦЛП), Садовническая</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="26" customHeight="1">
       <c r="A21" s="10" t="inlineStr">
         <is>
           <t>Roza Rossa (Роза Росса)</t>
@@ -2028,7 +2096,11 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q21" s="10" t="inlineStr"/>
+      <c r="Q21" s="10" t="inlineStr">
+        <is>
+          <t>Дом 6 эт. на 120 апартаментов по проекту Пьеро Лиссони, сервис отеля Метрополь, SPA, бассейн</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="26" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
@@ -2101,9 +2173,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q22" s="4" t="inlineStr"/>
-    </row>
-    <row r="23" ht="15" customHeight="1">
+      <c r="Q22" s="4" t="inlineStr">
+        <is>
+          <t>Собрание 7 клубных домов, ок. 90 лотов, исторические особняки и новые корпуса, у Третьяковки</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="26" customHeight="1">
       <c r="A23" s="10" t="inlineStr">
         <is>
           <t>Дом NV/9</t>
@@ -2174,7 +2250,11 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q23" s="10" t="inlineStr"/>
+      <c r="Q23" s="10" t="inlineStr">
+        <is>
+          <t>Два клубных корпуса 4–9 эт. на 77 квартир, 6 пентхаусов с каминами, патио, у Яузы</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="26" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
@@ -2247,7 +2327,11 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q24" s="4" t="inlineStr"/>
+      <c r="Q24" s="4" t="inlineStr">
+        <is>
+          <t>Клубный дом 6 эт. на 28 лотов с фасадом доходного дома 1908 г. (ЦЛП), у Малой Грузинской</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="26" customHeight="1">
       <c r="A25" s="10" t="inlineStr">
@@ -2320,9 +2404,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q25" s="10" t="inlineStr"/>
-    </row>
-    <row r="26" ht="15" customHeight="1">
+      <c r="Q25" s="10" t="inlineStr">
+        <is>
+          <t>Два клубных корпуса 6 эт. на 73 квартиры, 11 пентхаусов, стиль модерн, Космодамианская наб.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="26" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
         <is>
           <t>Софийский</t>
@@ -2393,9 +2481,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q26" s="4" t="inlineStr"/>
-    </row>
-    <row r="27" ht="15" customHeight="1">
+      <c r="Q26" s="4" t="inlineStr">
+        <is>
+          <t>Апарт-комплекс 8 эт. на Балчуге в 500 м от Кремля, окна в пол с видом на Кремль, отель-сервис</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="26" customHeight="1">
       <c r="A27" s="10" t="inlineStr">
         <is>
           <t>Дом на Тишинке</t>
@@ -2466,9 +2558,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q27" s="10" t="inlineStr"/>
-    </row>
-    <row r="28" ht="15" customHeight="1">
+      <c r="Q27" s="10" t="inlineStr">
+        <is>
+          <t>Два корпуса 18 эт. на 142 квартиры от 87 м², пентхаусы с патио и каминами, Тишинка</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="26" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
         <is>
           <t>Тессинский, 1</t>
@@ -2539,9 +2635,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q28" s="4" t="inlineStr"/>
-    </row>
-    <row r="29" ht="15" customHeight="1">
+      <c r="Q28" s="4" t="inlineStr">
+        <is>
+          <t>Клубный дом 8 эт. и особняк, 71 лот, пентхаусы с потолками 6,9 м и каминами, у Яузы</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="26" customHeight="1">
       <c r="A29" s="10" t="inlineStr">
         <is>
           <t>Lucky (Лаки)</t>
@@ -2612,9 +2712,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q29" s="10" t="inlineStr"/>
-    </row>
-    <row r="30" ht="15" customHeight="1">
+      <c r="Q29" s="10" t="inlineStr">
+        <is>
+          <t>Квартал из 8 корпусов 15–21 эт., 619 квартир, дворы без машин, 200 м от м. Улица 1905 года</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="26" customHeight="1">
       <c r="A30" s="4" t="inlineStr">
         <is>
           <t>Artisan (Артисан)</t>
@@ -2685,9 +2789,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q30" s="4" t="inlineStr"/>
-    </row>
-    <row r="31" ht="15" customHeight="1">
+      <c r="Q30" s="4" t="inlineStr">
+        <is>
+          <t>Клубный дом 5 эт. на 32 резиденции, воссозданный ампирный фасад, на Арбате</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="26" customHeight="1">
       <c r="A31" s="10" t="inlineStr">
         <is>
           <t>Абрикосов</t>
@@ -2758,7 +2866,11 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q31" s="10" t="inlineStr"/>
+      <c r="Q31" s="10" t="inlineStr">
+        <is>
+          <t>Реконструкция особняка Абрикосовых на палатах XVII в., 5 эт., 26 квартир, у Чистых прудов</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="26" customHeight="1">
       <c r="A32" s="4" t="inlineStr">
@@ -2831,7 +2943,11 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q32" s="4" t="inlineStr"/>
+      <c r="Q32" s="4" t="inlineStr">
+        <is>
+          <t>Дом 9 эт. на 91 квартиру с отделкой, 12 пентхаусов, каменные фасады, на месте гостиницы Варшава</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="26" customHeight="1">
       <c r="A33" s="10" t="inlineStr">
@@ -2904,9 +3020,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q33" s="10" t="inlineStr"/>
-    </row>
-    <row r="34" ht="15" customHeight="1">
+      <c r="Q33" s="10" t="inlineStr">
+        <is>
+          <t>Четыре корпуса 4–9 эт. на 169 квартир на Саввинской наб., окна в пол, виды на реку</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="26" customHeight="1">
       <c r="A34" s="4" t="inlineStr">
         <is>
           <t>Пироговская 14</t>
@@ -2977,9 +3097,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q34" s="4" t="inlineStr"/>
-    </row>
-    <row r="35" ht="15" customHeight="1">
+      <c r="Q34" s="4" t="inlineStr">
+        <is>
+          <t>Клубный апарт-дом 9 эт. на 53 лота, фитнес, библиотека, паркинг на 61 м/м, Хамовники у Усачёва</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="26" customHeight="1">
       <c r="A35" s="10" t="inlineStr">
         <is>
           <t>Cloud Nine (Клауд Найн)</t>
@@ -3050,7 +3174,11 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q35" s="10" t="inlineStr"/>
+      <c r="Q35" s="10" t="inlineStr">
+        <is>
+          <t>Реконструкция 4 исторических зданий, 7–9 эт., 45 квартир, паркинг на 70 м/м, 900 м от Кремля</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="26" customHeight="1">
       <c r="A36" s="4" t="inlineStr">
@@ -3123,9 +3251,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q36" s="4" t="inlineStr"/>
-    </row>
-    <row r="37" ht="15" customHeight="1">
+      <c r="Q36" s="4" t="inlineStr">
+        <is>
+          <t>Дом 8 эт. в стиле ампир на 53 квартиры, фасады из известняка, виды на Кремль и Зарядье</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="26" customHeight="1">
       <c r="A37" s="10" t="inlineStr">
         <is>
           <t>Садовые кварталы</t>
@@ -3196,9 +3328,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q37" s="10" t="inlineStr"/>
-    </row>
-    <row r="38" ht="15" customHeight="1">
+      <c r="Q37" s="10" t="inlineStr">
+        <is>
+          <t>Квартал из 33 клубных домов на 11 га с прудом и парком, ок. 920 квартир, у Новодевичьего</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="26" customHeight="1">
       <c r="A38" s="4" t="inlineStr">
         <is>
           <t>Малая Ордынка 19</t>
@@ -3269,9 +3405,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q38" s="4" t="inlineStr"/>
-    </row>
-    <row r="39" ht="15" customHeight="1">
+      <c r="Q38" s="4" t="inlineStr">
+        <is>
+          <t>Клубный дом 6 эт. на 67 квартир, потолки 3,3–3,6 м, паркинг на 124 м/м, у Третьяковской</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="26" customHeight="1">
       <c r="A39" s="10" t="inlineStr">
         <is>
           <t>Дом в Газетном</t>
@@ -3342,9 +3482,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q39" s="10" t="inlineStr"/>
-    </row>
-    <row r="40" ht="15" customHeight="1">
+      <c r="Q39" s="10" t="inlineStr">
+        <is>
+          <t>Клубный дом 5 эт. на 24 апартамента, пентхаусы и городская вилла, 1 км от Кремля</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="26" customHeight="1">
       <c r="A40" s="4" t="inlineStr">
         <is>
           <t>Zvonarsky Deluxe (Звонарский Делюкс)</t>
@@ -3415,9 +3559,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q40" s="4" t="inlineStr"/>
-    </row>
-    <row r="41" ht="15" customHeight="1">
+      <c r="Q40" s="4" t="inlineStr">
+        <is>
+          <t>Клубный дом 9 эт. на 27 квартир по 3 на этаже, между Неглинной и Рождественкой</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="26" customHeight="1">
       <c r="A41" s="10" t="inlineStr">
         <is>
           <t>White Khamovniki (Вайт Хамовники)</t>
@@ -3488,7 +3636,11 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q41" s="10" t="inlineStr"/>
+      <c r="Q41" s="10" t="inlineStr">
+        <is>
+          <t>Две башни 15 эт. на 76 квартир, архбетон и латунь, паркинг на 120 м/м, у Фрунзенской</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="26" customHeight="1">
       <c r="A42" s="4" t="inlineStr">
@@ -3561,9 +3713,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q42" s="4" t="inlineStr"/>
-    </row>
-    <row r="43" ht="15" customHeight="1">
+      <c r="Q42" s="4" t="inlineStr">
+        <is>
+          <t>Квартал 1,7 га на Софийской наб., 162 лота с террасами и садами, виды на Кремль, паркинг</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="26" customHeight="1">
       <c r="A43" s="10" t="inlineStr">
         <is>
           <t>Magnum (Магнум)</t>
@@ -3634,7 +3790,11 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q43" s="10" t="inlineStr"/>
+      <c r="Q43" s="10" t="inlineStr">
+        <is>
+          <t>Клубный дом 6 эт. на 44 квартиры, английский стиль, 4 пентхауса с зимними садами, Усачёва</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="26" customHeight="1">
       <c r="A44" s="4" t="inlineStr">
@@ -3707,9 +3867,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q44" s="4" t="inlineStr"/>
-    </row>
-    <row r="45" ht="15" customHeight="1">
+      <c r="Q44" s="4" t="inlineStr">
+        <is>
+          <t>Клубный дом 3–6 эт. на 18 квартир, панно по Баксту (арх. П. Андреев), у Патриарших</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="26" customHeight="1">
       <c r="A45" s="10" t="inlineStr">
         <is>
           <t>Villa Grace (Вилла Грейс)</t>
@@ -3780,9 +3944,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q45" s="10" t="inlineStr"/>
-    </row>
-    <row r="46" ht="15" customHeight="1">
+      <c r="Q45" s="10" t="inlineStr">
+        <is>
+          <t>Клубный дом 6–7 эт. на 20 квартир от 100 м², потолки 3,5 м, между Пречистенкой и набережной</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="26" customHeight="1">
       <c r="A46" s="4" t="inlineStr">
         <is>
           <t>Brodsky (Бродский)</t>
@@ -3853,7 +4021,11 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q46" s="4" t="inlineStr"/>
+      <c r="Q46" s="4" t="inlineStr">
+        <is>
+          <t>Дом 14 эт. на 65 квартир и 2 пентхауса (ЦЛП), детский клуб, wellness, у Новодевичьих прудов</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="26" customHeight="1">
       <c r="A47" s="10" t="inlineStr">
@@ -3926,9 +4098,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q47" s="10" t="inlineStr"/>
-    </row>
-    <row r="48" ht="15" customHeight="1">
+      <c r="Q47" s="10" t="inlineStr">
+        <is>
+          <t>Дом из 8 секций 7–13 эт. на 202 квартиры, неоклассика, у Плющихи в Хамовниках</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="26" customHeight="1">
       <c r="A48" s="4" t="inlineStr">
         <is>
           <t>Carré Blanc (Карре Бланк)</t>
@@ -3999,7 +4175,11 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q48" s="4" t="inlineStr"/>
+      <c r="Q48" s="4" t="inlineStr">
+        <is>
+          <t>Особняк 5 эт. на 46 квартир (Speech), 4 пентхауса, сад 660 м² с фонтаном, у Храма Христа</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="26" customHeight="1">
       <c r="A49" s="10" t="inlineStr">
@@ -4072,9 +4252,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q49" s="10" t="inlineStr"/>
-    </row>
-    <row r="50" ht="15" customHeight="1">
+      <c r="Q49" s="10" t="inlineStr">
+        <is>
+          <t>Квартал из 3 корпусов 8–14 эт. на 98 квартир, прямые виды на Кремль, у Третьяковки</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="26" customHeight="1">
       <c r="A50" s="4" t="inlineStr">
         <is>
           <t>Хамовники 12</t>
@@ -4145,7 +4329,11 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q50" s="4" t="inlineStr"/>
+      <c r="Q50" s="4" t="inlineStr">
+        <is>
+          <t>Клубный дом 14 эт. на 51 квартиру от 100 м² (арх. Е. Герасимов), 100 м от Саввинской наб.</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="26" customHeight="1">
       <c r="A51" s="10" t="inlineStr">
@@ -4218,7 +4406,11 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q51" s="10" t="inlineStr"/>
+      <c r="Q51" s="10" t="inlineStr">
+        <is>
+          <t>Отель 5* и 14 брендовых резиденций Bulgari, таунхаусы, пентхаус, SPA, на Большой Никитской</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="26" customHeight="1">
       <c r="A52" s="4" t="inlineStr">
@@ -4291,7 +4483,11 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q52" s="4" t="inlineStr"/>
+      <c r="Q52" s="4" t="inlineStr">
+        <is>
+          <t>Три корпуса 6 эт.: реконструкция особняка и 2 новых, окна в пол, потолки до 4,6 м, у Большого</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="26" customHeight="1">
       <c r="A53" s="10" t="inlineStr">
@@ -4364,9 +4560,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q53" s="10" t="inlineStr"/>
-    </row>
-    <row r="54" ht="15" customHeight="1">
+      <c r="Q53" s="10" t="inlineStr">
+        <is>
+          <t>Клубный дом 7 эт. на 23 квартиры, потолки от 3,6 м, современная классика, у Патриарших</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="26" customHeight="1">
       <c r="A54" s="4" t="inlineStr">
         <is>
           <t>Barkli Gallery (Баркли Галлери)</t>
@@ -4437,7 +4637,11 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="Q54" s="4" t="inlineStr"/>
+      <c r="Q54" s="4" t="inlineStr">
+        <is>
+          <t>Реконструкция домов 1875 и 1913 гг., 4–7 эт., 43 лота с отделкой, 200 м от Третьяковки</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A3:Q54"/>
@@ -4647,7 +4851,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1">
+    <row r="4" ht="26" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>ЖК «Слава»</t>
@@ -4709,9 +4913,13 @@
         </is>
       </c>
       <c r="O4" s="5" t="inlineStr"/>
-      <c r="P4" s="4" t="inlineStr"/>
-    </row>
-    <row r="5" ht="15" customHeight="1">
+      <c r="P4" s="4" t="inlineStr">
+        <is>
+          <t>Квартал из 3 корпусов 6–22 эт. на Ленинградском пр., панорамное остекление, паркинг на 782 м/м</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="26" customHeight="1">
       <c r="A5" s="10" t="inlineStr">
         <is>
           <t>ЖК «Дом Дау»</t>
@@ -4777,9 +4985,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="P5" s="10" t="inlineStr"/>
-    </row>
-    <row r="6" ht="15" customHeight="1">
+      <c r="P5" s="10" t="inlineStr">
+        <is>
+          <t>Башня 85 эт., 340 м, 866 квартир на 2-й линии Краснопресненской наб. у Сити, SPA, коворкинг</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="26" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>ЖК «Начало»</t>
@@ -4845,9 +5057,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="P6" s="4" t="inlineStr"/>
-    </row>
-    <row r="7" ht="15" customHeight="1">
+      <c r="P6" s="4" t="inlineStr">
+        <is>
+          <t>Квартал из 8 корпусов 12–55 эт. на ул. Сергея Макеева, потолки 3,4–4,1 м, у Пресни</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="26" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Оне</t>
@@ -4913,7 +5129,11 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="P7" s="10" t="inlineStr"/>
+      <c r="P7" s="10" t="inlineStr">
+        <is>
+          <t>Башня 90 эт., 379 м в Москва-Сити, две башни в форме ленты Мёбиуса, Sky Bridge, сад на 338 м</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="26" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
@@ -4979,9 +5199,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="P8" s="4" t="inlineStr"/>
-    </row>
-    <row r="9" ht="15" customHeight="1">
+      <c r="P8" s="4" t="inlineStr">
+        <is>
+          <t>Две башни 96 и 83 эт., 395 м в Сити-2, 1774 квартиры, парк с бассейнами на 7 эт., APEX</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="26" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
         <is>
           <t>ЖК «Монблан»</t>
@@ -5047,7 +5271,11 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="P9" s="10" t="inlineStr"/>
+      <c r="P9" s="10" t="inlineStr">
+        <is>
+          <t>Дом из 6 секций 7–27 эт. на Шлюзовой наб., 341 квартира, вид на реку, у Павелецкой</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="26" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
@@ -5115,7 +5343,11 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="P10" s="4" t="inlineStr"/>
+      <c r="P10" s="4" t="inlineStr">
+        <is>
+          <t>Квартал из 6 домов 10–23 эт. на ул. Сергея Макеева, 265 квартир, двор-парк 1,8 га</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="26" customHeight="1">
       <c r="A11" s="10" t="inlineStr">
@@ -5183,9 +5415,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="P11" s="10" t="inlineStr"/>
-    </row>
-    <row r="12" ht="15" customHeight="1">
+      <c r="P11" s="10" t="inlineStr">
+        <is>
+          <t>Квартал из 12 домов 12–18 эт. на Лужнецкой наб., парк 8 га, вид на реку и Сити</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="26" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Тессинский V</t>
@@ -5251,7 +5487,11 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="P12" s="4" t="inlineStr"/>
+      <c r="P12" s="4" t="inlineStr">
+        <is>
+          <t>Квартал из 4 клубных домов 5–12 эт., 146 резиденций, у Серебрянической наб., Таганка</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="26" customHeight="1">
       <c r="A13" s="10" t="inlineStr">
@@ -5319,7 +5559,11 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="P13" s="10" t="inlineStr"/>
+      <c r="P13" s="10" t="inlineStr">
+        <is>
+          <t>Реконструкция Кокоревского подворья 1864 г., 7–8 эт., 68 квартир, потолки 4–7 м, Софийская наб.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="26" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
@@ -5387,9 +5631,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="P14" s="4" t="inlineStr"/>
-    </row>
-    <row r="15" ht="15" customHeight="1">
+      <c r="P14" s="4" t="inlineStr">
+        <is>
+          <t>Квартал из 10 домов 6–14 эт. на Тишинке, 404 квартиры, парк-бульвар 1,9 га, бассейн</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="26" customHeight="1">
       <c r="A15" s="10" t="inlineStr">
         <is>
           <t>ЖК «Дом Франка»</t>
@@ -5455,9 +5703,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="P15" s="10" t="inlineStr"/>
-    </row>
-    <row r="16" ht="15" customHeight="1">
+      <c r="P15" s="10" t="inlineStr">
+        <is>
+          <t>Реконструкция торгового дома 1904 г. (Кекушев) и новый корпус в Б. Кисельном пер., у Лубянки</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="26" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
           <t>ЖК «Татарская 35»</t>
@@ -5523,7 +5775,11 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="P16" s="4" t="inlineStr"/>
+      <c r="P16" s="4" t="inlineStr">
+        <is>
+          <t>Три корпуса 15–24 эт., 472 квартиры, wellness с бассейном, у Озерковской наб., Замоскворечье</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="26" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
@@ -5591,9 +5847,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="P17" s="10" t="inlineStr"/>
-    </row>
-    <row r="18" ht="15" customHeight="1">
+      <c r="P17" s="10" t="inlineStr">
+        <is>
+          <t>Клубный дом из 2 корпусов, 75 резиденций, потолки до 5,96 м, каменный фасад, ул. Обуха</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="26" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
           <t>ЖК «Дом Соболева»</t>
@@ -5659,7 +5919,11 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="P18" s="4" t="inlineStr"/>
+      <c r="P18" s="4" t="inlineStr">
+        <is>
+          <t>Клубный дом 7–8 эт. на ул. Машкова, 33 резиденции и 2 пентхауса, потолки 3,55 м, Красные Ворота</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="26" customHeight="1">
       <c r="A19" s="10" t="inlineStr">
@@ -5727,7 +5991,11 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="P19" s="10" t="inlineStr"/>
+      <c r="P19" s="10" t="inlineStr">
+        <is>
+          <t>Клубный дом 7–9 эт. (арх. Чобан), 46 резиденций, стена доходного дома 1905 г. Нирнзее, Пресня</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="26" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
@@ -5795,9 +6063,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="P20" s="4" t="inlineStr"/>
-    </row>
-    <row r="21" ht="15" customHeight="1">
+      <c r="P20" s="4" t="inlineStr">
+        <is>
+          <t>Клубный дом 13 эт. на Садовом кольце, 48 квартир, бассейн 20 м, SPA, хаммам, у Сухаревской</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="26" customHeight="1">
       <c r="A21" s="10" t="inlineStr">
         <is>
           <t>ЖК «Камергер»</t>
@@ -5863,9 +6135,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="P21" s="10" t="inlineStr"/>
-    </row>
-    <row r="22" ht="15" customHeight="1">
+      <c r="P21" s="10" t="inlineStr">
+        <is>
+          <t>Комплекс из 5 особняков в 300 м от Кремля, 17 резиденций с террасами, SPA, подземный переход</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="26" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Казачий</t>
@@ -5931,7 +6207,11 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="P22" s="4" t="inlineStr"/>
+      <c r="P22" s="4" t="inlineStr">
+        <is>
+          <t>Клубный дом 9 эт. (бюро WALL) в 1-м Казачьем пер., 76 квартир и 4 пентхауса, потолки до 3,95 м</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="26" customHeight="1">
       <c r="A23" s="10" t="inlineStr">
@@ -5999,9 +6279,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="P23" s="10" t="inlineStr"/>
-    </row>
-    <row r="24" ht="15" customHeight="1">
+      <c r="P23" s="10" t="inlineStr">
+        <is>
+          <t>Клубный квартал из 4 домов 2–10 эт. на Садовнической наб., свой парк 1 га, виллы и пентхаусы</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="26" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
           <t>Саввинская 17</t>
@@ -6067,7 +6351,11 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="P24" s="4" t="inlineStr"/>
+      <c r="P24" s="4" t="inlineStr">
+        <is>
+          <t>Клубный дом 4 эт. на 1-й линии реки в Хамовниках, 22 квартиры, окна в пол, у Девичьего поля</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="26" customHeight="1">
       <c r="A25" s="10" t="inlineStr">
@@ -6135,9 +6423,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="P25" s="10" t="inlineStr"/>
-    </row>
-    <row r="26" ht="15" customHeight="1">
+      <c r="P25" s="10" t="inlineStr">
+        <is>
+          <t>Реконструкция доходного дома 1915 г. фон Дессина, 7 эт., 36 квартир, в 50 м от Чистых прудов</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="26" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
         <is>
           <t>ЖК «PHANTOM»</t>
@@ -6203,7 +6495,11 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="P26" s="4" t="inlineStr"/>
+      <c r="P26" s="4" t="inlineStr">
+        <is>
+          <t>Клубный дом 7–9 эт. на М. Сухаревской пл., 76 квартир, пентхаусы и дуплексы, у Сухаревской</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="26" customHeight="1">
       <c r="A27" s="10" t="inlineStr">
@@ -6271,7 +6567,11 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="P27" s="10" t="inlineStr"/>
+      <c r="P27" s="10" t="inlineStr">
+        <is>
+          <t>Клубный дом 8 эт. в Костянском пер., 118 квартир, каменный фасад, бассейн, SPA, у Чистых прудов</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="26" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
@@ -6339,9 +6639,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="P28" s="4" t="inlineStr"/>
-    </row>
-    <row r="29" ht="15" customHeight="1">
+      <c r="P28" s="4" t="inlineStr">
+        <is>
+          <t>Клубный дом 7 эт. (арх. Казамонти) в Крестовоздвиженском пер., 43 квартиры и 3 пентхауса</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="26" customHeight="1">
       <c r="A29" s="10" t="inlineStr">
         <is>
           <t>Кло 17</t>
@@ -6407,9 +6711,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="P29" s="10" t="inlineStr"/>
-    </row>
-    <row r="30" ht="15" customHeight="1">
+      <c r="P29" s="10" t="inlineStr">
+        <is>
+          <t>Клубный дом (бюро PCA) в Староваганьковском пер., 26 квартир и 2 пентхауса, вид на Кремль</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="26" customHeight="1">
       <c r="A30" s="4" t="inlineStr">
         <is>
           <t>ТИТУЛ Империал</t>
@@ -6475,7 +6783,11 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="P30" s="4" t="inlineStr"/>
+      <c r="P30" s="4" t="inlineStr">
+        <is>
+          <t>Клубный дом на 12 квартир в Б. Николоворобинском пер., у Яузы, Таганка</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="26" customHeight="1">
       <c r="A31" s="10" t="inlineStr">
@@ -6543,9 +6855,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="P31" s="10" t="inlineStr"/>
-    </row>
-    <row r="32" ht="15" customHeight="1">
+      <c r="P31" s="10" t="inlineStr">
+        <is>
+          <t>Клубный дом 6 эт. на Софийской наб. (Кокоревское подворье), 42 квартиры и 5 пентхаусов</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="26" customHeight="1">
       <c r="A32" s="4" t="inlineStr">
         <is>
           <t>Дом Спорта</t>
@@ -6611,7 +6927,11 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="P32" s="4" t="inlineStr"/>
+      <c r="P32" s="4" t="inlineStr">
+        <is>
+          <t>Три корпуса на Дружинниковской ул. у Дома правительства, спорткластер 20 тыс. м² с катками</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="26" customHeight="1">
       <c r="A33" s="10" t="inlineStr">
@@ -6679,7 +6999,11 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="P33" s="10" t="inlineStr"/>
+      <c r="P33" s="10" t="inlineStr">
+        <is>
+          <t>7 особняков 3–5 эт. в неорусском стиле в 160 м от Красной пл., 3 памятника XIX в., двор-сад</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="26" customHeight="1">
       <c r="A34" s="4" t="inlineStr">
@@ -6747,9 +7071,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="P34" s="4" t="inlineStr"/>
-    </row>
-    <row r="35" ht="15" customHeight="1">
+      <c r="P34" s="4" t="inlineStr">
+        <is>
+          <t>Клубный дом 4–5 эт. из 3 корпусов на Берсеневской наб., 21 квартира, у Стрелки</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="26" customHeight="1">
       <c r="A35" s="10" t="inlineStr">
         <is>
           <t>ЖК «Николь»</t>
@@ -6815,9 +7143,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="P35" s="10" t="inlineStr"/>
-    </row>
-    <row r="36" ht="15" customHeight="1">
+      <c r="P35" s="10" t="inlineStr">
+        <is>
+          <t>3 здания с реконструкцией исторических домов на Никольской ул. (Heatherwick), у Красной пл.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="26" customHeight="1">
       <c r="A36" s="4" t="inlineStr">
         <is>
           <t>MONO Kami</t>
@@ -6883,9 +7215,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="P36" s="4" t="inlineStr"/>
-    </row>
-    <row r="37" ht="15" customHeight="1">
+      <c r="P36" s="4" t="inlineStr">
+        <is>
+          <t>Комплекс из 4 клубных домов 9–14 эт. в Пыжевском пер., 74 квартиры, 5 мин до Третьяковки</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="26" customHeight="1">
       <c r="A37" s="10" t="inlineStr">
         <is>
           <t>ЖК «Никитский-6»</t>
@@ -6951,7 +7287,11 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="P37" s="10" t="inlineStr"/>
+      <c r="P37" s="10" t="inlineStr">
+        <is>
+          <t>Клубный дом 8 эт. на Никитском бул., 57 квартир и 4 пентхауса с каминами и террасами</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="26" customHeight="1">
       <c r="A38" s="4" t="inlineStr">
@@ -7019,9 +7359,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="P38" s="4" t="inlineStr"/>
-    </row>
-    <row r="39" ht="15" customHeight="1">
+      <c r="P38" s="4" t="inlineStr">
+        <is>
+          <t>Квартал из 3 домов 10 эт. и неоклассического корпуса на Фрунзенской наб., 137 квартир, парк</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="26" customHeight="1">
       <c r="A39" s="10" t="inlineStr">
         <is>
           <t>Kuznetsky Most 12 by Lalique (Кузнецкий Мост 12)</t>
@@ -7034,7 +7378,7 @@
       </c>
       <c r="C39" s="11" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>4 кв. 2026</t>
         </is>
       </c>
       <c r="D39" s="10" t="inlineStr">
@@ -7082,10 +7426,18 @@
           <t>бетон</t>
         </is>
       </c>
-      <c r="O39" s="11" t="inlineStr"/>
-      <c r="P39" s="10" t="inlineStr"/>
-    </row>
-    <row r="40" ht="15" customHeight="1">
+      <c r="O39" s="15" t="inlineStr">
+        <is>
+          <t>ссылка</t>
+        </is>
+      </c>
+      <c r="P39" s="10" t="inlineStr">
+        <is>
+          <t>Реконструкция здания XIX в. на Кузнецком Мосту, 3–6 эт., 59 квартир, потолки до 5,8 м, wellness</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="26" customHeight="1">
       <c r="A40" s="4" t="inlineStr">
         <is>
           <t>Саввинская 27</t>
@@ -7151,9 +7503,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="P40" s="4" t="inlineStr"/>
-    </row>
-    <row r="41" ht="15" customHeight="1">
+      <c r="P40" s="4" t="inlineStr">
+        <is>
+          <t>Клубный дом 6 эт. (ODA, APEX) на 1-й линии реки, 61 резиденция, 10 пентхаусов, SPA с бассейном</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="26" customHeight="1">
       <c r="A41" s="10" t="inlineStr">
         <is>
           <t>ДОМ XXII</t>
@@ -7166,7 +7522,7 @@
       </c>
       <c r="C41" s="11" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>4 кв. 2026</t>
         </is>
       </c>
       <c r="D41" s="10" t="inlineStr">
@@ -7219,9 +7575,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="P41" s="10" t="inlineStr"/>
-    </row>
-    <row r="42" ht="15" customHeight="1">
+      <c r="P41" s="10" t="inlineStr">
+        <is>
+          <t>Клубный дом из 2 корпусов 9–12 эт. у Новодевичьего, 109 квартир, потолки 3,5–4,5 м</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="26" customHeight="1">
       <c r="A42" s="4" t="inlineStr">
         <is>
           <t>Stoleshnikov 7 (Столешников 7)</t>
@@ -7287,9 +7647,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="P42" s="4" t="inlineStr"/>
-    </row>
-    <row r="43" ht="15" customHeight="1">
+      <c r="P42" s="4" t="inlineStr">
+        <is>
+          <t>Реконструкция доходного дома 1903 г. (Эрихсон), 5 эт., 12 квартир, камины и террасы</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="26" customHeight="1">
       <c r="A43" s="10" t="inlineStr">
         <is>
           <t>ЖК «Узоры»</t>
@@ -7355,9 +7719,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="P43" s="10" t="inlineStr"/>
-    </row>
-    <row r="44" ht="15" customHeight="1">
+      <c r="P43" s="10" t="inlineStr">
+        <is>
+          <t>Клубный дом из 2 секций 9–10 эт. на общем стилобате во 2-м Вражском пер., 72 квартиры</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="26" customHeight="1">
       <c r="A44" s="4" t="inlineStr">
         <is>
           <t>Annabels</t>
@@ -7423,7 +7791,11 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="P44" s="4" t="inlineStr"/>
+      <c r="P44" s="4" t="inlineStr">
+        <is>
+          <t>Клубный дом 7 эт. в Курсовом пер. на Золотой миле, 9 резиденций, пентхаус с террасами</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="26" customHeight="1">
       <c r="A45" s="10" t="inlineStr">
@@ -7491,7 +7863,11 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="P45" s="10" t="inlineStr"/>
+      <c r="P45" s="10" t="inlineStr">
+        <is>
+          <t>Реконструкция особняка Шехтеля в Трёхпрудном пер., 2–6 эт., 26 квартир, у Патриарших</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="26" customHeight="1">
       <c r="A46" s="4" t="inlineStr">
@@ -7559,7 +7935,11 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="P46" s="4" t="inlineStr"/>
+      <c r="P46" s="4" t="inlineStr">
+        <is>
+          <t>Клубный дом 3–6 эт. в Старомонетном пер., 27 резиденций, интерьеры Armani/Casa, у Полянки</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="26" customHeight="1">
       <c r="A47" s="10" t="inlineStr">
@@ -7627,7 +8007,11 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="P47" s="10" t="inlineStr"/>
+      <c r="P47" s="10" t="inlineStr">
+        <is>
+          <t>Клубный дом из 2 корпусов 11 эт. (GAFA) у Новодевичьего, 64 квартиры, бассейн 25 м</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="26" customHeight="1">
       <c r="A48" s="4" t="inlineStr">
@@ -7695,9 +8079,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="P48" s="4" t="inlineStr"/>
-    </row>
-    <row r="49" ht="15" customHeight="1">
+      <c r="P48" s="4" t="inlineStr">
+        <is>
+          <t>Клубный дом в 3-м Обыденском пер., 26 квартир, пентхаусы и виллы, в 150 м от ХХС</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="26" customHeight="1">
       <c r="A49" s="10" t="inlineStr">
         <is>
           <t>Лё Дом</t>
@@ -7763,9 +8151,13 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="P49" s="10" t="inlineStr"/>
-    </row>
-    <row r="50" ht="15" customHeight="1">
+      <c r="P49" s="10" t="inlineStr">
+        <is>
+          <t>Клубный дом 3–5 эт. в Соймоновском пр., более 70 квартир, вид на Храм Христа Спасителя</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="26" customHeight="1">
       <c r="A50" s="4" t="inlineStr">
         <is>
           <t>ЖК «БРЮСОВ»</t>
@@ -7831,7 +8223,11 @@
           <t>ссылка</t>
         </is>
       </c>
-      <c r="P50" s="4" t="inlineStr"/>
+      <c r="P50" s="4" t="inlineStr">
+        <is>
+          <t>Клубный дом 8 эт. в Брюсовом пер. (1508 London), 20 резиденций и пентхаус, 5 мин до Кремля</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A3:P50"/>
@@ -7886,17 +8282,18 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId46"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.35" bottom="0.35" header="0.2" footer="0.2"/>

</xml_diff>

<commit_message>
Planning sheet: filled gaps and descriptions; all ЖК cards collected
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Bv8NELxW2W7udnb3XUFGS2
</commit_message>
<xml_diff>
--- a/docs/premium-cao/premium-zhk-cao.xlsx
+++ b/docs/premium-cao/premium-zhk-cao.xlsx
@@ -213,16 +213,16 @@
     <xf numFmtId="0" fontId="5" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -8098,7 +8098,7 @@
       </c>
       <c r="C49" s="11" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>3 кв. 2026</t>
         </is>
       </c>
       <c r="D49" s="10" t="inlineStr">
@@ -8435,48 +8435,56 @@
     <row r="4" ht="26" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Клубный дом «Малая Никитская, 27»</t>
+          <t>Лёвшинский, 19</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Малая Никитская улица, 27 (два двухэтажных особняка 1861 г., бывший «Клуб 27»)</t>
+          <t>Большой Лёвшинский пер., 19</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>Пресненский</t>
+          <t>Хамовники</t>
         </is>
       </c>
       <c r="D4" s="19" t="inlineStr">
         <is>
-          <t>Садовое кольцо</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>не раскрыт (по данным форума pronovostroy.ru — Mono/ПИК; официально не подтверждено)</t>
+          <t>Хамовники</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>ТСИ Девелопмент</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>проект на согласовании (высотность 33 м); продажи не открыты</t>
+          <t>продажи открыты, котлован/фундамент (novostroy-m.ru, 2026) — вышел из стадии планирования</t>
         </is>
       </c>
       <c r="G4" s="5" t="n"/>
       <c r="H4" s="5" t="n"/>
-      <c r="I4" s="5" t="n"/>
-      <c r="J4" s="5" t="n"/>
-      <c r="K4" s="5" t="n"/>
-      <c r="L4" s="5" t="n"/>
+      <c r="I4" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="J4" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L4" s="5" t="inlineStr">
+        <is>
+          <t>2 кв. 2028</t>
+        </is>
+      </c>
       <c r="M4" s="8" t="n">
-        <v>3000000</v>
-      </c>
-      <c r="N4" s="5" t="inlineStr">
-        <is>
-          <t>2024-03-31</t>
-        </is>
-      </c>
+        <v>2800000</v>
+      </c>
+      <c r="N4" s="5" t="n"/>
       <c r="O4" s="9" t="inlineStr">
         <is>
           <t>ссылка</t>
@@ -8484,67 +8492,53 @@
       </c>
       <c r="P4" s="4" t="inlineStr">
         <is>
-          <t>Клубный дом высотой 33 м по проекту бюро WALL на месте двух двухэтажных особняков (бывший отель Club 27). Ориентировочная цена «от ~3 млн руб./м²» — оценка источника, не подтверждена застройщиком. В базе mskdeluxe.ru фигурирует как «Малая Никитская, 29-31».; Архитектура — бюро WALL (ярусные объемы, черно-белые фасады). Существующие здания ~4 000 м² сносятся. Цена ~3 млн руб./м² — предварительное рыночное ожидание (sosedi.life, https://sosedi.life/news/zhk-malaya-nikitskaya-27/), не оферта. Restate.ru (2025–2026) отмечал неопределенность со стартом: возможна продажа площадки вместо запуска.</t>
+          <t>Клубный дом 8 эт. на 16 резиденций 70–239 м², воссоздание фасада доходного дома Духовских 1904 г., паркинг 18 м/м, HADAA</t>
         </is>
       </c>
     </row>
     <row r="5" ht="26" customHeight="1">
       <c r="A5" s="10" t="inlineStr">
         <is>
-          <t>Палашёвский 11 (Большой Палашёвский, 11–13/15)</t>
+          <t>Клубный дом «Малая Никитская, 27»</t>
         </is>
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>Большой Палашёвский пер., 11–13</t>
+          <t>Малая Никитская улица, 27 (два двухэтажных особняка 1861 г., бывший «Клуб 27»)</t>
         </is>
       </c>
       <c r="C5" s="11" t="inlineStr">
         <is>
-          <t>Тверской</t>
-        </is>
-      </c>
-      <c r="D5" s="19" t="inlineStr">
+          <t>Пресненский</t>
+        </is>
+      </c>
+      <c r="D5" s="20" t="inlineStr">
         <is>
           <t>Садовое кольцо</t>
         </is>
       </c>
-      <c r="E5" s="10" t="inlineStr">
-        <is>
-          <t>Sminex (СЗ «Смайнэкс Палашёвский 11»)</t>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>не раскрыт</t>
         </is>
       </c>
       <c r="F5" s="10" t="inlineStr">
         <is>
-          <t>старт продаж без стройки (закрытый старт 22.04.2026)</t>
-        </is>
-      </c>
-      <c r="G5" s="13" t="n">
-        <v>15600</v>
-      </c>
+          <t>проектирование (kvartiravmoskve.ru, 02.03.2026); продажи не открыты, старт не анонсирован</t>
+        </is>
+      </c>
+      <c r="G5" s="11" t="n"/>
       <c r="H5" s="11" t="n"/>
-      <c r="I5" s="13" t="n">
-        <v>9</v>
-      </c>
-      <c r="J5" s="13" t="n">
-        <v>43</v>
-      </c>
-      <c r="K5" s="11" t="inlineStr">
-        <is>
-          <t>2026-04-22</t>
-        </is>
-      </c>
-      <c r="L5" s="11" t="inlineStr">
-        <is>
-          <t>1 кв. 2030</t>
-        </is>
-      </c>
+      <c r="I5" s="11" t="n"/>
+      <c r="J5" s="11" t="n"/>
+      <c r="K5" s="11" t="n"/>
+      <c r="L5" s="11" t="n"/>
       <c r="M5" s="14" t="n">
-        <v>3500000</v>
+        <v>3000000</v>
       </c>
       <c r="N5" s="11" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2024-03-31</t>
         </is>
       </c>
       <c r="O5" s="15" t="inlineStr">
@@ -8554,71 +8548,71 @@
       </c>
       <c r="P5" s="10" t="inlineStr">
         <is>
-          <t>Три корпуса 8–9 этажей с контрастными фасадами у Патриарших. Старт продаж 22.04.2026, лоты от 222,4 млн руб. (nngm.ru), от ~3,5 млн руб./м². Сдача 1 кв. 2030 (novostroev.ru, обзор делюкс-стартов 2026).</t>
+          <t>Клубный дом высотой 33 м (бюро WALL) на месте двух особняков 1861 г. у Патриарших; ярусные объёмы, чёрно-белые фасады</t>
         </is>
       </c>
     </row>
     <row r="6" ht="26" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>EDEN Private Residence</t>
+          <t>Палашёвский 11 (Большой Палашёвский, 11–13/15)</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Нижний Кисловский пер., 7, стр. 1–2</t>
+          <t>Большой Палашёвский пер., 11–13</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Пресненский</t>
-        </is>
-      </c>
-      <c r="D6" s="19" t="inlineStr">
+          <t>Тверской</t>
+        </is>
+      </c>
+      <c r="D6" s="20" t="inlineStr">
         <is>
           <t>Садовое кольцо</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>Sense Development (с ГК ПИК и Айсель Трудель)</t>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Sminex</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>старт продаж без стройки (закрытый формат, апрель 2026)</t>
+          <t>продажи открыты (апрель 2026), стадия котлована (проверено 03.09.2026) — вышел из стадии планирования</t>
         </is>
       </c>
       <c r="G6" s="7" t="n">
-        <v>17100</v>
-      </c>
-      <c r="H6" s="7" t="n">
-        <v>6200</v>
-      </c>
-      <c r="I6" s="7" t="n">
-        <v>9</v>
+        <v>15600</v>
+      </c>
+      <c r="H6" s="5" t="n"/>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>8–9</t>
+        </is>
       </c>
       <c r="J6" s="7" t="n">
-        <v>22</v>
+        <v>52</v>
       </c>
       <c r="K6" s="5" t="inlineStr">
         <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="L6" s="5" t="inlineStr">
+        <is>
+          <t>1 кв. 2030</t>
+        </is>
+      </c>
+      <c r="M6" s="8" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="N6" s="5" t="inlineStr">
+        <is>
           <t>2026-04</t>
         </is>
       </c>
-      <c r="L6" s="5" t="inlineStr">
-        <is>
-          <t>3 кв. 2029</t>
-        </is>
-      </c>
-      <c r="M6" s="8" t="n">
-        <v>5000000</v>
-      </c>
-      <c r="N6" s="5" t="inlineStr">
-        <is>
-          <t>2026-04</t>
-        </is>
-      </c>
       <c r="O6" s="9" t="inlineStr">
         <is>
           <t>ссылка</t>
@@ -8626,57 +8620,73 @@
       </c>
       <c r="P6" s="4" t="inlineStr">
         <is>
-          <t>Ultra luxury, 6–9 этажей, 22 резиденции, участок 0,3 га, архитектура Gregory Tuck Architects. Оценка цены ~5 млн руб./м² (около 1,1 млрд руб. за ~250 м²). Общая площадь в разных источниках 13–17,1 тыс. м².</t>
+          <t>Клубный дом 8–9 эт.: 45 квартир и 7 пентхаусов у Патриарших, три контрастных фасада, двор-сад с прудом, паркинг 88 м/м</t>
         </is>
       </c>
     </row>
     <row r="7" ht="26" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
-          <t>Большая Ордынка, 25</t>
+          <t>EDEN Private Residence</t>
         </is>
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>ул. Большая Ордынка, 25, стр. 1</t>
+          <t>Нижний Кисловский пер., 7, стр. 1–2</t>
         </is>
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>Замоскворечье</t>
-        </is>
-      </c>
-      <c r="D7" s="19" t="inlineStr">
+          <t>Пресненский</t>
+        </is>
+      </c>
+      <c r="D7" s="20" t="inlineStr">
         <is>
           <t>Садовое кольцо</t>
         </is>
       </c>
-      <c r="E7" s="10" t="inlineStr">
-        <is>
-          <t>Aurix Development (Группа «Эталон»)</t>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>Sense Development</t>
         </is>
       </c>
       <c r="F7" s="10" t="inlineStr">
         <is>
-          <t>концепция одобрена ГЗК, подготовка к строительству, старт продаж 2026</t>
+          <t>закрытые продажи (апрель 2026), стадия котлована; публичные продажи не открыты (novostroev.ru, 03.09.2026)</t>
         </is>
       </c>
       <c r="G7" s="13" t="n">
-        <v>17000</v>
-      </c>
-      <c r="H7" s="11" t="n"/>
-      <c r="I7" s="13" t="n">
-        <v>8</v>
-      </c>
-      <c r="J7" s="11" t="n"/>
+        <v>17100</v>
+      </c>
+      <c r="H7" s="13" t="n">
+        <v>6200</v>
+      </c>
+      <c r="I7" s="11" t="inlineStr">
+        <is>
+          <t>6–9</t>
+        </is>
+      </c>
+      <c r="J7" s="13" t="n">
+        <v>22</v>
+      </c>
       <c r="K7" s="11" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="L7" s="11" t="n"/>
-      <c r="M7" s="20" t="n"/>
-      <c r="N7" s="11" t="n"/>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="L7" s="11" t="inlineStr">
+        <is>
+          <t>3 кв. 2029</t>
+        </is>
+      </c>
+      <c r="M7" s="14" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="N7" s="11" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
       <c r="O7" s="15" t="inlineStr">
         <is>
           <t>ссылка</t>
@@ -8684,55 +8694,63 @@
       </c>
       <c r="P7" s="10" t="inlineStr">
         <is>
-          <t>7 этажей + мансардный уровень, &gt;17 тыс. м², на месте конструктивистской АТС 1927 г. Де-люкс. Одобрение ГЗК упоминает whitewill.ru.</t>
+          <t>Ultra luxury клубный дом 6–9 эт. на 22 резиденции 107–411 м² у Арбата, участок 0,3 га, Gregory Tuck Architects</t>
         </is>
       </c>
     </row>
     <row r="8" ht="26" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Большая Пироговская, 51 (общежития Института красной профессуры)</t>
+          <t>Большая Ордынка, 25</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>ул. Большая Пироговская, 51</t>
+          <t>ул. Большая Ордынка, 25, стр. 1</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Хамовники</t>
-        </is>
-      </c>
-      <c r="D8" s="21" t="inlineStr">
-        <is>
-          <t>Хамовники</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>Vesper (fee-девелопер) / собственник Capital Group</t>
+          <t>Замоскворечье</t>
+        </is>
+      </c>
+      <c r="D8" s="20" t="inlineStr">
+        <is>
+          <t>Садовое кольцо</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Aurix Development</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>анонсирован (fee-development), концепция</t>
+          <t>концепция одобрена ГЗК, подготовка к строительству; старт продаж заявлен на 2026, цены и планировки не опубликованы</t>
         </is>
       </c>
       <c r="G8" s="7" t="n">
-        <v>46700</v>
+        <v>17000</v>
       </c>
       <c r="H8" s="5" t="n"/>
-      <c r="I8" s="5" t="n"/>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>7 + мансарда</t>
+        </is>
+      </c>
       <c r="J8" s="5" t="n"/>
-      <c r="K8" s="5" t="n"/>
-      <c r="L8" s="5" t="n"/>
-      <c r="M8" s="22" t="n"/>
-      <c r="N8" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>4 кв. 2031</t>
+        </is>
+      </c>
+      <c r="M8" s="21" t="n"/>
+      <c r="N8" s="5" t="n"/>
       <c r="O8" s="9" t="inlineStr">
         <is>
           <t>ссылка</t>
@@ -8740,59 +8758,59 @@
       </c>
       <c r="P8" s="4" t="inlineStr">
         <is>
-          <t>Участок 1,5 га, ансамбль восьми 6-этажных корпусов 1929–32 гг. (арх. Осипов, Рухлядев; статус памятника утрачен в 2000-х). Планируемая площадь выросла с 39 до 46,7 тыс. м². Vesper — концепция, продукт и управление реализацией. В базе mskdeluxe.ru — «Б.Пироговская, 51».</t>
+          <t>Клубный дом 7 эт. + мансарда, &gt;17 тыс. м², на месте первой АТС Москвы 1927 г. в Замоскворечье; делюкс</t>
         </is>
       </c>
     </row>
     <row r="9" ht="26" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Большой Козихинский, 22</t>
+          <t>Большая Пироговская, 51 (общежития Института красной профессуры)</t>
         </is>
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>Большой Козихинский пер., 22</t>
+          <t>ул. Большая Пироговская, 51</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>Пресненский</t>
+          <t>Хамовники</t>
         </is>
       </c>
       <c r="D9" s="19" t="inlineStr">
         <is>
-          <t>Садовое кольцо</t>
+          <t>Хамовники</t>
         </is>
       </c>
       <c r="E9" s="11" t="inlineStr">
         <is>
-          <t>КОЛДИ / Доминанта</t>
+          <t>Vesper</t>
         </is>
       </c>
       <c r="F9" s="10" t="inlineStr">
         <is>
-          <t>проект, продажи не начаты</t>
+          <t>анонсирован (fee-development, июнь 2026), концепция; ГПЗУ получен в начале 2025; реализация не подтверждена</t>
         </is>
       </c>
       <c r="G9" s="13" t="n">
-        <v>9377</v>
+        <v>46700</v>
       </c>
       <c r="H9" s="11" t="n"/>
-      <c r="I9" s="13" t="n">
-        <v>9</v>
-      </c>
-      <c r="J9" s="13" t="n">
-        <v>98</v>
-      </c>
-      <c r="K9" s="11" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
+      <c r="I9" s="10" t="inlineStr">
+        <is>
+          <t>12–13 (концепция Buro 2+2, 8 корпусов)</t>
+        </is>
+      </c>
+      <c r="J9" s="11" t="n"/>
+      <c r="K9" s="11" t="n"/>
       <c r="L9" s="11" t="n"/>
-      <c r="M9" s="20" t="n"/>
-      <c r="N9" s="11" t="n"/>
+      <c r="M9" s="22" t="n"/>
+      <c r="N9" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
       <c r="O9" s="15" t="inlineStr">
         <is>
           <t>ссылка</t>
@@ -8800,52 +8818,58 @@
       </c>
       <c r="P9" s="10" t="inlineStr">
         <is>
-          <t>Патриаршие пруды. Статус «Проект / продажи не начаты» подтверждён novostroev.ru на 01.09.2026; включён в список перспективных стартов делюкс-класса 2026 (novostroev.ru). Официальный сайт kozihinsky22.ru недоступен (403).</t>
+          <t>Застройка 1,5 га бывших общежитий 1929–32 гг.: концепция 8 корпусов 12–13 эт. на стилобате в светлом камне, 46,7 тыс. м²</t>
         </is>
       </c>
     </row>
     <row r="10" ht="26" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Воздвиженка 7/6</t>
+          <t>Большой Козихинский, 22</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>ул. Воздвиженка, 7/6</t>
+          <t>Большой Козихинский пер., 22</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Арбат</t>
-        </is>
-      </c>
-      <c r="D10" s="19" t="inlineStr">
+          <t>Пресненский</t>
+        </is>
+      </c>
+      <c r="D10" s="20" t="inlineStr">
         <is>
           <t>Садовое кольцо</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>АПРИ (по данным vozdvizhenka7.ru)</t>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>КОЛДИ / Доминанта</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>анонсирован, старт продаж ожидается</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="n"/>
+          <t>проект, продажи не начаты (novostroev.ru, проверено 03.09.2026)</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="n">
+        <v>9377</v>
+      </c>
       <c r="H10" s="5" t="n"/>
-      <c r="I10" s="5" t="n"/>
-      <c r="J10" s="5" t="n"/>
+      <c r="I10" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="J10" s="7" t="n">
+        <v>98</v>
+      </c>
       <c r="K10" s="5" t="inlineStr">
         <is>
-          <t>2026–2027</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="L10" s="5" t="n"/>
-      <c r="M10" s="22" t="n"/>
+      <c r="M10" s="21" t="n"/>
       <c r="N10" s="5" t="n"/>
       <c r="O10" s="9" t="inlineStr">
         <is>
@@ -8854,55 +8878,53 @@
       </c>
       <c r="P10" s="4" t="inlineStr">
         <is>
-          <t>Указан в базе делюкс-стартов 2026–2027 mskdeluxe.ru. Агрегаторы описывают как бутик-дом на 10–15 квартир; ранее указывалась сдача 1 кв. 2025 — данные противоречивы, официальный сайт vozdvizhenka7.ru недоступен (503). Требует верификации.</t>
+          <t>Клубный дом 9 эт. на 98 квартир (9,4 тыс. м²) у Патриарших прудов, 5 мин. от м. Пушкинская; делюкс</t>
         </is>
       </c>
     </row>
     <row r="11" ht="26" customHeight="1">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>Квартал на Савинской набережной («Московский шёлк»)</t>
+          <t>Воздвиженка 7/6</t>
         </is>
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>Савинская наб. (территория БЦ «Московский шёлк»)</t>
+          <t>ул. Воздвиженка, 7/6</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>Хамовники</t>
-        </is>
-      </c>
-      <c r="D11" s="21" t="inlineStr">
-        <is>
-          <t>Хамовники</t>
+          <t>Арбат</t>
+        </is>
+      </c>
+      <c r="D11" s="20" t="inlineStr">
+        <is>
+          <t>Садовое кольцо</t>
         </is>
       </c>
       <c r="E11" s="11" t="inlineStr">
         <is>
-          <t>Sminex</t>
-        </is>
-      </c>
-      <c r="F11" s="11" t="inlineStr">
-        <is>
-          <t>проектирование</t>
-        </is>
-      </c>
-      <c r="G11" s="13" t="n">
-        <v>125000</v>
-      </c>
+          <t>АПРИ</t>
+        </is>
+      </c>
+      <c r="F11" s="10" t="inlineStr">
+        <is>
+          <t>анонсирован; в списке делюкс-стартов 2026–2027 mskdeluxe.ru; параметры не раскрыты, сайт проекта недоступен (08.09.2026)</t>
+        </is>
+      </c>
+      <c r="G11" s="11" t="n"/>
       <c r="H11" s="11" t="n"/>
       <c r="I11" s="11" t="n"/>
       <c r="J11" s="11" t="n"/>
-      <c r="K11" s="11" t="n"/>
+      <c r="K11" s="11" t="inlineStr">
+        <is>
+          <t>2026–2027</t>
+        </is>
+      </c>
       <c r="L11" s="11" t="n"/>
-      <c r="M11" s="20" t="n"/>
-      <c r="N11" s="11" t="inlineStr">
-        <is>
-          <t>2024-03-12</t>
-        </is>
-      </c>
+      <c r="M11" s="22" t="n"/>
+      <c r="N11" s="11" t="n"/>
       <c r="O11" s="15" t="inlineStr">
         <is>
           <t>ссылка</t>
@@ -8910,29 +8932,29 @@
       </c>
       <c r="P11" s="10" t="inlineStr">
         <is>
-          <t>ЖК ~125 тыс. м² на территории делового квартала «Московский шёлк». По данным Sminex на декабрь 2025 г. находится в стадии проектирования (вместе с Лужнецкой).</t>
+          <t>Бутик-дом делюкс ориентировочно на 10–15 квартир на Воздвиженке у Александровского сада; параметры не подтверждены</t>
         </is>
       </c>
     </row>
     <row r="12" ht="26" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Клубные дома на Берниковской набережной, 12 (Sminex)</t>
+          <t>Квартал на Савинской набережной («Московский шёлк»)</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Берниковская набережная, 12, стр. 1 (здание бывшей школы №1685, 1936 г., арх. А. Машинский)</t>
+          <t>Савинская наб. (территория БЦ «Московский шёлк»)</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Таганский</t>
+          <t>Хамовники</t>
         </is>
       </c>
       <c r="D12" s="19" t="inlineStr">
         <is>
-          <t>Садовое кольцо</t>
+          <t>Хамовники</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -8942,29 +8964,25 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>проектирование; предварительная архитектурная концепция (бюро 80/88) опубликована в марте 2026</t>
+          <t>проектирование (подтверждено Sminex в декабре 2025); начало реализации планировалось на 2026, старт продаж не объявлен</t>
         </is>
       </c>
       <c r="G12" s="7" t="n">
-        <v>23336</v>
-      </c>
-      <c r="H12" s="7" t="n">
-        <v>13000</v>
-      </c>
-      <c r="I12" s="4" t="inlineStr">
-        <is>
-          <t>9–13 (два корпуса; 9-этажный многосекционный вдоль набережной, 13-этажный в глубине со стороны Берникова переулка)</t>
-        </is>
-      </c>
-      <c r="J12" s="7" t="n">
-        <v>166</v>
-      </c>
-      <c r="K12" s="5" t="n"/>
+        <v>125000</v>
+      </c>
+      <c r="H12" s="5" t="n"/>
+      <c r="I12" s="5" t="n"/>
+      <c r="J12" s="5" t="n"/>
+      <c r="K12" s="4" t="inlineStr">
+        <is>
+          <t>2026 (начало реализации, план 2024 г.)</t>
+        </is>
+      </c>
       <c r="L12" s="5" t="n"/>
-      <c r="M12" s="22" t="n"/>
+      <c r="M12" s="21" t="n"/>
       <c r="N12" s="5" t="inlineStr">
         <is>
-          <t>2025-03-18</t>
+          <t>2024-03-12</t>
         </is>
       </c>
       <c r="O12" s="9" t="inlineStr">
@@ -8974,63 +8992,61 @@
       </c>
       <c r="P12" s="4" t="inlineStr">
         <is>
-          <t>Участок 0,6 га на первой линии Яузы, два корпуса 9–13 этажей, ~23 тыс. м², 166 квартир, «органический неоклассицизм». Делюкс. Застройщик не назван.; Sminex приобрел площадку в конце 2024 г.; по пресс-релизу — два элитных клубных дома 7–13 этажей, общая площадь 21,4 тыс. м², из них ~13 тыс. м² жилья. По концепции 80/88 (Москвич Mag, https://moskvichmag.ru/gorod/poyavilsya-proekt-mnogosektsionnogo-zhk-na-bernikovskoj-naberezhnoj-na-meste-zakrytoj-shkoly) — 23 336 м², 166 квартир; участок 0,6 га; отмечается, что окончательная реализация именно этого проекта не гарантирована. Агрегатор kvartiravmoskve.ru: стадия «проектирование», монолит-кирпич, подземный паркинг.</t>
+          <t>ЖК ~125 тыс. м² на 4,5 га бывшей фабрики «Московский шёлк» на Савинской наб.: новые корпуса и реставрация</t>
         </is>
       </c>
     </row>
     <row r="13" ht="26" customHeight="1">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>Клубный дом «Большая Никитская, 16» (R4S)</t>
+          <t>Клубные дома на Берниковской набережной, 12 (Sminex)</t>
         </is>
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>Большая Никитская улица, 16 (реконструкция доходного дома, объект культурного наследия)</t>
+          <t>Берниковская набережная, 12, стр. 1 (здание бывшей школы №1685, 1936 г., арх. А. Машинский)</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>Пресненский</t>
-        </is>
-      </c>
-      <c r="D13" s="19" t="inlineStr">
+          <t>Таганский</t>
+        </is>
+      </c>
+      <c r="D13" s="20" t="inlineStr">
         <is>
           <t>Садовое кольцо</t>
         </is>
       </c>
-      <c r="E13" s="10" t="inlineStr">
-        <is>
-          <t>R4S Group (генподрядчик — Спецжилремонт)</t>
+      <c r="E13" s="11" t="inlineStr">
+        <is>
+          <t>Sminex</t>
         </is>
       </c>
       <c r="F13" s="10" t="inlineStr">
         <is>
-          <t>реконструкция; старт продаж I кв. 2026; ввод III кв. 2026</t>
-        </is>
-      </c>
-      <c r="G13" s="11" t="n"/>
-      <c r="H13" s="11" t="n"/>
-      <c r="I13" s="13" t="n">
-        <v>4</v>
+          <t>проектирование; площадка подтверждена Sminex 17.03.2026, сроки и старт продаж не объявлены</t>
+        </is>
+      </c>
+      <c r="G13" s="13" t="n">
+        <v>21400</v>
+      </c>
+      <c r="H13" s="13" t="n">
+        <v>13000</v>
+      </c>
+      <c r="I13" s="11" t="inlineStr">
+        <is>
+          <t>7–13 (два корпуса)</t>
+        </is>
       </c>
       <c r="J13" s="13" t="n">
-        <v>4</v>
-      </c>
-      <c r="K13" s="10" t="inlineStr">
-        <is>
-          <t>2026 Q1 (старт продаж)</t>
-        </is>
-      </c>
-      <c r="L13" s="11" t="inlineStr">
-        <is>
-          <t>2026 Q3</t>
-        </is>
-      </c>
-      <c r="M13" s="20" t="n"/>
+        <v>166</v>
+      </c>
+      <c r="K13" s="11" t="n"/>
+      <c r="L13" s="11" t="n"/>
+      <c r="M13" s="22" t="n"/>
       <c r="N13" s="11" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2025-03-18</t>
         </is>
       </c>
       <c r="O13" s="15" t="inlineStr">
@@ -9040,59 +9056,63 @@
       </c>
       <c r="P13" s="10" t="inlineStr">
         <is>
-          <t>Единственная публичная новинка на Большой Никитской в 2025–2026: 4 квартиры 139,4 / 141,4 / 151 / 234 м². Другие участки на Большой Никитской в открытых анонсах не найдены.</t>
+          <t>Два клубных дома 7–13 эт., 166 квартир на 0,6 га на первой линии Яузы; двор-парк, пентхаусы с каминами; делюкс</t>
         </is>
       </c>
     </row>
     <row r="14" ht="26" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Клубный дом «Земледельческий, 15»</t>
+          <t>Клубный дом «Большая Никитская, 16» (R4S)</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Земледельческий переулок, 15 (на месте административного здания 1975 г., 5 этажей, 5 744 м²)</t>
+          <t>Большая Никитская улица, 16 (реконструкция доходного дома, объект культурного наследия)</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Хамовники</t>
-        </is>
-      </c>
-      <c r="D14" s="21" t="inlineStr">
-        <is>
-          <t>Хамовники</t>
+          <t>Пресненский</t>
+        </is>
+      </c>
+      <c r="D14" s="20" t="inlineStr">
+        <is>
+          <t>Садовое кольцо</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>не раскрыт</t>
+          <t>R4S Group</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>проектирование (агрегаторы; в списке ожидаемых стартов делюкс-класса 2026 на mskdeluxe.ru)</t>
-        </is>
-      </c>
-      <c r="G14" s="7" t="n">
-        <v>8000</v>
-      </c>
+          <t>проект/реконструкция; продажи не начаты (novostroev.ru, 02.09.2026); заявленный ввод 3 кв. 2026 не подтверждён</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="n"/>
       <c r="H14" s="5" t="n"/>
-      <c r="I14" s="5" t="n"/>
+      <c r="I14" s="7" t="n">
+        <v>4</v>
+      </c>
       <c r="J14" s="7" t="n">
-        <v>77</v>
-      </c>
-      <c r="K14" s="5" t="inlineStr">
-        <is>
-          <t>2026–2027</t>
-        </is>
-      </c>
-      <c r="L14" s="5" t="n"/>
-      <c r="M14" s="22" t="n"/>
+        <v>4</v>
+      </c>
+      <c r="K14" s="4" t="inlineStr">
+        <is>
+          <t>2026 Q1 (старт продаж, не состоялся на 02.09.2026)</t>
+        </is>
+      </c>
+      <c r="L14" s="5" t="inlineStr">
+        <is>
+          <t>2026 Q3</t>
+        </is>
+      </c>
+      <c r="M14" s="21" t="n"/>
       <c r="N14" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="O14" s="9" t="inlineStr">
@@ -9102,51 +9122,61 @@
       </c>
       <c r="P14" s="4" t="inlineStr">
         <is>
-          <t>Участок 0,3 га (сейчас административное здание 1975 г., 5 эт., 5,7 тыс. м²), клубный дом ~8 тыс. м², 77 квартир, коммерция, подземный паркинг. Делюкс.; Участок 0,3 га; делюкс; 77 квартир + коммерческая часть; подземный паркинг; монолит-кирпич; 1 км до м. Смоленская. Сделок по продаже БЦ и решений Москомархитектуры в открытых источниках не найдено.</t>
+          <t>Реконструкция исторического особняка (ОКН) в клубный дом 4 эт. на 4 квартиры 139–234 м² у Кремля, потолки 3,1–3,7 м</t>
         </is>
       </c>
     </row>
     <row r="15" ht="26" customHeight="1">
       <c r="A15" s="10" t="inlineStr">
         <is>
-          <t>Клубный дом на Курсовом переулке, 15 (проект бюро Дмитрия Великовского)</t>
+          <t>Клубный дом «Земледельческий, 15»</t>
         </is>
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>Курсовой переулок, 15</t>
-        </is>
-      </c>
-      <c r="C15" s="10" t="inlineStr">
-        <is>
-          <t>Хамовники (Остоженка)</t>
-        </is>
-      </c>
-      <c r="D15" s="21" t="inlineStr">
+          <t>Земледельческий переулок, 15 (на месте административного здания 1975 г., 5 этажей, 5 744 м²)</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
         <is>
           <t>Хамовники</t>
         </is>
       </c>
-      <c r="E15" s="10" t="inlineStr">
-        <is>
-          <t>не раскрыт (проект бюро Дмитрия Великовского)</t>
+      <c r="D15" s="19" t="inlineStr">
+        <is>
+          <t>Хамовники</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="inlineStr">
+        <is>
+          <t>не раскрыт</t>
         </is>
       </c>
       <c r="F15" s="10" t="inlineStr">
         <is>
-          <t>проект / предстарт; в открытых источниках только страница агрегатора</t>
-        </is>
-      </c>
-      <c r="G15" s="11" t="n"/>
+          <t>проектирование (kvartiravmoskve.ru, 21.06.2026); по адресу действует БЦ; сделок и решений МКА не найдено</t>
+        </is>
+      </c>
+      <c r="G15" s="13" t="n">
+        <v>8000</v>
+      </c>
       <c r="H15" s="11" t="n"/>
-      <c r="I15" s="13" t="n">
-        <v>6</v>
-      </c>
-      <c r="J15" s="11" t="n"/>
-      <c r="K15" s="11" t="n"/>
+      <c r="I15" s="11" t="n"/>
+      <c r="J15" s="13" t="n">
+        <v>77</v>
+      </c>
+      <c r="K15" s="11" t="inlineStr">
+        <is>
+          <t>2026–2027</t>
+        </is>
+      </c>
       <c r="L15" s="11" t="n"/>
-      <c r="M15" s="20" t="n"/>
-      <c r="N15" s="11" t="n"/>
+      <c r="M15" s="22" t="n"/>
+      <c r="N15" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
       <c r="O15" s="15" t="inlineStr">
         <is>
           <t>ссылка</t>
@@ -9154,57 +9184,51 @@
       </c>
       <c r="P15" s="10" t="inlineStr">
         <is>
-          <t>«Золотая миля», 6 этажей, камерный клубный дом. Подробные параметры и застройщик в открытых источниках не раскрыты.; По описанию агрегатора: 6-этажный дом по проекту бюро Дмитрия Великовского, панорамное остекление, локация «Золотой мили» рядом с Зачатьевским монастырем. Сейчас по адресу — детский клуб-студия «Пречистенские ворота». Пресса (Коммерсант, РБК, Ведомости, Москвич Mag) и Москомархитектура публикаций по площадке не имеют; девелопер и параметры не подтверждены.</t>
+          <t>Клубный дом ~8 тыс. м² на 77 квартир на 0,3 га на месте БЦ 1975 г. у Плющихи; коммерция, подземный паркинг; делюкс</t>
         </is>
       </c>
     </row>
     <row r="16" ht="26" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Льва Толстого, 14–16 (три клубных дома Sminex)</t>
+          <t>Клубный дом на Курсовом переулке, 15 (проект бюро Дмитрия Великовского)</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>ул. Льва Толстого, 14</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
+          <t>Курсовой переулок, 15</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Хамовники (Остоженка)</t>
+        </is>
+      </c>
+      <c r="D16" s="19" t="inlineStr">
         <is>
           <t>Хамовники</t>
         </is>
       </c>
-      <c r="D16" s="21" t="inlineStr">
-        <is>
-          <t>Хамовники</t>
-        </is>
-      </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>Sminex</t>
+          <t>не раскрыт</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>участок приобретён (декабрь 2025), концепция в финальной стадии, старт продаж не объявлен</t>
-        </is>
-      </c>
-      <c r="G16" s="7" t="n">
-        <v>20300</v>
-      </c>
-      <c r="H16" s="7" t="n">
-        <v>12400</v>
-      </c>
-      <c r="I16" s="5" t="n"/>
+          <t>проект / предстарт; в открытых источниках только страница агрегатора (08.09.2026)</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="n"/>
+      <c r="H16" s="5" t="n"/>
+      <c r="I16" s="7" t="n">
+        <v>6</v>
+      </c>
       <c r="J16" s="5" t="n"/>
       <c r="K16" s="5" t="n"/>
       <c r="L16" s="5" t="n"/>
-      <c r="M16" s="22" t="n"/>
-      <c r="N16" s="5" t="inlineStr">
-        <is>
-          <t>2025-12-18</t>
-        </is>
-      </c>
+      <c r="M16" s="21" t="n"/>
+      <c r="N16" s="5" t="n"/>
       <c r="O16" s="9" t="inlineStr">
         <is>
           <t>ссылка</t>
@@ -9212,19 +9236,19 @@
       </c>
       <c r="P16" s="4" t="inlineStr">
         <is>
-          <t>Участок ~0,6 га у делового квартала «Красная Роза», куплен у структур А. Клячина. Три камерных клубных дома, надземная площадь 20,3 тыс. м², квартиры 12,4 тыс. м². Сохраняется фасад бывшего доходного дома Трындина-Жиро.</t>
+          <t>Камерный клубный дом 6 эт. на «Золотой миле» у Зачатьевского монастыря; классика с панорамными окнами, башня с куполом</t>
         </is>
       </c>
     </row>
     <row r="17" ht="26" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t>Лёвшинский, 19</t>
+          <t>Льва Толстого, 14–16 (три клубных дома Sminex)</t>
         </is>
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>Большой Лёвшинский пер., 19</t>
+          <t>ул. Льва Толстого, 14</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
@@ -9232,41 +9256,37 @@
           <t>Хамовники</t>
         </is>
       </c>
-      <c r="D17" s="21" t="inlineStr">
+      <c r="D17" s="19" t="inlineStr">
         <is>
           <t>Хамовники</t>
         </is>
       </c>
-      <c r="E17" s="10" t="inlineStr">
-        <is>
-          <t>ТСИ Девелопмент (ГК «Трансстройинвест»)</t>
+      <c r="E17" s="11" t="inlineStr">
+        <is>
+          <t>Sminex</t>
         </is>
       </c>
       <c r="F17" s="10" t="inlineStr">
         <is>
-          <t>старт бронирования, старт продаж</t>
-        </is>
-      </c>
-      <c r="G17" s="11" t="n"/>
-      <c r="H17" s="11" t="n"/>
-      <c r="I17" s="13" t="n">
-        <v>8</v>
-      </c>
-      <c r="J17" s="13" t="n">
-        <v>16</v>
-      </c>
-      <c r="K17" s="11" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="L17" s="11" t="inlineStr">
-        <is>
-          <t>2 кв. 2028</t>
-        </is>
-      </c>
-      <c r="M17" s="20" t="n"/>
-      <c r="N17" s="11" t="n"/>
+          <t>участок приобретён (декабрь 2025), проектирование; старт продаж не объявлен (08.09.2026)</t>
+        </is>
+      </c>
+      <c r="G17" s="13" t="n">
+        <v>20300</v>
+      </c>
+      <c r="H17" s="13" t="n">
+        <v>12400</v>
+      </c>
+      <c r="I17" s="11" t="n"/>
+      <c r="J17" s="11" t="n"/>
+      <c r="K17" s="11" t="n"/>
+      <c r="L17" s="11" t="n"/>
+      <c r="M17" s="22" t="n"/>
+      <c r="N17" s="11" t="inlineStr">
+        <is>
+          <t>2025-12-18</t>
+        </is>
+      </c>
       <c r="O17" s="15" t="inlineStr">
         <is>
           <t>ссылка</t>
@@ -9274,7 +9294,7 @@
       </c>
       <c r="P17" s="10" t="inlineStr">
         <is>
-          <t>Воссоздание фасада доходного дома Духовских (1904, арх. Мейснер), проект HADAA Architects. 16 резиденций 70–239 м², паркинг 18 м/м. Цена от 197,12 млн руб. за лот. Стадия стройки в источниках не подтверждена.</t>
+          <t>Три камерных клубных дома у «Красной Розы» на 0,6 га; сохранение фасада дома Трындина-Жиро, виды на Кремль, клубхаус</t>
         </is>
       </c>
     </row>
@@ -9306,10 +9326,12 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>анонсирован, старт продаж ожидается</t>
-        </is>
-      </c>
-      <c r="G18" s="5" t="n"/>
+          <t>проект/анонс; сроки реализации и старт продаж не объявлены, предложений нет (сентябрь 2026)</t>
+        </is>
+      </c>
+      <c r="G18" s="7" t="n">
+        <v>90000</v>
+      </c>
       <c r="H18" s="5" t="n"/>
       <c r="I18" s="5" t="n"/>
       <c r="J18" s="5" t="n"/>
@@ -9319,8 +9341,12 @@
           <t>2030</t>
         </is>
       </c>
-      <c r="M18" s="22" t="n"/>
-      <c r="N18" s="5" t="n"/>
+      <c r="M18" s="21" t="n"/>
+      <c r="N18" s="5" t="inlineStr">
+        <is>
+          <t>2014-07-17</t>
+        </is>
+      </c>
       <c r="O18" s="9" t="inlineStr">
         <is>
           <t>ссылка</t>
@@ -9328,7 +9354,7 @@
       </c>
       <c r="P18" s="4" t="inlineStr">
         <is>
-          <t>Участок ~1,7 га с ОКН (фабрика Трёхгорной мануфактуры, будет сохранена/реконструирована). Апартаменты премиум-класса + офисы + wellness, подземный паркинг на 750 м/м. Сроки реализации официально не подтверждены; апартаменты, а не квартиры.</t>
+          <t>МФК с апартаментами, офисами и wellness на 1,7 га у Трёхгорной мануфактуры (ОКН сохраняется), паркинг 750 м/м</t>
         </is>
       </c>
     </row>
@@ -9348,7 +9374,7 @@
           <t>Тверской</t>
         </is>
       </c>
-      <c r="D19" s="19" t="inlineStr">
+      <c r="D19" s="20" t="inlineStr">
         <is>
           <t>Садовое кольцо</t>
         </is>
@@ -9360,15 +9386,17 @@
       </c>
       <c r="F19" s="10" t="inlineStr">
         <is>
-          <t>анонсирован, старт продаж ожидается в 2026 г.</t>
+          <t>предстарт; старт продаж ожидается в 2026 г. (на 08.09.2026 не объявлен)</t>
         </is>
       </c>
       <c r="G19" s="13" t="n">
         <v>12000</v>
       </c>
       <c r="H19" s="11" t="n"/>
-      <c r="I19" s="13" t="n">
-        <v>9</v>
+      <c r="I19" s="11" t="inlineStr">
+        <is>
+          <t>7–9</t>
+        </is>
       </c>
       <c r="J19" s="11" t="n"/>
       <c r="K19" s="11" t="inlineStr">
@@ -9377,7 +9405,7 @@
         </is>
       </c>
       <c r="L19" s="11" t="n"/>
-      <c r="M19" s="20" t="n"/>
+      <c r="M19" s="22" t="n"/>
       <c r="N19" s="11" t="n"/>
       <c r="O19" s="15" t="inlineStr">
         <is>
@@ -9386,7 +9414,7 @@
       </c>
       <c r="P19" s="10" t="inlineStr">
         <is>
-          <t>Участок ~0,4 га у сада «Эрмитаж», 2 корпуса 7–9 этажей, волнообразные фасады, делюкс-класс.</t>
+          <t>Два корпуса 7–9 эт. на 0,4 га у сада «Эрмитаж», волнообразные бионические фасады, камерный клубный формат; делюкс</t>
         </is>
       </c>
     </row>
@@ -9406,7 +9434,7 @@
           <t>Пресненский</t>
         </is>
       </c>
-      <c r="D20" s="19" t="inlineStr">
+      <c r="D20" s="20" t="inlineStr">
         <is>
           <t>Садовое кольцо</t>
         </is>
@@ -9418,7 +9446,7 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>в списке ожидаемых стартов делюкс-класса 2026 (агрегатор); подробностей нет</t>
+          <t>в списке ожидаемых стартов делюкс-класса 2026 (mskdeluxe.ru); подробностей нет (08.09.2026)</t>
         </is>
       </c>
       <c r="G20" s="5" t="n"/>
@@ -9427,7 +9455,7 @@
       <c r="J20" s="5" t="n"/>
       <c r="K20" s="5" t="n"/>
       <c r="L20" s="5" t="n"/>
-      <c r="M20" s="22" t="n"/>
+      <c r="M20" s="21" t="n"/>
       <c r="N20" s="5" t="n"/>
       <c r="O20" s="9" t="inlineStr">
         <is>
@@ -9436,7 +9464,7 @@
       </c>
       <c r="P20" s="4" t="inlineStr">
         <is>
-          <t>В том же списке mskdeluxe.ru: М. Дмитровка 5/9, Льва Толстого 14, Хилков 3, Б. Пироговская 51, Б. Харитоньевский 13, Олсуфьевский 10, Большая Ордынка 25, Воздвиженка 7/6, Малая Полянка 3 — без параметров и девелоперов.</t>
+          <t>Ожидаемый делюкс-старт на Малой Никитской у Красной Пресни; параметры не раскрыты, возможно тот же участок, что и №27</t>
         </is>
       </c>
     </row>
@@ -9456,7 +9484,7 @@
           <t>Замоскворечье</t>
         </is>
       </c>
-      <c r="D21" s="19" t="inlineStr">
+      <c r="D21" s="20" t="inlineStr">
         <is>
           <t>Садовое кольцо</t>
         </is>
@@ -9468,13 +9496,15 @@
       </c>
       <c r="F21" s="10" t="inlineStr">
         <is>
-          <t>старт продаж 06.04.2026</t>
+          <t>анонс старта продаж 06.04.2026; по novostroev.ru на 03.09.2026 — проект, продажи не начаты</t>
         </is>
       </c>
       <c r="G21" s="13" t="n">
         <v>3000</v>
       </c>
-      <c r="H21" s="11" t="n"/>
+      <c r="H21" s="13" t="n">
+        <v>2360</v>
+      </c>
       <c r="I21" s="13" t="n">
         <v>6</v>
       </c>
@@ -9487,7 +9517,7 @@
         </is>
       </c>
       <c r="L21" s="11" t="n"/>
-      <c r="M21" s="20" t="n"/>
+      <c r="M21" s="22" t="n"/>
       <c r="N21" s="11" t="inlineStr">
         <is>
           <t>2026-04-06</t>
@@ -9500,7 +9530,7 @@
       </c>
       <c r="P21" s="10" t="inlineStr">
         <is>
-          <t>Участок 0,1 га, 11 квартир, 14 подземных м/м, архитектура A2M. Делюкс.</t>
+          <t>Клубный дом 6 эт. на 11 квартир на участке 0,1 га в Замоскворечье, 14 м/м, архитектура A2M; делюкс</t>
         </is>
       </c>
     </row>
@@ -9520,25 +9550,27 @@
           <t>Хамовники</t>
         </is>
       </c>
-      <c r="D22" s="21" t="inlineStr">
+      <c r="D22" s="19" t="inlineStr">
         <is>
           <t>Хамовники</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>Грандор (Grandor)</t>
+          <t>Грандор</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>ГПЗУ получен (апрель 2021), старт продаж ожидается</t>
+          <t>проект (ГПЗУ апрель 2021); продажи не начаты, «скоро в продаже» (08.09.2026)</t>
         </is>
       </c>
       <c r="G22" s="5" t="n"/>
       <c r="H22" s="5" t="n"/>
-      <c r="I22" s="7" t="n">
-        <v>8</v>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>5–8</t>
+        </is>
       </c>
       <c r="J22" s="5" t="n"/>
       <c r="K22" s="5" t="inlineStr">
@@ -9547,7 +9579,7 @@
         </is>
       </c>
       <c r="L22" s="5" t="n"/>
-      <c r="M22" s="22" t="n"/>
+      <c r="M22" s="21" t="n"/>
       <c r="N22" s="5" t="n"/>
       <c r="O22" s="9" t="inlineStr">
         <is>
@@ -9556,7 +9588,7 @@
       </c>
       <c r="P22" s="4" t="inlineStr">
         <is>
-          <t>Участок 0,4 га, семь корпусов 5–8 этажей в индивидуальной архитектуре. В базе делюкс-стартов 2026–2027 mskdeluxe.ru.</t>
+          <t>Семь корпусов 5–8 эт. на 0,4 га в Хамовниках у м. Фрунзенская, индивидуальная архитектура; делюкс</t>
         </is>
       </c>
     </row>
@@ -9576,19 +9608,19 @@
           <t>Якиманка</t>
         </is>
       </c>
-      <c r="D23" s="19" t="inlineStr">
+      <c r="D23" s="20" t="inlineStr">
         <is>
           <t>Садовое кольцо</t>
         </is>
       </c>
-      <c r="E23" s="10" t="inlineStr">
-        <is>
-          <t>Aurix Development (Группа «Эталон»)</t>
-        </is>
-      </c>
-      <c r="F23" s="11" t="inlineStr">
-        <is>
-          <t>старт продаж 2026</t>
+      <c r="E23" s="11" t="inlineStr">
+        <is>
+          <t>Aurix Development</t>
+        </is>
+      </c>
+      <c r="F23" s="10" t="inlineStr">
+        <is>
+          <t>старт продаж 2026 (по сайту проекта); строительство не начато, цены не опубликованы (08.09.2026)</t>
         </is>
       </c>
       <c r="G23" s="11" t="n"/>
@@ -9605,7 +9637,7 @@
         </is>
       </c>
       <c r="L23" s="11" t="n"/>
-      <c r="M23" s="20" t="n"/>
+      <c r="M23" s="22" t="n"/>
       <c r="N23" s="11" t="n"/>
       <c r="O23" s="15" t="inlineStr">
         <is>
@@ -9614,7 +9646,7 @@
       </c>
       <c r="P23" s="10" t="inlineStr">
         <is>
-          <t>9 этажей, 34 квартиры, паркинг на 36 м/м, проект Etalon Project. Продажи открыты в 2026 г.; стадия строительства в открытых источниках не уточнена.</t>
+          <t>Клубный дом 9 эт. на 34 резиденции у Третьяковской галереи, паркинг 36 м/м, отделка премиум, мотивы русского фольклора</t>
         </is>
       </c>
     </row>
@@ -9634,7 +9666,7 @@
           <t>Хамовники</t>
         </is>
       </c>
-      <c r="D24" s="21" t="inlineStr">
+      <c r="D24" s="19" t="inlineStr">
         <is>
           <t>Хамовники</t>
         </is>
@@ -9646,20 +9678,24 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>проект утверждён (АГР, май 2026), начало строительства 2027</t>
+          <t>проект утверждён (АГР, май 2026); начало строительства 2027, старт продаж ожидается в 2027</t>
         </is>
       </c>
       <c r="G24" s="5" t="n"/>
       <c r="H24" s="5" t="n"/>
-      <c r="I24" s="5" t="n"/>
+      <c r="I24" s="4" t="inlineStr">
+        <is>
+          <t>8–24 (жилые корпуса переменной этажности)</t>
+        </is>
+      </c>
       <c r="J24" s="5" t="n"/>
-      <c r="K24" s="5" t="inlineStr">
-        <is>
-          <t>2027 (стройка)</t>
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t>2027 (стройка и старт продаж)</t>
         </is>
       </c>
       <c r="L24" s="5" t="n"/>
-      <c r="M24" s="22" t="n"/>
+      <c r="M24" s="21" t="n"/>
       <c r="N24" s="5" t="inlineStr">
         <is>
           <t>2026-05-28</t>
@@ -9672,7 +9708,7 @@
       </c>
       <c r="P24" s="4" t="inlineStr">
         <is>
-          <t>Два жилых корпуса переменной этажности в неоклассике + эллиптический БЦ 26 тыс. м² («яйцо Фаберже»). Концепция согласована Департаментом градостроительной политики (В. Овчинский). Параметры жилой части не раскрыты.</t>
+          <t>Квартал на 5,27 га у Лужников: два жилых корпуса 8–24 эт. в неоклассике + эллиптический БЦ «яйцо Фаберже» 26 тыс. м²</t>
         </is>
       </c>
     </row>
@@ -9692,7 +9728,7 @@
           <t>Басманный</t>
         </is>
       </c>
-      <c r="D25" s="19" t="inlineStr">
+      <c r="D25" s="20" t="inlineStr">
         <is>
           <t>Садовое кольцо</t>
         </is>
@@ -9704,7 +9740,7 @@
       </c>
       <c r="F25" s="10" t="inlineStr">
         <is>
-          <t>старт продаж июль–август 2026</t>
+          <t>проектирование (kvartiravmoskve.ru, 15.07.2026); старт продаж заявлен на июль–август 2026, цены не опубликованы</t>
         </is>
       </c>
       <c r="G25" s="11" t="n"/>
@@ -9719,7 +9755,7 @@
         </is>
       </c>
       <c r="L25" s="11" t="n"/>
-      <c r="M25" s="20" t="n"/>
+      <c r="M25" s="22" t="n"/>
       <c r="N25" s="11" t="inlineStr">
         <is>
           <t>2026-07</t>
@@ -9732,7 +9768,7 @@
       </c>
       <c r="P25" s="10" t="inlineStr">
         <is>
-          <t>Клубный дом делюкс-класса у Чистых прудов, 1 монолитный корпус 7 этажей, архитектура WALL. В обзоре делюкс-стартов 2026 novostroev.ru фигурировал как Veil, 9 этажей.</t>
+          <t>Камерный клубный дом 7 эт. у Чистых прудов, монолит-кирпич, двор без машин, архитектура WALL; делюкс</t>
         </is>
       </c>
     </row>
@@ -9752,23 +9788,23 @@
           <t>Мещанский</t>
         </is>
       </c>
-      <c r="D26" s="19" t="inlineStr">
+      <c r="D26" s="20" t="inlineStr">
         <is>
           <t>Садовое кольцо</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr">
-        <is>
-          <t>Sminex (проект выкуплен у «Галс-Девелопмент»)</t>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Sminex</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>проект приобретён, старт продаж ожидается</t>
+          <t>проект дорабатывается под стандарты Sminex; по gdeetotdom.ru — возведение стен; продажи по запросу, старт не объявлен</t>
         </is>
       </c>
       <c r="G26" s="7" t="n">
-        <v>36400</v>
+        <v>31000</v>
       </c>
       <c r="H26" s="7" t="n">
         <v>18000</v>
@@ -9780,8 +9816,12 @@
         <v>115</v>
       </c>
       <c r="K26" s="5" t="n"/>
-      <c r="L26" s="5" t="n"/>
-      <c r="M26" s="22" t="n"/>
+      <c r="L26" s="5" t="inlineStr">
+        <is>
+          <t>2 кв. 2030</t>
+        </is>
+      </c>
+      <c r="M26" s="21" t="n"/>
       <c r="N26" s="5" t="inlineStr">
         <is>
           <t>2025-12-12</t>
@@ -9794,7 +9834,7 @@
       </c>
       <c r="P26" s="4" t="inlineStr">
         <is>
-          <t>Семь корпусов 2–10 этажей, 115 квартир 61–426 м², таунхаусы и пентхаусы, двор-парк Scape, реставрация особняка конца XIX в. Сделка 12.12.2025.</t>
+          <t>Семь клубных домов 2–10 эт., 115 квартир 61–426 м² у Кузнецкого Моста, двор-парк, реставрация особняка XIX в.</t>
         </is>
       </c>
     </row>
@@ -9814,7 +9854,7 @@
           <t>Хамовники</t>
         </is>
       </c>
-      <c r="D27" s="21" t="inlineStr">
+      <c r="D27" s="19" t="inlineStr">
         <is>
           <t>Хамовники</t>
         </is>
@@ -9826,7 +9866,7 @@
       </c>
       <c r="F27" s="10" t="inlineStr">
         <is>
-          <t>участок приобретён (апрель 2026), проектирование</t>
+          <t>участок приобретён (апрель 2026), проектирование; сроки не объявлены (08.09.2026)</t>
         </is>
       </c>
       <c r="G27" s="13" t="n">
@@ -9839,7 +9879,7 @@
       <c r="J27" s="11" t="n"/>
       <c r="K27" s="11" t="n"/>
       <c r="L27" s="11" t="n"/>
-      <c r="M27" s="20" t="n"/>
+      <c r="M27" s="22" t="n"/>
       <c r="N27" s="11" t="inlineStr">
         <is>
           <t>2026-04-24</t>
@@ -9852,7 +9892,7 @@
       </c>
       <c r="P27" s="10" t="inlineStr">
         <is>
-          <t>Участок 0,5 га (бывшая шёлковая фабрика, 4 здания 5 тыс. м²), продавец KR Properties (А. Клячин), переход прав 23.04.2026. Камерный клубный дом: пентхаусы с видом на Кремль, виллы, двор-сад; фасады по ул. Тимура Фрунзе сохраняются.</t>
+          <t>Камерный клубный дом на 0,5 га бывшей шёлковой фабрики: пентхаусы с видом на Кремль, виллы, двор-сад среди ОКН</t>
         </is>
       </c>
     </row>
@@ -9872,7 +9912,7 @@
           <t>Замоскворечье</t>
         </is>
       </c>
-      <c r="D28" s="19" t="inlineStr">
+      <c r="D28" s="20" t="inlineStr">
         <is>
           <t>Садовое кольцо</t>
         </is>
@@ -9884,7 +9924,7 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>участок приобретён (март 2026), проектирование</t>
+          <t>участок приобретён (март 2026), проектирование; параметры и сроки не раскрыты (08.09.2026)</t>
         </is>
       </c>
       <c r="G28" s="5" t="n"/>
@@ -9893,7 +9933,7 @@
       <c r="J28" s="5" t="n"/>
       <c r="K28" s="5" t="n"/>
       <c r="L28" s="5" t="n"/>
-      <c r="M28" s="22" t="n"/>
+      <c r="M28" s="21" t="n"/>
       <c r="N28" s="5" t="inlineStr">
         <is>
           <t>2026-03-17</t>
@@ -9906,7 +9946,7 @@
       </c>
       <c r="P28" s="4" t="inlineStr">
         <is>
-          <t>Участок 1,8 га, 8 зданий 38,5 тыс. м², в т.ч. 3 корпуса типографии Сытина (ОКН, арх. Эрихсон/Шухов). Продавец — В. Погребенко, оценка сделки 12–14 млрд руб., инвестиции 25–30 млрд руб. План: реставрация + новые элитные клубные дома. Участок у Садового кольца (Валовая ул.).</t>
+          <t>Реставрация типографии Сытина (ОКН) и новые клубные дома на 1,8 га в Замоскворечье; двор-парк, виды на Кремль</t>
         </is>
       </c>
     </row>
@@ -9926,32 +9966,36 @@
           <t>Хамовники</t>
         </is>
       </c>
-      <c r="D29" s="21" t="inlineStr">
+      <c r="D29" s="19" t="inlineStr">
         <is>
           <t>Хамовники</t>
         </is>
       </c>
       <c r="E29" s="10" t="inlineStr">
         <is>
-          <t>ГК «Векторстройфинанс» (VSF)</t>
+          <t>ГК «Векторстройфинанс»</t>
         </is>
       </c>
       <c r="F29" s="10" t="inlineStr">
         <is>
-          <t>анонсирован (приобретение объекта), концепция</t>
+          <t>концепция бюро МЛА+ опубликована (январь 2026); сроки строительства не объявлены, реализация именно этой концепции не подтверждена</t>
         </is>
       </c>
       <c r="G29" s="13" t="n">
         <v>2500</v>
       </c>
       <c r="H29" s="11" t="n"/>
-      <c r="I29" s="13" t="n">
-        <v>4</v>
-      </c>
-      <c r="J29" s="11" t="n"/>
+      <c r="I29" s="10" t="inlineStr">
+        <is>
+          <t>4–10 (башня 10 эт. + клубный корпус 4 эт.)</t>
+        </is>
+      </c>
+      <c r="J29" s="13" t="n">
+        <v>27</v>
+      </c>
       <c r="K29" s="11" t="n"/>
       <c r="L29" s="11" t="n"/>
-      <c r="M29" s="20" t="n"/>
+      <c r="M29" s="22" t="n"/>
       <c r="N29" s="11" t="inlineStr">
         <is>
           <t>2025-07-09</t>
@@ -9964,7 +10008,7 @@
       </c>
       <c r="P29" s="10" t="inlineStr">
         <is>
-          <t>Четырёхэтажное здание 1889 г. и двухэтажное до 1812 г., ~2,5 тыс. м². Оценка инвестиций 3,5–4,5 млрд руб., стоимость объекта до 1,3 млрд руб. Планируется перестройка в элитный клубный дом.</t>
+          <t>Клубный дом на месте усадьбы Якунина: башня «Шёлк» 10 эт. и корпус «Кашемир» 4 эт., 27 квартир, вход-«игольное ушко»</t>
         </is>
       </c>
     </row>
@@ -9984,7 +10028,7 @@
           <t>Хамовники</t>
         </is>
       </c>
-      <c r="D30" s="21" t="inlineStr">
+      <c r="D30" s="19" t="inlineStr">
         <is>
           <t>Хамовники</t>
         </is>
@@ -9996,7 +10040,7 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>проект, продажи не начаты</t>
+          <t>проект, продажи не начаты (novostroev.ru, 03.09.2026); старт продаж заявлен на 2026</t>
         </is>
       </c>
       <c r="G30" s="7" t="n">
@@ -10012,8 +10056,12 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="L30" s="5" t="n"/>
-      <c r="M30" s="22" t="n"/>
+      <c r="L30" s="5" t="inlineStr">
+        <is>
+          <t>2030</t>
+        </is>
+      </c>
+      <c r="M30" s="21" t="n"/>
       <c r="N30" s="5" t="n"/>
       <c r="O30" s="9" t="inlineStr">
         <is>
@@ -10022,7 +10070,7 @@
       </c>
       <c r="P30" s="4" t="inlineStr">
         <is>
-          <t>Участок ~0,4 га, два корпуса ~14 и 18 этажей, архитектура Arch(e)type, двор без машин. Площадь 24,6 тыс. м² — по обзору делюкс-стартов 2026 novostroev.ru.</t>
+          <t>Два корпуса 14–18 эт. на 0,4 га у м. Спортивная, Arch(e)type, двор без машин, SPA с бассейном; делюкс</t>
         </is>
       </c>
     </row>
@@ -10054,7 +10102,7 @@
       </c>
       <c r="F31" s="10" t="inlineStr">
         <is>
-          <t>решение о КРТ (по данным заказчика — август 2026); оператор/правообладатель и торги в открытых источниках не найдены</t>
+          <t>решение о КРТ (август 2026); оператор/правообладатель и торги в открытых источниках не найдены (проверка 08.09.2026)</t>
         </is>
       </c>
       <c r="G31" s="13" t="n">
@@ -10067,7 +10115,7 @@
       <c r="J31" s="11" t="n"/>
       <c r="K31" s="11" t="n"/>
       <c r="L31" s="11" t="n"/>
-      <c r="M31" s="20" t="n"/>
+      <c r="M31" s="22" t="n"/>
       <c r="N31" s="11" t="inlineStr">
         <is>
           <t>2026-08</t>
@@ -10080,7 +10128,7 @@
       </c>
       <c r="P31" s="10" t="inlineStr">
         <is>
-          <t>Участок ~0,3 га включён в программу КРТ решением властей Москвы. Существующие здания реконструированы в 2004 г., в 2020 г. переоборудованы под хостелы. Оператор/девелопер в публикации не назван; в других открытых источниках на 07.09.2026 не найден. Локация — Пресненский район вне Садового кольца, между Б. Грузинской и Пресненским Валом (условно отнесено к зоне Пресня/Сити).; Поиск по mos.ru, krt.mos.ru, stroi.mos.ru, Ведомости, РБК, Интерфакс, М24, Известия (август–сентябрь 2026) не выявил отдельной публикации по этому участку: новости августа 2026 о КРТ (250 проектов, 63 договора с начала года) даются агрегированно. Ближайший крупный проект — квартал «Тишинский бульвар» Sminex (Электрический пер., 1), связь с участком №8 не подтверждена. Площадь 0,3 га / ~10 000 м² — из исходных данных запроса, независимого подтверждения нет.</t>
+          <t>Участок КРТ 0,3 га с двумя зданиями (хостелы) на Пресне между Б. Грузинской и Пресненским Валом; параметры не раскрыты</t>
         </is>
       </c>
     </row>
@@ -10100,7 +10148,7 @@
           <t>Хамовники</t>
         </is>
       </c>
-      <c r="D32" s="21" t="inlineStr">
+      <c r="D32" s="19" t="inlineStr">
         <is>
           <t>Хамовники</t>
         </is>
@@ -10112,7 +10160,7 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>проектирование (долгосрочный проект), старт продаж ожидается</t>
+          <t>статус противоречив: novostroy-m.ru — проект 2016 г. «скоро старт»; novostroev.ru (03.09.2026) — «строительство/продажи завершены»; mskdeluxe.ru — старт 2026–2027</t>
         </is>
       </c>
       <c r="G32" s="7" t="n">
@@ -10121,8 +10169,10 @@
       <c r="H32" s="7" t="n">
         <v>8800</v>
       </c>
-      <c r="I32" s="7" t="n">
-        <v>8</v>
+      <c r="I32" s="5" t="inlineStr">
+        <is>
+          <t>3–8</t>
+        </is>
       </c>
       <c r="J32" s="5" t="n"/>
       <c r="K32" s="5" t="inlineStr">
@@ -10131,7 +10181,7 @@
         </is>
       </c>
       <c r="L32" s="5" t="n"/>
-      <c r="M32" s="22" t="n"/>
+      <c r="M32" s="21" t="n"/>
       <c r="N32" s="5" t="n"/>
       <c r="O32" s="9" t="inlineStr">
         <is>
@@ -10140,7 +10190,7 @@
       </c>
       <c r="P32" s="4" t="inlineStr">
         <is>
-          <t>3–8 этажей, монолит-кирпич, коммерция 1,8 тыс. м², паркинг 170 м/м. Карточка novostroy-m.ru датирована 2016 г.; проект вновь фигурирует в списке делюкс-стартов 2026–2027 на mskdeluxe.ru. Актуальность требует проверки.</t>
+          <t>Клубный дом 3–8 эт. на «Золотой миле», 19,8 тыс. м², жильё 8,8 тыс. м², коммерция 1,8 тыс. м², паркинг 170 м/м</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix Slava ЖК link lookup
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Bv8NELxW2W7udnb3XUFGS2
</commit_message>
<xml_diff>
--- a/docs/premium-cao/premium-zhk-cao.xlsx
+++ b/docs/premium-cao/premium-zhk-cao.xlsx
@@ -4922,7 +4922,11 @@
           <t>бетон</t>
         </is>
       </c>
-      <c r="O4" s="5" t="inlineStr"/>
+      <c r="O4" s="9" t="inlineStr">
+        <is>
+          <t>ссылка</t>
+        </is>
+      </c>
       <c r="P4" s="10" t="inlineStr">
         <is>
           <t>Квартал из 3 корпусов 6–22 эт. на Ленинградском пр., панорамное остекление, паркинг на 782 м/м</t>
@@ -8258,52 +8262,53 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O5" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O4" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O5" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId47"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.35" bottom="0.35" header="0.2" footer="0.2"/>

</xml_diff>

<commit_message>
Workbook: auto row heights for wrapped text, wider narrow columns
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Bv8NELxW2W7udnb3XUFGS2
</commit_message>
<xml_diff>
--- a/docs/premium-cao/premium-zhk-cao.xlsx
+++ b/docs/premium-cao/premium-zhk-cao.xlsx
@@ -606,15 +606,15 @@
   <dimension ref="A1:Q54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
     <col width="6" customWidth="1" min="7" max="7"/>
     <col width="7" customWidth="1" min="8" max="8"/>
-    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
@@ -622,7 +622,7 @@
     <col width="9" customWidth="1" min="14" max="14"/>
     <col width="10" customWidth="1" min="15" max="15"/>
     <col width="7" customWidth="1" min="16" max="16"/>
-    <col width="74" customWidth="1" min="17" max="17"/>
+    <col width="70" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -635,7 +635,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>ЦАО, дома 2018+, активные объявления Циан на 2026-09-07; зоны: Садовое кольцо / Хамовники / Сити / Пресня / Белорусская. Сортировка по медиане ₽/м², цвет — от дешёвых (зелёный) к дорогим (красный)</t>
+          <t>ЦАО, дома 2018+, активные объявления Циан на 2026-09-07; зоны: Садовое кольцо / Хамовники / Сити / Пресня / Белорусская. Сортировка по медиане ₽/м², цвет — от дешёвых (зелёный) к дорогим (красный). Класс — по карточке ЖК на Циан</t>
         </is>
       </c>
     </row>
@@ -726,7 +726,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="24" customHeight="1">
+    <row r="4" ht="140.5" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Резиденция Тверская</t>
@@ -789,7 +789,7 @@
       </c>
       <c r="O4" s="5" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P4" s="9" t="inlineStr">
@@ -803,7 +803,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="24" customHeight="1">
+    <row r="5" ht="115.5" customHeight="1">
       <c r="A5" s="11" t="inlineStr">
         <is>
           <t>NEVA TOWERS (Нева Тауэрс)</t>
@@ -866,7 +866,7 @@
       </c>
       <c r="O5" s="12" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P5" s="16" t="inlineStr">
@@ -880,7 +880,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1">
+    <row r="6" ht="115.5" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Sinatra (Синатра)</t>
@@ -943,7 +943,7 @@
       </c>
       <c r="O6" s="5" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P6" s="9" t="inlineStr">
@@ -957,7 +957,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1">
+    <row r="7" ht="115.5" customHeight="1">
       <c r="A7" s="11" t="inlineStr">
         <is>
           <t>LUMIN (ЛЮМИН)</t>
@@ -1020,7 +1020,7 @@
       </c>
       <c r="O7" s="12" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P7" s="16" t="inlineStr">
@@ -1034,7 +1034,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1">
+    <row r="8" ht="115.5" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Уланский, 13</t>
@@ -1097,7 +1097,7 @@
       </c>
       <c r="O8" s="5" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P8" s="9" t="inlineStr">
@@ -1111,7 +1111,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1">
+    <row r="9" ht="115.5" customHeight="1">
       <c r="A9" s="11" t="inlineStr">
         <is>
           <t>Современник</t>
@@ -1174,7 +1174,7 @@
       </c>
       <c r="O9" s="12" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P9" s="16" t="inlineStr">
@@ -1188,7 +1188,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1">
+    <row r="10" ht="115.5" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Репаблик</t>
@@ -1251,7 +1251,7 @@
       </c>
       <c r="O10" s="5" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P10" s="9" t="inlineStr">
@@ -1265,7 +1265,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="24" customHeight="1">
+    <row r="11" ht="115.5" customHeight="1">
       <c r="A11" s="11" t="inlineStr">
         <is>
           <t>City Park (Сити Парк)</t>
@@ -1328,7 +1328,7 @@
       </c>
       <c r="O11" s="12" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P11" s="16" t="inlineStr">
@@ -1342,7 +1342,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1">
+    <row r="12" ht="115.5" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t>SkyView</t>
@@ -1405,7 +1405,7 @@
       </c>
       <c r="O12" s="5" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P12" s="9" t="inlineStr">
@@ -1419,7 +1419,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1">
+    <row r="13" ht="115.5" customHeight="1">
       <c r="A13" s="11" t="inlineStr">
         <is>
           <t>Полянка/44</t>
@@ -1482,7 +1482,7 @@
       </c>
       <c r="O13" s="12" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P13" s="16" t="inlineStr">
@@ -1496,7 +1496,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1">
+    <row r="14" ht="140.5" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Титул на Серебрянической</t>
@@ -1559,7 +1559,7 @@
       </c>
       <c r="O14" s="5" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P14" s="9" t="inlineStr">
@@ -1573,7 +1573,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="15" customHeight="1">
+    <row r="15" ht="115.5" customHeight="1">
       <c r="A15" s="11" t="inlineStr">
         <is>
           <t>Bogenhouse (Богенхаус)</t>
@@ -1636,7 +1636,7 @@
       </c>
       <c r="O15" s="12" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P15" s="16" t="inlineStr">
@@ -1650,7 +1650,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1">
+    <row r="16" ht="128" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Capital Towers (Капитал Тауэрс)</t>
@@ -1713,7 +1713,7 @@
       </c>
       <c r="O16" s="5" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P16" s="9" t="inlineStr">
@@ -1727,7 +1727,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="24" customHeight="1">
+    <row r="17" ht="128" customHeight="1">
       <c r="A17" s="11" t="inlineStr">
         <is>
           <t>BALCHUG VIEWPOINT (Балчуг Вьюпоинт)</t>
@@ -1790,7 +1790,7 @@
       </c>
       <c r="O17" s="12" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P17" s="16" t="inlineStr">
@@ -1804,7 +1804,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1">
+    <row r="18" ht="128" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Титул на Якиманке</t>
@@ -1867,7 +1867,7 @@
       </c>
       <c r="O18" s="5" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P18" s="9" t="inlineStr">
@@ -1881,7 +1881,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="15" customHeight="1">
+    <row r="19" ht="128" customHeight="1">
       <c r="A19" s="11" t="inlineStr">
         <is>
           <t>Клубный дом ЦВЕТ32</t>
@@ -1944,7 +1944,7 @@
       </c>
       <c r="O19" s="12" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P19" s="16" t="inlineStr">
@@ -1958,7 +1958,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="15" customHeight="1">
+    <row r="20" ht="115.5" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
           <t>A.Residence (А Резиденс)</t>
@@ -2021,7 +2021,7 @@
       </c>
       <c r="O20" s="5" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P20" s="9" t="inlineStr">
@@ -2035,7 +2035,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1">
+    <row r="21" ht="115.5" customHeight="1">
       <c r="A21" s="11" t="inlineStr">
         <is>
           <t>Roza Rossa (Роза Росса)</t>
@@ -2098,7 +2098,7 @@
       </c>
       <c r="O21" s="12" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P21" s="16" t="inlineStr">
@@ -2112,7 +2112,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="15" customHeight="1">
+    <row r="22" ht="153" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Собрание клубных домов ORDYNKA (Ордынка)</t>
@@ -2175,7 +2175,7 @@
       </c>
       <c r="O22" s="5" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P22" s="9" t="inlineStr">
@@ -2189,7 +2189,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="15" customHeight="1">
+    <row r="23" ht="115.5" customHeight="1">
       <c r="A23" s="11" t="inlineStr">
         <is>
           <t>Дом NV/9</t>
@@ -2252,7 +2252,7 @@
       </c>
       <c r="O23" s="12" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P23" s="16" t="inlineStr">
@@ -2266,7 +2266,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="15" customHeight="1">
+    <row r="24" ht="128" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
           <t>Fantastic House (Фантастик Хаус)</t>
@@ -2329,7 +2329,7 @@
       </c>
       <c r="O24" s="5" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P24" s="9" t="inlineStr">
@@ -2343,7 +2343,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="15" customHeight="1">
+    <row r="25" ht="140.5" customHeight="1">
       <c r="A25" s="11" t="inlineStr">
         <is>
           <t>Клубный дом Космо 4/22</t>
@@ -2406,7 +2406,7 @@
       </c>
       <c r="O25" s="12" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P25" s="16" t="inlineStr">
@@ -2420,7 +2420,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="24" customHeight="1">
+    <row r="26" ht="115.5" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
         <is>
           <t>Софийский</t>
@@ -2483,7 +2483,7 @@
       </c>
       <c r="O26" s="5" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P26" s="9" t="inlineStr">
@@ -2497,7 +2497,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="15" customHeight="1">
+    <row r="27" ht="128" customHeight="1">
       <c r="A27" s="11" t="inlineStr">
         <is>
           <t>Дом на Тишинке</t>
@@ -2560,7 +2560,7 @@
       </c>
       <c r="O27" s="12" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P27" s="16" t="inlineStr">
@@ -2574,7 +2574,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="15" customHeight="1">
+    <row r="28" ht="128" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
         <is>
           <t>Тессинский, 1</t>
@@ -2637,7 +2637,7 @@
       </c>
       <c r="O28" s="5" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P28" s="9" t="inlineStr">
@@ -2651,7 +2651,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="15" customHeight="1">
+    <row r="29" ht="103" customHeight="1">
       <c r="A29" s="11" t="inlineStr">
         <is>
           <t>Lucky (Лаки)</t>
@@ -2714,7 +2714,7 @@
       </c>
       <c r="O29" s="12" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P29" s="16" t="inlineStr">
@@ -2728,7 +2728,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="15" customHeight="1">
+    <row r="30" ht="115.5" customHeight="1">
       <c r="A30" s="4" t="inlineStr">
         <is>
           <t>Artisan (Артисан)</t>
@@ -2791,7 +2791,7 @@
       </c>
       <c r="O30" s="5" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P30" s="9" t="inlineStr">
@@ -2805,7 +2805,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="15" customHeight="1">
+    <row r="31" ht="115.5" customHeight="1">
       <c r="A31" s="11" t="inlineStr">
         <is>
           <t>Абрикосов</t>
@@ -2868,7 +2868,7 @@
       </c>
       <c r="O31" s="12" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P31" s="16" t="inlineStr">
@@ -2882,7 +2882,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="24" customHeight="1">
+    <row r="32" ht="128" customHeight="1">
       <c r="A32" s="4" t="inlineStr">
         <is>
           <t>Клубный дом CULT (Клубный дом Культ)</t>
@@ -2945,7 +2945,7 @@
       </c>
       <c r="O32" s="5" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P32" s="9" t="inlineStr">
@@ -2959,7 +2959,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="15" customHeight="1">
+    <row r="33" ht="140.5" customHeight="1">
       <c r="A33" s="11" t="inlineStr">
         <is>
           <t>SAVVIN RIVER RESIDENCE (Саввин Ривер Резиденс)</t>
@@ -3022,7 +3022,7 @@
       </c>
       <c r="O33" s="12" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P33" s="16" t="inlineStr">
@@ -3036,7 +3036,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="24" customHeight="1">
+    <row r="34" ht="128" customHeight="1">
       <c r="A34" s="4" t="inlineStr">
         <is>
           <t>Пироговская 14</t>
@@ -3099,7 +3099,7 @@
       </c>
       <c r="O34" s="5" t="inlineStr">
         <is>
-          <t>бизнес (Циан)</t>
+          <t>бизнес</t>
         </is>
       </c>
       <c r="P34" s="9" t="inlineStr">
@@ -3113,7 +3113,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="15" customHeight="1">
+    <row r="35" ht="115.5" customHeight="1">
       <c r="A35" s="11" t="inlineStr">
         <is>
           <t>Cloud Nine (Клауд Найн)</t>
@@ -3176,7 +3176,7 @@
       </c>
       <c r="O35" s="12" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P35" s="16" t="inlineStr">
@@ -3190,7 +3190,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="15" customHeight="1">
+    <row r="36" ht="140.5" customHeight="1">
       <c r="A36" s="4" t="inlineStr">
         <is>
           <t>Симфония набережных (Котельническая 21)</t>
@@ -3253,7 +3253,7 @@
       </c>
       <c r="O36" s="5" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P36" s="9" t="inlineStr">
@@ -3267,7 +3267,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="15" customHeight="1">
+    <row r="37" ht="128" customHeight="1">
       <c r="A37" s="11" t="inlineStr">
         <is>
           <t>Садовые кварталы</t>
@@ -3330,7 +3330,7 @@
       </c>
       <c r="O37" s="12" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P37" s="16" t="inlineStr">
@@ -3344,7 +3344,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="15" customHeight="1">
+    <row r="38" ht="128" customHeight="1">
       <c r="A38" s="4" t="inlineStr">
         <is>
           <t>Малая Ордынка 19</t>
@@ -3407,7 +3407,7 @@
       </c>
       <c r="O38" s="5" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P38" s="9" t="inlineStr">
@@ -3421,7 +3421,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="15" customHeight="1">
+    <row r="39" ht="128" customHeight="1">
       <c r="A39" s="11" t="inlineStr">
         <is>
           <t>Дом в Газетном</t>
@@ -3484,7 +3484,7 @@
       </c>
       <c r="O39" s="12" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P39" s="16" t="inlineStr">
@@ -3498,7 +3498,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="15" customHeight="1">
+    <row r="40" ht="128" customHeight="1">
       <c r="A40" s="4" t="inlineStr">
         <is>
           <t>Zvonarsky Deluxe (Звонарский Делюкс)</t>
@@ -3561,7 +3561,7 @@
       </c>
       <c r="O40" s="5" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P40" s="9" t="inlineStr">
@@ -3575,7 +3575,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="15" customHeight="1">
+    <row r="41" ht="128" customHeight="1">
       <c r="A41" s="11" t="inlineStr">
         <is>
           <t>White Khamovniki (Вайт Хамовники)</t>
@@ -3638,7 +3638,7 @@
       </c>
       <c r="O41" s="12" t="inlineStr">
         <is>
-          <t>бизнес (Циан)</t>
+          <t>бизнес</t>
         </is>
       </c>
       <c r="P41" s="16" t="inlineStr">
@@ -3652,7 +3652,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="15" customHeight="1">
+    <row r="42" ht="140.5" customHeight="1">
       <c r="A42" s="4" t="inlineStr">
         <is>
           <t>Золотой, жилой квартал</t>
@@ -3715,7 +3715,7 @@
       </c>
       <c r="O42" s="5" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P42" s="9" t="inlineStr">
@@ -3729,7 +3729,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="15" customHeight="1">
+    <row r="43" ht="103" customHeight="1">
       <c r="A43" s="11" t="inlineStr">
         <is>
           <t>Magnum (Магнум)</t>
@@ -3792,7 +3792,7 @@
       </c>
       <c r="O43" s="12" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P43" s="16" t="inlineStr">
@@ -3806,7 +3806,7 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="15" customHeight="1">
+    <row r="44" ht="140.5" customHeight="1">
       <c r="A44" s="4" t="inlineStr">
         <is>
           <t>Дом Бакст на Патриарших</t>
@@ -3869,7 +3869,7 @@
       </c>
       <c r="O44" s="5" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P44" s="9" t="inlineStr">
@@ -3883,7 +3883,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="15" customHeight="1">
+    <row r="45" ht="115.5" customHeight="1">
       <c r="A45" s="11" t="inlineStr">
         <is>
           <t>Villa Grace (Вилла Грейс)</t>
@@ -3946,7 +3946,7 @@
       </c>
       <c r="O45" s="12" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P45" s="16" t="inlineStr">
@@ -3960,7 +3960,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="15" customHeight="1">
+    <row r="46" ht="115.5" customHeight="1">
       <c r="A46" s="4" t="inlineStr">
         <is>
           <t>Brodsky (Бродский)</t>
@@ -4023,7 +4023,7 @@
       </c>
       <c r="O46" s="5" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P46" s="9" t="inlineStr">
@@ -4037,7 +4037,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="15" customHeight="1">
+    <row r="47" ht="128" customHeight="1">
       <c r="A47" s="11" t="inlineStr">
         <is>
           <t>Жизнь на Плющихе</t>
@@ -4100,7 +4100,7 @@
       </c>
       <c r="O47" s="12" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P47" s="16" t="inlineStr">
@@ -4114,7 +4114,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="15" customHeight="1">
+    <row r="48" ht="115.5" customHeight="1">
       <c r="A48" s="4" t="inlineStr">
         <is>
           <t>Carré Blanc (Карре Бланк)</t>
@@ -4177,7 +4177,7 @@
       </c>
       <c r="O48" s="5" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P48" s="9" t="inlineStr">
@@ -4191,7 +4191,7 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="15" customHeight="1">
+    <row r="49" ht="128" customHeight="1">
       <c r="A49" s="11" t="inlineStr">
         <is>
           <t>Дом Лаврушинский</t>
@@ -4254,7 +4254,7 @@
       </c>
       <c r="O49" s="12" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P49" s="16" t="inlineStr">
@@ -4268,7 +4268,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="15" customHeight="1">
+    <row r="50" ht="128" customHeight="1">
       <c r="A50" s="4" t="inlineStr">
         <is>
           <t>Хамовники 12</t>
@@ -4331,7 +4331,7 @@
       </c>
       <c r="O50" s="5" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P50" s="9" t="inlineStr">
@@ -4345,7 +4345,7 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="15" customHeight="1">
+    <row r="51" ht="153" customHeight="1">
       <c r="A51" s="11" t="inlineStr">
         <is>
           <t>Stella di Mosca Hotel &amp; Residences (Стелла ди Моска Хотел энд Резиденсиз)</t>
@@ -4408,7 +4408,7 @@
       </c>
       <c r="O51" s="12" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P51" s="16" t="inlineStr">
@@ -4422,7 +4422,7 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="24" customHeight="1">
+    <row r="52" ht="140.5" customHeight="1">
       <c r="A52" s="4" t="inlineStr">
         <is>
           <t>Большая Дмитровка IX</t>
@@ -4485,7 +4485,7 @@
       </c>
       <c r="O52" s="5" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P52" s="9" t="inlineStr">
@@ -4499,7 +4499,7 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="15" customHeight="1">
+    <row r="53" ht="128" customHeight="1">
       <c r="A53" s="11" t="inlineStr">
         <is>
           <t>Малая Бронная 15</t>
@@ -4562,7 +4562,7 @@
       </c>
       <c r="O53" s="12" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P53" s="16" t="inlineStr">
@@ -4576,7 +4576,7 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="15" customHeight="1">
+    <row r="54" ht="128" customHeight="1">
       <c r="A54" s="4" t="inlineStr">
         <is>
           <t>Barkli Gallery (Баркли Галлери)</t>
@@ -4639,7 +4639,7 @@
       </c>
       <c r="O54" s="5" t="inlineStr">
         <is>
-          <t>премиум (Циан)</t>
+          <t>премиум</t>
         </is>
       </c>
       <c r="P54" s="9" t="inlineStr">
@@ -4747,22 +4747,22 @@
   <dimension ref="A1:P50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
     <col width="6" customWidth="1" min="7" max="7"/>
     <col width="7" customWidth="1" min="8" max="8"/>
-    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
     <col width="6" customWidth="1" min="13" max="13"/>
     <col width="8" customWidth="1" min="14" max="14"/>
     <col width="7" customWidth="1" min="15" max="15"/>
-    <col width="74" customWidth="1" min="16" max="16"/>
+    <col width="70" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -4861,7 +4861,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="24" customHeight="1">
+    <row r="4" ht="103" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>ЖК «Слава»</t>
@@ -4933,7 +4933,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1">
+    <row r="5" ht="115.5" customHeight="1">
       <c r="A5" s="11" t="inlineStr">
         <is>
           <t>ЖК «Дом Дау»</t>
@@ -5005,7 +5005,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1">
+    <row r="6" ht="115.5" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>ЖК «Начало»</t>
@@ -5077,7 +5077,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1">
+    <row r="7" ht="103" customHeight="1">
       <c r="A7" s="11" t="inlineStr">
         <is>
           <t>Оне</t>
@@ -5149,7 +5149,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1">
+    <row r="8" ht="128" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>АУРУС Резиденции</t>
@@ -5219,7 +5219,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1">
+    <row r="9" ht="115.5" customHeight="1">
       <c r="A9" s="11" t="inlineStr">
         <is>
           <t>ЖК «Монблан»</t>
@@ -5291,7 +5291,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1">
+    <row r="10" ht="128" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>ЖК «Квартал Life Time»</t>
@@ -5363,7 +5363,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1">
+    <row r="11" ht="140.5" customHeight="1">
       <c r="A11" s="11" t="inlineStr">
         <is>
           <t>ЖК «Коллекция Лужники»</t>
@@ -5435,7 +5435,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1">
+    <row r="12" ht="128" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Тессинский V</t>
@@ -5507,7 +5507,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="24" customHeight="1">
+    <row r="13" ht="128" customHeight="1">
       <c r="A13" s="11" t="inlineStr">
         <is>
           <t>Резиденция 1864</t>
@@ -5579,7 +5579,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1">
+    <row r="14" ht="165.5" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
           <t>ЖК «Элитный квартал Тишинский бульвар»</t>
@@ -5651,7 +5651,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="15" customHeight="1">
+    <row r="15" ht="115.5" customHeight="1">
       <c r="A15" s="11" t="inlineStr">
         <is>
           <t>ЖК «Дом Франка»</t>
@@ -5723,7 +5723,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1">
+    <row r="16" ht="128" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
           <t>ЖК «Татарская 35»</t>
@@ -5795,7 +5795,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="15" customHeight="1">
+    <row r="17" ht="153" customHeight="1">
       <c r="A17" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve"> Клубный дом «Резиденции Воронцова»</t>
@@ -5867,7 +5867,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="24" customHeight="1">
+    <row r="18" ht="128" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
           <t>ЖК «Дом Соболева»</t>
@@ -5939,7 +5939,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="24" customHeight="1">
+    <row r="19" ht="128" customHeight="1">
       <c r="A19" s="11" t="inlineStr">
         <is>
           <t>ЖК «Климашкина 7/11»</t>
@@ -6011,7 +6011,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="15" customHeight="1">
+    <row r="20" ht="128" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
           <t>ЖК «Клубный дом Форум»</t>
@@ -6083,7 +6083,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1">
+    <row r="21" ht="115.5" customHeight="1">
       <c r="A21" s="11" t="inlineStr">
         <is>
           <t>ЖК «Камергер»</t>
@@ -6155,7 +6155,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="24" customHeight="1">
+    <row r="22" ht="115.5" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Казачий</t>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="15" customHeight="1">
+    <row r="23" ht="128" customHeight="1">
       <c r="A23" s="11" t="inlineStr">
         <is>
           <t>ЖК «Садовническая 69»</t>
@@ -6299,7 +6299,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="15" customHeight="1">
+    <row r="24" ht="128" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
           <t>Саввинская 17</t>
@@ -6371,7 +6371,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="15" customHeight="1">
+    <row r="25" ht="140.5" customHeight="1">
       <c r="A25" s="11" t="inlineStr">
         <is>
           <t>ЖК «Исторический дом «Чистые Пруды»</t>
@@ -6443,7 +6443,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="15" customHeight="1">
+    <row r="26" ht="115.5" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
         <is>
           <t>ЖК «PHANTOM»</t>
@@ -6515,7 +6515,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="24" customHeight="1">
+    <row r="27" ht="140.5" customHeight="1">
       <c r="A27" s="11" t="inlineStr">
         <is>
           <t>Клубный дом TURGENEV (Тургенев)</t>
@@ -6587,7 +6587,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="15" customHeight="1">
+    <row r="28" ht="140.5" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
         <is>
           <t>Фамильный дом Люче</t>
@@ -6659,7 +6659,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="15" customHeight="1">
+    <row r="29" ht="115.5" customHeight="1">
       <c r="A29" s="11" t="inlineStr">
         <is>
           <t>Кло 17</t>
@@ -6731,7 +6731,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="15" customHeight="1">
+    <row r="30" ht="128" customHeight="1">
       <c r="A30" s="4" t="inlineStr">
         <is>
           <t>ТИТУЛ Империал</t>
@@ -6803,7 +6803,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="15" customHeight="1">
+    <row r="31" ht="128" customHeight="1">
       <c r="A31" s="11" t="inlineStr">
         <is>
           <t>Клубный дом DUO (Дуо)</t>
@@ -6875,7 +6875,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="15" customHeight="1">
+    <row r="32" ht="115.5" customHeight="1">
       <c r="A32" s="4" t="inlineStr">
         <is>
           <t>Дом Спорта</t>
@@ -6947,7 +6947,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="15" customHeight="1">
+    <row r="33" ht="165.5" customHeight="1">
       <c r="A33" s="11" t="inlineStr">
         <is>
           <t>«Ильинка 3/8»</t>
@@ -7019,7 +7019,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="15" customHeight="1">
+    <row r="34" ht="128" customHeight="1">
       <c r="A34" s="4" t="inlineStr">
         <is>
           <t>ЖК «Красный Октябрь»</t>
@@ -7091,7 +7091,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="15" customHeight="1">
+    <row r="35" ht="115.5" customHeight="1">
       <c r="A35" s="11" t="inlineStr">
         <is>
           <t>ЖК «Николь»</t>
@@ -7163,7 +7163,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="15" customHeight="1">
+    <row r="36" ht="115.5" customHeight="1">
       <c r="A36" s="4" t="inlineStr">
         <is>
           <t>MONO Kami</t>
@@ -7235,7 +7235,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="15" customHeight="1">
+    <row r="37" ht="115.5" customHeight="1">
       <c r="A37" s="11" t="inlineStr">
         <is>
           <t>ЖК «Никитский-6»</t>
@@ -7307,7 +7307,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="15" customHeight="1">
+    <row r="38" ht="153" customHeight="1">
       <c r="A38" s="4" t="inlineStr">
         <is>
           <t>ЖК «Фрунзенская набережная»</t>
@@ -7379,7 +7379,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="24" customHeight="1">
+    <row r="39" ht="153" customHeight="1">
       <c r="A39" s="11" t="inlineStr">
         <is>
           <t>Kuznetsky Most 12 by Lalique (Кузнецкий Мост 12)</t>
@@ -7451,7 +7451,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="24" customHeight="1">
+    <row r="40" ht="128" customHeight="1">
       <c r="A40" s="4" t="inlineStr">
         <is>
           <t>Саввинская 27</t>
@@ -7523,7 +7523,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="15" customHeight="1">
+    <row r="41" ht="115.5" customHeight="1">
       <c r="A41" s="11" t="inlineStr">
         <is>
           <t>ДОМ XXII</t>
@@ -7595,7 +7595,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="15" customHeight="1">
+    <row r="42" ht="128" customHeight="1">
       <c r="A42" s="4" t="inlineStr">
         <is>
           <t>Stoleshnikov 7 (Столешников 7)</t>
@@ -7667,7 +7667,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="15" customHeight="1">
+    <row r="43" ht="115.5" customHeight="1">
       <c r="A43" s="11" t="inlineStr">
         <is>
           <t>ЖК «Узоры»</t>
@@ -7739,7 +7739,7 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="15" customHeight="1">
+    <row r="44" ht="115.5" customHeight="1">
       <c r="A44" s="4" t="inlineStr">
         <is>
           <t>Annabels</t>
@@ -7811,7 +7811,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="15" customHeight="1">
+    <row r="45" ht="140.5" customHeight="1">
       <c r="A45" s="11" t="inlineStr">
         <is>
           <t>ЖК «Клубный дом Левенсон»</t>
@@ -7883,7 +7883,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="15" customHeight="1">
+    <row r="46" ht="153" customHeight="1">
       <c r="A46" s="4" t="inlineStr">
         <is>
           <t>Armani/Casa Moscow Residences (Армани/Каса Москоу Резиденсес)</t>
@@ -7955,7 +7955,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="15" customHeight="1">
+    <row r="47" ht="140.5" customHeight="1">
       <c r="A47" s="11" t="inlineStr">
         <is>
           <t>ЖК «Погодинская»</t>
@@ -8027,7 +8027,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="15" customHeight="1">
+    <row r="48" ht="140.5" customHeight="1">
       <c r="A48" s="4" t="inlineStr">
         <is>
           <t>ЖК «Клубный дом Обыденский №1»</t>
@@ -8099,7 +8099,7 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="15" customHeight="1">
+    <row r="49" ht="115.5" customHeight="1">
       <c r="A49" s="11" t="inlineStr">
         <is>
           <t>Лё Дом</t>
@@ -8171,7 +8171,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="15" customHeight="1">
+    <row r="50" ht="115.5" customHeight="1">
       <c r="A50" s="4" t="inlineStr">
         <is>
           <t>ЖК «БРЮСОВ»</t>
@@ -8333,22 +8333,22 @@
   <dimension ref="A1:P32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
     <col width="10" customWidth="1" min="13" max="13"/>
     <col width="10" customWidth="1" min="14" max="14"/>
     <col width="7" customWidth="1" min="15" max="15"/>
-    <col width="74" customWidth="1" min="16" max="16"/>
+    <col width="70" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -8447,7 +8447,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="24" customHeight="1">
+    <row r="4" ht="90.5" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Лёвшинский, 19</t>
@@ -8511,7 +8511,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="24" customHeight="1">
+    <row r="5" ht="215.5" customHeight="1">
       <c r="A5" s="11" t="inlineStr">
         <is>
           <t>Клубный дом «Малая Никитская, 27»</t>
@@ -8567,7 +8567,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="24" customHeight="1">
+    <row r="6" ht="128" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Палашёвский 11 (Большой Палашёвский, 11–13/15)</t>
@@ -8639,7 +8639,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="24" customHeight="1">
+    <row r="7" ht="115.5" customHeight="1">
       <c r="A7" s="11" t="inlineStr">
         <is>
           <t>EDEN Private Residence</t>
@@ -8713,7 +8713,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="24" customHeight="1">
+    <row r="8" ht="103" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Большая Ордынка, 25</t>
@@ -8777,7 +8777,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="24" customHeight="1">
+    <row r="9" ht="103" customHeight="1">
       <c r="A9" s="11" t="inlineStr">
         <is>
           <t>Большая Пироговская, 51 (общежития Института красной профессуры)</t>
@@ -8837,7 +8837,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="24" customHeight="1">
+    <row r="10" ht="153" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Большой Козихинский, 22</t>
@@ -8897,7 +8897,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="24" customHeight="1">
+    <row r="11" ht="65.5" customHeight="1">
       <c r="A11" s="11" t="inlineStr">
         <is>
           <t>Воздвиженка 7/6</t>
@@ -8951,7 +8951,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="24" customHeight="1">
+    <row r="12" ht="103" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Квартал на Савинской набережной («Московский шёлк»)</t>
@@ -9011,7 +9011,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="24" customHeight="1">
+    <row r="13" ht="178" customHeight="1">
       <c r="A13" s="11" t="inlineStr">
         <is>
           <t>Клубные дома на Берниковской набережной, 12 (Sminex)</t>
@@ -9075,7 +9075,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="24" customHeight="1">
+    <row r="14" ht="153" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Клубный дом «Большая Никитская, 16» (R4S)</t>
@@ -9141,7 +9141,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="24" customHeight="1">
+    <row r="15" ht="115.5" customHeight="1">
       <c r="A15" s="11" t="inlineStr">
         <is>
           <t>Клубный дом «Земледельческий, 15»</t>
@@ -9203,7 +9203,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="24" customHeight="1">
+    <row r="16" ht="78" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Клубный дом на Курсовом переулке, 15 (проект бюро Дмитрия Великовского)</t>
@@ -9255,7 +9255,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="24" customHeight="1">
+    <row r="17" ht="228" customHeight="1">
       <c r="A17" s="11" t="inlineStr">
         <is>
           <t>Льва Толстого, 14–16 (три клубных дома Sminex)</t>
@@ -9313,7 +9313,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="24" customHeight="1">
+    <row r="18" ht="140.5" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
           <t>МФК «На Краснопресненской набережной» (Трёхгорная мануфактура)</t>
@@ -9373,7 +9373,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="24" customHeight="1">
+    <row r="19" ht="115.5" customHeight="1">
       <c r="A19" s="11" t="inlineStr">
         <is>
           <t>Малая Дмитровка, 5/9</t>
@@ -9433,7 +9433,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="24" customHeight="1">
+    <row r="20" ht="53" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Малая Никитская, 29–31 (ожидаемый делюкс-старт)</t>
@@ -9483,7 +9483,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="24" customHeight="1">
+    <row r="21" ht="140.5" customHeight="1">
       <c r="A21" s="11" t="inlineStr">
         <is>
           <t>Малая Ордынка, 14/1</t>
@@ -9549,7 +9549,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="24" customHeight="1">
+    <row r="22" ht="53" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Олсуфьевский 10</t>
@@ -9607,7 +9607,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="24" customHeight="1">
+    <row r="23" ht="53" customHeight="1">
       <c r="A23" s="11" t="inlineStr">
         <is>
           <t>Полянка-3</t>
@@ -9665,7 +9665,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="24" customHeight="1">
+    <row r="24" ht="103" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
           <t>Премиальный квартал на Лужнецкой набережной, 10А</t>
@@ -9727,7 +9727,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="24" customHeight="1">
+    <row r="25" ht="165.5" customHeight="1">
       <c r="A25" s="11" t="inlineStr">
         <is>
           <t>Роден (ранее анонсировался как Veil)</t>
@@ -9787,7 +9787,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="24" customHeight="1">
+    <row r="26" ht="228" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
         <is>
           <t>Рождественка 8</t>
@@ -9853,7 +9853,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="24" customHeight="1">
+    <row r="27" ht="103" customHeight="1">
       <c r="A27" s="11" t="inlineStr">
         <is>
           <t>Тимура Фрунзе, 11 (клубный дом Sminex)</t>
@@ -9911,7 +9911,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="24" customHeight="1">
+    <row r="28" ht="115.5" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
         <is>
           <t>Типография Сытина (Пятницкая, 71/5)</t>
@@ -9965,7 +9965,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="24" customHeight="1">
+    <row r="29" ht="240.5" customHeight="1">
       <c r="A29" s="11" t="inlineStr">
         <is>
           <t>Усадьба в Большом Саввинском переулке (клубный дом VSF)</t>
@@ -10027,7 +10027,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="24" customHeight="1">
+    <row r="30" ht="128" customHeight="1">
       <c r="A30" s="4" t="inlineStr">
         <is>
           <t>Усачёва, 22</t>
@@ -10089,7 +10089,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="24" customHeight="1">
+    <row r="31" ht="65.5" customHeight="1">
       <c r="A31" s="11" t="inlineStr">
         <is>
           <t>Участок КРТ «Большой Тишинский переулок, 8»</t>
@@ -10147,7 +10147,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="24" customHeight="1">
+    <row r="32" ht="90.5" customHeight="1">
       <c r="A32" s="4" t="inlineStr">
         <is>
           <t>Хилков (Хилков переулок, вл. 3)</t>

</xml_diff>

<commit_message>
Workbook: ignore link cells when sizing rows
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Bv8NELxW2W7udnb3XUFGS2
</commit_message>
<xml_diff>
--- a/docs/premium-cao/premium-zhk-cao.xlsx
+++ b/docs/premium-cao/premium-zhk-cao.xlsx
@@ -726,7 +726,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="140.5" customHeight="1">
+    <row r="4" ht="28" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Резиденция Тверская</t>
@@ -803,7 +803,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="115.5" customHeight="1">
+    <row r="5" ht="28" customHeight="1">
       <c r="A5" s="11" t="inlineStr">
         <is>
           <t>NEVA TOWERS (Нева Тауэрс)</t>
@@ -880,7 +880,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="115.5" customHeight="1">
+    <row r="6" ht="28" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Sinatra (Синатра)</t>
@@ -957,7 +957,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="115.5" customHeight="1">
+    <row r="7" ht="28" customHeight="1">
       <c r="A7" s="11" t="inlineStr">
         <is>
           <t>LUMIN (ЛЮМИН)</t>
@@ -1034,7 +1034,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="115.5" customHeight="1">
+    <row r="8" ht="15" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Уланский, 13</t>
@@ -1111,7 +1111,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="115.5" customHeight="1">
+    <row r="9" ht="28" customHeight="1">
       <c r="A9" s="11" t="inlineStr">
         <is>
           <t>Современник</t>
@@ -1188,7 +1188,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="115.5" customHeight="1">
+    <row r="10" ht="28" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Репаблик</t>
@@ -1265,7 +1265,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="115.5" customHeight="1">
+    <row r="11" ht="28" customHeight="1">
       <c r="A11" s="11" t="inlineStr">
         <is>
           <t>City Park (Сити Парк)</t>
@@ -1342,7 +1342,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="115.5" customHeight="1">
+    <row r="12" ht="28" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t>SkyView</t>
@@ -1419,7 +1419,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="115.5" customHeight="1">
+    <row r="13" ht="28" customHeight="1">
       <c r="A13" s="11" t="inlineStr">
         <is>
           <t>Полянка/44</t>
@@ -1496,7 +1496,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="140.5" customHeight="1">
+    <row r="14" ht="28" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Титул на Серебрянической</t>
@@ -1573,7 +1573,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="115.5" customHeight="1">
+    <row r="15" ht="28" customHeight="1">
       <c r="A15" s="11" t="inlineStr">
         <is>
           <t>Bogenhouse (Богенхаус)</t>
@@ -1650,7 +1650,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="128" customHeight="1">
+    <row r="16" ht="28" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Capital Towers (Капитал Тауэрс)</t>
@@ -1727,7 +1727,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="128" customHeight="1">
+    <row r="17" ht="28" customHeight="1">
       <c r="A17" s="11" t="inlineStr">
         <is>
           <t>BALCHUG VIEWPOINT (Балчуг Вьюпоинт)</t>
@@ -1804,7 +1804,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="128" customHeight="1">
+    <row r="18" ht="15" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Титул на Якиманке</t>
@@ -1881,7 +1881,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="128" customHeight="1">
+    <row r="19" ht="15" customHeight="1">
       <c r="A19" s="11" t="inlineStr">
         <is>
           <t>Клубный дом ЦВЕТ32</t>
@@ -1958,7 +1958,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="115.5" customHeight="1">
+    <row r="20" ht="28" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
           <t>A.Residence (А Резиденс)</t>
@@ -2035,7 +2035,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="115.5" customHeight="1">
+    <row r="21" ht="28" customHeight="1">
       <c r="A21" s="11" t="inlineStr">
         <is>
           <t>Roza Rossa (Роза Росса)</t>
@@ -2112,7 +2112,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="153" customHeight="1">
+    <row r="22" ht="28" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Собрание клубных домов ORDYNKA (Ордынка)</t>
@@ -2189,7 +2189,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="115.5" customHeight="1">
+    <row r="23" ht="28" customHeight="1">
       <c r="A23" s="11" t="inlineStr">
         <is>
           <t>Дом NV/9</t>
@@ -2266,7 +2266,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="128" customHeight="1">
+    <row r="24" ht="28" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
           <t>Fantastic House (Фантастик Хаус)</t>
@@ -2343,7 +2343,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="140.5" customHeight="1">
+    <row r="25" ht="28" customHeight="1">
       <c r="A25" s="11" t="inlineStr">
         <is>
           <t>Клубный дом Космо 4/22</t>
@@ -2420,7 +2420,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="115.5" customHeight="1">
+    <row r="26" ht="28" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
         <is>
           <t>Софийский</t>
@@ -2497,7 +2497,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="128" customHeight="1">
+    <row r="27" ht="15" customHeight="1">
       <c r="A27" s="11" t="inlineStr">
         <is>
           <t>Дом на Тишинке</t>
@@ -2574,7 +2574,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="128" customHeight="1">
+    <row r="28" ht="15" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
         <is>
           <t>Тессинский, 1</t>
@@ -2651,7 +2651,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="103" customHeight="1">
+    <row r="29" ht="28" customHeight="1">
       <c r="A29" s="11" t="inlineStr">
         <is>
           <t>Lucky (Лаки)</t>
@@ -2728,7 +2728,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="115.5" customHeight="1">
+    <row r="30" ht="15" customHeight="1">
       <c r="A30" s="4" t="inlineStr">
         <is>
           <t>Artisan (Артисан)</t>
@@ -2805,7 +2805,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="115.5" customHeight="1">
+    <row r="31" ht="28" customHeight="1">
       <c r="A31" s="11" t="inlineStr">
         <is>
           <t>Абрикосов</t>
@@ -2882,7 +2882,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="128" customHeight="1">
+    <row r="32" ht="28" customHeight="1">
       <c r="A32" s="4" t="inlineStr">
         <is>
           <t>Клубный дом CULT (Клубный дом Культ)</t>
@@ -2959,7 +2959,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="140.5" customHeight="1">
+    <row r="33" ht="28" customHeight="1">
       <c r="A33" s="11" t="inlineStr">
         <is>
           <t>SAVVIN RIVER RESIDENCE (Саввин Ривер Резиденс)</t>
@@ -3036,7 +3036,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="128" customHeight="1">
+    <row r="34" ht="28" customHeight="1">
       <c r="A34" s="4" t="inlineStr">
         <is>
           <t>Пироговская 14</t>
@@ -3113,7 +3113,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="115.5" customHeight="1">
+    <row r="35" ht="28" customHeight="1">
       <c r="A35" s="11" t="inlineStr">
         <is>
           <t>Cloud Nine (Клауд Найн)</t>
@@ -3190,7 +3190,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="140.5" customHeight="1">
+    <row r="36" ht="28" customHeight="1">
       <c r="A36" s="4" t="inlineStr">
         <is>
           <t>Симфония набережных (Котельническая 21)</t>
@@ -3267,7 +3267,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="128" customHeight="1">
+    <row r="37" ht="28" customHeight="1">
       <c r="A37" s="11" t="inlineStr">
         <is>
           <t>Садовые кварталы</t>
@@ -3344,7 +3344,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="128" customHeight="1">
+    <row r="38" ht="28" customHeight="1">
       <c r="A38" s="4" t="inlineStr">
         <is>
           <t>Малая Ордынка 19</t>
@@ -3421,7 +3421,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="128" customHeight="1">
+    <row r="39" ht="15" customHeight="1">
       <c r="A39" s="11" t="inlineStr">
         <is>
           <t>Дом в Газетном</t>
@@ -3498,7 +3498,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="128" customHeight="1">
+    <row r="40" ht="28" customHeight="1">
       <c r="A40" s="4" t="inlineStr">
         <is>
           <t>Zvonarsky Deluxe (Звонарский Делюкс)</t>
@@ -3575,7 +3575,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="128" customHeight="1">
+    <row r="41" ht="28" customHeight="1">
       <c r="A41" s="11" t="inlineStr">
         <is>
           <t>White Khamovniki (Вайт Хамовники)</t>
@@ -3652,7 +3652,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="140.5" customHeight="1">
+    <row r="42" ht="28" customHeight="1">
       <c r="A42" s="4" t="inlineStr">
         <is>
           <t>Золотой, жилой квартал</t>
@@ -3729,7 +3729,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="103" customHeight="1">
+    <row r="43" ht="28" customHeight="1">
       <c r="A43" s="11" t="inlineStr">
         <is>
           <t>Magnum (Магнум)</t>
@@ -3806,7 +3806,7 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="140.5" customHeight="1">
+    <row r="44" ht="28" customHeight="1">
       <c r="A44" s="4" t="inlineStr">
         <is>
           <t>Дом Бакст на Патриарших</t>
@@ -3883,7 +3883,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="115.5" customHeight="1">
+    <row r="45" ht="28" customHeight="1">
       <c r="A45" s="11" t="inlineStr">
         <is>
           <t>Villa Grace (Вилла Грейс)</t>
@@ -3960,7 +3960,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="115.5" customHeight="1">
+    <row r="46" ht="28" customHeight="1">
       <c r="A46" s="4" t="inlineStr">
         <is>
           <t>Brodsky (Бродский)</t>
@@ -4037,7 +4037,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="128" customHeight="1">
+    <row r="47" ht="15" customHeight="1">
       <c r="A47" s="11" t="inlineStr">
         <is>
           <t>Жизнь на Плющихе</t>
@@ -4114,7 +4114,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="115.5" customHeight="1">
+    <row r="48" ht="28" customHeight="1">
       <c r="A48" s="4" t="inlineStr">
         <is>
           <t>Carré Blanc (Карре Бланк)</t>
@@ -4191,7 +4191,7 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="128" customHeight="1">
+    <row r="49" ht="28" customHeight="1">
       <c r="A49" s="11" t="inlineStr">
         <is>
           <t>Дом Лаврушинский</t>
@@ -4268,7 +4268,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="128" customHeight="1">
+    <row r="50" ht="28" customHeight="1">
       <c r="A50" s="4" t="inlineStr">
         <is>
           <t>Хамовники 12</t>
@@ -4345,7 +4345,7 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="153" customHeight="1">
+    <row r="51" ht="40.5" customHeight="1">
       <c r="A51" s="11" t="inlineStr">
         <is>
           <t>Stella di Mosca Hotel &amp; Residences (Стелла ди Моска Хотел энд Резиденсиз)</t>
@@ -4422,7 +4422,7 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="140.5" customHeight="1">
+    <row r="52" ht="28" customHeight="1">
       <c r="A52" s="4" t="inlineStr">
         <is>
           <t>Большая Дмитровка IX</t>
@@ -4499,7 +4499,7 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="128" customHeight="1">
+    <row r="53" ht="15" customHeight="1">
       <c r="A53" s="11" t="inlineStr">
         <is>
           <t>Малая Бронная 15</t>
@@ -4576,7 +4576,7 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="128" customHeight="1">
+    <row r="54" ht="28" customHeight="1">
       <c r="A54" s="4" t="inlineStr">
         <is>
           <t>Barkli Gallery (Баркли Галлери)</t>
@@ -4861,7 +4861,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="103" customHeight="1">
+    <row r="4" ht="28" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>ЖК «Слава»</t>
@@ -4933,7 +4933,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="115.5" customHeight="1">
+    <row r="5" ht="28" customHeight="1">
       <c r="A5" s="11" t="inlineStr">
         <is>
           <t>ЖК «Дом Дау»</t>
@@ -5005,7 +5005,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="115.5" customHeight="1">
+    <row r="6" ht="28" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>ЖК «Начало»</t>
@@ -5077,7 +5077,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="103" customHeight="1">
+    <row r="7" ht="28" customHeight="1">
       <c r="A7" s="11" t="inlineStr">
         <is>
           <t>Оне</t>
@@ -5149,7 +5149,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="128" customHeight="1">
+    <row r="8" ht="28" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>АУРУС Резиденции</t>
@@ -5219,7 +5219,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="115.5" customHeight="1">
+    <row r="9" ht="15" customHeight="1">
       <c r="A9" s="11" t="inlineStr">
         <is>
           <t>ЖК «Монблан»</t>
@@ -5291,7 +5291,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="128" customHeight="1">
+    <row r="10" ht="40.5" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>ЖК «Квартал Life Time»</t>
@@ -5363,7 +5363,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="140.5" customHeight="1">
+    <row r="11" ht="15" customHeight="1">
       <c r="A11" s="11" t="inlineStr">
         <is>
           <t>ЖК «Коллекция Лужники»</t>
@@ -5435,7 +5435,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="128" customHeight="1">
+    <row r="12" ht="28" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Тессинский V</t>
@@ -5507,7 +5507,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="128" customHeight="1">
+    <row r="13" ht="40.5" customHeight="1">
       <c r="A13" s="11" t="inlineStr">
         <is>
           <t>Резиденция 1864</t>
@@ -5579,7 +5579,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="165.5" customHeight="1">
+    <row r="14" ht="28" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
           <t>ЖК «Элитный квартал Тишинский бульвар»</t>
@@ -5651,7 +5651,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="115.5" customHeight="1">
+    <row r="15" ht="40.5" customHeight="1">
       <c r="A15" s="11" t="inlineStr">
         <is>
           <t>ЖК «Дом Франка»</t>
@@ -5723,7 +5723,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="128" customHeight="1">
+    <row r="16" ht="28" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
           <t>ЖК «Татарская 35»</t>
@@ -5795,7 +5795,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="153" customHeight="1">
+    <row r="17" ht="28" customHeight="1">
       <c r="A17" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve"> Клубный дом «Резиденции Воронцова»</t>
@@ -5867,7 +5867,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="128" customHeight="1">
+    <row r="18" ht="28" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
           <t>ЖК «Дом Соболева»</t>
@@ -5939,7 +5939,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="128" customHeight="1">
+    <row r="19" ht="28" customHeight="1">
       <c r="A19" s="11" t="inlineStr">
         <is>
           <t>ЖК «Климашкина 7/11»</t>
@@ -6011,7 +6011,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="128" customHeight="1">
+    <row r="20" ht="40.5" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
           <t>ЖК «Клубный дом Форум»</t>
@@ -6083,7 +6083,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="115.5" customHeight="1">
+    <row r="21" ht="28" customHeight="1">
       <c r="A21" s="11" t="inlineStr">
         <is>
           <t>ЖК «Камергер»</t>
@@ -6155,7 +6155,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="115.5" customHeight="1">
+    <row r="22" ht="28" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Казачий</t>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="128" customHeight="1">
+    <row r="23" ht="28" customHeight="1">
       <c r="A23" s="11" t="inlineStr">
         <is>
           <t>ЖК «Садовническая 69»</t>
@@ -6299,7 +6299,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="128" customHeight="1">
+    <row r="24" ht="28" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
           <t>Саввинская 17</t>
@@ -6371,7 +6371,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="140.5" customHeight="1">
+    <row r="25" ht="28" customHeight="1">
       <c r="A25" s="11" t="inlineStr">
         <is>
           <t>ЖК «Исторический дом «Чистые Пруды»</t>
@@ -6443,7 +6443,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="115.5" customHeight="1">
+    <row r="26" ht="28" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
         <is>
           <t>ЖК «PHANTOM»</t>
@@ -6515,7 +6515,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="140.5" customHeight="1">
+    <row r="27" ht="28" customHeight="1">
       <c r="A27" s="11" t="inlineStr">
         <is>
           <t>Клубный дом TURGENEV (Тургенев)</t>
@@ -6587,7 +6587,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="140.5" customHeight="1">
+    <row r="28" ht="28" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
         <is>
           <t>Фамильный дом Люче</t>
@@ -6659,7 +6659,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="115.5" customHeight="1">
+    <row r="29" ht="28" customHeight="1">
       <c r="A29" s="11" t="inlineStr">
         <is>
           <t>Кло 17</t>
@@ -6731,7 +6731,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="128" customHeight="1">
+    <row r="30" ht="28" customHeight="1">
       <c r="A30" s="4" t="inlineStr">
         <is>
           <t>ТИТУЛ Империал</t>
@@ -6803,7 +6803,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="128" customHeight="1">
+    <row r="31" ht="15" customHeight="1">
       <c r="A31" s="11" t="inlineStr">
         <is>
           <t>Клубный дом DUO (Дуо)</t>
@@ -6875,7 +6875,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="115.5" customHeight="1">
+    <row r="32" ht="28" customHeight="1">
       <c r="A32" s="4" t="inlineStr">
         <is>
           <t>Дом Спорта</t>
@@ -6947,7 +6947,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="165.5" customHeight="1">
+    <row r="33" ht="40.5" customHeight="1">
       <c r="A33" s="11" t="inlineStr">
         <is>
           <t>«Ильинка 3/8»</t>
@@ -7019,7 +7019,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="128" customHeight="1">
+    <row r="34" ht="28" customHeight="1">
       <c r="A34" s="4" t="inlineStr">
         <is>
           <t>ЖК «Красный Октябрь»</t>
@@ -7091,7 +7091,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="115.5" customHeight="1">
+    <row r="35" ht="28" customHeight="1">
       <c r="A35" s="11" t="inlineStr">
         <is>
           <t>ЖК «Николь»</t>
@@ -7163,7 +7163,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="115.5" customHeight="1">
+    <row r="36" ht="40.5" customHeight="1">
       <c r="A36" s="4" t="inlineStr">
         <is>
           <t>MONO Kami</t>
@@ -7235,7 +7235,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="115.5" customHeight="1">
+    <row r="37" ht="28" customHeight="1">
       <c r="A37" s="11" t="inlineStr">
         <is>
           <t>ЖК «Никитский-6»</t>
@@ -7307,7 +7307,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="153" customHeight="1">
+    <row r="38" ht="28" customHeight="1">
       <c r="A38" s="4" t="inlineStr">
         <is>
           <t>ЖК «Фрунзенская набережная»</t>
@@ -7379,7 +7379,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="153" customHeight="1">
+    <row r="39" ht="28" customHeight="1">
       <c r="A39" s="11" t="inlineStr">
         <is>
           <t>Kuznetsky Most 12 by Lalique (Кузнецкий Мост 12)</t>
@@ -7451,7 +7451,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="128" customHeight="1">
+    <row r="40" ht="28" customHeight="1">
       <c r="A40" s="4" t="inlineStr">
         <is>
           <t>Саввинская 27</t>
@@ -7523,7 +7523,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="115.5" customHeight="1">
+    <row r="41" ht="15" customHeight="1">
       <c r="A41" s="11" t="inlineStr">
         <is>
           <t>ДОМ XXII</t>
@@ -7595,7 +7595,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="128" customHeight="1">
+    <row r="42" ht="28" customHeight="1">
       <c r="A42" s="4" t="inlineStr">
         <is>
           <t>Stoleshnikov 7 (Столешников 7)</t>
@@ -7667,7 +7667,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="115.5" customHeight="1">
+    <row r="43" ht="28" customHeight="1">
       <c r="A43" s="11" t="inlineStr">
         <is>
           <t>ЖК «Узоры»</t>
@@ -7739,7 +7739,7 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="115.5" customHeight="1">
+    <row r="44" ht="40.5" customHeight="1">
       <c r="A44" s="4" t="inlineStr">
         <is>
           <t>Annabels</t>
@@ -7811,7 +7811,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="140.5" customHeight="1">
+    <row r="45" ht="15" customHeight="1">
       <c r="A45" s="11" t="inlineStr">
         <is>
           <t>ЖК «Клубный дом Левенсон»</t>
@@ -7883,7 +7883,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="153" customHeight="1">
+    <row r="46" ht="40.5" customHeight="1">
       <c r="A46" s="4" t="inlineStr">
         <is>
           <t>Armani/Casa Moscow Residences (Армани/Каса Москоу Резиденсес)</t>
@@ -7955,7 +7955,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="140.5" customHeight="1">
+    <row r="47" ht="15" customHeight="1">
       <c r="A47" s="11" t="inlineStr">
         <is>
           <t>ЖК «Погодинская»</t>
@@ -8027,7 +8027,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="140.5" customHeight="1">
+    <row r="48" ht="40.5" customHeight="1">
       <c r="A48" s="4" t="inlineStr">
         <is>
           <t>ЖК «Клубный дом Обыденский №1»</t>
@@ -8099,7 +8099,7 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="115.5" customHeight="1">
+    <row r="49" ht="15" customHeight="1">
       <c r="A49" s="11" t="inlineStr">
         <is>
           <t>Лё Дом</t>
@@ -8171,7 +8171,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="115.5" customHeight="1">
+    <row r="50" ht="40.5" customHeight="1">
       <c r="A50" s="4" t="inlineStr">
         <is>
           <t>ЖК «БРЮСОВ»</t>
@@ -8447,7 +8447,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="90.5" customHeight="1">
+    <row r="4" ht="53" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Лёвшинский, 19</t>
@@ -8511,7 +8511,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="215.5" customHeight="1">
+    <row r="5" ht="53" customHeight="1">
       <c r="A5" s="11" t="inlineStr">
         <is>
           <t>Клубный дом «Малая Никитская, 27»</t>
@@ -8567,7 +8567,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="128" customHeight="1">
+    <row r="6" ht="65.5" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Палашёвский 11 (Большой Палашёвский, 11–13/15)</t>
@@ -8639,7 +8639,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="115.5" customHeight="1">
+    <row r="7" ht="65.5" customHeight="1">
       <c r="A7" s="11" t="inlineStr">
         <is>
           <t>EDEN Private Residence</t>
@@ -8713,7 +8713,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="103" customHeight="1">
+    <row r="8" ht="65.5" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Большая Ордынка, 25</t>
@@ -8777,7 +8777,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="103" customHeight="1">
+    <row r="9" ht="65.5" customHeight="1">
       <c r="A9" s="11" t="inlineStr">
         <is>
           <t>Большая Пироговская, 51 (общежития Института красной профессуры)</t>
@@ -8837,7 +8837,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="153" customHeight="1">
+    <row r="10" ht="40.5" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Большой Козихинский, 22</t>
@@ -8951,7 +8951,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="103" customHeight="1">
+    <row r="12" ht="65.5" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Квартал на Савинской набережной («Московский шёлк»)</t>
@@ -9011,7 +9011,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="178" customHeight="1">
+    <row r="13" ht="53" customHeight="1">
       <c r="A13" s="11" t="inlineStr">
         <is>
           <t>Клубные дома на Берниковской набережной, 12 (Sminex)</t>
@@ -9075,7 +9075,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="153" customHeight="1">
+    <row r="14" ht="65.5" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Клубный дом «Большая Никитская, 16» (R4S)</t>
@@ -9141,7 +9141,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="115.5" customHeight="1">
+    <row r="15" ht="65.5" customHeight="1">
       <c r="A15" s="11" t="inlineStr">
         <is>
           <t>Клубный дом «Земледельческий, 15»</t>
@@ -9203,7 +9203,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="78" customHeight="1">
+    <row r="16" ht="53" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Клубный дом на Курсовом переулке, 15 (проект бюро Дмитрия Великовского)</t>
@@ -9255,7 +9255,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="228" customHeight="1">
+    <row r="17" ht="53" customHeight="1">
       <c r="A17" s="11" t="inlineStr">
         <is>
           <t>Льва Толстого, 14–16 (три клубных дома Sminex)</t>
@@ -9313,7 +9313,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="140.5" customHeight="1">
+    <row r="18" ht="53" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
           <t>МФК «На Краснопресненской набережной» (Трёхгорная мануфактура)</t>
@@ -9373,7 +9373,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="115.5" customHeight="1">
+    <row r="19" ht="40.5" customHeight="1">
       <c r="A19" s="11" t="inlineStr">
         <is>
           <t>Малая Дмитровка, 5/9</t>
@@ -9483,7 +9483,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="140.5" customHeight="1">
+    <row r="21" ht="53" customHeight="1">
       <c r="A21" s="11" t="inlineStr">
         <is>
           <t>Малая Ордынка, 14/1</t>
@@ -9665,7 +9665,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="103" customHeight="1">
+    <row r="24" ht="78" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
           <t>Премиальный квартал на Лужнецкой набережной, 10А</t>
@@ -9727,7 +9727,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="165.5" customHeight="1">
+    <row r="25" ht="65.5" customHeight="1">
       <c r="A25" s="11" t="inlineStr">
         <is>
           <t>Роден (ранее анонсировался как Veil)</t>
@@ -9787,7 +9787,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="228" customHeight="1">
+    <row r="26" ht="65.5" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
         <is>
           <t>Рождественка 8</t>
@@ -9853,7 +9853,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="103" customHeight="1">
+    <row r="27" ht="53" customHeight="1">
       <c r="A27" s="11" t="inlineStr">
         <is>
           <t>Тимура Фрунзе, 11 (клубный дом Sminex)</t>
@@ -9911,7 +9911,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="115.5" customHeight="1">
+    <row r="28" ht="53" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
         <is>
           <t>Типография Сытина (Пятницкая, 71/5)</t>
@@ -9965,7 +9965,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="240.5" customHeight="1">
+    <row r="29" ht="78" customHeight="1">
       <c r="A29" s="11" t="inlineStr">
         <is>
           <t>Усадьба в Большом Саввинском переулке (клубный дом VSF)</t>
@@ -10027,7 +10027,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="128" customHeight="1">
+    <row r="30" ht="53" customHeight="1">
       <c r="A30" s="4" t="inlineStr">
         <is>
           <t>Усачёва, 22</t>

</xml_diff>

<commit_message>
Workbook: one-line cells where possible, rows sized to wrapped text
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Bv8NELxW2W7udnb3XUFGS2
</commit_message>
<xml_diff>
--- a/docs/premium-cao/premium-zhk-cao.xlsx
+++ b/docs/premium-cao/premium-zhk-cao.xlsx
@@ -606,10 +606,10 @@
   <dimension ref="A1:Q54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
     <col width="6" customWidth="1" min="7" max="7"/>
@@ -622,7 +622,7 @@
     <col width="9" customWidth="1" min="14" max="14"/>
     <col width="10" customWidth="1" min="15" max="15"/>
     <col width="7" customWidth="1" min="16" max="16"/>
-    <col width="70" customWidth="1" min="17" max="17"/>
+    <col width="84" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -726,7 +726,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="28" customHeight="1">
+    <row r="4" ht="15" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Резиденция Тверская</t>
@@ -734,7 +734,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Kovaks (Ковакс)</t>
+          <t>Kovaks</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
@@ -744,7 +744,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Москва, 2-я Брестская, 6</t>
+          <t>2-я Брестская, 6</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -806,7 +806,7 @@
     <row r="5" ht="28" customHeight="1">
       <c r="A5" s="11" t="inlineStr">
         <is>
-          <t>NEVA TOWERS (Нева Тауэрс)</t>
+          <t>NEVA TOWERS</t>
         </is>
       </c>
       <c r="B5" s="11" t="inlineStr">
@@ -821,7 +821,7 @@
       </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t>Москва, 1-й Красногвардейский, 22с2</t>
+          <t>1-й Красногвардейский, 22с2</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
@@ -880,10 +880,10 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="28" customHeight="1">
+    <row r="6" ht="15" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Sinatra (Синатра)</t>
+          <t>Sinatra</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -898,7 +898,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Москва, Большой Тишинский, 38</t>
+          <t>Большой Тишинский, 38</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -957,10 +957,10 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="28" customHeight="1">
+    <row r="7" ht="15" customHeight="1">
       <c r="A7" s="11" t="inlineStr">
         <is>
-          <t>LUMIN (ЛЮМИН)</t>
+          <t>LUMIN</t>
         </is>
       </c>
       <c r="B7" s="12" t="inlineStr">
@@ -975,7 +975,7 @@
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>Москва, Славянская, 2/5с1</t>
+          <t>Славянская, 2/5с1</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
@@ -1052,7 +1052,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Москва, Уланский, 13С1</t>
+          <t>Уланский, 13С1</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -1111,7 +1111,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="28" customHeight="1">
+    <row r="9" ht="15" customHeight="1">
       <c r="A9" s="11" t="inlineStr">
         <is>
           <t>Современник</t>
@@ -1129,7 +1129,7 @@
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>Москва, Машкова, 13С1</t>
+          <t>Машкова, 13С1</t>
         </is>
       </c>
       <c r="E9" s="12" t="inlineStr">
@@ -1188,7 +1188,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="28" customHeight="1">
+    <row r="10" ht="15" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Репаблик</t>
@@ -1206,7 +1206,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Москва, Пресненский Вал, 27к5</t>
+          <t>Пресненский Вал, 27к5</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -1265,10 +1265,10 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="28" customHeight="1">
+    <row r="11" ht="15" customHeight="1">
       <c r="A11" s="11" t="inlineStr">
         <is>
-          <t>City Park (Сити Парк)</t>
+          <t>City Park</t>
         </is>
       </c>
       <c r="B11" s="12" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>Москва, Мантулинская, 9к4</t>
+          <t>Мантулинская, 9к4</t>
         </is>
       </c>
       <c r="E11" s="12" t="inlineStr">
@@ -1342,7 +1342,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="28" customHeight="1">
+    <row r="12" ht="15" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t>SkyView</t>
@@ -1360,7 +1360,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Москва, Дружинниковская, 15А</t>
+          <t>Дружинниковская, 15А</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -1419,7 +1419,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="28" customHeight="1">
+    <row r="13" ht="15" customHeight="1">
       <c r="A13" s="11" t="inlineStr">
         <is>
           <t>Полянка/44</t>
@@ -1437,7 +1437,7 @@
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>Москва, Большая Полянка, 44</t>
+          <t>Большая Полянка, 44</t>
         </is>
       </c>
       <c r="E13" s="12" t="inlineStr">
@@ -1496,7 +1496,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="28" customHeight="1">
+    <row r="14" ht="15" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Титул на Серебрянической</t>
@@ -1514,7 +1514,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Москва, Серебрянический, 8</t>
+          <t>Серебрянический, 8</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -1576,7 +1576,7 @@
     <row r="15" ht="28" customHeight="1">
       <c r="A15" s="11" t="inlineStr">
         <is>
-          <t>Bogenhouse (Богенхаус)</t>
+          <t>Bogenhouse</t>
         </is>
       </c>
       <c r="B15" s="12" t="inlineStr">
@@ -1591,7 +1591,7 @@
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>Москва, Озерковская, 6</t>
+          <t>Озерковская, 6</t>
         </is>
       </c>
       <c r="E15" s="12" t="inlineStr">
@@ -1650,10 +1650,10 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="28" customHeight="1">
+    <row r="16" ht="15" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Capital Towers (Капитал Тауэрс)</t>
+          <t>Capital Towers</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
@@ -1668,7 +1668,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Москва, Краснопресненская, 14Ак3</t>
+          <t>Краснопресненская, 14Ак3</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -1727,10 +1727,10 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="28" customHeight="1">
+    <row r="17" ht="15" customHeight="1">
       <c r="A17" s="11" t="inlineStr">
         <is>
-          <t>BALCHUG VIEWPOINT (Балчуг Вьюпоинт)</t>
+          <t>BALCHUG VIEWPOINT</t>
         </is>
       </c>
       <c r="B17" s="12" t="inlineStr">
@@ -1745,7 +1745,7 @@
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>Москва, Садовническая, 7</t>
+          <t>Садовническая, 7</t>
         </is>
       </c>
       <c r="E17" s="12" t="inlineStr">
@@ -1822,7 +1822,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Москва, 2-й Хвостов, 8</t>
+          <t>2-й Хвостов, 8</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -1899,7 +1899,7 @@
       </c>
       <c r="D19" s="11" t="inlineStr">
         <is>
-          <t>Москва, Цветной, 32А</t>
+          <t>Цветной, 32А</t>
         </is>
       </c>
       <c r="E19" s="12" t="inlineStr">
@@ -1958,15 +1958,15 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="28" customHeight="1">
+    <row r="20" ht="15" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>A.Residence (А Резиденс)</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>O1 Properties (СЗ А-Резиденс)</t>
+          <t>A.Residence</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>O1 Properties</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
@@ -1976,7 +1976,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Москва, Садовническая, 82</t>
+          <t>Садовническая, 82</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -2035,10 +2035,10 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="28" customHeight="1">
+    <row r="21" ht="15" customHeight="1">
       <c r="A21" s="11" t="inlineStr">
         <is>
-          <t>Roza Rossa (Роза Росса)</t>
+          <t>Roza Rossa</t>
         </is>
       </c>
       <c r="B21" s="12" t="inlineStr">
@@ -2053,7 +2053,7 @@
       </c>
       <c r="D21" s="11" t="inlineStr">
         <is>
-          <t>Москва, Зубовская, 7</t>
+          <t>Зубовская, 7</t>
         </is>
       </c>
       <c r="E21" s="12" t="inlineStr">
@@ -2115,7 +2115,7 @@
     <row r="22" ht="28" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>Собрание клубных домов ORDYNKA (Ордынка)</t>
+          <t>Собрание клубных домов ORDYNKA</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
@@ -2130,7 +2130,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Москва, Большой Ордынский, 4С4</t>
+          <t>Большой Ордынский, 4С4</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -2207,7 +2207,7 @@
       </c>
       <c r="D23" s="11" t="inlineStr">
         <is>
-          <t>Москва, Большой Николоворобинский, 9к1</t>
+          <t>Большой Николоворобинский, 9к1</t>
         </is>
       </c>
       <c r="E23" s="12" t="inlineStr">
@@ -2266,10 +2266,10 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="28" customHeight="1">
+    <row r="24" ht="15" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>Fantastic House (Фантастик Хаус)</t>
+          <t>Fantastic House</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
@@ -2284,7 +2284,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Москва, Большой Тишинский, 30</t>
+          <t>Большой Тишинский, 30</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -2343,7 +2343,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="28" customHeight="1">
+    <row r="25" ht="15" customHeight="1">
       <c r="A25" s="11" t="inlineStr">
         <is>
           <t>Клубный дом Космо 4/22</t>
@@ -2361,7 +2361,7 @@
       </c>
       <c r="D25" s="11" t="inlineStr">
         <is>
-          <t>Москва, Космодамианская, 4/22</t>
+          <t>Космодамианская, 4/22</t>
         </is>
       </c>
       <c r="E25" s="12" t="inlineStr">
@@ -2420,7 +2420,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="28" customHeight="1">
+    <row r="26" ht="15" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
         <is>
           <t>Софийский</t>
@@ -2438,7 +2438,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Москва, Софийская, 34</t>
+          <t>Софийская, 34</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -2515,7 +2515,7 @@
       </c>
       <c r="D27" s="11" t="inlineStr">
         <is>
-          <t>Москва, Средний Тишинский, 5</t>
+          <t>Средний Тишинский, 5</t>
         </is>
       </c>
       <c r="E27" s="12" t="inlineStr">
@@ -2592,7 +2592,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Москва, Тессинский, 1</t>
+          <t>Тессинский, 1</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -2651,10 +2651,10 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="28" customHeight="1">
+    <row r="29" ht="15" customHeight="1">
       <c r="A29" s="11" t="inlineStr">
         <is>
-          <t>Lucky (Лаки)</t>
+          <t>Lucky</t>
         </is>
       </c>
       <c r="B29" s="12" t="inlineStr">
@@ -2669,7 +2669,7 @@
       </c>
       <c r="D29" s="11" t="inlineStr">
         <is>
-          <t>Москва, Костикова, 4к1</t>
+          <t>Костикова, 4к1</t>
         </is>
       </c>
       <c r="E29" s="12" t="inlineStr">
@@ -2731,7 +2731,7 @@
     <row r="30" ht="15" customHeight="1">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>Artisan (Артисан)</t>
+          <t>Artisan</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
@@ -2746,7 +2746,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Москва, Арбат, 39</t>
+          <t>Арбат, 39</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -2805,7 +2805,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="28" customHeight="1">
+    <row r="31" ht="15" customHeight="1">
       <c r="A31" s="11" t="inlineStr">
         <is>
           <t>Абрикосов</t>
@@ -2823,7 +2823,7 @@
       </c>
       <c r="D31" s="11" t="inlineStr">
         <is>
-          <t>Москва, Потаповский, 6С1</t>
+          <t>Потаповский, 6С1</t>
         </is>
       </c>
       <c r="E31" s="12" t="inlineStr">
@@ -2882,10 +2882,10 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="28" customHeight="1">
+    <row r="32" ht="15" customHeight="1">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>Клубный дом CULT (Клубный дом Культ)</t>
+          <t>Клубный дом CULT</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
@@ -2900,7 +2900,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Москва, Ленинский, 2</t>
+          <t>Ленинский, 2</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -2959,10 +2959,10 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="28" customHeight="1">
+    <row r="33" ht="15" customHeight="1">
       <c r="A33" s="11" t="inlineStr">
         <is>
-          <t>SAVVIN RIVER RESIDENCE (Саввин Ривер Резиденс)</t>
+          <t>SAVVIN RIVER RESIDENCE</t>
         </is>
       </c>
       <c r="B33" s="12" t="inlineStr">
@@ -2977,7 +2977,7 @@
       </c>
       <c r="D33" s="11" t="inlineStr">
         <is>
-          <t>Москва, Саввинская, 13</t>
+          <t>Саввинская, 13</t>
         </is>
       </c>
       <c r="E33" s="12" t="inlineStr">
@@ -3054,7 +3054,7 @@
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Москва, Малая Пироговская, 12</t>
+          <t>Малая Пироговская, 12</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -3116,7 +3116,7 @@
     <row r="35" ht="28" customHeight="1">
       <c r="A35" s="11" t="inlineStr">
         <is>
-          <t>Cloud Nine (Клауд Найн)</t>
+          <t>Cloud Nine</t>
         </is>
       </c>
       <c r="B35" s="12" t="inlineStr">
@@ -3131,7 +3131,7 @@
       </c>
       <c r="D35" s="11" t="inlineStr">
         <is>
-          <t>Москва, Большая Полянка, 9С2</t>
+          <t>Большая Полянка, 9С2</t>
         </is>
       </c>
       <c r="E35" s="12" t="inlineStr">
@@ -3208,7 +3208,7 @@
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>Москва, Котельническая, 21</t>
+          <t>Котельническая, 21</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -3267,7 +3267,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="28" customHeight="1">
+    <row r="37" ht="15" customHeight="1">
       <c r="A37" s="11" t="inlineStr">
         <is>
           <t>Садовые кварталы</t>
@@ -3285,7 +3285,7 @@
       </c>
       <c r="D37" s="11" t="inlineStr">
         <is>
-          <t>Москва, Усачева, 15А</t>
+          <t>Усачева, 15А</t>
         </is>
       </c>
       <c r="E37" s="12" t="inlineStr">
@@ -3362,7 +3362,7 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>Москва, Малая Ордынка, 19</t>
+          <t>Малая Ордынка, 19</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
@@ -3439,7 +3439,7 @@
       </c>
       <c r="D39" s="11" t="inlineStr">
         <is>
-          <t>Москва, Газетный, 13с2</t>
+          <t>Газетный, 13с2</t>
         </is>
       </c>
       <c r="E39" s="12" t="inlineStr">
@@ -3498,10 +3498,10 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="28" customHeight="1">
+    <row r="40" ht="15" customHeight="1">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>Zvonarsky Deluxe (Звонарский Делюкс)</t>
+          <t>Zvonarsky Deluxe</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr">
@@ -3516,7 +3516,7 @@
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>Москва, Звонарский, 3</t>
+          <t>Звонарский, 3</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -3575,10 +3575,10 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="28" customHeight="1">
+    <row r="41" ht="15" customHeight="1">
       <c r="A41" s="11" t="inlineStr">
         <is>
-          <t>White Khamovniki (Вайт Хамовники)</t>
+          <t>White Khamovniki</t>
         </is>
       </c>
       <c r="B41" s="12" t="inlineStr">
@@ -3593,7 +3593,7 @@
       </c>
       <c r="D41" s="11" t="inlineStr">
         <is>
-          <t>Москва, Олсуфьевский, 9к1</t>
+          <t>Олсуфьевский, 9к1</t>
         </is>
       </c>
       <c r="E41" s="12" t="inlineStr">
@@ -3652,7 +3652,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="28" customHeight="1">
+    <row r="42" ht="15" customHeight="1">
       <c r="A42" s="4" t="inlineStr">
         <is>
           <t>Золотой, жилой квартал</t>
@@ -3670,7 +3670,7 @@
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Москва, Софийская, 18</t>
+          <t>Софийская, 18</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -3732,7 +3732,7 @@
     <row r="43" ht="28" customHeight="1">
       <c r="A43" s="11" t="inlineStr">
         <is>
-          <t>Magnum (Магнум)</t>
+          <t>Magnum</t>
         </is>
       </c>
       <c r="B43" s="12" t="inlineStr">
@@ -3747,7 +3747,7 @@
       </c>
       <c r="D43" s="11" t="inlineStr">
         <is>
-          <t>Москва, Усачева, 9</t>
+          <t>Усачева, 9</t>
         </is>
       </c>
       <c r="E43" s="12" t="inlineStr">
@@ -3806,7 +3806,7 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="28" customHeight="1">
+    <row r="44" ht="15" customHeight="1">
       <c r="A44" s="4" t="inlineStr">
         <is>
           <t>Дом Бакст на Патриарших</t>
@@ -3824,7 +3824,7 @@
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Москва, Большой Козихинский, 15</t>
+          <t>Большой Козихинский, 15</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
@@ -3883,10 +3883,10 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="28" customHeight="1">
+    <row r="45" ht="15" customHeight="1">
       <c r="A45" s="11" t="inlineStr">
         <is>
-          <t>Villa Grace (Вилла Грейс)</t>
+          <t>Villa Grace</t>
         </is>
       </c>
       <c r="B45" s="12" t="inlineStr">
@@ -3901,7 +3901,7 @@
       </c>
       <c r="D45" s="11" t="inlineStr">
         <is>
-          <t>Москва, Пожарский, 3</t>
+          <t>Пожарский, 3</t>
         </is>
       </c>
       <c r="E45" s="12" t="inlineStr">
@@ -3960,10 +3960,10 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="28" customHeight="1">
+    <row r="46" ht="15" customHeight="1">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>Brodsky (Бродский)</t>
+          <t>Brodsky</t>
         </is>
       </c>
       <c r="B46" s="5" t="inlineStr">
@@ -3978,7 +3978,7 @@
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>Москва, 1-й Тружеников, 16</t>
+          <t>1-й Тружеников, 16</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -4055,7 +4055,7 @@
       </c>
       <c r="D47" s="11" t="inlineStr">
         <is>
-          <t>Москва, Погодинская, 2</t>
+          <t>Погодинская, 2</t>
         </is>
       </c>
       <c r="E47" s="12" t="inlineStr">
@@ -4114,10 +4114,10 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="28" customHeight="1">
+    <row r="48" ht="15" customHeight="1">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>Carré Blanc (Карре Бланк)</t>
+          <t>Carré Blanc</t>
         </is>
       </c>
       <c r="B48" s="5" t="inlineStr">
@@ -4132,7 +4132,7 @@
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>Москва, Пречистенская, 43</t>
+          <t>Пречистенская, 43</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
@@ -4191,7 +4191,7 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="28" customHeight="1">
+    <row r="49" ht="15" customHeight="1">
       <c r="A49" s="11" t="inlineStr">
         <is>
           <t>Дом Лаврушинский</t>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="D49" s="11" t="inlineStr">
         <is>
-          <t>Москва, Большой Толмачевский, 5С1</t>
+          <t>Большой Толмачевский, 5С1</t>
         </is>
       </c>
       <c r="E49" s="12" t="inlineStr">
@@ -4268,7 +4268,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="28" customHeight="1">
+    <row r="50" ht="15" customHeight="1">
       <c r="A50" s="4" t="inlineStr">
         <is>
           <t>Хамовники 12</t>
@@ -4286,7 +4286,7 @@
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>Москва, 1-й Тружеников, 12</t>
+          <t>1-й Тружеников, 12</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
@@ -4345,10 +4345,10 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="40.5" customHeight="1">
+    <row r="51" ht="28" customHeight="1">
       <c r="A51" s="11" t="inlineStr">
         <is>
-          <t>Stella di Mosca Hotel &amp; Residences (Стелла ди Моска Хотел энд Резиденсиз)</t>
+          <t>Stella di Mosca Hotel &amp; Residences</t>
         </is>
       </c>
       <c r="B51" s="11" t="inlineStr">
@@ -4363,7 +4363,7 @@
       </c>
       <c r="D51" s="11" t="inlineStr">
         <is>
-          <t>Москва, Большая Никитская, 9</t>
+          <t>Большая Никитская, 9</t>
         </is>
       </c>
       <c r="E51" s="12" t="inlineStr">
@@ -4422,7 +4422,7 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="28" customHeight="1">
+    <row r="52" ht="15" customHeight="1">
       <c r="A52" s="4" t="inlineStr">
         <is>
           <t>Большая Дмитровка IX</t>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>Москва, Большая Дмитровка, 9А</t>
+          <t>Большая Дмитровка, 9А</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
@@ -4517,7 +4517,7 @@
       </c>
       <c r="D53" s="11" t="inlineStr">
         <is>
-          <t>Москва, Малая Бронная, 15Б</t>
+          <t>Малая Бронная, 15Б</t>
         </is>
       </c>
       <c r="E53" s="12" t="inlineStr">
@@ -4576,10 +4576,10 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="28" customHeight="1">
+    <row r="54" ht="15" customHeight="1">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>Barkli Gallery (Баркли Галлери)</t>
+          <t>Barkli Gallery</t>
         </is>
       </c>
       <c r="B54" s="5" t="inlineStr">
@@ -4594,7 +4594,7 @@
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>Москва, Ордынский, 4А</t>
+          <t>Ордынский, 4А</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
@@ -4747,10 +4747,10 @@
   <dimension ref="A1:P50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
     <col width="6" customWidth="1" min="7" max="7"/>
@@ -4762,7 +4762,7 @@
     <col width="6" customWidth="1" min="13" max="13"/>
     <col width="8" customWidth="1" min="14" max="14"/>
     <col width="7" customWidth="1" min="15" max="15"/>
-    <col width="70" customWidth="1" min="16" max="16"/>
+    <col width="84" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -4879,7 +4879,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Москва, Ленинградский проспект, вл8</t>
+          <t>Ленинградский проспект, вл8</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -4951,7 +4951,7 @@
       </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t>Москва, Краснопресненская набережная</t>
+          <t>Краснопресненская набережная</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
@@ -5005,7 +5005,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="28" customHeight="1">
+    <row r="6" ht="15" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>ЖК «Начало»</t>
@@ -5016,14 +5016,14 @@
           <t>ДОНСТРОЙ</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>2029 (Циан: 2029–2030)</t>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>2029–2030</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Москва, улица Сергея Макеева, 7</t>
+          <t>улица Сергея Макеева, 7</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -5077,7 +5077,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="28" customHeight="1">
+    <row r="7" ht="15" customHeight="1">
       <c r="A7" s="11" t="inlineStr">
         <is>
           <t>Оне</t>
@@ -5095,7 +5095,7 @@
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>Москва, 1-й Красногвардейский, 13</t>
+          <t>1-й Красногвардейский, 13</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
@@ -5149,7 +5149,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="28" customHeight="1">
+    <row r="8" ht="15" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>АУРУС Резиденции</t>
@@ -5237,7 +5237,7 @@
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>Москва, Шлюзовая набережная</t>
+          <t>Шлюзовая набережная</t>
         </is>
       </c>
       <c r="E9" s="12" t="inlineStr">
@@ -5291,7 +5291,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="40.5" customHeight="1">
+    <row r="10" ht="15" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>ЖК «Квартал Life Time»</t>
@@ -5302,14 +5302,14 @@
           <t>Sminex</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>2 кв. 2026 (Циан: 3 кв. 2026)</t>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>3 кв. 2026</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Москва, улица Сергея Макеева</t>
+          <t>улица Сергея Макеева</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -5381,7 +5381,7 @@
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>Москва, Лужнецкая набережная</t>
+          <t>Лужнецкая набережная</t>
         </is>
       </c>
       <c r="E11" s="12" t="inlineStr">
@@ -5453,7 +5453,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Москва, Тессинский, 5С11</t>
+          <t>Тессинский, 5С11</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -5525,7 +5525,7 @@
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>Москва, Софийская, 36</t>
+          <t>Софийская, 36</t>
         </is>
       </c>
       <c r="E13" s="12" t="inlineStr">
@@ -5597,7 +5597,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Москва, Электрический переулок</t>
+          <t>Электрический переулок</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -5651,7 +5651,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="40.5" customHeight="1">
+    <row r="15" ht="28" customHeight="1">
       <c r="A15" s="11" t="inlineStr">
         <is>
           <t>ЖК «Дом Франка»</t>
@@ -5662,14 +5662,14 @@
           <t>Трансстройинвест</t>
         </is>
       </c>
-      <c r="C15" s="11" t="inlineStr">
-        <is>
-          <t>2 кв. 2026 (Циан: 4 кв. 2026)</t>
+      <c r="C15" s="12" t="inlineStr">
+        <is>
+          <t>4 кв. 2026</t>
         </is>
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>Москва, Большой Кисельный переулок, 11</t>
+          <t>Большой Кисельный переулок, 11</t>
         </is>
       </c>
       <c r="E15" s="12" t="inlineStr">
@@ -5723,7 +5723,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="28" customHeight="1">
+    <row r="16" ht="15" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
           <t>ЖК «Татарская 35»</t>
@@ -5741,7 +5741,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Москва, Большая Татарская улица</t>
+          <t>Большая Татарская улица</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -5798,7 +5798,7 @@
     <row r="17" ht="28" customHeight="1">
       <c r="A17" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Клубный дом «Резиденции Воронцова»</t>
+          <t>Клубный дом «Резиденции Воронцова»</t>
         </is>
       </c>
       <c r="B17" s="12" t="inlineStr">
@@ -5813,7 +5813,7 @@
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>Москва, Обуха</t>
+          <t>Обуха</t>
         </is>
       </c>
       <c r="E17" s="12" t="inlineStr">
@@ -5885,7 +5885,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Москва, Машкова улица, 18</t>
+          <t>Машкова улица, 18</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -5939,7 +5939,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="28" customHeight="1">
+    <row r="19" ht="15" customHeight="1">
       <c r="A19" s="11" t="inlineStr">
         <is>
           <t>ЖК «Климашкина 7/11»</t>
@@ -5957,7 +5957,7 @@
       </c>
       <c r="D19" s="11" t="inlineStr">
         <is>
-          <t>Москва, улица Климашкина, 7/11</t>
+          <t>улица Климашкина, 7/11</t>
         </is>
       </c>
       <c r="E19" s="12" t="inlineStr">
@@ -6011,7 +6011,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="40.5" customHeight="1">
+    <row r="20" ht="28" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
           <t>ЖК «Клубный дом Форум»</t>
@@ -6022,14 +6022,14 @@
           <t>MR Group</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>1 кв. 2026 (Циан: 4 кв. 2027)</t>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>4 кв. 2027</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Москва, Садовая-Сухаревская улица, 14</t>
+          <t>Садовая-Сухаревская улица, 14</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -6083,7 +6083,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="28" customHeight="1">
+    <row r="21" ht="15" customHeight="1">
       <c r="A21" s="11" t="inlineStr">
         <is>
           <t>ЖК «Камергер»</t>
@@ -6101,7 +6101,7 @@
       </c>
       <c r="D21" s="11" t="inlineStr">
         <is>
-          <t>Москва, Георгиевский переулок, 1</t>
+          <t>Георгиевский переулок, 1</t>
         </is>
       </c>
       <c r="E21" s="12" t="inlineStr">
@@ -6155,7 +6155,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="28" customHeight="1">
+    <row r="22" ht="15" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Казачий</t>
@@ -6173,7 +6173,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Москва, 1-й Казачий, 10С1</t>
+          <t>1-й Казачий, 10С1</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -6245,7 +6245,7 @@
       </c>
       <c r="D23" s="11" t="inlineStr">
         <is>
-          <t>Москва, Садовническая улица</t>
+          <t>Садовническая улица</t>
         </is>
       </c>
       <c r="E23" s="12" t="inlineStr">
@@ -6299,7 +6299,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="28" customHeight="1">
+    <row r="24" ht="15" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
           <t>Саввинская 17</t>
@@ -6317,7 +6317,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Москва, Саввинская, 17</t>
+          <t>Саввинская, 17</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -6389,7 +6389,7 @@
       </c>
       <c r="D25" s="11" t="inlineStr">
         <is>
-          <t>Москва, Потаповский переулок, 5с4</t>
+          <t>Потаповский переулок, 5с4</t>
         </is>
       </c>
       <c r="E25" s="12" t="inlineStr">
@@ -6443,7 +6443,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="28" customHeight="1">
+    <row r="26" ht="15" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
         <is>
           <t>ЖК «PHANTOM»</t>
@@ -6461,7 +6461,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Москва, Малая Сухаревская площадь</t>
+          <t>Малая Сухаревская площадь</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -6515,10 +6515,10 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="28" customHeight="1">
+    <row r="27" ht="15" customHeight="1">
       <c r="A27" s="11" t="inlineStr">
         <is>
-          <t>Клубный дом TURGENEV (Тургенев)</t>
+          <t>Клубный дом TURGENEV</t>
         </is>
       </c>
       <c r="B27" s="12" t="inlineStr">
@@ -6533,7 +6533,7 @@
       </c>
       <c r="D27" s="11" t="inlineStr">
         <is>
-          <t>Москва, Костянский, 13</t>
+          <t>Костянский, 13</t>
         </is>
       </c>
       <c r="E27" s="12" t="inlineStr">
@@ -6587,7 +6587,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="28" customHeight="1">
+    <row r="28" ht="15" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
         <is>
           <t>Фамильный дом Люче</t>
@@ -6605,7 +6605,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Москва, Крестовоздвиженский, 4</t>
+          <t>Крестовоздвиженский, 4</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -6659,7 +6659,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="28" customHeight="1">
+    <row r="29" ht="15" customHeight="1">
       <c r="A29" s="11" t="inlineStr">
         <is>
           <t>Кло 17</t>
@@ -6677,7 +6677,7 @@
       </c>
       <c r="D29" s="11" t="inlineStr">
         <is>
-          <t>Москва, Староваганьковский, 17С4</t>
+          <t>Староваганьковский, 17С4</t>
         </is>
       </c>
       <c r="E29" s="12" t="inlineStr">
@@ -6749,7 +6749,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Москва, Большой Николоворобинский, 12/11</t>
+          <t>Большой Николоворобинский, 12/11</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -6806,7 +6806,7 @@
     <row r="31" ht="15" customHeight="1">
       <c r="A31" s="11" t="inlineStr">
         <is>
-          <t>Клубный дом DUO (Дуо)</t>
+          <t>Клубный дом DUO</t>
         </is>
       </c>
       <c r="B31" s="12" t="inlineStr">
@@ -6821,7 +6821,7 @@
       </c>
       <c r="D31" s="11" t="inlineStr">
         <is>
-          <t>Москва, Софийская, 34С3</t>
+          <t>Софийская, 34С3</t>
         </is>
       </c>
       <c r="E31" s="12" t="inlineStr">
@@ -6875,7 +6875,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="28" customHeight="1">
+    <row r="32" ht="15" customHeight="1">
       <c r="A32" s="4" t="inlineStr">
         <is>
           <t>Дом Спорта</t>
@@ -6893,7 +6893,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Москва, Дружинниковская, 18</t>
+          <t>Дружинниковская, 18</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -6947,7 +6947,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="40.5" customHeight="1">
+    <row r="33" ht="28" customHeight="1">
       <c r="A33" s="11" t="inlineStr">
         <is>
           <t>«Ильинка 3/8»</t>
@@ -6958,14 +6958,14 @@
           <t>Sminex</t>
         </is>
       </c>
-      <c r="C33" s="11" t="inlineStr">
-        <is>
-          <t>1 кв. 2026 (Циан: 3 кв. 2025)</t>
+      <c r="C33" s="12" t="inlineStr">
+        <is>
+          <t>3 кв. 2025</t>
         </is>
       </c>
       <c r="D33" s="11" t="inlineStr">
         <is>
-          <t>Москва, улица Ильинка</t>
+          <t>улица Ильинка</t>
         </is>
       </c>
       <c r="E33" s="12" t="inlineStr">
@@ -7019,7 +7019,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="28" customHeight="1">
+    <row r="34" ht="15" customHeight="1">
       <c r="A34" s="4" t="inlineStr">
         <is>
           <t>ЖК «Красный Октябрь»</t>
@@ -7037,7 +7037,7 @@
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Москва, Берсеневская набережная</t>
+          <t>Берсеневская набережная</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -7109,7 +7109,7 @@
       </c>
       <c r="D35" s="11" t="inlineStr">
         <is>
-          <t>Москва, Никольская улица, 8/1с1</t>
+          <t>Никольская улица, 8/1с1</t>
         </is>
       </c>
       <c r="E35" s="12" t="inlineStr">
@@ -7163,20 +7163,20 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="40.5" customHeight="1">
+    <row r="36" ht="15" customHeight="1">
       <c r="A36" s="4" t="inlineStr">
         <is>
           <t>MONO Kami</t>
         </is>
       </c>
-      <c r="B36" s="4" t="inlineStr">
-        <is>
-          <t>Tekta Group (ранее ПИК / MONO)</t>
-        </is>
-      </c>
-      <c r="C36" s="4" t="inlineStr">
-        <is>
-          <t>4 кв. 2028 (Циан: 2 кв. 2029)</t>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Tekta Group</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>2 кв. 2029</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
@@ -7235,7 +7235,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="28" customHeight="1">
+    <row r="37" ht="15" customHeight="1">
       <c r="A37" s="11" t="inlineStr">
         <is>
           <t>ЖК «Никитский-6»</t>
@@ -7253,7 +7253,7 @@
       </c>
       <c r="D37" s="11" t="inlineStr">
         <is>
-          <t>Москва, Никитский бульвар, 6/20</t>
+          <t>Никитский бульвар, 6/20</t>
         </is>
       </c>
       <c r="E37" s="12" t="inlineStr">
@@ -7307,7 +7307,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="28" customHeight="1">
+    <row r="38" ht="15" customHeight="1">
       <c r="A38" s="4" t="inlineStr">
         <is>
           <t>ЖК «Фрунзенская набережная»</t>
@@ -7325,7 +7325,7 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>Москва, Фрунзенская набережная, 30</t>
+          <t>Фрунзенская набережная, 30</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
@@ -7379,10 +7379,10 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="28" customHeight="1">
+    <row r="39" ht="15" customHeight="1">
       <c r="A39" s="11" t="inlineStr">
         <is>
-          <t>Kuznetsky Most 12 by Lalique (Кузнецкий Мост 12)</t>
+          <t>Kuznetsky Most 12 by Lalique</t>
         </is>
       </c>
       <c r="B39" s="12" t="inlineStr">
@@ -7397,7 +7397,7 @@
       </c>
       <c r="D39" s="11" t="inlineStr">
         <is>
-          <t>Москва, Кузнецкий Мост, 12/3С1</t>
+          <t>Кузнецкий Мост, 12/3С1</t>
         </is>
       </c>
       <c r="E39" s="12" t="inlineStr">
@@ -7451,7 +7451,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="28" customHeight="1">
+    <row r="40" ht="15" customHeight="1">
       <c r="A40" s="4" t="inlineStr">
         <is>
           <t>Саввинская 27</t>
@@ -7469,7 +7469,7 @@
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>Москва, Саввинская, 27</t>
+          <t>Саввинская, 27</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -7541,7 +7541,7 @@
       </c>
       <c r="D41" s="11" t="inlineStr">
         <is>
-          <t>Москва, Новодевичий, 6С2</t>
+          <t>Новодевичий, 6С2</t>
         </is>
       </c>
       <c r="E41" s="12" t="inlineStr">
@@ -7595,10 +7595,10 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="28" customHeight="1">
+    <row r="42" ht="15" customHeight="1">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>Stoleshnikov 7 (Столешников 7)</t>
+          <t>Stoleshnikov 7</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
@@ -7613,7 +7613,7 @@
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Москва, Столешников, 7С1</t>
+          <t>Столешников, 7С1</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -7667,7 +7667,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="28" customHeight="1">
+    <row r="43" ht="15" customHeight="1">
       <c r="A43" s="11" t="inlineStr">
         <is>
           <t>ЖК «Узоры»</t>
@@ -7685,7 +7685,7 @@
       </c>
       <c r="D43" s="11" t="inlineStr">
         <is>
-          <t>Москва, 2-й Вражский переулок, 8с2</t>
+          <t>2-й Вражский переулок, 8с2</t>
         </is>
       </c>
       <c r="E43" s="12" t="inlineStr">
@@ -7739,7 +7739,7 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="40.5" customHeight="1">
+    <row r="44" ht="15" customHeight="1">
       <c r="A44" s="4" t="inlineStr">
         <is>
           <t>Annabels</t>
@@ -7750,14 +7750,14 @@
           <t>СЗ ЮНИКС</t>
         </is>
       </c>
-      <c r="C44" s="4" t="inlineStr">
-        <is>
-          <t>1 кв. 2026 (Циан: 4 кв. 2026)</t>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>4 кв. 2026</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Москва, Курсовой переулок</t>
+          <t>Курсовой переулок</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
@@ -7829,7 +7829,7 @@
       </c>
       <c r="D45" s="11" t="inlineStr">
         <is>
-          <t>Москва, Трёхпрудный переулок</t>
+          <t>Трёхпрудный переулок</t>
         </is>
       </c>
       <c r="E45" s="12" t="inlineStr">
@@ -7883,10 +7883,10 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="40.5" customHeight="1">
+    <row r="46" ht="28" customHeight="1">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>Armani/Casa Moscow Residences (Армани/Каса Москоу Резиденсес)</t>
+          <t>Armani/Casa Moscow Residences</t>
         </is>
       </c>
       <c r="B46" s="5" t="inlineStr">
@@ -7901,7 +7901,7 @@
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>Москва, Старомонетный, 19/11</t>
+          <t>Старомонетный, 19/11</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -7973,7 +7973,7 @@
       </c>
       <c r="D47" s="11" t="inlineStr">
         <is>
-          <t>Москва, Погодинская улица</t>
+          <t>Погодинская улица</t>
         </is>
       </c>
       <c r="E47" s="12" t="inlineStr">
@@ -8027,7 +8027,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="40.5" customHeight="1">
+    <row r="48" ht="28" customHeight="1">
       <c r="A48" s="4" t="inlineStr">
         <is>
           <t>ЖК «Клубный дом Обыденский №1»</t>
@@ -8038,14 +8038,14 @@
           <t>Sminex</t>
         </is>
       </c>
-      <c r="C48" s="4" t="inlineStr">
-        <is>
-          <t>1 кв. 2026 (Циан: 1 кв. 2030)</t>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>1 кв. 2030</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>Москва, 3-й Обыденский переулок, 1</t>
+          <t>3-й Обыденский переулок, 1</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
@@ -8117,7 +8117,7 @@
       </c>
       <c r="D49" s="11" t="inlineStr">
         <is>
-          <t>Москва, Соймоновский, 3</t>
+          <t>Соймоновский, 3</t>
         </is>
       </c>
       <c r="E49" s="12" t="inlineStr">
@@ -8171,7 +8171,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="40.5" customHeight="1">
+    <row r="50" ht="15" customHeight="1">
       <c r="A50" s="4" t="inlineStr">
         <is>
           <t>ЖК «БРЮСОВ»</t>
@@ -8182,14 +8182,14 @@
           <t>VOSHOD</t>
         </is>
       </c>
-      <c r="C50" s="4" t="inlineStr">
-        <is>
-          <t>2 кв. 2026 (Циан: 4 кв. 2026)</t>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>4 кв. 2026</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>Москва, Брюсов переулок, 2/14с10</t>
+          <t>Брюсов переулок, 2/14с10</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
@@ -8333,22 +8333,22 @@
   <dimension ref="A1:P32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
     <col width="11" customWidth="1" min="12" max="12"/>
     <col width="10" customWidth="1" min="13" max="13"/>
     <col width="10" customWidth="1" min="14" max="14"/>
     <col width="7" customWidth="1" min="15" max="15"/>
-    <col width="70" customWidth="1" min="16" max="16"/>
+    <col width="84" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -8447,7 +8447,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="53" customHeight="1">
+    <row r="4" ht="28" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Лёвшинский, 19</t>
@@ -8475,7 +8475,7 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>продажи открыты, котлован/фундамент (novostroy-m.ru, 2026) — вышел из стадии планирования</t>
+          <t>продажи открыты, котлован/фундамент</t>
         </is>
       </c>
       <c r="G4" s="5" t="n"/>
@@ -8511,7 +8511,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="53" customHeight="1">
+    <row r="5" ht="28" customHeight="1">
       <c r="A5" s="11" t="inlineStr">
         <is>
           <t>Клубный дом «Малая Никитская, 27»</t>
@@ -8519,7 +8519,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>Малая Никитская улица, 27 (два двухэтажных особняка 1861 г., бывший «Клуб 27»)</t>
+          <t>Малая Никитская улица, 27</t>
         </is>
       </c>
       <c r="C5" s="12" t="inlineStr">
@@ -8537,9 +8537,9 @@
           <t>не раскрыт</t>
         </is>
       </c>
-      <c r="F5" s="11" t="inlineStr">
-        <is>
-          <t>проектирование (kvartiravmoskve.ru, 02.03.2026); продажи не открыты, старт не анонсирован</t>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>проектирование</t>
         </is>
       </c>
       <c r="G5" s="12" t="n"/>
@@ -8567,10 +8567,10 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="65.5" customHeight="1">
+    <row r="6" ht="28" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Палашёвский 11 (Большой Палашёвский, 11–13/15)</t>
+          <t>Палашёвский 11</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -8595,7 +8595,7 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>продажи открыты (апрель 2026), стадия котлована (проверено 03.09.2026) — вышел из стадии планирования</t>
+          <t>продажи открыты, стадия котлована</t>
         </is>
       </c>
       <c r="G6" s="7" t="n">
@@ -8639,7 +8639,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="65.5" customHeight="1">
+    <row r="7" ht="28" customHeight="1">
       <c r="A7" s="11" t="inlineStr">
         <is>
           <t>EDEN Private Residence</t>
@@ -8667,7 +8667,7 @@
       </c>
       <c r="F7" s="11" t="inlineStr">
         <is>
-          <t>закрытые продажи (апрель 2026), стадия котлована; публичные продажи не открыты (novostroev.ru, 03.09.2026)</t>
+          <t>закрытые продажи, стадия котлована</t>
         </is>
       </c>
       <c r="G7" s="14" t="n">
@@ -8713,7 +8713,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="65.5" customHeight="1">
+    <row r="8" ht="28" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Большая Ордынка, 25</t>
@@ -8741,7 +8741,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>концепция одобрена ГЗК, подготовка к строительству; старт продаж заявлен на 2026, цены и планировки не опубликованы</t>
+          <t>концепция одобрена ГЗК, подготовка к строительст</t>
         </is>
       </c>
       <c r="G8" s="7" t="n">
@@ -8780,7 +8780,7 @@
     <row r="9" ht="65.5" customHeight="1">
       <c r="A9" s="11" t="inlineStr">
         <is>
-          <t>Большая Пироговская, 51 (общежития Института красной профессуры)</t>
+          <t>Большая Пироговская, 51</t>
         </is>
       </c>
       <c r="B9" s="11" t="inlineStr">
@@ -8805,7 +8805,7 @@
       </c>
       <c r="F9" s="11" t="inlineStr">
         <is>
-          <t>анонсирован (fee-development, июнь 2026), концепция; ГПЗУ получен в начале 2025; реализация не подтверждена</t>
+          <t>анонсирован, концепция</t>
         </is>
       </c>
       <c r="G9" s="14" t="n">
@@ -8837,7 +8837,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="40.5" customHeight="1">
+    <row r="10" ht="15" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Большой Козихинский, 22</t>
@@ -8865,7 +8865,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>проект, продажи не начаты (novostroev.ru, проверено 03.09.2026)</t>
+          <t>проект, продажи не начаты</t>
         </is>
       </c>
       <c r="G10" s="7" t="n">
@@ -8897,7 +8897,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="65.5" customHeight="1">
+    <row r="11" ht="28" customHeight="1">
       <c r="A11" s="11" t="inlineStr">
         <is>
           <t>Воздвиженка 7/6</t>
@@ -8923,9 +8923,9 @@
           <t>АПРИ</t>
         </is>
       </c>
-      <c r="F11" s="11" t="inlineStr">
-        <is>
-          <t>анонсирован; в списке делюкс-стартов 2026–2027 mskdeluxe.ru; параметры не раскрыты, сайт проекта недоступен (08.09.2026)</t>
+      <c r="F11" s="12" t="inlineStr">
+        <is>
+          <t>анонсирован</t>
         </is>
       </c>
       <c r="G11" s="12" t="n"/>
@@ -8951,15 +8951,15 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="65.5" customHeight="1">
+    <row r="12" ht="40.5" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Квартал на Савинской набережной («Московский шёлк»)</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>Савинская наб. (территория БЦ «Московский шёлк»)</t>
+          <t>Квартал на Савинской набережной</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Савинская наб.</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -8977,9 +8977,9 @@
           <t>Sminex</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
-        <is>
-          <t>проектирование (подтверждено Sminex в декабре 2025); начало реализации планировалось на 2026, старт продаж не объявлен</t>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>проектирование</t>
         </is>
       </c>
       <c r="G12" s="7" t="n">
@@ -9011,15 +9011,15 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="53" customHeight="1">
+    <row r="13" ht="28" customHeight="1">
       <c r="A13" s="11" t="inlineStr">
         <is>
-          <t>Клубные дома на Берниковской набережной, 12 (Sminex)</t>
+          <t>Клубные дома на Берниковской набережной, 12</t>
         </is>
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>Берниковская набережная, 12, стр. 1 (здание бывшей школы №1685, 1936 г., арх. А. Машинский)</t>
+          <t>Берниковская набережная, 12, стр. 1</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
@@ -9037,9 +9037,9 @@
           <t>Sminex</t>
         </is>
       </c>
-      <c r="F13" s="11" t="inlineStr">
-        <is>
-          <t>проектирование; площадка подтверждена Sminex 17.03.2026, сроки и старт продаж не объявлены</t>
+      <c r="F13" s="12" t="inlineStr">
+        <is>
+          <t>проектирование</t>
         </is>
       </c>
       <c r="G13" s="14" t="n">
@@ -9075,15 +9075,15 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="65.5" customHeight="1">
+    <row r="14" ht="53" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Клубный дом «Большая Никитская, 16» (R4S)</t>
+          <t>Клубный дом «Большая Никитская, 16»</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Большая Никитская улица, 16 (реконструкция доходного дома, объект культурного наследия)</t>
+          <t>Большая Никитская улица, 16</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
@@ -9103,7 +9103,7 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>проект/реконструкция; продажи не начаты (novostroev.ru, 02.09.2026); заявленный ввод 3 кв. 2026 не подтверждён</t>
+          <t>проект/реконструкция</t>
         </is>
       </c>
       <c r="G14" s="5" t="n"/>
@@ -9141,7 +9141,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="65.5" customHeight="1">
+    <row r="15" ht="28" customHeight="1">
       <c r="A15" s="11" t="inlineStr">
         <is>
           <t>Клубный дом «Земледельческий, 15»</t>
@@ -9149,7 +9149,7 @@
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>Земледельческий переулок, 15 (на месте административного здания 1975 г., 5 этажей, 5 744 м²)</t>
+          <t>Земледельческий переулок, 15</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
@@ -9167,9 +9167,9 @@
           <t>не раскрыт</t>
         </is>
       </c>
-      <c r="F15" s="11" t="inlineStr">
-        <is>
-          <t>проектирование (kvartiravmoskve.ru, 21.06.2026); по адресу действует БЦ; сделок и решений МКА не найдено</t>
+      <c r="F15" s="12" t="inlineStr">
+        <is>
+          <t>проектирование</t>
         </is>
       </c>
       <c r="G15" s="14" t="n">
@@ -9203,10 +9203,10 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="53" customHeight="1">
+    <row r="16" ht="28" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Клубный дом на Курсовом переулке, 15 (проект бюро Дмитрия Великовского)</t>
+          <t>Клубный дом на Курсовом переулке, 15</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
@@ -9229,9 +9229,9 @@
           <t>не раскрыт</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t>проект / предстарт; в открытых источниках только страница агрегатора (08.09.2026)</t>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>проект / предстарт</t>
         </is>
       </c>
       <c r="G16" s="5" t="n"/>
@@ -9255,10 +9255,10 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="53" customHeight="1">
+    <row r="17" ht="28" customHeight="1">
       <c r="A17" s="11" t="inlineStr">
         <is>
-          <t>Льва Толстого, 14–16 (три клубных дома Sminex)</t>
+          <t>Льва Толстого, 14–16</t>
         </is>
       </c>
       <c r="B17" s="11" t="inlineStr">
@@ -9283,7 +9283,7 @@
       </c>
       <c r="F17" s="11" t="inlineStr">
         <is>
-          <t>участок приобретён (декабрь 2025), проектирование; старт продаж не объявлен (08.09.2026)</t>
+          <t>участок приобретён, проектирование</t>
         </is>
       </c>
       <c r="G17" s="14" t="n">
@@ -9313,10 +9313,10 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="53" customHeight="1">
+    <row r="18" ht="28" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>МФК «На Краснопресненской набережной» (Трёхгорная мануфактура)</t>
+          <t>МФК «На Краснопресненской набережной»</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
@@ -9339,9 +9339,9 @@
           <t>ГК Ташир</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr">
-        <is>
-          <t>проект/анонс; сроки реализации и старт продаж не объявлены, предложений нет (сентябрь 2026)</t>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>проект/анонс</t>
         </is>
       </c>
       <c r="G18" s="7" t="n">
@@ -9373,7 +9373,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="40.5" customHeight="1">
+    <row r="19" ht="28" customHeight="1">
       <c r="A19" s="11" t="inlineStr">
         <is>
           <t>Малая Дмитровка, 5/9</t>
@@ -9399,9 +9399,9 @@
           <t>Группа «Эталон»</t>
         </is>
       </c>
-      <c r="F19" s="11" t="inlineStr">
-        <is>
-          <t>предстарт; старт продаж ожидается в 2026 г. (на 08.09.2026 не объявлен)</t>
+      <c r="F19" s="12" t="inlineStr">
+        <is>
+          <t>предстарт</t>
         </is>
       </c>
       <c r="G19" s="14" t="n">
@@ -9433,10 +9433,10 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="53" customHeight="1">
+    <row r="20" ht="28" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Малая Никитская, 29–31 (ожидаемый делюкс-старт)</t>
+          <t>Малая Никитская, 29–31</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
@@ -9461,7 +9461,7 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>в списке ожидаемых стартов делюкс-класса 2026 (mskdeluxe.ru); подробностей нет (08.09.2026)</t>
+          <t>в списке ожидаемых стартов делюкс-класса 2026</t>
         </is>
       </c>
       <c r="G20" s="5" t="n"/>
@@ -9483,7 +9483,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="53" customHeight="1">
+    <row r="21" ht="15" customHeight="1">
       <c r="A21" s="11" t="inlineStr">
         <is>
           <t>Малая Ордынка, 14/1</t>
@@ -9511,7 +9511,7 @@
       </c>
       <c r="F21" s="11" t="inlineStr">
         <is>
-          <t>анонс старта продаж 06.04.2026; по novostroev.ru на 03.09.2026 — проект, продажи не начаты</t>
+          <t>анонс старта продаж 06.04.2026</t>
         </is>
       </c>
       <c r="G21" s="14" t="n">
@@ -9549,7 +9549,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="53" customHeight="1">
+    <row r="22" ht="15" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Олсуфьевский 10</t>
@@ -9575,9 +9575,9 @@
           <t>Грандор</t>
         </is>
       </c>
-      <c r="F22" s="4" t="inlineStr">
-        <is>
-          <t>проект (ГПЗУ апрель 2021); продажи не начаты, «скоро в продаже» (08.09.2026)</t>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>проект</t>
         </is>
       </c>
       <c r="G22" s="5" t="n"/>
@@ -9607,7 +9607,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="53" customHeight="1">
+    <row r="23" ht="28" customHeight="1">
       <c r="A23" s="11" t="inlineStr">
         <is>
           <t>Полянка-3</t>
@@ -9633,9 +9633,9 @@
           <t>Aurix Development</t>
         </is>
       </c>
-      <c r="F23" s="11" t="inlineStr">
-        <is>
-          <t>старт продаж 2026 (по сайту проекта); строительство не начато, цены не опубликованы (08.09.2026)</t>
+      <c r="F23" s="12" t="inlineStr">
+        <is>
+          <t>старт продаж 2026</t>
         </is>
       </c>
       <c r="G23" s="12" t="n"/>
@@ -9665,7 +9665,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="78" customHeight="1">
+    <row r="24" ht="65.5" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
           <t>Премиальный квартал на Лужнецкой набережной, 10А</t>
@@ -9691,9 +9691,9 @@
           <t>Sminex</t>
         </is>
       </c>
-      <c r="F24" s="4" t="inlineStr">
-        <is>
-          <t>проект утверждён (АГР, май 2026); начало строительства 2027, старт продаж ожидается в 2027</t>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>проект утверждён</t>
         </is>
       </c>
       <c r="G24" s="5" t="n"/>
@@ -9727,10 +9727,10 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="65.5" customHeight="1">
+    <row r="25" ht="28" customHeight="1">
       <c r="A25" s="11" t="inlineStr">
         <is>
-          <t>Роден (ранее анонсировался как Veil)</t>
+          <t>Роден</t>
         </is>
       </c>
       <c r="B25" s="11" t="inlineStr">
@@ -9753,9 +9753,9 @@
           <t>MR Group</t>
         </is>
       </c>
-      <c r="F25" s="11" t="inlineStr">
-        <is>
-          <t>проектирование (kvartiravmoskve.ru, 15.07.2026); старт продаж заявлен на июль–август 2026, цены не опубликованы</t>
+      <c r="F25" s="12" t="inlineStr">
+        <is>
+          <t>проектирование</t>
         </is>
       </c>
       <c r="G25" s="12" t="n"/>
@@ -9787,7 +9787,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="65.5" customHeight="1">
+    <row r="26" ht="28" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
         <is>
           <t>Рождественка 8</t>
@@ -9815,7 +9815,7 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>проект дорабатывается под стандарты Sminex; по gdeetotdom.ru — возведение стен; продажи по запросу, старт не объявлен</t>
+          <t>проект дорабатывается под стандарты Sminex</t>
         </is>
       </c>
       <c r="G26" s="7" t="n">
@@ -9853,10 +9853,10 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="53" customHeight="1">
+    <row r="27" ht="28" customHeight="1">
       <c r="A27" s="11" t="inlineStr">
         <is>
-          <t>Тимура Фрунзе, 11 (клубный дом Sminex)</t>
+          <t>Тимура Фрунзе, 11</t>
         </is>
       </c>
       <c r="B27" s="11" t="inlineStr">
@@ -9881,7 +9881,7 @@
       </c>
       <c r="F27" s="11" t="inlineStr">
         <is>
-          <t>участок приобретён (апрель 2026), проектирование; сроки не объявлены (08.09.2026)</t>
+          <t>участок приобретён, проектирование</t>
         </is>
       </c>
       <c r="G27" s="14" t="n">
@@ -9911,15 +9911,15 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="53" customHeight="1">
+    <row r="28" ht="28" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>Типография Сытина (Пятницкая, 71/5)</t>
+          <t>Типография Сытина</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>ул. Пятницкая, 71/5 (2-й Монетчиковский пер., 5)</t>
+          <t>ул. Пятницкая, 71/5</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
@@ -9939,7 +9939,7 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>участок приобретён (март 2026), проектирование; параметры и сроки не раскрыты (08.09.2026)</t>
+          <t>участок приобретён, проектирование</t>
         </is>
       </c>
       <c r="G28" s="5" t="n"/>
@@ -9965,15 +9965,15 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="78" customHeight="1">
+    <row r="29" ht="65.5" customHeight="1">
       <c r="A29" s="11" t="inlineStr">
         <is>
-          <t>Усадьба в Большом Саввинском переулке (клубный дом VSF)</t>
+          <t>Усадьба в Большом Саввинском переулке</t>
         </is>
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>Большой Саввинский пер. (усадьба купца Якунина)</t>
+          <t>Большой Саввинский пер.</t>
         </is>
       </c>
       <c r="C29" s="12" t="inlineStr">
@@ -9993,7 +9993,7 @@
       </c>
       <c r="F29" s="11" t="inlineStr">
         <is>
-          <t>концепция бюро МЛА+ опубликована (январь 2026); сроки строительства не объявлены, реализация именно этой концепции не подтверждена</t>
+          <t>концепция бюро МЛА+ опубликована</t>
         </is>
       </c>
       <c r="G29" s="14" t="n">
@@ -10027,7 +10027,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="53" customHeight="1">
+    <row r="30" ht="15" customHeight="1">
       <c r="A30" s="4" t="inlineStr">
         <is>
           <t>Усачёва, 22</t>
@@ -10055,7 +10055,7 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>проект, продажи не начаты (novostroev.ru, 03.09.2026); старт продаж заявлен на 2026</t>
+          <t>проект, продажи не начаты</t>
         </is>
       </c>
       <c r="G30" s="7" t="n">
@@ -10089,7 +10089,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="65.5" customHeight="1">
+    <row r="31" ht="28" customHeight="1">
       <c r="A31" s="11" t="inlineStr">
         <is>
           <t>Участок КРТ «Большой Тишинский переулок, 8»</t>
@@ -10097,7 +10097,7 @@
       </c>
       <c r="B31" s="11" t="inlineStr">
         <is>
-          <t>Большой Тишинский переулок, 8 (стр. 1, 2)</t>
+          <t>Большой Тишинский переулок, 8</t>
         </is>
       </c>
       <c r="C31" s="12" t="inlineStr">
@@ -10115,9 +10115,9 @@
           <t>не раскрыт</t>
         </is>
       </c>
-      <c r="F31" s="11" t="inlineStr">
-        <is>
-          <t>решение о КРТ (август 2026); оператор/правообладатель и торги в открытых источниках не найдены (проверка 08.09.2026)</t>
+      <c r="F31" s="12" t="inlineStr">
+        <is>
+          <t>решение о КРТ</t>
         </is>
       </c>
       <c r="G31" s="14" t="n">
@@ -10147,10 +10147,10 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="90.5" customHeight="1">
+    <row r="32" ht="28" customHeight="1">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>Хилков (Хилков переулок, вл. 3)</t>
+          <t>Хилков</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
@@ -10175,7 +10175,7 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>статус противоречив: novostroy-m.ru — проект 2016 г. «скоро старт»; novostroev.ru (03.09.2026) — «строительство/продажи завершены»; mskdeluxe.ru — старт 2026–2027</t>
+          <t>статус противоречив: novostroy-m.ru</t>
         </is>
       </c>
       <c r="G32" s="7" t="n">

</xml_diff>

<commit_message>
Workbook: realistic chars-per-column for Cyrillic, taller wrapped rows
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Bv8NELxW2W7udnb3XUFGS2
</commit_message>
<xml_diff>
--- a/docs/premium-cao/premium-zhk-cao.xlsx
+++ b/docs/premium-cao/premium-zhk-cao.xlsx
@@ -607,14 +607,14 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
     <col width="6" customWidth="1" min="7" max="7"/>
     <col width="7" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
@@ -726,7 +726,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1">
+    <row r="4" ht="30" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Резиденция Тверская</t>
@@ -803,7 +803,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="28" customHeight="1">
+    <row r="5" ht="30" customHeight="1">
       <c r="A5" s="11" t="inlineStr">
         <is>
           <t>NEVA TOWERS</t>
@@ -880,7 +880,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1">
+    <row r="6" ht="30" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Sinatra</t>
@@ -957,7 +957,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1">
+    <row r="7" ht="30" customHeight="1">
       <c r="A7" s="11" t="inlineStr">
         <is>
           <t>LUMIN</t>
@@ -1034,7 +1034,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1">
+    <row r="8" ht="30" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Уланский, 13</t>
@@ -1111,7 +1111,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1">
+    <row r="9" ht="30" customHeight="1">
       <c r="A9" s="11" t="inlineStr">
         <is>
           <t>Современник</t>
@@ -1188,7 +1188,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1">
+    <row r="10" ht="30" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Репаблик</t>
@@ -1265,7 +1265,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1">
+    <row r="11" ht="30" customHeight="1">
       <c r="A11" s="11" t="inlineStr">
         <is>
           <t>City Park</t>
@@ -1342,7 +1342,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1">
+    <row r="12" ht="30" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t>SkyView</t>
@@ -1419,7 +1419,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1">
+    <row r="13" ht="30" customHeight="1">
       <c r="A13" s="11" t="inlineStr">
         <is>
           <t>Полянка/44</t>
@@ -1496,7 +1496,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1">
+    <row r="14" ht="30" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Титул на Серебрянической</t>
@@ -1573,7 +1573,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="28" customHeight="1">
+    <row r="15" ht="30" customHeight="1">
       <c r="A15" s="11" t="inlineStr">
         <is>
           <t>Bogenhouse</t>
@@ -1650,7 +1650,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1">
+    <row r="16" ht="30" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Capital Towers</t>
@@ -1727,7 +1727,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="15" customHeight="1">
+    <row r="17" ht="30" customHeight="1">
       <c r="A17" s="11" t="inlineStr">
         <is>
           <t>BALCHUG VIEWPOINT</t>
@@ -1958,7 +1958,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="15" customHeight="1">
+    <row r="20" ht="30" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
           <t>A.Residence</t>
@@ -2035,7 +2035,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1">
+    <row r="21" ht="30" customHeight="1">
       <c r="A21" s="11" t="inlineStr">
         <is>
           <t>Roza Rossa</t>
@@ -2112,7 +2112,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="28" customHeight="1">
+    <row r="22" ht="30" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Собрание клубных домов ORDYNKA</t>
@@ -2189,7 +2189,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="28" customHeight="1">
+    <row r="23" ht="30" customHeight="1">
       <c r="A23" s="11" t="inlineStr">
         <is>
           <t>Дом NV/9</t>
@@ -2343,7 +2343,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="15" customHeight="1">
+    <row r="25" ht="30" customHeight="1">
       <c r="A25" s="11" t="inlineStr">
         <is>
           <t>Клубный дом Космо 4/22</t>
@@ -2420,7 +2420,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="15" customHeight="1">
+    <row r="26" ht="30" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
         <is>
           <t>Софийский</t>
@@ -2651,7 +2651,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="15" customHeight="1">
+    <row r="29" ht="30" customHeight="1">
       <c r="A29" s="11" t="inlineStr">
         <is>
           <t>Lucky</t>
@@ -2805,7 +2805,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="15" customHeight="1">
+    <row r="31" ht="30" customHeight="1">
       <c r="A31" s="11" t="inlineStr">
         <is>
           <t>Абрикосов</t>
@@ -2882,7 +2882,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="15" customHeight="1">
+    <row r="32" ht="30" customHeight="1">
       <c r="A32" s="4" t="inlineStr">
         <is>
           <t>Клубный дом CULT</t>
@@ -3036,7 +3036,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="28" customHeight="1">
+    <row r="34" ht="30" customHeight="1">
       <c r="A34" s="4" t="inlineStr">
         <is>
           <t>Пироговская 14</t>
@@ -3113,7 +3113,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="28" customHeight="1">
+    <row r="35" ht="30" customHeight="1">
       <c r="A35" s="11" t="inlineStr">
         <is>
           <t>Cloud Nine</t>
@@ -3190,7 +3190,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="28" customHeight="1">
+    <row r="36" ht="30" customHeight="1">
       <c r="A36" s="4" t="inlineStr">
         <is>
           <t>Симфония набережных (Котельническая 21)</t>
@@ -3344,7 +3344,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="28" customHeight="1">
+    <row r="38" ht="30" customHeight="1">
       <c r="A38" s="4" t="inlineStr">
         <is>
           <t>Малая Ордынка 19</t>
@@ -3652,7 +3652,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="15" customHeight="1">
+    <row r="42" ht="30" customHeight="1">
       <c r="A42" s="4" t="inlineStr">
         <is>
           <t>Золотой, жилой квартал</t>
@@ -3729,7 +3729,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="28" customHeight="1">
+    <row r="43" ht="30" customHeight="1">
       <c r="A43" s="11" t="inlineStr">
         <is>
           <t>Magnum</t>
@@ -3883,7 +3883,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="15" customHeight="1">
+    <row r="45" ht="30" customHeight="1">
       <c r="A45" s="11" t="inlineStr">
         <is>
           <t>Villa Grace</t>
@@ -3960,7 +3960,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="15" customHeight="1">
+    <row r="46" ht="30" customHeight="1">
       <c r="A46" s="4" t="inlineStr">
         <is>
           <t>Brodsky</t>
@@ -4191,7 +4191,7 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="15" customHeight="1">
+    <row r="49" ht="30" customHeight="1">
       <c r="A49" s="11" t="inlineStr">
         <is>
           <t>Дом Лаврушинский</t>
@@ -4268,7 +4268,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="15" customHeight="1">
+    <row r="50" ht="30" customHeight="1">
       <c r="A50" s="4" t="inlineStr">
         <is>
           <t>Хамовники 12</t>
@@ -4345,7 +4345,7 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="28" customHeight="1">
+    <row r="51" ht="30" customHeight="1">
       <c r="A51" s="11" t="inlineStr">
         <is>
           <t>Stella di Mosca Hotel &amp; Residences</t>
@@ -4422,7 +4422,7 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="15" customHeight="1">
+    <row r="52" ht="30" customHeight="1">
       <c r="A52" s="4" t="inlineStr">
         <is>
           <t>Большая Дмитровка IX</t>
@@ -4748,14 +4748,14 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
     <col width="6" customWidth="1" min="7" max="7"/>
     <col width="7" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
@@ -4861,7 +4861,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="28" customHeight="1">
+    <row r="4" ht="30" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>ЖК «Слава»</t>
@@ -4933,7 +4933,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="28" customHeight="1">
+    <row r="5" ht="30" customHeight="1">
       <c r="A5" s="11" t="inlineStr">
         <is>
           <t>ЖК «Дом Дау»</t>
@@ -5077,7 +5077,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1">
+    <row r="7" ht="30" customHeight="1">
       <c r="A7" s="11" t="inlineStr">
         <is>
           <t>Оне</t>
@@ -5149,7 +5149,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1">
+    <row r="8" ht="30" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>АУРУС Резиденции</t>
@@ -5435,7 +5435,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="28" customHeight="1">
+    <row r="12" ht="30" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Тессинский V</t>
@@ -5507,7 +5507,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="40.5" customHeight="1">
+    <row r="13" ht="43.5" customHeight="1">
       <c r="A13" s="11" t="inlineStr">
         <is>
           <t>Резиденция 1864</t>
@@ -5579,7 +5579,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="28" customHeight="1">
+    <row r="14" ht="30" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
           <t>ЖК «Элитный квартал Тишинский бульвар»</t>
@@ -5651,7 +5651,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="28" customHeight="1">
+    <row r="15" ht="30" customHeight="1">
       <c r="A15" s="11" t="inlineStr">
         <is>
           <t>ЖК «Дом Франка»</t>
@@ -5723,7 +5723,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1">
+    <row r="16" ht="30" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
           <t>ЖК «Татарская 35»</t>
@@ -5795,7 +5795,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="28" customHeight="1">
+    <row r="17" ht="30" customHeight="1">
       <c r="A17" s="11" t="inlineStr">
         <is>
           <t>Клубный дом «Резиденции Воронцова»</t>
@@ -5867,7 +5867,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="28" customHeight="1">
+    <row r="18" ht="30" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
           <t>ЖК «Дом Соболева»</t>
@@ -5939,7 +5939,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="15" customHeight="1">
+    <row r="19" ht="30" customHeight="1">
       <c r="A19" s="11" t="inlineStr">
         <is>
           <t>ЖК «Климашкина 7/11»</t>
@@ -6011,7 +6011,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="28" customHeight="1">
+    <row r="20" ht="30" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
           <t>ЖК «Клубный дом Форум»</t>
@@ -6083,7 +6083,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1">
+    <row r="21" ht="30" customHeight="1">
       <c r="A21" s="11" t="inlineStr">
         <is>
           <t>ЖК «Камергер»</t>
@@ -6155,7 +6155,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="15" customHeight="1">
+    <row r="22" ht="30" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Казачий</t>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="28" customHeight="1">
+    <row r="23" ht="30" customHeight="1">
       <c r="A23" s="11" t="inlineStr">
         <is>
           <t>ЖК «Садовническая 69»</t>
@@ -6299,7 +6299,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="15" customHeight="1">
+    <row r="24" ht="30" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
           <t>Саввинская 17</t>
@@ -6371,7 +6371,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="28" customHeight="1">
+    <row r="25" ht="30" customHeight="1">
       <c r="A25" s="11" t="inlineStr">
         <is>
           <t>ЖК «Исторический дом «Чистые Пруды»</t>
@@ -6443,7 +6443,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="15" customHeight="1">
+    <row r="26" ht="30" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
         <is>
           <t>ЖК «PHANTOM»</t>
@@ -6515,7 +6515,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="15" customHeight="1">
+    <row r="27" ht="30" customHeight="1">
       <c r="A27" s="11" t="inlineStr">
         <is>
           <t>Клубный дом TURGENEV</t>
@@ -6659,7 +6659,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="15" customHeight="1">
+    <row r="29" ht="30" customHeight="1">
       <c r="A29" s="11" t="inlineStr">
         <is>
           <t>Кло 17</t>
@@ -6731,7 +6731,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="28" customHeight="1">
+    <row r="30" ht="30" customHeight="1">
       <c r="A30" s="4" t="inlineStr">
         <is>
           <t>ТИТУЛ Империал</t>
@@ -6875,7 +6875,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="15" customHeight="1">
+    <row r="32" ht="30" customHeight="1">
       <c r="A32" s="4" t="inlineStr">
         <is>
           <t>Дом Спорта</t>
@@ -6947,7 +6947,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="28" customHeight="1">
+    <row r="33" ht="30" customHeight="1">
       <c r="A33" s="11" t="inlineStr">
         <is>
           <t>«Ильинка 3/8»</t>
@@ -7091,7 +7091,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="28" customHeight="1">
+    <row r="35" ht="30" customHeight="1">
       <c r="A35" s="11" t="inlineStr">
         <is>
           <t>ЖК «Николь»</t>
@@ -7307,7 +7307,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="15" customHeight="1">
+    <row r="38" ht="30" customHeight="1">
       <c r="A38" s="4" t="inlineStr">
         <is>
           <t>ЖК «Фрунзенская набережная»</t>
@@ -7379,7 +7379,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="15" customHeight="1">
+    <row r="39" ht="30" customHeight="1">
       <c r="A39" s="11" t="inlineStr">
         <is>
           <t>Kuznetsky Most 12 by Lalique</t>
@@ -7451,7 +7451,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="15" customHeight="1">
+    <row r="40" ht="30" customHeight="1">
       <c r="A40" s="4" t="inlineStr">
         <is>
           <t>Саввинская 27</t>
@@ -7667,7 +7667,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="15" customHeight="1">
+    <row r="43" ht="30" customHeight="1">
       <c r="A43" s="11" t="inlineStr">
         <is>
           <t>ЖК «Узоры»</t>
@@ -7811,7 +7811,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="15" customHeight="1">
+    <row r="45" ht="30" customHeight="1">
       <c r="A45" s="11" t="inlineStr">
         <is>
           <t>ЖК «Клубный дом Левенсон»</t>
@@ -7883,7 +7883,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="28" customHeight="1">
+    <row r="46" ht="30" customHeight="1">
       <c r="A46" s="4" t="inlineStr">
         <is>
           <t>Armani/Casa Moscow Residences</t>
@@ -8027,7 +8027,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="28" customHeight="1">
+    <row r="48" ht="30" customHeight="1">
       <c r="A48" s="4" t="inlineStr">
         <is>
           <t>ЖК «Клубный дом Обыденский №1»</t>
@@ -8171,7 +8171,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="15" customHeight="1">
+    <row r="50" ht="30" customHeight="1">
       <c r="A50" s="4" t="inlineStr">
         <is>
           <t>ЖК «БРЮСОВ»</t>
@@ -8335,8 +8335,8 @@
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="30" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
@@ -8447,7 +8447,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="28" customHeight="1">
+    <row r="4" ht="30" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Лёвшинский, 19</t>
@@ -8511,7 +8511,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="28" customHeight="1">
+    <row r="5" ht="30" customHeight="1">
       <c r="A5" s="11" t="inlineStr">
         <is>
           <t>Клубный дом «Малая Никитская, 27»</t>
@@ -8567,7 +8567,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="28" customHeight="1">
+    <row r="6" ht="30" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Палашёвский 11</t>
@@ -8639,7 +8639,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="28" customHeight="1">
+    <row r="7" ht="30" customHeight="1">
       <c r="A7" s="11" t="inlineStr">
         <is>
           <t>EDEN Private Residence</t>
@@ -8713,7 +8713,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="28" customHeight="1">
+    <row r="8" ht="30" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Большая Ордынка, 25</t>
@@ -8777,7 +8777,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="65.5" customHeight="1">
+    <row r="9" ht="70.5" customHeight="1">
       <c r="A9" s="11" t="inlineStr">
         <is>
           <t>Большая Пироговская, 51</t>
@@ -8837,7 +8837,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1">
+    <row r="10" ht="30" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Большой Козихинский, 22</t>
@@ -8897,7 +8897,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="28" customHeight="1">
+    <row r="11" ht="30" customHeight="1">
       <c r="A11" s="11" t="inlineStr">
         <is>
           <t>Воздвиженка 7/6</t>
@@ -8951,7 +8951,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="40.5" customHeight="1">
+    <row r="12" ht="57" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Квартал на Савинской набережной</t>
@@ -9011,7 +9011,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="28" customHeight="1">
+    <row r="13" ht="43.5" customHeight="1">
       <c r="A13" s="11" t="inlineStr">
         <is>
           <t>Клубные дома на Берниковской набережной, 12</t>
@@ -9075,7 +9075,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="53" customHeight="1">
+    <row r="14" ht="70.5" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Клубный дом «Большая Никитская, 16»</t>
@@ -9141,7 +9141,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="28" customHeight="1">
+    <row r="15" ht="30" customHeight="1">
       <c r="A15" s="11" t="inlineStr">
         <is>
           <t>Клубный дом «Земледельческий, 15»</t>
@@ -9203,7 +9203,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="28" customHeight="1">
+    <row r="16" ht="30" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Клубный дом на Курсовом переулке, 15</t>
@@ -9255,7 +9255,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="28" customHeight="1">
+    <row r="17" ht="30" customHeight="1">
       <c r="A17" s="11" t="inlineStr">
         <is>
           <t>Льва Толстого, 14–16</t>
@@ -9313,7 +9313,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="28" customHeight="1">
+    <row r="18" ht="30" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
           <t>МФК «На Краснопресненской набережной»</t>
@@ -9373,7 +9373,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="28" customHeight="1">
+    <row r="19" ht="30" customHeight="1">
       <c r="A19" s="11" t="inlineStr">
         <is>
           <t>Малая Дмитровка, 5/9</t>
@@ -9433,7 +9433,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="28" customHeight="1">
+    <row r="20" ht="30" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Малая Никитская, 29–31</t>
@@ -9483,7 +9483,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1">
+    <row r="21" ht="30" customHeight="1">
       <c r="A21" s="11" t="inlineStr">
         <is>
           <t>Малая Ордынка, 14/1</t>
@@ -9549,7 +9549,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="15" customHeight="1">
+    <row r="22" ht="30" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Олсуфьевский 10</t>
@@ -9607,7 +9607,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="28" customHeight="1">
+    <row r="23" ht="30" customHeight="1">
       <c r="A23" s="11" t="inlineStr">
         <is>
           <t>Полянка-3</t>
@@ -9665,7 +9665,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="65.5" customHeight="1">
+    <row r="24" ht="84" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
           <t>Премиальный квартал на Лужнецкой набережной, 10А</t>
@@ -9727,7 +9727,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="28" customHeight="1">
+    <row r="25" ht="30" customHeight="1">
       <c r="A25" s="11" t="inlineStr">
         <is>
           <t>Роден</t>
@@ -9787,7 +9787,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="28" customHeight="1">
+    <row r="26" ht="43.5" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
         <is>
           <t>Рождественка 8</t>
@@ -9853,7 +9853,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="28" customHeight="1">
+    <row r="27" ht="30" customHeight="1">
       <c r="A27" s="11" t="inlineStr">
         <is>
           <t>Тимура Фрунзе, 11</t>
@@ -9911,7 +9911,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="28" customHeight="1">
+    <row r="28" ht="30" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
         <is>
           <t>Типография Сытина</t>
@@ -9965,7 +9965,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="65.5" customHeight="1">
+    <row r="29" ht="84" customHeight="1">
       <c r="A29" s="11" t="inlineStr">
         <is>
           <t>Усадьба в Большом Саввинском переулке</t>
@@ -10027,7 +10027,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="15" customHeight="1">
+    <row r="30" ht="30" customHeight="1">
       <c r="A30" s="4" t="inlineStr">
         <is>
           <t>Усачёва, 22</t>
@@ -10089,7 +10089,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="28" customHeight="1">
+    <row r="31" ht="30" customHeight="1">
       <c r="A31" s="11" t="inlineStr">
         <is>
           <t>Участок КРТ «Большой Тишинский переулок, 8»</t>
@@ -10147,7 +10147,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="28" customHeight="1">
+    <row r="32" ht="30" customHeight="1">
       <c r="A32" s="4" t="inlineStr">
         <is>
           <t>Хилков</t>

</xml_diff>

<commit_message>
Workbook: wider notes column so most descriptions stay on one line
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Bv8NELxW2W7udnb3XUFGS2
</commit_message>
<xml_diff>
--- a/docs/premium-cao/premium-zhk-cao.xlsx
+++ b/docs/premium-cao/premium-zhk-cao.xlsx
@@ -622,7 +622,7 @@
     <col width="9" customWidth="1" min="14" max="14"/>
     <col width="10" customWidth="1" min="15" max="15"/>
     <col width="7" customWidth="1" min="16" max="16"/>
-    <col width="84" customWidth="1" min="17" max="17"/>
+    <col width="90" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -726,7 +726,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="30" customHeight="1">
+    <row r="4" ht="15" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Резиденция Тверская</t>
@@ -880,7 +880,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="30" customHeight="1">
+    <row r="6" ht="15" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Sinatra</t>
@@ -957,7 +957,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="30" customHeight="1">
+    <row r="7" ht="15" customHeight="1">
       <c r="A7" s="11" t="inlineStr">
         <is>
           <t>LUMIN</t>
@@ -1111,7 +1111,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="30" customHeight="1">
+    <row r="9" ht="15" customHeight="1">
       <c r="A9" s="11" t="inlineStr">
         <is>
           <t>Современник</t>
@@ -1265,7 +1265,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="30" customHeight="1">
+    <row r="11" ht="15" customHeight="1">
       <c r="A11" s="11" t="inlineStr">
         <is>
           <t>City Park</t>
@@ -1727,7 +1727,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="30" customHeight="1">
+    <row r="17" ht="15" customHeight="1">
       <c r="A17" s="11" t="inlineStr">
         <is>
           <t>BALCHUG VIEWPOINT</t>
@@ -2035,7 +2035,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="30" customHeight="1">
+    <row r="21" ht="15" customHeight="1">
       <c r="A21" s="11" t="inlineStr">
         <is>
           <t>Roza Rossa</t>
@@ -2420,7 +2420,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="30" customHeight="1">
+    <row r="26" ht="15" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
         <is>
           <t>Софийский</t>
@@ -2805,7 +2805,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="30" customHeight="1">
+    <row r="31" ht="15" customHeight="1">
       <c r="A31" s="11" t="inlineStr">
         <is>
           <t>Абрикосов</t>
@@ -2882,7 +2882,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="30" customHeight="1">
+    <row r="32" ht="15" customHeight="1">
       <c r="A32" s="4" t="inlineStr">
         <is>
           <t>Клубный дом CULT</t>
@@ -3883,7 +3883,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="30" customHeight="1">
+    <row r="45" ht="15" customHeight="1">
       <c r="A45" s="11" t="inlineStr">
         <is>
           <t>Villa Grace</t>
@@ -3960,7 +3960,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="30" customHeight="1">
+    <row r="46" ht="15" customHeight="1">
       <c r="A46" s="4" t="inlineStr">
         <is>
           <t>Brodsky</t>
@@ -4268,7 +4268,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="30" customHeight="1">
+    <row r="50" ht="15" customHeight="1">
       <c r="A50" s="4" t="inlineStr">
         <is>
           <t>Хамовники 12</t>
@@ -4762,7 +4762,7 @@
     <col width="6" customWidth="1" min="13" max="13"/>
     <col width="8" customWidth="1" min="14" max="14"/>
     <col width="7" customWidth="1" min="15" max="15"/>
-    <col width="84" customWidth="1" min="16" max="16"/>
+    <col width="90" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -5723,7 +5723,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="30" customHeight="1">
+    <row r="16" ht="15" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
           <t>ЖК «Татарская 35»</t>
@@ -5939,7 +5939,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="30" customHeight="1">
+    <row r="19" ht="15" customHeight="1">
       <c r="A19" s="11" t="inlineStr">
         <is>
           <t>ЖК «Климашкина 7/11»</t>
@@ -6155,7 +6155,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="30" customHeight="1">
+    <row r="22" ht="15" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Казачий</t>
@@ -6299,7 +6299,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="30" customHeight="1">
+    <row r="24" ht="15" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
           <t>Саввинская 17</t>
@@ -6515,7 +6515,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="30" customHeight="1">
+    <row r="27" ht="15" customHeight="1">
       <c r="A27" s="11" t="inlineStr">
         <is>
           <t>Клубный дом TURGENEV</t>
@@ -6875,7 +6875,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="30" customHeight="1">
+    <row r="32" ht="15" customHeight="1">
       <c r="A32" s="4" t="inlineStr">
         <is>
           <t>Дом Спорта</t>
@@ -7451,7 +7451,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="30" customHeight="1">
+    <row r="40" ht="15" customHeight="1">
       <c r="A40" s="4" t="inlineStr">
         <is>
           <t>Саввинская 27</t>
@@ -8348,7 +8348,7 @@
     <col width="10" customWidth="1" min="13" max="13"/>
     <col width="10" customWidth="1" min="14" max="14"/>
     <col width="7" customWidth="1" min="15" max="15"/>
-    <col width="84" customWidth="1" min="16" max="16"/>
+    <col width="90" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -9549,7 +9549,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="30" customHeight="1">
+    <row r="22" ht="15" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Олсуфьевский 10</t>

</xml_diff>

<commit_message>
Workbook: widen year/address/date columns
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Bv8NELxW2W7udnb3XUFGS2
</commit_message>
<xml_diff>
--- a/docs/premium-cao/premium-zhk-cao.xlsx
+++ b/docs/premium-cao/premium-zhk-cao.xlsx
@@ -608,8 +608,8 @@
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="6" customWidth="1" min="7" max="7"/>
@@ -1188,7 +1188,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="30" customHeight="1">
+    <row r="10" ht="15" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Репаблик</t>
@@ -1342,7 +1342,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="30" customHeight="1">
+    <row r="12" ht="15" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t>SkyView</t>
@@ -1419,7 +1419,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="30" customHeight="1">
+    <row r="13" ht="15" customHeight="1">
       <c r="A13" s="11" t="inlineStr">
         <is>
           <t>Полянка/44</t>
@@ -1650,7 +1650,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="30" customHeight="1">
+    <row r="16" ht="15" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Capital Towers</t>
@@ -1958,7 +1958,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="30" customHeight="1">
+    <row r="20" ht="15" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
           <t>A.Residence</t>
@@ -2343,7 +2343,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="30" customHeight="1">
+    <row r="25" ht="15" customHeight="1">
       <c r="A25" s="11" t="inlineStr">
         <is>
           <t>Клубный дом Космо 4/22</t>
@@ -2651,7 +2651,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="30" customHeight="1">
+    <row r="29" ht="15" customHeight="1">
       <c r="A29" s="11" t="inlineStr">
         <is>
           <t>Lucky</t>
@@ -3652,7 +3652,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="30" customHeight="1">
+    <row r="42" ht="15" customHeight="1">
       <c r="A42" s="4" t="inlineStr">
         <is>
           <t>Золотой, жилой квартал</t>
@@ -4191,7 +4191,7 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="30" customHeight="1">
+    <row r="49" ht="15" customHeight="1">
       <c r="A49" s="11" t="inlineStr">
         <is>
           <t>Дом Лаврушинский</t>
@@ -4422,7 +4422,7 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="30" customHeight="1">
+    <row r="52" ht="15" customHeight="1">
       <c r="A52" s="4" t="inlineStr">
         <is>
           <t>Большая Дмитровка IX</t>
@@ -4749,8 +4749,8 @@
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="6" customWidth="1" min="7" max="7"/>
@@ -5077,7 +5077,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="30" customHeight="1">
+    <row r="7" ht="15" customHeight="1">
       <c r="A7" s="11" t="inlineStr">
         <is>
           <t>Оне</t>
@@ -6443,7 +6443,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="30" customHeight="1">
+    <row r="26" ht="15" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
         <is>
           <t>ЖК «PHANTOM»</t>
@@ -6659,7 +6659,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="30" customHeight="1">
+    <row r="29" ht="15" customHeight="1">
       <c r="A29" s="11" t="inlineStr">
         <is>
           <t>Кло 17</t>
@@ -8171,7 +8171,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="30" customHeight="1">
+    <row r="50" ht="15" customHeight="1">
       <c r="A50" s="4" t="inlineStr">
         <is>
           <t>ЖК «БРЮСОВ»</t>
@@ -8334,7 +8334,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
@@ -8344,9 +8344,9 @@
     <col width="9" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
     <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
     <col width="7" customWidth="1" min="15" max="15"/>
     <col width="90" customWidth="1" min="16" max="16"/>
   </cols>

</xml_diff>